<commit_message>
QQQ exp 103 CatBoost depth=6 -0.87 DISCARD (depth=4 baseline confirmed)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>105</row>
+      <row>106</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T103"/>
+  <dimension ref="A1:T104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7361,7 +7361,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.02 n_est=2000 - combine best CatBoost findings (lr from exp 98, capacity fro</t>
+          <t>CatBoost depth=6 lr=0.01 n_est=1000 - depth axis test</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7379,51 +7379,51 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>-0.8764</v>
+        <v>-0.8688</v>
       </c>
       <c r="F79" t="n">
-        <v>-0.1626</v>
+        <v>0.7087</v>
       </c>
       <c r="G79" t="n">
-        <v>-0.4764</v>
+        <v>-0.6688</v>
       </c>
       <c r="I79" t="n">
-        <v>-23.11</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="J79" t="n">
-        <v>768.9</v>
+        <v>1767.6</v>
       </c>
       <c r="K79" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L79" t="n">
         <v>1</v>
       </c>
       <c r="N79" t="n">
-        <v>0.0008</v>
+        <v>0.0031</v>
       </c>
       <c r="O79" t="n">
-        <v>46.43</v>
+        <v>49.34</v>
       </c>
       <c r="P79" t="n">
-        <v>0.5760999999999999</v>
+        <v>0.5827</v>
       </c>
       <c r="Q79" t="n">
-        <v>0.3655</v>
+        <v>0.5127</v>
       </c>
       <c r="R79" t="n">
-        <v>0.4472</v>
+        <v>0.5455</v>
       </c>
       <c r="S79" t="n">
-        <v>-0.0257</v>
+        <v>-0.0203</v>
       </c>
       <c r="T79" t="n">
-        <v>2594.9</v>
+        <v>4289.1</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -7432,7 +7432,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
+          <t>CatBoost lr=0.02 n_est=2000 - combine best CatBoost findings (lr from exp 98, capacity fro</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7441,60 +7441,60 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>-0.9217</v>
+        <v>-0.8764</v>
       </c>
       <c r="F80" t="n">
-        <v>0.5942</v>
+        <v>-0.1626</v>
       </c>
       <c r="G80" t="n">
-        <v>-0.7217</v>
+        <v>-0.4764</v>
       </c>
       <c r="I80" t="n">
-        <v>58.5</v>
+        <v>-23.11</v>
       </c>
       <c r="J80" t="n">
-        <v>1585</v>
+        <v>768.9</v>
       </c>
       <c r="K80" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N80" t="n">
-        <v>0.019</v>
+        <v>0.0008</v>
       </c>
       <c r="O80" t="n">
-        <v>48.5</v>
+        <v>46.43</v>
       </c>
       <c r="P80" t="n">
-        <v>0.5986</v>
+        <v>0.5760999999999999</v>
       </c>
       <c r="Q80" t="n">
-        <v>0.3987</v>
+        <v>0.3655</v>
       </c>
       <c r="R80" t="n">
-        <v>0.4786</v>
+        <v>0.4472</v>
       </c>
       <c r="S80" t="n">
-        <v>0.0103</v>
+        <v>-0.0257</v>
       </c>
       <c r="T80" t="n">
-        <v>18919.4</v>
+        <v>2594.9</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
+          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -7503,51 +7503,51 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="F81" t="n">
-        <v>-0.2367</v>
+        <v>0.5942</v>
       </c>
       <c r="G81" t="n">
-        <v>-0.5226</v>
+        <v>-0.7217</v>
       </c>
       <c r="I81" t="n">
-        <v>-43.21</v>
+        <v>58.5</v>
       </c>
       <c r="J81" t="n">
-        <v>567.9000000000001</v>
+        <v>1585</v>
       </c>
       <c r="K81" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N81" t="n">
-        <v>-0.0164</v>
+        <v>0.019</v>
       </c>
       <c r="O81" t="n">
-        <v>45.63</v>
+        <v>48.5</v>
       </c>
       <c r="P81" t="n">
-        <v>0.5938</v>
+        <v>0.5986</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.1648</v>
+        <v>0.3987</v>
       </c>
       <c r="R81" t="n">
-        <v>0.258</v>
+        <v>0.4786</v>
       </c>
       <c r="S81" t="n">
-        <v>0.0188</v>
+        <v>0.0103</v>
       </c>
       <c r="T81" t="n">
-        <v>33.8</v>
+        <v>18919.4</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7565,60 +7565,60 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="F82" t="n">
-        <v>0.1045</v>
+        <v>-0.2367</v>
       </c>
       <c r="G82" t="n">
-        <v>-0.6746</v>
+        <v>-0.5226</v>
       </c>
       <c r="I82" t="n">
-        <v>-4.63</v>
+        <v>-43.21</v>
       </c>
       <c r="J82" t="n">
-        <v>953.7</v>
+        <v>567.9000000000001</v>
       </c>
       <c r="K82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N82" t="n">
-        <v>-0.0374</v>
+        <v>-0.0164</v>
       </c>
       <c r="O82" t="n">
-        <v>51.03</v>
+        <v>45.63</v>
       </c>
       <c r="P82" t="n">
-        <v>0.5765</v>
+        <v>0.5938</v>
       </c>
       <c r="Q82" t="n">
-        <v>0.5415</v>
+        <v>0.1648</v>
       </c>
       <c r="R82" t="n">
-        <v>0.5585</v>
+        <v>0.258</v>
       </c>
       <c r="S82" t="n">
-        <v>0.0091</v>
+        <v>0.0188</v>
       </c>
       <c r="T82" t="n">
-        <v>30.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7627,60 +7627,60 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="F83" t="n">
-        <v>0.8788</v>
+        <v>0.1045</v>
       </c>
       <c r="G83" t="n">
-        <v>-0.866</v>
+        <v>-0.6746</v>
       </c>
       <c r="I83" t="n">
-        <v>107.82</v>
+        <v>-4.63</v>
       </c>
       <c r="J83" t="n">
-        <v>2078.2</v>
+        <v>953.7</v>
       </c>
       <c r="K83" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L83" t="n">
         <v>2</v>
       </c>
       <c r="N83" t="n">
-        <v>0.0329</v>
+        <v>-0.0374</v>
       </c>
       <c r="O83" t="n">
-        <v>54.14</v>
+        <v>51.03</v>
       </c>
       <c r="P83" t="n">
-        <v>0.6011</v>
+        <v>0.5765</v>
       </c>
       <c r="Q83" t="n">
-        <v>0.6725</v>
+        <v>0.5415</v>
       </c>
       <c r="R83" t="n">
-        <v>0.6348</v>
+        <v>0.5585</v>
       </c>
       <c r="S83" t="n">
-        <v>0.0251</v>
+        <v>0.0091</v>
       </c>
       <c r="T83" t="n">
-        <v>75.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -7689,51 +7689,51 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F84" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G84" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I84" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J84" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K84" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L84" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N84" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O84" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P84" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q84" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R84" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S84" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T84" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -7742,7 +7742,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -7751,60 +7751,60 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F85" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G85" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I85" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J85" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N85" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O85" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P85" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q85" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R85" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S85" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T85" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7813,60 +7813,60 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F86" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G86" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I86" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J86" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K86" t="n">
         <v>2</v>
       </c>
       <c r="L86" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N86" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O86" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P86" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q86" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R86" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S86" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T86" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7875,60 +7875,60 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F87" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G87" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I87" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J87" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K87" t="n">
+        <v>2</v>
+      </c>
+      <c r="L87" t="n">
         <v>5</v>
       </c>
-      <c r="L87" t="n">
-        <v>2</v>
-      </c>
       <c r="N87" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O87" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P87" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q87" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R87" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S87" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T87" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -7937,60 +7937,60 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F88" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G88" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I88" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J88" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K88" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L88" t="n">
         <v>2</v>
       </c>
       <c r="N88" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O88" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P88" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q88" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R88" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S88" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T88" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -7999,51 +7999,51 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F89" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G89" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I89" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J89" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L89" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N89" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O89" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P89" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q89" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R89" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S89" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T89" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -8052,7 +8052,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -8061,51 +8061,51 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F90" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G90" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I90" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J90" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K90" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L90" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N90" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O90" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P90" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q90" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R90" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S90" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T90" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8123,60 +8123,60 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F91" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G91" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I91" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J91" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K91" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L91" t="n">
         <v>2</v>
       </c>
       <c r="N91" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O91" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P91" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q91" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R91" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S91" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T91" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8185,60 +8185,60 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F92" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G92" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I92" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J92" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K92" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L92" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N92" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O92" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P92" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q92" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R92" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S92" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T92" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8247,60 +8247,60 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>-1.4347</v>
+        <v>-1.3564</v>
       </c>
       <c r="F93" t="n">
-        <v>-0.6758999999999999</v>
+        <v>0.011</v>
       </c>
       <c r="G93" t="n">
-        <v>-0.8347</v>
+        <v>-0.9564</v>
       </c>
       <c r="I93" t="n">
-        <v>-70.84999999999999</v>
+        <v>-17.26</v>
       </c>
       <c r="J93" t="n">
-        <v>291.5000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K93" t="n">
+        <v>3</v>
+      </c>
+      <c r="L93" t="n">
         <v>1</v>
       </c>
-      <c r="L93" t="n">
-        <v>2</v>
-      </c>
       <c r="N93" t="n">
-        <v>0.0284</v>
+        <v>-0.0003</v>
       </c>
       <c r="O93" t="n">
-        <v>44.07</v>
+        <v>48.19</v>
       </c>
       <c r="P93" t="n">
-        <v>0.5588</v>
+        <v>0.5666</v>
       </c>
       <c r="Q93" t="n">
-        <v>0.1177</v>
+        <v>0.4114</v>
       </c>
       <c r="R93" t="n">
-        <v>0.1945</v>
+        <v>0.4767</v>
       </c>
       <c r="S93" t="n">
-        <v>-0.0101</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T93" t="n">
-        <v>79.8</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8309,39 +8309,51 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F94" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G94" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I94" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J94" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K94" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L94" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N94" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O94" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P94" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R94" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S94" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T94" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -8350,7 +8362,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -8359,51 +8371,39 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F95" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G95" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I95" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J95" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K95" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L95" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N95" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O95" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P95" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q95" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R95" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S95" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T95" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -8412,7 +8412,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8421,51 +8421,51 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F96" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G96" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I96" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J96" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L96" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N96" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O96" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P96" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q96" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R96" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S96" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T96" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -8474,7 +8474,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8483,113 +8483,113 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F97" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G97" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I97" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J97" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K97" t="n">
         <v>1</v>
       </c>
       <c r="L97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N97" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O97" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P97" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q97" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R97" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S97" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T97" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
+        <v>59</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F98" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G98" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I98" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J98" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K98" t="n">
         <v>1</v>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E98" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F98" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G98" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I98" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J98" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K98" t="n">
-        <v>5</v>
       </c>
       <c r="L98" t="n">
         <v>1</v>
       </c>
       <c r="N98" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O98" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P98" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R98" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S98" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T98" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -8598,12 +8598,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E99" t="n">
@@ -8646,21 +8646,21 @@
         <v>0.0098</v>
       </c>
       <c r="T99" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8669,19 +8669,19 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F100" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G100" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I100" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J100" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K100" t="n">
         <v>5</v>
@@ -8690,39 +8690,39 @@
         <v>1</v>
       </c>
       <c r="N100" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O100" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P100" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q100" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R100" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S100" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T100" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8731,113 +8731,113 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F101" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G101" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I101" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J101" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K101" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L101" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N101" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O101" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P101" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q101" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R101" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S101" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T101" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
+        <v>22</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F102" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G102" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I102" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J102" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K102" t="n">
+        <v>4</v>
+      </c>
+      <c r="L102" t="n">
         <v>2</v>
       </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E102" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F102" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G102" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I102" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J102" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K102" t="n">
-        <v>5</v>
-      </c>
-      <c r="L102" t="n">
-        <v>1</v>
-      </c>
       <c r="N102" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O102" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P102" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q102" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R102" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S102" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T102" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8846,7 +8846,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8855,51 +8855,113 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F103" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G103" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I103" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J103" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K103" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L103" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N103" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O103" t="n">
         <v>47.65</v>
       </c>
       <c r="P103" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R103" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S103" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T103" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>41</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F104" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G104" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I104" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J104" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K104" t="n">
+        <v>4</v>
+      </c>
+      <c r="L104" t="n">
+        <v>2</v>
+      </c>
+      <c r="N104" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O104" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P104" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q103" t="n">
+      <c r="Q104" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R103" t="n">
+      <c r="R104" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S103" t="n">
+      <c r="S104" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T103" t="n">
+      <c r="T104" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T103"/>
-  <conditionalFormatting sqref="E2:E103">
+  <autoFilter ref="A1:T104"/>
+  <conditionalFormatting sqref="E2:E104">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -8921,7 +8983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K103"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11845,7 +11907,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -11853,36 +11915,36 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>-0.8764</v>
+        <v>-0.8688</v>
       </c>
       <c r="D79" t="n">
         <v>1000</v>
       </c>
       <c r="E79" t="n">
-        <v>762</v>
+        <v>1120</v>
       </c>
       <c r="F79" t="n">
-        <v>937.8695999999999</v>
+        <v>1237.6</v>
       </c>
       <c r="G79" t="n">
-        <v>946.9669351199999</v>
+        <v>1385.61696</v>
       </c>
       <c r="H79" t="n">
-        <v>929.2586534332559</v>
+        <v>1253.429102016</v>
       </c>
       <c r="I79" t="n">
-        <v>802.1360696435864</v>
+        <v>1143.378026858995</v>
       </c>
       <c r="J79" t="n">
-        <v>902.5635055629634</v>
+        <v>1478.502126531366</v>
       </c>
       <c r="K79" t="n">
-        <v>768.8035940385322</v>
+        <v>1767.549292268249</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
@@ -11890,73 +11952,73 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>-0.9217</v>
+        <v>-0.8764</v>
       </c>
       <c r="D80" t="n">
         <v>1000</v>
       </c>
       <c r="E80" t="n">
-        <v>1206.3</v>
+        <v>762</v>
       </c>
       <c r="F80" t="n">
-        <v>1403.65068</v>
+        <v>937.8695999999999</v>
       </c>
       <c r="G80" t="n">
-        <v>1572.930952008</v>
+        <v>946.9669351199999</v>
       </c>
       <c r="H80" t="n">
-        <v>1622.320983901051</v>
+        <v>929.2586534332559</v>
       </c>
       <c r="I80" t="n">
-        <v>1560.023858119251</v>
+        <v>802.1360696435864</v>
       </c>
       <c r="J80" t="n">
-        <v>2085.595895919627</v>
+        <v>902.5635055629634</v>
       </c>
       <c r="K80" t="n">
-        <v>1584.844321309324</v>
+        <v>768.8035940385322</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="D81" t="n">
         <v>1000</v>
       </c>
       <c r="E81" t="n">
-        <v>1141.9</v>
+        <v>1206.3</v>
       </c>
       <c r="F81" t="n">
-        <v>983.4042799999999</v>
+        <v>1403.65068</v>
       </c>
       <c r="G81" t="n">
-        <v>1002.482323032</v>
+        <v>1572.930952008</v>
       </c>
       <c r="H81" t="n">
-        <v>1006.392004091825</v>
+        <v>1622.320983901051</v>
       </c>
       <c r="I81" t="n">
-        <v>968.1491079363354</v>
+        <v>1560.023858119251</v>
       </c>
       <c r="J81" t="n">
-        <v>739.9563631957411</v>
+        <v>2085.595895919627</v>
       </c>
       <c r="K81" t="n">
-        <v>567.8425131164117</v>
+        <v>1584.844321309324</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -11964,110 +12026,110 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="D82" t="n">
         <v>1000</v>
       </c>
       <c r="E82" t="n">
-        <v>823.5</v>
+        <v>1141.9</v>
       </c>
       <c r="F82" t="n">
-        <v>939.36645</v>
+        <v>983.4042799999999</v>
       </c>
       <c r="G82" t="n">
-        <v>1037.24843409</v>
+        <v>1002.482323032</v>
       </c>
       <c r="H82" t="n">
-        <v>968.582587753242</v>
+        <v>1006.392004091825</v>
       </c>
       <c r="I82" t="n">
-        <v>996.38090802176</v>
+        <v>968.1491079363354</v>
       </c>
       <c r="J82" t="n">
-        <v>1251.255144293726</v>
+        <v>739.9563631957411</v>
       </c>
       <c r="K82" t="n">
-        <v>953.7066709806782</v>
+        <v>567.8425131164117</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="D83" t="n">
         <v>1000</v>
       </c>
       <c r="E83" t="n">
-        <v>1390.6</v>
+        <v>823.5</v>
       </c>
       <c r="F83" t="n">
-        <v>1715.16604</v>
+        <v>939.36645</v>
       </c>
       <c r="G83" t="n">
-        <v>1928.018145564</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H83" t="n">
-        <v>1842.799743530072</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I83" t="n">
-        <v>1932.359811065633</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J83" t="n">
-        <v>2502.212719348888</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K83" t="n">
-        <v>2078.337884691186</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D84" t="n">
         <v>1000</v>
       </c>
       <c r="E84" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F84" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G84" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H84" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I84" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J84" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K84" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -12075,184 +12137,184 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D85" t="n">
         <v>1000</v>
       </c>
       <c r="E85" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F85" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G85" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H85" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I85" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J85" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K85" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D86" t="n">
         <v>1000</v>
       </c>
       <c r="E86" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F86" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G86" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H86" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I86" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J86" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K86" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D87" t="n">
         <v>1000</v>
       </c>
       <c r="E87" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F87" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G87" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H87" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I87" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J87" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K87" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D88" t="n">
         <v>1000</v>
       </c>
       <c r="E88" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F88" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G88" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H88" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I88" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J88" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K88" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D89" t="n">
         <v>1000</v>
       </c>
       <c r="E89" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F89" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G89" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H89" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I89" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J89" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K89" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -12260,36 +12322,36 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D90" t="n">
         <v>1000</v>
       </c>
       <c r="E90" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F90" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G90" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H90" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I90" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J90" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K90" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -12297,147 +12359,147 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D91" t="n">
         <v>1000</v>
       </c>
       <c r="E91" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F91" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G91" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H91" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I91" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J91" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K91" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D92" t="n">
         <v>1000</v>
       </c>
       <c r="E92" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F92" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G92" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H92" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I92" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J92" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K92" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>-1.4347</v>
+        <v>-1.3564</v>
       </c>
       <c r="D93" t="n">
         <v>1000</v>
       </c>
       <c r="E93" t="n">
-        <v>743.8000000000001</v>
+        <v>799.9</v>
       </c>
       <c r="F93" t="n">
-        <v>692.62656</v>
+        <v>677.35532</v>
       </c>
       <c r="G93" t="n">
-        <v>666.7223266560001</v>
+        <v>658.660313168</v>
       </c>
       <c r="H93" t="n">
-        <v>724.7938413077377</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I93" t="n">
-        <v>681.3786902134042</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J93" t="n">
-        <v>441.2608397822005</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K93" t="n">
-        <v>291.4527846761434</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D94" t="n">
         <v>1000</v>
       </c>
       <c r="E94" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F94" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G94" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H94" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I94" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J94" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K94" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
@@ -12445,36 +12507,36 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D95" t="n">
         <v>1000</v>
       </c>
       <c r="E95" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F95" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G95" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H95" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I95" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J95" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K95" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
@@ -12482,36 +12544,36 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D96" t="n">
         <v>1000</v>
       </c>
       <c r="E96" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F96" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G96" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H96" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I96" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J96" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K96" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -12519,73 +12581,73 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D97" t="n">
         <v>1000</v>
       </c>
       <c r="E97" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F97" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G97" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H97" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I97" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J97" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K97" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D98" t="n">
         <v>1000</v>
       </c>
       <c r="E98" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F98" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G98" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H98" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I98" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J98" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K98" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -12622,81 +12684,81 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D100" t="n">
         <v>1000</v>
       </c>
       <c r="E100" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F100" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G100" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H100" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I100" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J100" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K100" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D101" t="n">
         <v>1000</v>
       </c>
       <c r="E101" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F101" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G101" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H101" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I101" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J101" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K101" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -12704,36 +12766,36 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D102" t="n">
         <v>1000</v>
       </c>
       <c r="E102" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F102" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G102" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H102" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I102" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J102" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K102" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -12741,30 +12803,67 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D103" t="n">
         <v>1000</v>
       </c>
       <c r="E103" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F103" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G103" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H103" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I103" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J103" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K103" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>41</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D104" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E104" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F103" t="n">
+      <c r="F104" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G103" t="n">
+      <c r="G104" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H103" t="n">
+      <c r="H104" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I103" t="n">
+      <c r="I104" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J103" t="n">
+      <c r="J104" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K103" t="n">
+      <c r="K104" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 106 xLSTM seed=0: -0.75 (exp 105 was lucky seed; F1 mean +1.52)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>108</row>
+      <row>109</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T106"/>
+  <dimension ref="A1:T107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7051,16 +7051,16 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>LightGBM @ exp 10 n_est=500 (down from 1000) - capacity sweet-spot test between 300 and 10</t>
+          <t>xLSTM @ exp 105 RECORD hidden=64 seed=0 - multi-seed verify (was +0.08 seed=42 F1 +3.10 ex</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -7069,60 +7069,60 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>-0.7554</v>
+        <v>-0.7528</v>
       </c>
       <c r="F74" t="n">
-        <v>0.7433</v>
+        <v>0.6044</v>
       </c>
       <c r="G74" t="n">
-        <v>-0.5554</v>
+        <v>-0.6528</v>
       </c>
       <c r="I74" t="n">
-        <v>82.7</v>
+        <v>103.48</v>
       </c>
       <c r="J74" t="n">
-        <v>1827</v>
+        <v>2034.8</v>
       </c>
       <c r="K74" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L74" t="n">
         <v>4</v>
       </c>
       <c r="N74" t="n">
-        <v>0.0283</v>
+        <v>0.0487</v>
       </c>
       <c r="O74" t="n">
-        <v>48.5</v>
+        <v>53.73</v>
       </c>
       <c r="P74" t="n">
-        <v>0.5928</v>
+        <v>0.5816</v>
       </c>
       <c r="Q74" t="n">
-        <v>0.4193</v>
+        <v>0.6803</v>
       </c>
       <c r="R74" t="n">
-        <v>0.4912</v>
+        <v>0.6271</v>
       </c>
       <c r="S74" t="n">
-        <v>0.0009</v>
+        <v>0.0265</v>
       </c>
       <c r="T74" t="n">
-        <v>117.6</v>
+        <v>140.8</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>lightgbm</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer warmup=5 (up from 0) - Goyal 2017 LR warmup on 1-layer</t>
+          <t>LightGBM @ exp 10 n_est=500 (down from 1000) - capacity sweet-spot test between 300 and 10</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -7131,60 +7131,60 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>-0.7729</v>
+        <v>-0.7554</v>
       </c>
       <c r="F75" t="n">
-        <v>-0.2729</v>
+        <v>0.7433</v>
       </c>
       <c r="G75" t="n">
-        <v>0.3166</v>
+        <v>-0.5554</v>
       </c>
       <c r="I75" t="n">
-        <v>-46.29</v>
+        <v>82.7</v>
       </c>
       <c r="J75" t="n">
-        <v>537.1</v>
+        <v>1827</v>
       </c>
       <c r="K75" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N75" t="n">
-        <v>0.0109</v>
+        <v>0.0283</v>
       </c>
       <c r="O75" t="n">
-        <v>46.06</v>
+        <v>48.5</v>
       </c>
       <c r="P75" t="n">
-        <v>0.5444</v>
+        <v>0.5928</v>
       </c>
       <c r="Q75" t="n">
-        <v>0.3569</v>
+        <v>0.4193</v>
       </c>
       <c r="R75" t="n">
-        <v>0.4311</v>
+        <v>0.4912</v>
       </c>
       <c r="S75" t="n">
-        <v>-0.0437</v>
+        <v>0.0009</v>
       </c>
       <c r="T75" t="n">
-        <v>87.40000000000001</v>
+        <v>117.6</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>LightGBM @ exp 10 gbm_lr=0.005 (down from 0.01) - slower learning at fixed n_est</t>
+          <t>LSTM @ exp 71 1-layer warmup=5 (up from 0) - Goyal 2017 LR warmup on 1-layer</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -7193,122 +7193,122 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>-0.8</v>
+        <v>-0.7729</v>
       </c>
       <c r="F76" t="n">
-        <v>0.4079</v>
+        <v>-0.2729</v>
       </c>
       <c r="G76" t="n">
-        <v>-0.5</v>
+        <v>0.3166</v>
       </c>
       <c r="I76" t="n">
-        <v>32.66</v>
+        <v>-46.29</v>
       </c>
       <c r="J76" t="n">
-        <v>1326.6</v>
+        <v>537.1</v>
       </c>
       <c r="K76" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N76" t="n">
-        <v>0.0255</v>
+        <v>0.0109</v>
       </c>
       <c r="O76" t="n">
-        <v>47.74</v>
+        <v>46.06</v>
       </c>
       <c r="P76" t="n">
-        <v>0.5764</v>
+        <v>0.5444</v>
       </c>
       <c r="Q76" t="n">
-        <v>0.4478</v>
+        <v>0.3569</v>
       </c>
       <c r="R76" t="n">
-        <v>0.504</v>
+        <v>0.4311</v>
       </c>
       <c r="S76" t="n">
-        <v>-0.0299</v>
+        <v>-0.0437</v>
       </c>
       <c r="T76" t="n">
-        <v>217.8</v>
+        <v>87.40000000000001</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
+        <v>93</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>lightgbm</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>LightGBM @ exp 10 gbm_lr=0.005 (down from 0.01) - slower learning at fixed n_est</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0.4079</v>
+      </c>
+      <c r="G77" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="I77" t="n">
+        <v>32.66</v>
+      </c>
+      <c r="J77" t="n">
+        <v>1326.6</v>
+      </c>
+      <c r="K77" t="n">
         <v>4</v>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>mlp</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>mlp seq=20 + stronger reg head_dropout=0.25 wd=1e-4 patience=15 (Gu-Kelly-Xiu 2020); hill-</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E77" t="n">
-        <v>-0.8341</v>
-      </c>
-      <c r="F77" t="n">
-        <v>-0.4341</v>
-      </c>
-      <c r="G77" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="I77" t="n">
-        <v>-54.77</v>
-      </c>
-      <c r="J77" t="n">
-        <v>452.2999999999999</v>
-      </c>
-      <c r="K77" t="n">
-        <v>3</v>
-      </c>
       <c r="L77" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N77" t="n">
-        <v>-0.0036</v>
+        <v>0.0255</v>
       </c>
       <c r="O77" t="n">
-        <v>49.07</v>
+        <v>47.74</v>
       </c>
       <c r="P77" t="n">
-        <v>0.5674</v>
+        <v>0.5764</v>
       </c>
       <c r="Q77" t="n">
-        <v>0.4955</v>
+        <v>0.4478</v>
       </c>
       <c r="R77" t="n">
-        <v>0.529</v>
+        <v>0.504</v>
       </c>
       <c r="S77" t="n">
-        <v>-0.0193</v>
+        <v>-0.0299</v>
       </c>
       <c r="T77" t="n">
-        <v>32.6</v>
+        <v>217.8</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">CatBoost @ LightGBM-exp10 config (depth=4 lr=0.01 n_est=1000 seq=60) - 3-way GBM ensemble </t>
+          <t>mlp seq=20 + stronger reg head_dropout=0.25 wd=1e-4 patience=15 (Gu-Kelly-Xiu 2020); hill-</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -7317,51 +7317,51 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>-0.8395</v>
+        <v>-0.8341</v>
       </c>
       <c r="F78" t="n">
-        <v>0.2322</v>
+        <v>-0.4341</v>
       </c>
       <c r="G78" t="n">
-        <v>-0.5395</v>
+        <v>1.203</v>
       </c>
       <c r="I78" t="n">
-        <v>12.15</v>
+        <v>-54.77</v>
       </c>
       <c r="J78" t="n">
-        <v>1121.5</v>
+        <v>452.2999999999999</v>
       </c>
       <c r="K78" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L78" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N78" t="n">
-        <v>0.011</v>
+        <v>-0.0036</v>
       </c>
       <c r="O78" t="n">
-        <v>48.87</v>
+        <v>49.07</v>
       </c>
       <c r="P78" t="n">
-        <v>0.5893</v>
+        <v>0.5674</v>
       </c>
       <c r="Q78" t="n">
-        <v>0.4541</v>
+        <v>0.4955</v>
       </c>
       <c r="R78" t="n">
-        <v>0.513</v>
+        <v>0.529</v>
       </c>
       <c r="S78" t="n">
-        <v>-0.0056</v>
+        <v>-0.0193</v>
       </c>
       <c r="T78" t="n">
-        <v>1316.8</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -7370,7 +7370,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.02 n_est=500 - smaller capacity at productive lr</t>
+          <t xml:space="preserve">CatBoost @ LightGBM-exp10 config (depth=4 lr=0.01 n_est=1000 seq=60) - 3-way GBM ensemble </t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -7379,60 +7379,60 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>-0.8456</v>
+        <v>-0.8395</v>
       </c>
       <c r="F79" t="n">
-        <v>0.2334</v>
+        <v>0.2322</v>
       </c>
       <c r="G79" t="n">
-        <v>-0.4456</v>
+        <v>-0.5395</v>
       </c>
       <c r="I79" t="n">
-        <v>12.26</v>
+        <v>12.15</v>
       </c>
       <c r="J79" t="n">
-        <v>1122.6</v>
+        <v>1121.5</v>
       </c>
       <c r="K79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L79" t="n">
         <v>2</v>
       </c>
       <c r="N79" t="n">
-        <v>0.0108</v>
+        <v>0.011</v>
       </c>
       <c r="O79" t="n">
-        <v>49.72</v>
+        <v>48.87</v>
       </c>
       <c r="P79" t="n">
-        <v>0.5938</v>
+        <v>0.5893</v>
       </c>
       <c r="Q79" t="n">
-        <v>0.481</v>
+        <v>0.4541</v>
       </c>
       <c r="R79" t="n">
-        <v>0.5315</v>
+        <v>0.513</v>
       </c>
       <c r="S79" t="n">
-        <v>0.0028</v>
+        <v>-0.0056</v>
       </c>
       <c r="T79" t="n">
-        <v>673.8</v>
+        <v>1316.8</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t xml:space="preserve">dMamba @ FX-Mamba-winner config seed=99 — 3rd seed for stable champion declaration (seeds </t>
+          <t>CatBoost lr=0.02 n_est=500 - smaller capacity at productive lr</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -7441,60 +7441,60 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>-0.862</v>
+        <v>-0.8456</v>
       </c>
       <c r="F80" t="n">
-        <v>-0.462</v>
+        <v>0.2334</v>
       </c>
       <c r="G80" t="n">
-        <v>1.3122</v>
+        <v>-0.4456</v>
       </c>
       <c r="I80" t="n">
-        <v>-42.07</v>
+        <v>12.26</v>
       </c>
       <c r="J80" t="n">
-        <v>579.3</v>
+        <v>1122.6</v>
       </c>
       <c r="K80" t="n">
         <v>3</v>
       </c>
       <c r="L80" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N80" t="n">
-        <v>0.0467</v>
+        <v>0.0108</v>
       </c>
       <c r="O80" t="n">
-        <v>43.33</v>
+        <v>49.72</v>
       </c>
       <c r="P80" t="n">
-        <v>0.5858</v>
+        <v>0.5938</v>
       </c>
       <c r="Q80" t="n">
-        <v>0.1576</v>
+        <v>0.481</v>
       </c>
       <c r="R80" t="n">
-        <v>0.2484</v>
+        <v>0.5315</v>
       </c>
       <c r="S80" t="n">
-        <v>-0.0059</v>
+        <v>0.0028</v>
       </c>
       <c r="T80" t="n">
-        <v>705.3</v>
+        <v>673.8</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CatBoost depth=6 lr=0.01 n_est=1000 - depth axis test</t>
+          <t xml:space="preserve">dMamba @ FX-Mamba-winner config seed=99 — 3rd seed for stable champion declaration (seeds </t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -7503,51 +7503,51 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>-0.8688</v>
+        <v>-0.862</v>
       </c>
       <c r="F81" t="n">
-        <v>0.7087</v>
+        <v>-0.462</v>
       </c>
       <c r="G81" t="n">
-        <v>-0.6688</v>
+        <v>1.3122</v>
       </c>
       <c r="I81" t="n">
-        <v>76.76000000000001</v>
+        <v>-42.07</v>
       </c>
       <c r="J81" t="n">
-        <v>1767.6</v>
+        <v>579.3</v>
       </c>
       <c r="K81" t="n">
+        <v>3</v>
+      </c>
+      <c r="L81" t="n">
         <v>5</v>
       </c>
-      <c r="L81" t="n">
-        <v>1</v>
-      </c>
       <c r="N81" t="n">
-        <v>0.0031</v>
+        <v>0.0467</v>
       </c>
       <c r="O81" t="n">
-        <v>49.34</v>
+        <v>43.33</v>
       </c>
       <c r="P81" t="n">
-        <v>0.5827</v>
+        <v>0.5858</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.5127</v>
+        <v>0.1576</v>
       </c>
       <c r="R81" t="n">
-        <v>0.5455</v>
+        <v>0.2484</v>
       </c>
       <c r="S81" t="n">
-        <v>-0.0203</v>
+        <v>-0.0059</v>
       </c>
       <c r="T81" t="n">
-        <v>4289.1</v>
+        <v>705.3</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -7556,7 +7556,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.02 n_est=2000 - combine best CatBoost findings (lr from exp 98, capacity fro</t>
+          <t>CatBoost depth=6 lr=0.01 n_est=1000 - depth axis test</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -7565,51 +7565,51 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>-0.8764</v>
+        <v>-0.8688</v>
       </c>
       <c r="F82" t="n">
-        <v>-0.1626</v>
+        <v>0.7087</v>
       </c>
       <c r="G82" t="n">
-        <v>-0.4764</v>
+        <v>-0.6688</v>
       </c>
       <c r="I82" t="n">
-        <v>-23.11</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="J82" t="n">
-        <v>768.9</v>
+        <v>1767.6</v>
       </c>
       <c r="K82" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L82" t="n">
         <v>1</v>
       </c>
       <c r="N82" t="n">
-        <v>0.0008</v>
+        <v>0.0031</v>
       </c>
       <c r="O82" t="n">
-        <v>46.43</v>
+        <v>49.34</v>
       </c>
       <c r="P82" t="n">
-        <v>0.5760999999999999</v>
+        <v>0.5827</v>
       </c>
       <c r="Q82" t="n">
-        <v>0.3655</v>
+        <v>0.5127</v>
       </c>
       <c r="R82" t="n">
-        <v>0.4472</v>
+        <v>0.5455</v>
       </c>
       <c r="S82" t="n">
-        <v>-0.0257</v>
+        <v>-0.0203</v>
       </c>
       <c r="T82" t="n">
-        <v>2594.9</v>
+        <v>4289.1</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
+          <t>CatBoost lr=0.02 n_est=2000 - combine best CatBoost findings (lr from exp 98, capacity fro</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -7627,60 +7627,60 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>-0.9217</v>
+        <v>-0.8764</v>
       </c>
       <c r="F83" t="n">
-        <v>0.5942</v>
+        <v>-0.1626</v>
       </c>
       <c r="G83" t="n">
-        <v>-0.7217</v>
+        <v>-0.4764</v>
       </c>
       <c r="I83" t="n">
-        <v>58.5</v>
+        <v>-23.11</v>
       </c>
       <c r="J83" t="n">
-        <v>1585</v>
+        <v>768.9</v>
       </c>
       <c r="K83" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L83" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N83" t="n">
-        <v>0.019</v>
+        <v>0.0008</v>
       </c>
       <c r="O83" t="n">
-        <v>48.5</v>
+        <v>46.43</v>
       </c>
       <c r="P83" t="n">
-        <v>0.5986</v>
+        <v>0.5760999999999999</v>
       </c>
       <c r="Q83" t="n">
-        <v>0.3987</v>
+        <v>0.3655</v>
       </c>
       <c r="R83" t="n">
-        <v>0.4786</v>
+        <v>0.4472</v>
       </c>
       <c r="S83" t="n">
-        <v>0.0103</v>
+        <v>-0.0257</v>
       </c>
       <c r="T83" t="n">
-        <v>18919.4</v>
+        <v>2594.9</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
+          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -7689,51 +7689,51 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="F84" t="n">
-        <v>-0.2367</v>
+        <v>0.5942</v>
       </c>
       <c r="G84" t="n">
-        <v>-0.5226</v>
+        <v>-0.7217</v>
       </c>
       <c r="I84" t="n">
-        <v>-43.21</v>
+        <v>58.5</v>
       </c>
       <c r="J84" t="n">
-        <v>567.9000000000001</v>
+        <v>1585</v>
       </c>
       <c r="K84" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N84" t="n">
-        <v>-0.0164</v>
+        <v>0.019</v>
       </c>
       <c r="O84" t="n">
-        <v>45.63</v>
+        <v>48.5</v>
       </c>
       <c r="P84" t="n">
-        <v>0.5938</v>
+        <v>0.5986</v>
       </c>
       <c r="Q84" t="n">
-        <v>0.1648</v>
+        <v>0.3987</v>
       </c>
       <c r="R84" t="n">
-        <v>0.258</v>
+        <v>0.4786</v>
       </c>
       <c r="S84" t="n">
-        <v>0.0188</v>
+        <v>0.0103</v>
       </c>
       <c r="T84" t="n">
-        <v>33.8</v>
+        <v>18919.4</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -7742,7 +7742,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -7751,60 +7751,60 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="F85" t="n">
-        <v>0.1045</v>
+        <v>-0.2367</v>
       </c>
       <c r="G85" t="n">
-        <v>-0.6746</v>
+        <v>-0.5226</v>
       </c>
       <c r="I85" t="n">
-        <v>-4.63</v>
+        <v>-43.21</v>
       </c>
       <c r="J85" t="n">
-        <v>953.7</v>
+        <v>567.9000000000001</v>
       </c>
       <c r="K85" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L85" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N85" t="n">
-        <v>-0.0374</v>
+        <v>-0.0164</v>
       </c>
       <c r="O85" t="n">
-        <v>51.03</v>
+        <v>45.63</v>
       </c>
       <c r="P85" t="n">
-        <v>0.5765</v>
+        <v>0.5938</v>
       </c>
       <c r="Q85" t="n">
-        <v>0.5415</v>
+        <v>0.1648</v>
       </c>
       <c r="R85" t="n">
-        <v>0.5585</v>
+        <v>0.258</v>
       </c>
       <c r="S85" t="n">
-        <v>0.0091</v>
+        <v>0.0188</v>
       </c>
       <c r="T85" t="n">
-        <v>30.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -7813,60 +7813,60 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="F86" t="n">
-        <v>0.8788</v>
+        <v>0.1045</v>
       </c>
       <c r="G86" t="n">
-        <v>-0.866</v>
+        <v>-0.6746</v>
       </c>
       <c r="I86" t="n">
-        <v>107.82</v>
+        <v>-4.63</v>
       </c>
       <c r="J86" t="n">
-        <v>2078.2</v>
+        <v>953.7</v>
       </c>
       <c r="K86" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L86" t="n">
         <v>2</v>
       </c>
       <c r="N86" t="n">
-        <v>0.0329</v>
+        <v>-0.0374</v>
       </c>
       <c r="O86" t="n">
-        <v>54.14</v>
+        <v>51.03</v>
       </c>
       <c r="P86" t="n">
-        <v>0.6011</v>
+        <v>0.5765</v>
       </c>
       <c r="Q86" t="n">
-        <v>0.6725</v>
+        <v>0.5415</v>
       </c>
       <c r="R86" t="n">
-        <v>0.6348</v>
+        <v>0.5585</v>
       </c>
       <c r="S86" t="n">
-        <v>0.0251</v>
+        <v>0.0091</v>
       </c>
       <c r="T86" t="n">
-        <v>75.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -7875,51 +7875,51 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F87" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G87" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I87" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J87" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K87" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L87" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N87" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O87" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P87" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q87" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R87" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S87" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T87" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -7928,7 +7928,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -7937,60 +7937,60 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F88" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G88" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I88" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J88" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K88" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L88" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N88" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O88" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P88" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q88" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R88" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S88" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T88" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -7999,60 +7999,60 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F89" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G89" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I89" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J89" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K89" t="n">
         <v>2</v>
       </c>
       <c r="L89" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N89" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O89" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P89" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q89" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R89" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S89" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T89" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -8061,60 +8061,60 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F90" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G90" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I90" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J90" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K90" t="n">
+        <v>2</v>
+      </c>
+      <c r="L90" t="n">
         <v>5</v>
       </c>
-      <c r="L90" t="n">
-        <v>2</v>
-      </c>
       <c r="N90" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O90" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P90" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q90" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R90" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S90" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T90" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -8123,60 +8123,60 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F91" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G91" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I91" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J91" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K91" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L91" t="n">
         <v>2</v>
       </c>
       <c r="N91" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O91" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P91" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q91" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R91" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S91" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T91" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8185,51 +8185,51 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F92" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G92" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I92" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J92" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L92" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N92" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O92" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P92" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q92" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R92" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S92" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T92" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -8238,7 +8238,7 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8247,51 +8247,51 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F93" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G93" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I93" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J93" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K93" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L93" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N93" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O93" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P93" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q93" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R93" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S93" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T93" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -8300,7 +8300,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8309,60 +8309,60 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F94" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G94" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I94" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J94" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K94" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L94" t="n">
         <v>2</v>
       </c>
       <c r="N94" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O94" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P94" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q94" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R94" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S94" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T94" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -8371,60 +8371,60 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F95" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G95" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I95" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J95" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K95" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N95" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O95" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P95" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q95" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R95" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S95" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T95" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8433,60 +8433,60 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>-1.4347</v>
+        <v>-1.3564</v>
       </c>
       <c r="F96" t="n">
-        <v>-0.6758999999999999</v>
+        <v>0.011</v>
       </c>
       <c r="G96" t="n">
-        <v>-0.8347</v>
+        <v>-0.9564</v>
       </c>
       <c r="I96" t="n">
-        <v>-70.84999999999999</v>
+        <v>-17.26</v>
       </c>
       <c r="J96" t="n">
-        <v>291.5000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K96" t="n">
+        <v>3</v>
+      </c>
+      <c r="L96" t="n">
         <v>1</v>
       </c>
-      <c r="L96" t="n">
-        <v>2</v>
-      </c>
       <c r="N96" t="n">
-        <v>0.0284</v>
+        <v>-0.0003</v>
       </c>
       <c r="O96" t="n">
-        <v>44.07</v>
+        <v>48.19</v>
       </c>
       <c r="P96" t="n">
-        <v>0.5588</v>
+        <v>0.5666</v>
       </c>
       <c r="Q96" t="n">
-        <v>0.1177</v>
+        <v>0.4114</v>
       </c>
       <c r="R96" t="n">
-        <v>0.1945</v>
+        <v>0.4767</v>
       </c>
       <c r="S96" t="n">
-        <v>-0.0101</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T96" t="n">
-        <v>79.8</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8495,39 +8495,51 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F97" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G97" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I97" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J97" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K97" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L97" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N97" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O97" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P97" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R97" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S97" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T97" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -8536,7 +8548,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8545,51 +8557,39 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F98" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G98" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I98" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J98" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K98" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L98" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N98" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O98" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P98" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q98" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R98" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S98" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T98" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -8598,7 +8598,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8607,51 +8607,51 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F99" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G99" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I99" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J99" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L99" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N99" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O99" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P99" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q99" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R99" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S99" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T99" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -8660,7 +8660,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8669,113 +8669,113 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F100" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G100" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I100" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J100" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K100" t="n">
         <v>1</v>
       </c>
       <c r="L100" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N100" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O100" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P100" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q100" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R100" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S100" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T100" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
+        <v>59</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F101" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G101" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I101" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J101" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K101" t="n">
         <v>1</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C101" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E101" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F101" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G101" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I101" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J101" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K101" t="n">
-        <v>5</v>
       </c>
       <c r="L101" t="n">
         <v>1</v>
       </c>
       <c r="N101" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O101" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P101" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q101" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R101" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S101" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T101" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -8784,12 +8784,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -8832,21 +8832,21 @@
         <v>0.0098</v>
       </c>
       <c r="T102" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8855,19 +8855,19 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F103" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G103" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I103" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J103" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K103" t="n">
         <v>5</v>
@@ -8876,39 +8876,39 @@
         <v>1</v>
       </c>
       <c r="N103" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O103" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P103" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R103" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S103" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T103" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -8917,113 +8917,113 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F104" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G104" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I104" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J104" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K104" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N104" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O104" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P104" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q104" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R104" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S104" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T104" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
+        <v>22</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F105" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G105" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I105" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J105" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K105" t="n">
+        <v>4</v>
+      </c>
+      <c r="L105" t="n">
         <v>2</v>
       </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E105" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F105" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G105" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I105" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J105" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K105" t="n">
-        <v>5</v>
-      </c>
-      <c r="L105" t="n">
-        <v>1</v>
-      </c>
       <c r="N105" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O105" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P105" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q105" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R105" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S105" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T105" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -9032,7 +9032,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9041,51 +9041,113 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F106" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G106" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I106" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J106" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K106" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N106" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O106" t="n">
         <v>47.65</v>
       </c>
       <c r="P106" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R106" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S106" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T106" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>41</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F107" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G107" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I107" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J107" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K107" t="n">
+        <v>4</v>
+      </c>
+      <c r="L107" t="n">
+        <v>2</v>
+      </c>
+      <c r="N107" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O107" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P107" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q106" t="n">
+      <c r="Q107" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R106" t="n">
+      <c r="R107" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S106" t="n">
+      <c r="S107" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T106" t="n">
+      <c r="T107" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T106"/>
-  <conditionalFormatting sqref="E2:E106">
+  <autoFilter ref="A1:T107"/>
+  <conditionalFormatting sqref="E2:E107">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -9107,7 +9169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K106"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11846,192 +11908,192 @@
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>-0.7554</v>
+        <v>-0.7528</v>
       </c>
       <c r="D74" t="n">
         <v>1000</v>
       </c>
       <c r="E74" t="n">
-        <v>1025.7</v>
+        <v>843.7</v>
       </c>
       <c r="F74" t="n">
-        <v>1138.527</v>
+        <v>922.41721</v>
       </c>
       <c r="G74" t="n">
-        <v>1222.777998</v>
+        <v>936.714676755</v>
       </c>
       <c r="H74" t="n">
-        <v>1085.4600288246</v>
+        <v>1095.019457126595</v>
       </c>
       <c r="I74" t="n">
-        <v>915.6940803164325</v>
+        <v>1178.897947542492</v>
       </c>
       <c r="J74" t="n">
-        <v>1284.718794683955</v>
+        <v>1454.406397883173</v>
       </c>
       <c r="K74" t="n">
-        <v>1827.255541678989</v>
+        <v>2034.859991278347</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>lightgbm</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>-0.7729</v>
+        <v>-0.7554</v>
       </c>
       <c r="D75" t="n">
         <v>1000</v>
       </c>
       <c r="E75" t="n">
-        <v>879.3</v>
+        <v>1025.7</v>
       </c>
       <c r="F75" t="n">
-        <v>936.7182899999999</v>
+        <v>1138.527</v>
       </c>
       <c r="G75" t="n">
-        <v>835.646386509</v>
+        <v>1222.777998</v>
       </c>
       <c r="H75" t="n">
-        <v>799.4628979731602</v>
+        <v>1085.4600288246</v>
       </c>
       <c r="I75" t="n">
-        <v>859.0228838721607</v>
+        <v>915.6940803164325</v>
       </c>
       <c r="J75" t="n">
-        <v>659.1282587951089</v>
+        <v>1284.718794683955</v>
       </c>
       <c r="K75" t="n">
-        <v>537.1895309180137</v>
+        <v>1827.255541678989</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>-0.8</v>
+        <v>-0.7729</v>
       </c>
       <c r="D76" t="n">
         <v>1000</v>
       </c>
       <c r="E76" t="n">
-        <v>936.6999999999999</v>
+        <v>879.3</v>
       </c>
       <c r="F76" t="n">
-        <v>1011.26132</v>
+        <v>936.7182899999999</v>
       </c>
       <c r="G76" t="n">
-        <v>1048.779114972</v>
+        <v>835.646386509</v>
       </c>
       <c r="H76" t="n">
-        <v>1000.849909417779</v>
+        <v>799.4628979731602</v>
       </c>
       <c r="I76" t="n">
-        <v>1051.592999825261</v>
+        <v>859.0228838721607</v>
       </c>
       <c r="J76" t="n">
-        <v>1570.133508039097</v>
+        <v>659.1282587951089</v>
       </c>
       <c r="K76" t="n">
-        <v>1326.605800942233</v>
+        <v>537.1895309180137</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>4</v>
+        <v>93</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lightgbm</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>-0.8341</v>
+        <v>-0.8</v>
       </c>
       <c r="D77" t="n">
         <v>1000</v>
       </c>
       <c r="E77" t="n">
-        <v>909.6999999999999</v>
+        <v>936.6999999999999</v>
       </c>
       <c r="F77" t="n">
-        <v>831.10192</v>
+        <v>1011.26132</v>
       </c>
       <c r="G77" t="n">
-        <v>866.4237515999999</v>
+        <v>1048.779114972</v>
       </c>
       <c r="H77" t="n">
-        <v>873.0952144873199</v>
+        <v>1000.849909417779</v>
       </c>
       <c r="I77" t="n">
-        <v>662.4173392315297</v>
+        <v>1051.592999825261</v>
       </c>
       <c r="J77" t="n">
-        <v>447.3966709169752</v>
+        <v>1570.133508039097</v>
       </c>
       <c r="K77" t="n">
-        <v>452.3180342970618</v>
+        <v>1326.605800942233</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>-0.8395</v>
+        <v>-0.8341</v>
       </c>
       <c r="D78" t="n">
         <v>1000</v>
       </c>
       <c r="E78" t="n">
-        <v>1011.7</v>
+        <v>909.6999999999999</v>
       </c>
       <c r="F78" t="n">
-        <v>1220.21137</v>
+        <v>831.10192</v>
       </c>
       <c r="G78" t="n">
-        <v>1383.963735854</v>
+        <v>866.4237515999999</v>
       </c>
       <c r="H78" t="n">
-        <v>1276.56814995173</v>
+        <v>873.0952144873199</v>
       </c>
       <c r="I78" t="n">
-        <v>1150.570873551494</v>
+        <v>662.4173392315297</v>
       </c>
       <c r="J78" t="n">
-        <v>1502.300389596186</v>
+        <v>447.3966709169752</v>
       </c>
       <c r="K78" t="n">
-        <v>1121.617470872512</v>
+        <v>452.3180342970618</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
@@ -12039,110 +12101,110 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>-0.8456</v>
+        <v>-0.8395</v>
       </c>
       <c r="D79" t="n">
         <v>1000</v>
       </c>
       <c r="E79" t="n">
-        <v>953</v>
+        <v>1011.7</v>
       </c>
       <c r="F79" t="n">
-        <v>1234.8974</v>
+        <v>1220.21137</v>
       </c>
       <c r="G79" t="n">
-        <v>1386.04884176</v>
+        <v>1383.963735854</v>
       </c>
       <c r="H79" t="n">
-        <v>1167.330334530272</v>
+        <v>1276.56814995173</v>
       </c>
       <c r="I79" t="n">
-        <v>993.3981146852617</v>
+        <v>1150.570873551494</v>
       </c>
       <c r="J79" t="n">
-        <v>1310.689472515734</v>
+        <v>1502.300389596186</v>
       </c>
       <c r="K79" t="n">
-        <v>1122.605533209726</v>
+        <v>1121.617470872512</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>-0.862</v>
+        <v>-0.8456</v>
       </c>
       <c r="D80" t="n">
         <v>1000</v>
       </c>
       <c r="E80" t="n">
-        <v>1064.8</v>
+        <v>953</v>
       </c>
       <c r="F80" t="n">
-        <v>857.3769599999999</v>
+        <v>1234.8974</v>
       </c>
       <c r="G80" t="n">
-        <v>754.4917247999999</v>
+        <v>1386.04884176</v>
       </c>
       <c r="H80" t="n">
-        <v>689.30363977728</v>
+        <v>1167.330334530272</v>
       </c>
       <c r="I80" t="n">
-        <v>835.2981506821078</v>
+        <v>993.3981146852617</v>
       </c>
       <c r="J80" t="n">
-        <v>582.2028110254292</v>
+        <v>1310.689472515734</v>
       </c>
       <c r="K80" t="n">
-        <v>579.3500172514047</v>
+        <v>1122.605533209726</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>-0.8688</v>
+        <v>-0.862</v>
       </c>
       <c r="D81" t="n">
         <v>1000</v>
       </c>
       <c r="E81" t="n">
-        <v>1120</v>
+        <v>1064.8</v>
       </c>
       <c r="F81" t="n">
-        <v>1237.6</v>
+        <v>857.3769599999999</v>
       </c>
       <c r="G81" t="n">
-        <v>1385.61696</v>
+        <v>754.4917247999999</v>
       </c>
       <c r="H81" t="n">
-        <v>1253.429102016</v>
+        <v>689.30363977728</v>
       </c>
       <c r="I81" t="n">
-        <v>1143.378026858995</v>
+        <v>835.2981506821078</v>
       </c>
       <c r="J81" t="n">
-        <v>1478.502126531366</v>
+        <v>582.2028110254292</v>
       </c>
       <c r="K81" t="n">
-        <v>1767.549292268249</v>
+        <v>579.3500172514047</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -12150,36 +12212,36 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>-0.8764</v>
+        <v>-0.8688</v>
       </c>
       <c r="D82" t="n">
         <v>1000</v>
       </c>
       <c r="E82" t="n">
-        <v>762</v>
+        <v>1120</v>
       </c>
       <c r="F82" t="n">
-        <v>937.8695999999999</v>
+        <v>1237.6</v>
       </c>
       <c r="G82" t="n">
-        <v>946.9669351199999</v>
+        <v>1385.61696</v>
       </c>
       <c r="H82" t="n">
-        <v>929.2586534332559</v>
+        <v>1253.429102016</v>
       </c>
       <c r="I82" t="n">
-        <v>802.1360696435864</v>
+        <v>1143.378026858995</v>
       </c>
       <c r="J82" t="n">
-        <v>902.5635055629634</v>
+        <v>1478.502126531366</v>
       </c>
       <c r="K82" t="n">
-        <v>768.8035940385322</v>
+        <v>1767.549292268249</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>18</v>
+        <v>100</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -12187,73 +12249,73 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>-0.9217</v>
+        <v>-0.8764</v>
       </c>
       <c r="D83" t="n">
         <v>1000</v>
       </c>
       <c r="E83" t="n">
-        <v>1206.3</v>
+        <v>762</v>
       </c>
       <c r="F83" t="n">
-        <v>1403.65068</v>
+        <v>937.8695999999999</v>
       </c>
       <c r="G83" t="n">
-        <v>1572.930952008</v>
+        <v>946.9669351199999</v>
       </c>
       <c r="H83" t="n">
-        <v>1622.320983901051</v>
+        <v>929.2586534332559</v>
       </c>
       <c r="I83" t="n">
-        <v>1560.023858119251</v>
+        <v>802.1360696435864</v>
       </c>
       <c r="J83" t="n">
-        <v>2085.595895919627</v>
+        <v>902.5635055629634</v>
       </c>
       <c r="K83" t="n">
-        <v>1584.844321309324</v>
+        <v>768.8035940385322</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="D84" t="n">
         <v>1000</v>
       </c>
       <c r="E84" t="n">
-        <v>1141.9</v>
+        <v>1206.3</v>
       </c>
       <c r="F84" t="n">
-        <v>983.4042799999999</v>
+        <v>1403.65068</v>
       </c>
       <c r="G84" t="n">
-        <v>1002.482323032</v>
+        <v>1572.930952008</v>
       </c>
       <c r="H84" t="n">
-        <v>1006.392004091825</v>
+        <v>1622.320983901051</v>
       </c>
       <c r="I84" t="n">
-        <v>968.1491079363354</v>
+        <v>1560.023858119251</v>
       </c>
       <c r="J84" t="n">
-        <v>739.9563631957411</v>
+        <v>2085.595895919627</v>
       </c>
       <c r="K84" t="n">
-        <v>567.8425131164117</v>
+        <v>1584.844321309324</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
@@ -12261,110 +12323,110 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="D85" t="n">
         <v>1000</v>
       </c>
       <c r="E85" t="n">
-        <v>823.5</v>
+        <v>1141.9</v>
       </c>
       <c r="F85" t="n">
-        <v>939.36645</v>
+        <v>983.4042799999999</v>
       </c>
       <c r="G85" t="n">
-        <v>1037.24843409</v>
+        <v>1002.482323032</v>
       </c>
       <c r="H85" t="n">
-        <v>968.582587753242</v>
+        <v>1006.392004091825</v>
       </c>
       <c r="I85" t="n">
-        <v>996.38090802176</v>
+        <v>968.1491079363354</v>
       </c>
       <c r="J85" t="n">
-        <v>1251.255144293726</v>
+        <v>739.9563631957411</v>
       </c>
       <c r="K85" t="n">
-        <v>953.7066709806782</v>
+        <v>567.8425131164117</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="D86" t="n">
         <v>1000</v>
       </c>
       <c r="E86" t="n">
-        <v>1390.6</v>
+        <v>823.5</v>
       </c>
       <c r="F86" t="n">
-        <v>1715.16604</v>
+        <v>939.36645</v>
       </c>
       <c r="G86" t="n">
-        <v>1928.018145564</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H86" t="n">
-        <v>1842.799743530072</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I86" t="n">
-        <v>1932.359811065633</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J86" t="n">
-        <v>2502.212719348888</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K86" t="n">
-        <v>2078.337884691186</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D87" t="n">
         <v>1000</v>
       </c>
       <c r="E87" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F87" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G87" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H87" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I87" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J87" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K87" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -12372,184 +12434,184 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D88" t="n">
         <v>1000</v>
       </c>
       <c r="E88" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F88" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G88" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H88" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I88" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J88" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K88" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D89" t="n">
         <v>1000</v>
       </c>
       <c r="E89" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F89" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G89" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H89" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I89" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J89" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K89" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D90" t="n">
         <v>1000</v>
       </c>
       <c r="E90" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F90" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G90" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H90" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I90" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J90" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K90" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D91" t="n">
         <v>1000</v>
       </c>
       <c r="E91" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F91" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G91" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H91" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I91" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J91" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K91" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D92" t="n">
         <v>1000</v>
       </c>
       <c r="E92" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F92" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G92" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H92" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I92" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J92" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K92" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
@@ -12557,36 +12619,36 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D93" t="n">
         <v>1000</v>
       </c>
       <c r="E93" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F93" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G93" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H93" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I93" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J93" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K93" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -12594,147 +12656,147 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D94" t="n">
         <v>1000</v>
       </c>
       <c r="E94" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F94" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G94" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H94" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I94" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J94" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K94" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D95" t="n">
         <v>1000</v>
       </c>
       <c r="E95" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F95" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G95" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H95" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I95" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J95" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K95" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>-1.4347</v>
+        <v>-1.3564</v>
       </c>
       <c r="D96" t="n">
         <v>1000</v>
       </c>
       <c r="E96" t="n">
-        <v>743.8000000000001</v>
+        <v>799.9</v>
       </c>
       <c r="F96" t="n">
-        <v>692.62656</v>
+        <v>677.35532</v>
       </c>
       <c r="G96" t="n">
-        <v>666.7223266560001</v>
+        <v>658.660313168</v>
       </c>
       <c r="H96" t="n">
-        <v>724.7938413077377</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I96" t="n">
-        <v>681.3786902134042</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J96" t="n">
-        <v>441.2608397822005</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K96" t="n">
-        <v>291.4527846761434</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D97" t="n">
         <v>1000</v>
       </c>
       <c r="E97" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F97" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G97" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H97" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I97" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J97" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K97" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
@@ -12742,36 +12804,36 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D98" t="n">
         <v>1000</v>
       </c>
       <c r="E98" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F98" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G98" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H98" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I98" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J98" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K98" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
@@ -12779,36 +12841,36 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D99" t="n">
         <v>1000</v>
       </c>
       <c r="E99" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F99" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G99" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H99" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I99" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J99" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K99" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -12816,73 +12878,73 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D100" t="n">
         <v>1000</v>
       </c>
       <c r="E100" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F100" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G100" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H100" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I100" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J100" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K100" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D101" t="n">
         <v>1000</v>
       </c>
       <c r="E101" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F101" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G101" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H101" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I101" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J101" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K101" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -12919,81 +12981,81 @@
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D103" t="n">
         <v>1000</v>
       </c>
       <c r="E103" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F103" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G103" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H103" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I103" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J103" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K103" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D104" t="n">
         <v>1000</v>
       </c>
       <c r="E104" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F104" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G104" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H104" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I104" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J104" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K104" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
@@ -13001,36 +13063,36 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D105" t="n">
         <v>1000</v>
       </c>
       <c r="E105" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F105" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G105" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H105" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I105" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J105" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K105" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -13038,30 +13100,67 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D106" t="n">
         <v>1000</v>
       </c>
       <c r="E106" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F106" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G106" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H106" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I106" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J106" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K106" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>41</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D107" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E107" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F106" t="n">
+      <c r="F107" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G106" t="n">
+      <c r="G107" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H106" t="n">
+      <c r="H107" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I106" t="n">
+      <c r="I107" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J106" t="n">
+      <c r="J107" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K106" t="n">
+      <c r="K107" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 108 iTransformer baseline -1.41 (FX result reproduced; F4 +2.89 alpha but mass-variance)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$109</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>110</row>
+      <row>111</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T108"/>
+  <dimension ref="A1:T109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8539,16 +8539,16 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>35</v>
+        <v>108</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8557,60 +8557,60 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>-1.4347</v>
+        <v>-1.4054</v>
       </c>
       <c r="F98" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6131</v>
       </c>
       <c r="G98" t="n">
-        <v>-0.8347</v>
+        <v>-0.9054</v>
       </c>
       <c r="I98" t="n">
-        <v>-70.84999999999999</v>
+        <v>-49.86</v>
       </c>
       <c r="J98" t="n">
-        <v>291.5000000000001</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N98" t="n">
-        <v>0.0284</v>
+        <v>0.0074</v>
       </c>
       <c r="O98" t="n">
-        <v>44.07</v>
+        <v>44.37</v>
       </c>
       <c r="P98" t="n">
-        <v>0.5588</v>
+        <v>0.6127</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.1177</v>
+        <v>0.1688</v>
       </c>
       <c r="R98" t="n">
-        <v>0.1945</v>
+        <v>0.2647</v>
       </c>
       <c r="S98" t="n">
-        <v>-0.0101</v>
+        <v>0.0182</v>
       </c>
       <c r="T98" t="n">
-        <v>79.8</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8619,39 +8619,51 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F99" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G99" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I99" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J99" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K99" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N99" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O99" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P99" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R99" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S99" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T99" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -8660,7 +8672,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8669,51 +8681,39 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F100" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G100" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I100" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J100" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K100" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L100" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N100" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O100" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P100" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q100" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R100" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S100" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T100" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -8722,7 +8722,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8731,51 +8731,51 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F101" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G101" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I101" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J101" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L101" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N101" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O101" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P101" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q101" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R101" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S101" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T101" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -8793,113 +8793,113 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F102" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G102" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I102" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J102" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K102" t="n">
         <v>1</v>
       </c>
       <c r="L102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N102" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O102" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P102" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q102" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R102" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S102" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T102" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
+        <v>59</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F103" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G103" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I103" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J103" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K103" t="n">
         <v>1</v>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C103" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E103" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F103" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G103" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I103" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J103" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K103" t="n">
-        <v>5</v>
       </c>
       <c r="L103" t="n">
         <v>1</v>
       </c>
       <c r="N103" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O103" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P103" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R103" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S103" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T103" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -8908,12 +8908,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -8956,21 +8956,21 @@
         <v>0.0098</v>
       </c>
       <c r="T104" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -8979,19 +8979,19 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F105" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G105" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I105" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J105" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K105" t="n">
         <v>5</v>
@@ -9000,39 +9000,39 @@
         <v>1</v>
       </c>
       <c r="N105" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O105" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P105" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q105" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R105" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S105" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T105" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9041,113 +9041,113 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F106" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G106" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I106" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J106" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K106" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L106" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N106" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O106" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P106" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q106" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R106" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S106" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T106" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
+        <v>22</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F107" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G107" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I107" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J107" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K107" t="n">
+        <v>4</v>
+      </c>
+      <c r="L107" t="n">
         <v>2</v>
       </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E107" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F107" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G107" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I107" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J107" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K107" t="n">
-        <v>5</v>
-      </c>
-      <c r="L107" t="n">
-        <v>1</v>
-      </c>
       <c r="N107" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O107" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P107" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q107" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R107" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S107" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T107" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -9156,7 +9156,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9165,51 +9165,113 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F108" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G108" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I108" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J108" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K108" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L108" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N108" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O108" t="n">
         <v>47.65</v>
       </c>
       <c r="P108" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R108" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S108" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T108" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>41</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F109" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G109" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I109" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J109" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K109" t="n">
+        <v>4</v>
+      </c>
+      <c r="L109" t="n">
+        <v>2</v>
+      </c>
+      <c r="N109" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O109" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P109" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q108" t="n">
+      <c r="Q109" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R108" t="n">
+      <c r="R109" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S108" t="n">
+      <c r="S109" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T108" t="n">
+      <c r="T109" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T108"/>
-  <conditionalFormatting sqref="E2:E108">
+  <autoFilter ref="A1:T109"/>
+  <conditionalFormatting sqref="E2:E109">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -9231,7 +9293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K108"/>
+  <dimension ref="A1:K109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12858,81 +12920,81 @@
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>35</v>
+        <v>108</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-1.4347</v>
+        <v>-1.4054</v>
       </c>
       <c r="D98" t="n">
         <v>1000</v>
       </c>
       <c r="E98" t="n">
-        <v>743.8000000000001</v>
+        <v>951.8</v>
       </c>
       <c r="F98" t="n">
-        <v>692.62656</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G98" t="n">
-        <v>666.7223266560001</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H98" t="n">
-        <v>724.7938413077377</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I98" t="n">
-        <v>681.3786902134042</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J98" t="n">
-        <v>441.2608397822005</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K98" t="n">
-        <v>291.4527846761434</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D99" t="n">
         <v>1000</v>
       </c>
       <c r="E99" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F99" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G99" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H99" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I99" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J99" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K99" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -12940,36 +13002,36 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D100" t="n">
         <v>1000</v>
       </c>
       <c r="E100" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F100" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G100" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H100" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I100" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J100" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K100" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
@@ -12977,36 +13039,36 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D101" t="n">
         <v>1000</v>
       </c>
       <c r="E101" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F101" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G101" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H101" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I101" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J101" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K101" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -13014,73 +13076,73 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D102" t="n">
         <v>1000</v>
       </c>
       <c r="E102" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F102" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G102" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H102" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I102" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J102" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K102" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D103" t="n">
         <v>1000</v>
       </c>
       <c r="E103" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F103" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G103" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H103" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I103" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J103" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K103" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -13117,81 +13179,81 @@
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D105" t="n">
         <v>1000</v>
       </c>
       <c r="E105" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F105" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G105" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H105" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I105" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J105" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K105" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D106" t="n">
         <v>1000</v>
       </c>
       <c r="E106" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F106" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G106" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H106" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I106" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J106" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K106" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -13199,36 +13261,36 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D107" t="n">
         <v>1000</v>
       </c>
       <c r="E107" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F107" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G107" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H107" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I107" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J107" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K107" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -13236,30 +13298,67 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D108" t="n">
         <v>1000</v>
       </c>
       <c r="E108" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F108" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G108" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H108" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I108" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J108" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K108" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>41</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D109" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E109" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F108" t="n">
+      <c r="F109" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G108" t="n">
+      <c r="G109" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H108" t="n">
+      <c r="H109" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I108" t="n">
+      <c r="I109" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J108" t="n">
+      <c r="J109" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K108" t="n">
+      <c r="K109" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 110 PatchTST -1.42 (FX failure mode reproduced)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>112</row>
+      <row>113</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T110"/>
+  <dimension ref="A1:T111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8663,16 +8663,16 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8681,60 +8681,60 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="F100" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.8189</v>
       </c>
       <c r="G100" t="n">
-        <v>-0.8347</v>
+        <v>1.1456</v>
       </c>
       <c r="I100" t="n">
-        <v>-70.84999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J100" t="n">
-        <v>291.5000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K100" t="n">
         <v>1</v>
       </c>
       <c r="L100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N100" t="n">
-        <v>0.0284</v>
+        <v>0.0089</v>
       </c>
       <c r="O100" t="n">
-        <v>44.07</v>
+        <v>41.44</v>
       </c>
       <c r="P100" t="n">
-        <v>0.5588</v>
+        <v>0.68</v>
       </c>
       <c r="Q100" t="n">
-        <v>0.1177</v>
+        <v>0.0271</v>
       </c>
       <c r="R100" t="n">
-        <v>0.1945</v>
+        <v>0.0521</v>
       </c>
       <c r="S100" t="n">
-        <v>-0.0101</v>
+        <v>0.0277</v>
       </c>
       <c r="T100" t="n">
-        <v>79.8</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8743,39 +8743,51 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F101" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G101" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I101" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J101" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K101" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N101" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O101" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P101" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R101" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S101" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T101" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -8784,7 +8796,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -8793,51 +8805,39 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F102" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G102" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I102" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J102" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K102" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L102" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N102" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O102" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P102" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q102" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R102" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S102" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T102" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8846,7 +8846,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8855,51 +8855,51 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F103" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G103" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I103" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J103" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L103" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N103" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O103" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P103" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R103" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S103" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T103" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -8908,7 +8908,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -8917,113 +8917,113 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F104" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G104" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I104" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J104" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K104" t="n">
         <v>1</v>
       </c>
       <c r="L104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N104" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O104" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P104" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q104" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R104" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S104" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T104" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
+        <v>59</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F105" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G105" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I105" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J105" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K105" t="n">
         <v>1</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C105" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E105" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F105" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G105" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I105" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J105" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K105" t="n">
-        <v>5</v>
       </c>
       <c r="L105" t="n">
         <v>1</v>
       </c>
       <c r="N105" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O105" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P105" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q105" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R105" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S105" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T105" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -9032,12 +9032,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E106" t="n">
@@ -9080,21 +9080,21 @@
         <v>0.0098</v>
       </c>
       <c r="T106" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9103,19 +9103,19 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F107" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G107" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I107" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J107" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K107" t="n">
         <v>5</v>
@@ -9124,39 +9124,39 @@
         <v>1</v>
       </c>
       <c r="N107" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O107" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P107" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q107" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R107" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S107" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T107" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9165,113 +9165,113 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F108" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G108" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I108" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J108" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K108" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L108" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N108" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O108" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P108" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q108" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R108" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S108" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T108" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
+        <v>22</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F109" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G109" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I109" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J109" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K109" t="n">
+        <v>4</v>
+      </c>
+      <c r="L109" t="n">
         <v>2</v>
       </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E109" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F109" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G109" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I109" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J109" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K109" t="n">
-        <v>5</v>
-      </c>
-      <c r="L109" t="n">
-        <v>1</v>
-      </c>
       <c r="N109" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O109" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P109" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q109" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R109" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S109" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T109" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -9280,7 +9280,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9289,51 +9289,113 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F110" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G110" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I110" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J110" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K110" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L110" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N110" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O110" t="n">
         <v>47.65</v>
       </c>
       <c r="P110" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R110" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S110" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T110" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>41</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F111" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G111" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I111" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J111" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K111" t="n">
+        <v>4</v>
+      </c>
+      <c r="L111" t="n">
+        <v>2</v>
+      </c>
+      <c r="N111" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O111" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P111" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q110" t="n">
+      <c r="Q111" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R110" t="n">
+      <c r="R111" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S110" t="n">
+      <c r="S111" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T110" t="n">
+      <c r="T111" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T110"/>
-  <conditionalFormatting sqref="E2:E110">
+  <autoFilter ref="A1:T111"/>
+  <conditionalFormatting sqref="E2:E111">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -9355,7 +9417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K110"/>
+  <dimension ref="A1:K111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13056,81 +13118,81 @@
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="D100" t="n">
         <v>1000</v>
       </c>
       <c r="E100" t="n">
-        <v>743.8000000000001</v>
+        <v>942</v>
       </c>
       <c r="F100" t="n">
-        <v>692.62656</v>
+        <v>730.2384</v>
       </c>
       <c r="G100" t="n">
-        <v>666.7223266560001</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H100" t="n">
-        <v>724.7938413077377</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I100" t="n">
-        <v>681.3786902134042</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J100" t="n">
-        <v>441.2608397822005</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K100" t="n">
-        <v>291.4527846761434</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D101" t="n">
         <v>1000</v>
       </c>
       <c r="E101" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F101" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G101" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H101" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I101" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J101" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K101" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -13138,36 +13200,36 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D102" t="n">
         <v>1000</v>
       </c>
       <c r="E102" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F102" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G102" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H102" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I102" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J102" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K102" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -13175,36 +13237,36 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D103" t="n">
         <v>1000</v>
       </c>
       <c r="E103" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F103" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G103" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H103" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I103" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J103" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K103" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -13212,73 +13274,73 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D104" t="n">
         <v>1000</v>
       </c>
       <c r="E104" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F104" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G104" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H104" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I104" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J104" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K104" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D105" t="n">
         <v>1000</v>
       </c>
       <c r="E105" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F105" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G105" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H105" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I105" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J105" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K105" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
@@ -13315,81 +13377,81 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D107" t="n">
         <v>1000</v>
       </c>
       <c r="E107" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F107" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G107" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H107" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I107" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J107" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K107" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D108" t="n">
         <v>1000</v>
       </c>
       <c r="E108" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F108" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G108" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H108" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I108" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J108" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K108" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -13397,36 +13459,36 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D109" t="n">
         <v>1000</v>
       </c>
       <c r="E109" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F109" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G109" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H109" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I109" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J109" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K109" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -13434,30 +13496,67 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D110" t="n">
         <v>1000</v>
       </c>
       <c r="E110" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F110" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G110" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H110" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I110" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J110" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K110" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>41</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D111" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E111" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F110" t="n">
+      <c r="F111" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G110" t="n">
+      <c r="G111" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H110" t="n">
+      <c r="H111" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I110" t="n">
+      <c r="I111" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J110" t="n">
+      <c r="J111" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K110" t="n">
+      <c r="K111" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 117 LSTM+features seed=42 -0.88 (features HURT LSTM, opposite of MLP)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$118</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>119</row>
+      <row>120</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T117"/>
+  <dimension ref="A1:T118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8167,16 +8167,16 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>18</v>
+        <v>117</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
+          <t>LSTM 1-layer + new features seed=42 - 2nd seed feature-impact assessment</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -8185,19 +8185,19 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>-0.9217</v>
+        <v>-0.8773</v>
       </c>
       <c r="F92" t="n">
-        <v>0.5942</v>
+        <v>0.388</v>
       </c>
       <c r="G92" t="n">
-        <v>-0.7217</v>
+        <v>-0.6773</v>
       </c>
       <c r="I92" t="n">
-        <v>58.5</v>
+        <v>46.95</v>
       </c>
       <c r="J92" t="n">
-        <v>1585</v>
+        <v>1469.5</v>
       </c>
       <c r="K92" t="n">
         <v>5</v>
@@ -8206,39 +8206,39 @@
         <v>2</v>
       </c>
       <c r="N92" t="n">
-        <v>0.019</v>
+        <v>0.0197</v>
       </c>
       <c r="O92" t="n">
-        <v>48.5</v>
+        <v>47.05</v>
       </c>
       <c r="P92" t="n">
-        <v>0.5986</v>
+        <v>0.5664</v>
       </c>
       <c r="Q92" t="n">
-        <v>0.3987</v>
+        <v>0.3222</v>
       </c>
       <c r="R92" t="n">
-        <v>0.4786</v>
+        <v>0.4107</v>
       </c>
       <c r="S92" t="n">
-        <v>0.0103</v>
+        <v>-0.0083</v>
       </c>
       <c r="T92" t="n">
-        <v>18919.4</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
+          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8247,51 +8247,51 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="F93" t="n">
-        <v>-0.2367</v>
+        <v>0.5942</v>
       </c>
       <c r="G93" t="n">
-        <v>-0.5226</v>
+        <v>-0.7217</v>
       </c>
       <c r="I93" t="n">
-        <v>-43.21</v>
+        <v>58.5</v>
       </c>
       <c r="J93" t="n">
-        <v>567.9000000000001</v>
+        <v>1585</v>
       </c>
       <c r="K93" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L93" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N93" t="n">
-        <v>-0.0164</v>
+        <v>0.019</v>
       </c>
       <c r="O93" t="n">
-        <v>45.63</v>
+        <v>48.5</v>
       </c>
       <c r="P93" t="n">
-        <v>0.5938</v>
+        <v>0.5986</v>
       </c>
       <c r="Q93" t="n">
-        <v>0.1648</v>
+        <v>0.3987</v>
       </c>
       <c r="R93" t="n">
-        <v>0.258</v>
+        <v>0.4786</v>
       </c>
       <c r="S93" t="n">
-        <v>0.0188</v>
+        <v>0.0103</v>
       </c>
       <c r="T93" t="n">
-        <v>33.8</v>
+        <v>18919.4</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -8300,7 +8300,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8309,60 +8309,60 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="F94" t="n">
-        <v>0.1045</v>
+        <v>-0.2367</v>
       </c>
       <c r="G94" t="n">
-        <v>-0.6746</v>
+        <v>-0.5226</v>
       </c>
       <c r="I94" t="n">
-        <v>-4.63</v>
+        <v>-43.21</v>
       </c>
       <c r="J94" t="n">
-        <v>953.7</v>
+        <v>567.9000000000001</v>
       </c>
       <c r="K94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L94" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N94" t="n">
-        <v>-0.0374</v>
+        <v>-0.0164</v>
       </c>
       <c r="O94" t="n">
-        <v>51.03</v>
+        <v>45.63</v>
       </c>
       <c r="P94" t="n">
-        <v>0.5765</v>
+        <v>0.5938</v>
       </c>
       <c r="Q94" t="n">
-        <v>0.5415</v>
+        <v>0.1648</v>
       </c>
       <c r="R94" t="n">
-        <v>0.5585</v>
+        <v>0.258</v>
       </c>
       <c r="S94" t="n">
-        <v>0.0091</v>
+        <v>0.0188</v>
       </c>
       <c r="T94" t="n">
-        <v>30.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -8371,60 +8371,60 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="F95" t="n">
-        <v>0.8788</v>
+        <v>0.1045</v>
       </c>
       <c r="G95" t="n">
-        <v>-0.866</v>
+        <v>-0.6746</v>
       </c>
       <c r="I95" t="n">
-        <v>107.82</v>
+        <v>-4.63</v>
       </c>
       <c r="J95" t="n">
-        <v>2078.2</v>
+        <v>953.7</v>
       </c>
       <c r="K95" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L95" t="n">
         <v>2</v>
       </c>
       <c r="N95" t="n">
-        <v>0.0329</v>
+        <v>-0.0374</v>
       </c>
       <c r="O95" t="n">
-        <v>54.14</v>
+        <v>51.03</v>
       </c>
       <c r="P95" t="n">
-        <v>0.6011</v>
+        <v>0.5765</v>
       </c>
       <c r="Q95" t="n">
-        <v>0.6725</v>
+        <v>0.5415</v>
       </c>
       <c r="R95" t="n">
-        <v>0.6348</v>
+        <v>0.5585</v>
       </c>
       <c r="S95" t="n">
-        <v>0.0251</v>
+        <v>0.0091</v>
       </c>
       <c r="T95" t="n">
-        <v>75.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8433,51 +8433,51 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F96" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G96" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I96" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J96" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K96" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L96" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N96" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O96" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P96" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q96" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R96" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S96" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T96" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -8486,7 +8486,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8495,60 +8495,60 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F97" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G97" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I97" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J97" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K97" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N97" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O97" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P97" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q97" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R97" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S97" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T97" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8557,60 +8557,60 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F98" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G98" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I98" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J98" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K98" t="n">
         <v>2</v>
       </c>
       <c r="L98" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N98" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O98" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P98" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R98" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S98" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T98" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8619,60 +8619,60 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F99" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G99" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I99" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J99" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K99" t="n">
+        <v>2</v>
+      </c>
+      <c r="L99" t="n">
         <v>5</v>
       </c>
-      <c r="L99" t="n">
-        <v>2</v>
-      </c>
       <c r="N99" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O99" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P99" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q99" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R99" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S99" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T99" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8681,60 +8681,60 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F100" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G100" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I100" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J100" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K100" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L100" t="n">
         <v>2</v>
       </c>
       <c r="N100" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O100" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P100" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q100" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R100" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S100" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T100" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8743,51 +8743,51 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F101" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G101" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I101" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J101" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K101" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L101" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N101" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O101" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P101" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q101" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R101" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S101" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T101" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -8796,7 +8796,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -8805,51 +8805,51 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F102" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G102" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I102" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J102" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K102" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L102" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N102" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O102" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P102" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q102" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R102" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S102" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T102" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -8858,7 +8858,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8867,60 +8867,60 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F103" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G103" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I103" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J103" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K103" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L103" t="n">
         <v>2</v>
       </c>
       <c r="N103" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O103" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P103" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R103" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S103" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T103" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -8929,60 +8929,60 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F104" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G104" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I104" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J104" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K104" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L104" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N104" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O104" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P104" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q104" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R104" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S104" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T104" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -8991,60 +8991,60 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F105" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G105" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I105" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J105" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K105" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L105" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N105" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O105" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P105" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q105" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R105" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S105" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T105" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9053,60 +9053,60 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F106" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G106" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I106" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J106" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K106" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L106" t="n">
         <v>3</v>
       </c>
       <c r="N106" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O106" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P106" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q106" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R106" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S106" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T106" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9115,60 +9115,60 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="F107" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.8189</v>
       </c>
       <c r="G107" t="n">
-        <v>-0.8347</v>
+        <v>1.1456</v>
       </c>
       <c r="I107" t="n">
-        <v>-70.84999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J107" t="n">
-        <v>291.5000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K107" t="n">
         <v>1</v>
       </c>
       <c r="L107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N107" t="n">
-        <v>0.0284</v>
+        <v>0.0089</v>
       </c>
       <c r="O107" t="n">
-        <v>44.07</v>
+        <v>41.44</v>
       </c>
       <c r="P107" t="n">
-        <v>0.5588</v>
+        <v>0.68</v>
       </c>
       <c r="Q107" t="n">
-        <v>0.1177</v>
+        <v>0.0271</v>
       </c>
       <c r="R107" t="n">
-        <v>0.1945</v>
+        <v>0.0521</v>
       </c>
       <c r="S107" t="n">
-        <v>-0.0101</v>
+        <v>0.0277</v>
       </c>
       <c r="T107" t="n">
-        <v>79.8</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9177,39 +9177,51 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F108" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G108" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I108" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J108" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K108" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N108" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O108" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P108" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R108" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S108" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T108" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -9218,7 +9230,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9227,51 +9239,39 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F109" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G109" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I109" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J109" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K109" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L109" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N109" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O109" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P109" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q109" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R109" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S109" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T109" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -9280,7 +9280,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9289,51 +9289,51 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F110" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G110" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I110" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J110" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L110" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N110" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O110" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P110" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q110" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R110" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S110" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T110" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -9342,7 +9342,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9351,113 +9351,113 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F111" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G111" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I111" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J111" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K111" t="n">
         <v>1</v>
       </c>
       <c r="L111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N111" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O111" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P111" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q111" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R111" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S111" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T111" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
+        <v>59</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F112" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G112" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I112" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J112" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K112" t="n">
         <v>1</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E112" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F112" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G112" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I112" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J112" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K112" t="n">
-        <v>5</v>
       </c>
       <c r="L112" t="n">
         <v>1</v>
       </c>
       <c r="N112" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O112" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P112" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q112" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R112" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S112" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T112" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -9466,12 +9466,12 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -9514,21 +9514,21 @@
         <v>0.0098</v>
       </c>
       <c r="T113" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -9537,19 +9537,19 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F114" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G114" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I114" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J114" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K114" t="n">
         <v>5</v>
@@ -9558,39 +9558,39 @@
         <v>1</v>
       </c>
       <c r="N114" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O114" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P114" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q114" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R114" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S114" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T114" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -9599,113 +9599,113 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F115" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G115" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I115" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J115" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K115" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L115" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N115" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O115" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P115" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q115" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R115" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S115" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T115" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
+        <v>22</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F116" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G116" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I116" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J116" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K116" t="n">
+        <v>4</v>
+      </c>
+      <c r="L116" t="n">
         <v>2</v>
       </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E116" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F116" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G116" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I116" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J116" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K116" t="n">
-        <v>5</v>
-      </c>
-      <c r="L116" t="n">
-        <v>1</v>
-      </c>
       <c r="N116" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O116" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P116" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q116" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R116" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S116" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T116" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -9723,51 +9723,113 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F117" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G117" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I117" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J117" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K117" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L117" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N117" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O117" t="n">
         <v>47.65</v>
       </c>
       <c r="P117" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R117" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S117" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T117" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>41</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F118" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G118" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I118" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J118" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K118" t="n">
+        <v>4</v>
+      </c>
+      <c r="L118" t="n">
+        <v>2</v>
+      </c>
+      <c r="N118" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O118" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P118" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q117" t="n">
+      <c r="Q118" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R117" t="n">
+      <c r="R118" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S117" t="n">
+      <c r="S118" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T117" t="n">
+      <c r="T118" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T117"/>
-  <conditionalFormatting sqref="E2:E117">
+  <autoFilter ref="A1:T118"/>
+  <conditionalFormatting sqref="E2:E118">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -9789,7 +9851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K117"/>
+  <dimension ref="A1:K118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13194,81 +13256,81 @@
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>18</v>
+        <v>117</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>-0.9217</v>
+        <v>-0.8773</v>
       </c>
       <c r="D92" t="n">
         <v>1000</v>
       </c>
       <c r="E92" t="n">
-        <v>1206.3</v>
+        <v>813.4</v>
       </c>
       <c r="F92" t="n">
-        <v>1403.65068</v>
+        <v>777.12236</v>
       </c>
       <c r="G92" t="n">
-        <v>1572.930952008</v>
+        <v>782.873065464</v>
       </c>
       <c r="H92" t="n">
-        <v>1622.320983901051</v>
+        <v>886.2905974117942</v>
       </c>
       <c r="I92" t="n">
-        <v>1560.023858119251</v>
+        <v>1154.925277487309</v>
       </c>
       <c r="J92" t="n">
-        <v>2085.595895919627</v>
+        <v>1312.572577864327</v>
       </c>
       <c r="K92" t="n">
-        <v>1584.844321309324</v>
+        <v>1469.425000919113</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="D93" t="n">
         <v>1000</v>
       </c>
       <c r="E93" t="n">
-        <v>1141.9</v>
+        <v>1206.3</v>
       </c>
       <c r="F93" t="n">
-        <v>983.4042799999999</v>
+        <v>1403.65068</v>
       </c>
       <c r="G93" t="n">
-        <v>1002.482323032</v>
+        <v>1572.930952008</v>
       </c>
       <c r="H93" t="n">
-        <v>1006.392004091825</v>
+        <v>1622.320983901051</v>
       </c>
       <c r="I93" t="n">
-        <v>968.1491079363354</v>
+        <v>1560.023858119251</v>
       </c>
       <c r="J93" t="n">
-        <v>739.9563631957411</v>
+        <v>2085.595895919627</v>
       </c>
       <c r="K93" t="n">
-        <v>567.8425131164117</v>
+        <v>1584.844321309324</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
@@ -13276,110 +13338,110 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="D94" t="n">
         <v>1000</v>
       </c>
       <c r="E94" t="n">
-        <v>823.5</v>
+        <v>1141.9</v>
       </c>
       <c r="F94" t="n">
-        <v>939.36645</v>
+        <v>983.4042799999999</v>
       </c>
       <c r="G94" t="n">
-        <v>1037.24843409</v>
+        <v>1002.482323032</v>
       </c>
       <c r="H94" t="n">
-        <v>968.582587753242</v>
+        <v>1006.392004091825</v>
       </c>
       <c r="I94" t="n">
-        <v>996.38090802176</v>
+        <v>968.1491079363354</v>
       </c>
       <c r="J94" t="n">
-        <v>1251.255144293726</v>
+        <v>739.9563631957411</v>
       </c>
       <c r="K94" t="n">
-        <v>953.7066709806782</v>
+        <v>567.8425131164117</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="D95" t="n">
         <v>1000</v>
       </c>
       <c r="E95" t="n">
-        <v>1390.6</v>
+        <v>823.5</v>
       </c>
       <c r="F95" t="n">
-        <v>1715.16604</v>
+        <v>939.36645</v>
       </c>
       <c r="G95" t="n">
-        <v>1928.018145564</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H95" t="n">
-        <v>1842.799743530072</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I95" t="n">
-        <v>1932.359811065633</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J95" t="n">
-        <v>2502.212719348888</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K95" t="n">
-        <v>2078.337884691186</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D96" t="n">
         <v>1000</v>
       </c>
       <c r="E96" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F96" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G96" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H96" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I96" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J96" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K96" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
@@ -13387,184 +13449,184 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D97" t="n">
         <v>1000</v>
       </c>
       <c r="E97" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F97" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G97" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H97" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I97" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J97" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K97" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D98" t="n">
         <v>1000</v>
       </c>
       <c r="E98" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F98" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G98" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H98" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I98" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J98" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K98" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D99" t="n">
         <v>1000</v>
       </c>
       <c r="E99" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F99" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G99" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H99" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I99" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J99" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K99" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D100" t="n">
         <v>1000</v>
       </c>
       <c r="E100" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F100" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G100" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H100" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I100" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J100" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K100" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D101" t="n">
         <v>1000</v>
       </c>
       <c r="E101" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F101" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G101" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H101" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I101" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J101" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K101" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
@@ -13572,36 +13634,36 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D102" t="n">
         <v>1000</v>
       </c>
       <c r="E102" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F102" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G102" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H102" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I102" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J102" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K102" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
@@ -13609,221 +13671,221 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D103" t="n">
         <v>1000</v>
       </c>
       <c r="E103" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F103" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G103" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H103" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I103" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J103" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K103" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D104" t="n">
         <v>1000</v>
       </c>
       <c r="E104" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F104" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G104" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H104" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I104" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J104" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K104" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D105" t="n">
         <v>1000</v>
       </c>
       <c r="E105" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F105" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G105" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H105" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I105" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J105" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K105" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D106" t="n">
         <v>1000</v>
       </c>
       <c r="E106" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F106" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G106" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H106" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I106" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J106" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K106" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="D107" t="n">
         <v>1000</v>
       </c>
       <c r="E107" t="n">
-        <v>743.8000000000001</v>
+        <v>942</v>
       </c>
       <c r="F107" t="n">
-        <v>692.62656</v>
+        <v>730.2384</v>
       </c>
       <c r="G107" t="n">
-        <v>666.7223266560001</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H107" t="n">
-        <v>724.7938413077377</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I107" t="n">
-        <v>681.3786902134042</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J107" t="n">
-        <v>441.2608397822005</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K107" t="n">
-        <v>291.4527846761434</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D108" t="n">
         <v>1000</v>
       </c>
       <c r="E108" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F108" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G108" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H108" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I108" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J108" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K108" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -13831,36 +13893,36 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D109" t="n">
         <v>1000</v>
       </c>
       <c r="E109" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F109" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G109" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H109" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I109" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J109" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K109" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -13868,36 +13930,36 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D110" t="n">
         <v>1000</v>
       </c>
       <c r="E110" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F110" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G110" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H110" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I110" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J110" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K110" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -13905,73 +13967,73 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D111" t="n">
         <v>1000</v>
       </c>
       <c r="E111" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F111" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G111" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H111" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I111" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J111" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K111" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D112" t="n">
         <v>1000</v>
       </c>
       <c r="E112" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F112" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G112" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H112" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I112" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J112" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K112" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -14008,81 +14070,81 @@
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D114" t="n">
         <v>1000</v>
       </c>
       <c r="E114" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F114" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G114" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H114" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I114" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J114" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K114" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D115" t="n">
         <v>1000</v>
       </c>
       <c r="E115" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F115" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G115" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H115" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I115" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J115" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K115" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -14090,36 +14152,36 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D116" t="n">
         <v>1000</v>
       </c>
       <c r="E116" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F116" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G116" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H116" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I116" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J116" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K116" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -14127,30 +14189,67 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D117" t="n">
         <v>1000</v>
       </c>
       <c r="E117" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F117" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G117" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H117" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I117" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J117" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K117" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>41</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D118" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E118" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F117" t="n">
+      <c r="F118" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G117" t="n">
+      <c r="G118" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H117" t="n">
+      <c r="H118" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I117" t="n">
+      <c r="I118" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J117" t="n">
+      <c r="J118" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K117" t="n">
+      <c r="K118" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 127 MLP+features lr=1e-4 seed=0 -0.84 (exp 126 was lucky seed)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$127</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$128</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>129</row>
+      <row>130</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T127"/>
+  <dimension ref="A1:T128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8477,16 +8477,16 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.02 n_est=500 - smaller capacity at productive lr</t>
+          <t>MLP @ exp 126 lr=1e-4 + features seed=0 - 2nd seed verify</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8495,60 +8495,60 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>-0.8456</v>
+        <v>-0.8429</v>
       </c>
       <c r="F97" t="n">
-        <v>0.2334</v>
+        <v>0.3863</v>
       </c>
       <c r="G97" t="n">
-        <v>-0.4456</v>
+        <v>-0.6429</v>
       </c>
       <c r="I97" t="n">
-        <v>12.26</v>
+        <v>46.31</v>
       </c>
       <c r="J97" t="n">
-        <v>1122.6</v>
+        <v>1463.1</v>
       </c>
       <c r="K97" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L97" t="n">
         <v>2</v>
       </c>
       <c r="N97" t="n">
-        <v>0.0108</v>
+        <v>0.0055</v>
       </c>
       <c r="O97" t="n">
-        <v>49.72</v>
+        <v>51.67</v>
       </c>
       <c r="P97" t="n">
-        <v>0.5938</v>
+        <v>0.5765</v>
       </c>
       <c r="Q97" t="n">
-        <v>0.481</v>
+        <v>0.5836</v>
       </c>
       <c r="R97" t="n">
-        <v>0.5315</v>
+        <v>0.58</v>
       </c>
       <c r="S97" t="n">
-        <v>0.0028</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="T97" t="n">
-        <v>673.8</v>
+        <v>49.6</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">dMamba @ FX-Mamba-winner config seed=99 — 3rd seed for stable champion declaration (seeds </t>
+          <t>CatBoost lr=0.02 n_est=500 - smaller capacity at productive lr</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -8557,60 +8557,60 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>-0.862</v>
+        <v>-0.8456</v>
       </c>
       <c r="F98" t="n">
-        <v>-0.462</v>
+        <v>0.2334</v>
       </c>
       <c r="G98" t="n">
-        <v>1.3122</v>
+        <v>-0.4456</v>
       </c>
       <c r="I98" t="n">
-        <v>-42.07</v>
+        <v>12.26</v>
       </c>
       <c r="J98" t="n">
-        <v>579.3</v>
+        <v>1122.6</v>
       </c>
       <c r="K98" t="n">
         <v>3</v>
       </c>
       <c r="L98" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N98" t="n">
-        <v>0.0467</v>
+        <v>0.0108</v>
       </c>
       <c r="O98" t="n">
-        <v>43.33</v>
+        <v>49.72</v>
       </c>
       <c r="P98" t="n">
-        <v>0.5858</v>
+        <v>0.5938</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.1576</v>
+        <v>0.481</v>
       </c>
       <c r="R98" t="n">
-        <v>0.2484</v>
+        <v>0.5315</v>
       </c>
       <c r="S98" t="n">
-        <v>-0.0059</v>
+        <v>0.0028</v>
       </c>
       <c r="T98" t="n">
-        <v>705.3</v>
+        <v>673.8</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>CatBoost depth=6 lr=0.01 n_est=1000 - depth axis test</t>
+          <t xml:space="preserve">dMamba @ FX-Mamba-winner config seed=99 — 3rd seed for stable champion declaration (seeds </t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8619,51 +8619,51 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>-0.8688</v>
+        <v>-0.862</v>
       </c>
       <c r="F99" t="n">
-        <v>0.7087</v>
+        <v>-0.462</v>
       </c>
       <c r="G99" t="n">
-        <v>-0.6688</v>
+        <v>1.3122</v>
       </c>
       <c r="I99" t="n">
-        <v>76.76000000000001</v>
+        <v>-42.07</v>
       </c>
       <c r="J99" t="n">
-        <v>1767.6</v>
+        <v>579.3</v>
       </c>
       <c r="K99" t="n">
+        <v>3</v>
+      </c>
+      <c r="L99" t="n">
         <v>5</v>
       </c>
-      <c r="L99" t="n">
-        <v>1</v>
-      </c>
       <c r="N99" t="n">
-        <v>0.0031</v>
+        <v>0.0467</v>
       </c>
       <c r="O99" t="n">
-        <v>49.34</v>
+        <v>43.33</v>
       </c>
       <c r="P99" t="n">
-        <v>0.5827</v>
+        <v>0.5858</v>
       </c>
       <c r="Q99" t="n">
-        <v>0.5127</v>
+        <v>0.1576</v>
       </c>
       <c r="R99" t="n">
-        <v>0.5455</v>
+        <v>0.2484</v>
       </c>
       <c r="S99" t="n">
-        <v>-0.0203</v>
+        <v>-0.0059</v>
       </c>
       <c r="T99" t="n">
-        <v>4289.1</v>
+        <v>705.3</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -8672,7 +8672,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.02 n_est=2000 - combine best CatBoost findings (lr from exp 98, capacity fro</t>
+          <t>CatBoost depth=6 lr=0.01 n_est=1000 - depth axis test</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8681,60 +8681,60 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>-0.8764</v>
+        <v>-0.8688</v>
       </c>
       <c r="F100" t="n">
-        <v>-0.1626</v>
+        <v>0.7087</v>
       </c>
       <c r="G100" t="n">
-        <v>-0.4764</v>
+        <v>-0.6688</v>
       </c>
       <c r="I100" t="n">
-        <v>-23.11</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="J100" t="n">
-        <v>768.9</v>
+        <v>1767.6</v>
       </c>
       <c r="K100" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L100" t="n">
         <v>1</v>
       </c>
       <c r="N100" t="n">
-        <v>0.0008</v>
+        <v>0.0031</v>
       </c>
       <c r="O100" t="n">
-        <v>46.43</v>
+        <v>49.34</v>
       </c>
       <c r="P100" t="n">
-        <v>0.5760999999999999</v>
+        <v>0.5827</v>
       </c>
       <c r="Q100" t="n">
-        <v>0.3655</v>
+        <v>0.5127</v>
       </c>
       <c r="R100" t="n">
-        <v>0.4472</v>
+        <v>0.5455</v>
       </c>
       <c r="S100" t="n">
-        <v>-0.0257</v>
+        <v>-0.0203</v>
       </c>
       <c r="T100" t="n">
-        <v>2594.9</v>
+        <v>4289.1</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LSTM 1-layer + new features seed=42 - 2nd seed feature-impact assessment</t>
+          <t>CatBoost lr=0.02 n_est=2000 - combine best CatBoost findings (lr from exp 98, capacity fro</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8743,60 +8743,60 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>-0.8773</v>
+        <v>-0.8764</v>
       </c>
       <c r="F101" t="n">
-        <v>0.388</v>
+        <v>-0.1626</v>
       </c>
       <c r="G101" t="n">
-        <v>-0.6773</v>
+        <v>-0.4764</v>
       </c>
       <c r="I101" t="n">
-        <v>46.95</v>
+        <v>-23.11</v>
       </c>
       <c r="J101" t="n">
-        <v>1469.5</v>
+        <v>768.9</v>
       </c>
       <c r="K101" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L101" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N101" t="n">
-        <v>0.0197</v>
+        <v>0.0008</v>
       </c>
       <c r="O101" t="n">
-        <v>47.05</v>
+        <v>46.43</v>
       </c>
       <c r="P101" t="n">
-        <v>0.5664</v>
+        <v>0.5760999999999999</v>
       </c>
       <c r="Q101" t="n">
-        <v>0.3222</v>
+        <v>0.3655</v>
       </c>
       <c r="R101" t="n">
-        <v>0.4107</v>
+        <v>0.4472</v>
       </c>
       <c r="S101" t="n">
-        <v>-0.0083</v>
+        <v>-0.0257</v>
       </c>
       <c r="T101" t="n">
-        <v>74.59999999999999</v>
+        <v>2594.9</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>18</v>
+        <v>117</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
+          <t>LSTM 1-layer + new features seed=42 - 2nd seed feature-impact assessment</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -8805,19 +8805,19 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>-0.9217</v>
+        <v>-0.8773</v>
       </c>
       <c r="F102" t="n">
-        <v>0.5942</v>
+        <v>0.388</v>
       </c>
       <c r="G102" t="n">
-        <v>-0.7217</v>
+        <v>-0.6773</v>
       </c>
       <c r="I102" t="n">
-        <v>58.5</v>
+        <v>46.95</v>
       </c>
       <c r="J102" t="n">
-        <v>1585</v>
+        <v>1469.5</v>
       </c>
       <c r="K102" t="n">
         <v>5</v>
@@ -8826,39 +8826,39 @@
         <v>2</v>
       </c>
       <c r="N102" t="n">
-        <v>0.019</v>
+        <v>0.0197</v>
       </c>
       <c r="O102" t="n">
-        <v>48.5</v>
+        <v>47.05</v>
       </c>
       <c r="P102" t="n">
-        <v>0.5986</v>
+        <v>0.5664</v>
       </c>
       <c r="Q102" t="n">
-        <v>0.3987</v>
+        <v>0.3222</v>
       </c>
       <c r="R102" t="n">
-        <v>0.4786</v>
+        <v>0.4107</v>
       </c>
       <c r="S102" t="n">
-        <v>0.0103</v>
+        <v>-0.0083</v>
       </c>
       <c r="T102" t="n">
-        <v>18919.4</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
+          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8867,51 +8867,51 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="F103" t="n">
-        <v>-0.2367</v>
+        <v>0.5942</v>
       </c>
       <c r="G103" t="n">
-        <v>-0.5226</v>
+        <v>-0.7217</v>
       </c>
       <c r="I103" t="n">
-        <v>-43.21</v>
+        <v>58.5</v>
       </c>
       <c r="J103" t="n">
-        <v>567.9000000000001</v>
+        <v>1585</v>
       </c>
       <c r="K103" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L103" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N103" t="n">
-        <v>-0.0164</v>
+        <v>0.019</v>
       </c>
       <c r="O103" t="n">
-        <v>45.63</v>
+        <v>48.5</v>
       </c>
       <c r="P103" t="n">
-        <v>0.5938</v>
+        <v>0.5986</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.1648</v>
+        <v>0.3987</v>
       </c>
       <c r="R103" t="n">
-        <v>0.258</v>
+        <v>0.4786</v>
       </c>
       <c r="S103" t="n">
-        <v>0.0188</v>
+        <v>0.0103</v>
       </c>
       <c r="T103" t="n">
-        <v>33.8</v>
+        <v>18919.4</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -8920,7 +8920,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -8929,60 +8929,60 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="F104" t="n">
-        <v>0.1045</v>
+        <v>-0.2367</v>
       </c>
       <c r="G104" t="n">
-        <v>-0.6746</v>
+        <v>-0.5226</v>
       </c>
       <c r="I104" t="n">
-        <v>-4.63</v>
+        <v>-43.21</v>
       </c>
       <c r="J104" t="n">
-        <v>953.7</v>
+        <v>567.9000000000001</v>
       </c>
       <c r="K104" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L104" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N104" t="n">
-        <v>-0.0374</v>
+        <v>-0.0164</v>
       </c>
       <c r="O104" t="n">
-        <v>51.03</v>
+        <v>45.63</v>
       </c>
       <c r="P104" t="n">
-        <v>0.5765</v>
+        <v>0.5938</v>
       </c>
       <c r="Q104" t="n">
-        <v>0.5415</v>
+        <v>0.1648</v>
       </c>
       <c r="R104" t="n">
-        <v>0.5585</v>
+        <v>0.258</v>
       </c>
       <c r="S104" t="n">
-        <v>0.0091</v>
+        <v>0.0188</v>
       </c>
       <c r="T104" t="n">
-        <v>30.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -8991,60 +8991,60 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="F105" t="n">
-        <v>0.8788</v>
+        <v>0.1045</v>
       </c>
       <c r="G105" t="n">
-        <v>-0.866</v>
+        <v>-0.6746</v>
       </c>
       <c r="I105" t="n">
-        <v>107.82</v>
+        <v>-4.63</v>
       </c>
       <c r="J105" t="n">
-        <v>2078.2</v>
+        <v>953.7</v>
       </c>
       <c r="K105" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L105" t="n">
         <v>2</v>
       </c>
       <c r="N105" t="n">
-        <v>0.0329</v>
+        <v>-0.0374</v>
       </c>
       <c r="O105" t="n">
-        <v>54.14</v>
+        <v>51.03</v>
       </c>
       <c r="P105" t="n">
-        <v>0.6011</v>
+        <v>0.5765</v>
       </c>
       <c r="Q105" t="n">
-        <v>0.6725</v>
+        <v>0.5415</v>
       </c>
       <c r="R105" t="n">
-        <v>0.6348</v>
+        <v>0.5585</v>
       </c>
       <c r="S105" t="n">
-        <v>0.0251</v>
+        <v>0.0091</v>
       </c>
       <c r="T105" t="n">
-        <v>75.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9053,51 +9053,51 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F106" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G106" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I106" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J106" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K106" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L106" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N106" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O106" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P106" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q106" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R106" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S106" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T106" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -9106,7 +9106,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9115,60 +9115,60 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F107" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G107" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I107" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J107" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K107" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L107" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N107" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O107" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P107" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q107" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R107" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S107" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T107" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9177,60 +9177,60 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F108" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G108" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I108" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J108" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K108" t="n">
         <v>2</v>
       </c>
       <c r="L108" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N108" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O108" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P108" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q108" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R108" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S108" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T108" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9239,60 +9239,60 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F109" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G109" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I109" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J109" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K109" t="n">
+        <v>2</v>
+      </c>
+      <c r="L109" t="n">
         <v>5</v>
       </c>
-      <c r="L109" t="n">
-        <v>2</v>
-      </c>
       <c r="N109" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O109" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P109" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q109" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R109" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S109" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T109" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9301,60 +9301,60 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F110" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G110" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I110" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J110" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K110" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L110" t="n">
         <v>2</v>
       </c>
       <c r="N110" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O110" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P110" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q110" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R110" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S110" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T110" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9363,51 +9363,51 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F111" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G111" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I111" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J111" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K111" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L111" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N111" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O111" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P111" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q111" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R111" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S111" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T111" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -9416,7 +9416,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -9425,51 +9425,51 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F112" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G112" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I112" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J112" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K112" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L112" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N112" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O112" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P112" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q112" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R112" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S112" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T112" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -9478,7 +9478,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -9487,60 +9487,60 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F113" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G113" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I113" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J113" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K113" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L113" t="n">
         <v>2</v>
       </c>
       <c r="N113" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O113" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P113" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q113" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R113" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S113" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T113" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -9549,60 +9549,60 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F114" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G114" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I114" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J114" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K114" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L114" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N114" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O114" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P114" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q114" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R114" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S114" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T114" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -9611,60 +9611,60 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F115" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G115" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I115" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J115" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L115" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N115" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O115" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P115" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q115" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R115" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S115" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T115" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -9673,60 +9673,60 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F116" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G116" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I116" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J116" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L116" t="n">
         <v>3</v>
       </c>
       <c r="N116" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O116" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P116" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q116" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R116" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S116" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T116" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -9735,60 +9735,60 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="F117" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.8189</v>
       </c>
       <c r="G117" t="n">
-        <v>-0.8347</v>
+        <v>1.1456</v>
       </c>
       <c r="I117" t="n">
-        <v>-70.84999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J117" t="n">
-        <v>291.5000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K117" t="n">
         <v>1</v>
       </c>
       <c r="L117" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N117" t="n">
-        <v>0.0284</v>
+        <v>0.0089</v>
       </c>
       <c r="O117" t="n">
-        <v>44.07</v>
+        <v>41.44</v>
       </c>
       <c r="P117" t="n">
-        <v>0.5588</v>
+        <v>0.68</v>
       </c>
       <c r="Q117" t="n">
-        <v>0.1177</v>
+        <v>0.0271</v>
       </c>
       <c r="R117" t="n">
-        <v>0.1945</v>
+        <v>0.0521</v>
       </c>
       <c r="S117" t="n">
-        <v>-0.0101</v>
+        <v>0.0277</v>
       </c>
       <c r="T117" t="n">
-        <v>79.8</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -9797,39 +9797,51 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F118" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G118" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I118" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J118" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K118" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L118" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N118" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O118" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P118" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R118" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S118" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T118" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -9838,7 +9850,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -9847,51 +9859,39 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F119" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G119" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I119" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J119" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K119" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L119" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N119" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O119" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P119" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q119" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R119" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S119" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T119" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -9900,7 +9900,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -9909,51 +9909,51 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F120" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G120" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I120" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J120" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L120" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N120" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O120" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P120" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q120" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R120" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S120" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T120" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -9962,7 +9962,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -9971,113 +9971,113 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F121" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G121" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I121" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J121" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K121" t="n">
         <v>1</v>
       </c>
       <c r="L121" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N121" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O121" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P121" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q121" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R121" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S121" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T121" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
+        <v>59</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F122" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G122" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I122" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J122" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K122" t="n">
         <v>1</v>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C122" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D122" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E122" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F122" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G122" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I122" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J122" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K122" t="n">
-        <v>5</v>
       </c>
       <c r="L122" t="n">
         <v>1</v>
       </c>
       <c r="N122" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O122" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P122" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q122" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R122" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S122" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T122" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -10086,12 +10086,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E123" t="n">
@@ -10134,21 +10134,21 @@
         <v>0.0098</v>
       </c>
       <c r="T123" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -10157,19 +10157,19 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F124" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G124" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I124" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J124" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K124" t="n">
         <v>5</v>
@@ -10178,39 +10178,39 @@
         <v>1</v>
       </c>
       <c r="N124" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O124" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P124" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q124" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R124" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S124" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T124" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -10219,113 +10219,113 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F125" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G125" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I125" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J125" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K125" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L125" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N125" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O125" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P125" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q125" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R125" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S125" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T125" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
+        <v>22</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F126" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G126" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I126" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J126" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K126" t="n">
+        <v>4</v>
+      </c>
+      <c r="L126" t="n">
         <v>2</v>
       </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E126" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F126" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G126" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I126" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J126" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K126" t="n">
-        <v>5</v>
-      </c>
-      <c r="L126" t="n">
-        <v>1</v>
-      </c>
       <c r="N126" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O126" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P126" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q126" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R126" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S126" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T126" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -10334,7 +10334,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -10343,51 +10343,113 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F127" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G127" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I127" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J127" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K127" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L127" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N127" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O127" t="n">
         <v>47.65</v>
       </c>
       <c r="P127" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R127" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S127" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T127" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>41</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F128" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G128" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I128" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J128" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K128" t="n">
+        <v>4</v>
+      </c>
+      <c r="L128" t="n">
+        <v>2</v>
+      </c>
+      <c r="N128" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O128" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P128" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q127" t="n">
+      <c r="Q128" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R127" t="n">
+      <c r="R128" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S127" t="n">
+      <c r="S128" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T127" t="n">
+      <c r="T128" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T127"/>
-  <conditionalFormatting sqref="E2:E127">
+  <autoFilter ref="A1:T128"/>
+  <conditionalFormatting sqref="E2:E128">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -10409,7 +10471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K127"/>
+  <dimension ref="A1:K128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13999,118 +14061,118 @@
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-0.8456</v>
+        <v>-0.8429</v>
       </c>
       <c r="D97" t="n">
         <v>1000</v>
       </c>
       <c r="E97" t="n">
-        <v>953</v>
+        <v>861.6</v>
       </c>
       <c r="F97" t="n">
-        <v>1234.8974</v>
+        <v>960.85632</v>
       </c>
       <c r="G97" t="n">
-        <v>1386.04884176</v>
+        <v>989.7780952319999</v>
       </c>
       <c r="H97" t="n">
-        <v>1167.330334530272</v>
+        <v>1153.289436564326</v>
       </c>
       <c r="I97" t="n">
-        <v>993.3981146852617</v>
+        <v>1482.553570703441</v>
       </c>
       <c r="J97" t="n">
-        <v>1310.689472515734</v>
+        <v>1616.428158137962</v>
       </c>
       <c r="K97" t="n">
-        <v>1122.605533209726</v>
+        <v>1463.190768746483</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-0.862</v>
+        <v>-0.8456</v>
       </c>
       <c r="D98" t="n">
         <v>1000</v>
       </c>
       <c r="E98" t="n">
-        <v>1064.8</v>
+        <v>953</v>
       </c>
       <c r="F98" t="n">
-        <v>857.3769599999999</v>
+        <v>1234.8974</v>
       </c>
       <c r="G98" t="n">
-        <v>754.4917247999999</v>
+        <v>1386.04884176</v>
       </c>
       <c r="H98" t="n">
-        <v>689.30363977728</v>
+        <v>1167.330334530272</v>
       </c>
       <c r="I98" t="n">
-        <v>835.2981506821078</v>
+        <v>993.3981146852617</v>
       </c>
       <c r="J98" t="n">
-        <v>582.2028110254292</v>
+        <v>1310.689472515734</v>
       </c>
       <c r="K98" t="n">
-        <v>579.3500172514047</v>
+        <v>1122.605533209726</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>-0.8688</v>
+        <v>-0.862</v>
       </c>
       <c r="D99" t="n">
         <v>1000</v>
       </c>
       <c r="E99" t="n">
-        <v>1120</v>
+        <v>1064.8</v>
       </c>
       <c r="F99" t="n">
-        <v>1237.6</v>
+        <v>857.3769599999999</v>
       </c>
       <c r="G99" t="n">
-        <v>1385.61696</v>
+        <v>754.4917247999999</v>
       </c>
       <c r="H99" t="n">
-        <v>1253.429102016</v>
+        <v>689.30363977728</v>
       </c>
       <c r="I99" t="n">
-        <v>1143.378026858995</v>
+        <v>835.2981506821078</v>
       </c>
       <c r="J99" t="n">
-        <v>1478.502126531366</v>
+        <v>582.2028110254292</v>
       </c>
       <c r="K99" t="n">
-        <v>1767.549292268249</v>
+        <v>579.3500172514047</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
@@ -14118,147 +14180,147 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-0.8764</v>
+        <v>-0.8688</v>
       </c>
       <c r="D100" t="n">
         <v>1000</v>
       </c>
       <c r="E100" t="n">
-        <v>762</v>
+        <v>1120</v>
       </c>
       <c r="F100" t="n">
-        <v>937.8695999999999</v>
+        <v>1237.6</v>
       </c>
       <c r="G100" t="n">
-        <v>946.9669351199999</v>
+        <v>1385.61696</v>
       </c>
       <c r="H100" t="n">
-        <v>929.2586534332559</v>
+        <v>1253.429102016</v>
       </c>
       <c r="I100" t="n">
-        <v>802.1360696435864</v>
+        <v>1143.378026858995</v>
       </c>
       <c r="J100" t="n">
-        <v>902.5635055629634</v>
+        <v>1478.502126531366</v>
       </c>
       <c r="K100" t="n">
-        <v>768.8035940385322</v>
+        <v>1767.549292268249</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-0.8773</v>
+        <v>-0.8764</v>
       </c>
       <c r="D101" t="n">
         <v>1000</v>
       </c>
       <c r="E101" t="n">
-        <v>813.4</v>
+        <v>762</v>
       </c>
       <c r="F101" t="n">
-        <v>777.12236</v>
+        <v>937.8695999999999</v>
       </c>
       <c r="G101" t="n">
-        <v>782.873065464</v>
+        <v>946.9669351199999</v>
       </c>
       <c r="H101" t="n">
-        <v>886.2905974117942</v>
+        <v>929.2586534332559</v>
       </c>
       <c r="I101" t="n">
-        <v>1154.925277487309</v>
+        <v>802.1360696435864</v>
       </c>
       <c r="J101" t="n">
-        <v>1312.572577864327</v>
+        <v>902.5635055629634</v>
       </c>
       <c r="K101" t="n">
-        <v>1469.425000919113</v>
+        <v>768.8035940385322</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>18</v>
+        <v>117</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>-0.9217</v>
+        <v>-0.8773</v>
       </c>
       <c r="D102" t="n">
         <v>1000</v>
       </c>
       <c r="E102" t="n">
-        <v>1206.3</v>
+        <v>813.4</v>
       </c>
       <c r="F102" t="n">
-        <v>1403.65068</v>
+        <v>777.12236</v>
       </c>
       <c r="G102" t="n">
-        <v>1572.930952008</v>
+        <v>782.873065464</v>
       </c>
       <c r="H102" t="n">
-        <v>1622.320983901051</v>
+        <v>886.2905974117942</v>
       </c>
       <c r="I102" t="n">
-        <v>1560.023858119251</v>
+        <v>1154.925277487309</v>
       </c>
       <c r="J102" t="n">
-        <v>2085.595895919627</v>
+        <v>1312.572577864327</v>
       </c>
       <c r="K102" t="n">
-        <v>1584.844321309324</v>
+        <v>1469.425000919113</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="D103" t="n">
         <v>1000</v>
       </c>
       <c r="E103" t="n">
-        <v>1141.9</v>
+        <v>1206.3</v>
       </c>
       <c r="F103" t="n">
-        <v>983.4042799999999</v>
+        <v>1403.65068</v>
       </c>
       <c r="G103" t="n">
-        <v>1002.482323032</v>
+        <v>1572.930952008</v>
       </c>
       <c r="H103" t="n">
-        <v>1006.392004091825</v>
+        <v>1622.320983901051</v>
       </c>
       <c r="I103" t="n">
-        <v>968.1491079363354</v>
+        <v>1560.023858119251</v>
       </c>
       <c r="J103" t="n">
-        <v>739.9563631957411</v>
+        <v>2085.595895919627</v>
       </c>
       <c r="K103" t="n">
-        <v>567.8425131164117</v>
+        <v>1584.844321309324</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -14266,110 +14328,110 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="D104" t="n">
         <v>1000</v>
       </c>
       <c r="E104" t="n">
-        <v>823.5</v>
+        <v>1141.9</v>
       </c>
       <c r="F104" t="n">
-        <v>939.36645</v>
+        <v>983.4042799999999</v>
       </c>
       <c r="G104" t="n">
-        <v>1037.24843409</v>
+        <v>1002.482323032</v>
       </c>
       <c r="H104" t="n">
-        <v>968.582587753242</v>
+        <v>1006.392004091825</v>
       </c>
       <c r="I104" t="n">
-        <v>996.38090802176</v>
+        <v>968.1491079363354</v>
       </c>
       <c r="J104" t="n">
-        <v>1251.255144293726</v>
+        <v>739.9563631957411</v>
       </c>
       <c r="K104" t="n">
-        <v>953.7066709806782</v>
+        <v>567.8425131164117</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="D105" t="n">
         <v>1000</v>
       </c>
       <c r="E105" t="n">
-        <v>1390.6</v>
+        <v>823.5</v>
       </c>
       <c r="F105" t="n">
-        <v>1715.16604</v>
+        <v>939.36645</v>
       </c>
       <c r="G105" t="n">
-        <v>1928.018145564</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H105" t="n">
-        <v>1842.799743530072</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I105" t="n">
-        <v>1932.359811065633</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J105" t="n">
-        <v>2502.212719348888</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K105" t="n">
-        <v>2078.337884691186</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D106" t="n">
         <v>1000</v>
       </c>
       <c r="E106" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F106" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G106" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H106" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I106" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J106" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K106" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
@@ -14377,184 +14439,184 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D107" t="n">
         <v>1000</v>
       </c>
       <c r="E107" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F107" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G107" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H107" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I107" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J107" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K107" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D108" t="n">
         <v>1000</v>
       </c>
       <c r="E108" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F108" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G108" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H108" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I108" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J108" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K108" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D109" t="n">
         <v>1000</v>
       </c>
       <c r="E109" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F109" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G109" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H109" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I109" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J109" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K109" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D110" t="n">
         <v>1000</v>
       </c>
       <c r="E110" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F110" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G110" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H110" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I110" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J110" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K110" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D111" t="n">
         <v>1000</v>
       </c>
       <c r="E111" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F111" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G111" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H111" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I111" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J111" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K111" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -14562,36 +14624,36 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D112" t="n">
         <v>1000</v>
       </c>
       <c r="E112" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F112" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G112" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H112" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I112" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J112" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K112" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -14599,221 +14661,221 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D113" t="n">
         <v>1000</v>
       </c>
       <c r="E113" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F113" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G113" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H113" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I113" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J113" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K113" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D114" t="n">
         <v>1000</v>
       </c>
       <c r="E114" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F114" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G114" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H114" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I114" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J114" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K114" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D115" t="n">
         <v>1000</v>
       </c>
       <c r="E115" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F115" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G115" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H115" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I115" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J115" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K115" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D116" t="n">
         <v>1000</v>
       </c>
       <c r="E116" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F116" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G116" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H116" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I116" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J116" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K116" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="D117" t="n">
         <v>1000</v>
       </c>
       <c r="E117" t="n">
-        <v>743.8000000000001</v>
+        <v>942</v>
       </c>
       <c r="F117" t="n">
-        <v>692.62656</v>
+        <v>730.2384</v>
       </c>
       <c r="G117" t="n">
-        <v>666.7223266560001</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H117" t="n">
-        <v>724.7938413077377</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I117" t="n">
-        <v>681.3786902134042</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J117" t="n">
-        <v>441.2608397822005</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K117" t="n">
-        <v>291.4527846761434</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D118" t="n">
         <v>1000</v>
       </c>
       <c r="E118" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F118" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G118" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H118" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I118" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J118" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K118" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -14821,36 +14883,36 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D119" t="n">
         <v>1000</v>
       </c>
       <c r="E119" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F119" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G119" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H119" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I119" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J119" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K119" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -14858,36 +14920,36 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D120" t="n">
         <v>1000</v>
       </c>
       <c r="E120" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F120" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G120" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H120" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I120" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J120" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K120" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
@@ -14895,73 +14957,73 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D121" t="n">
         <v>1000</v>
       </c>
       <c r="E121" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F121" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G121" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H121" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I121" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J121" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K121" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D122" t="n">
         <v>1000</v>
       </c>
       <c r="E122" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F122" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G122" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H122" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I122" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J122" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K122" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -14998,81 +15060,81 @@
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D124" t="n">
         <v>1000</v>
       </c>
       <c r="E124" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F124" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G124" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H124" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I124" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J124" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K124" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D125" t="n">
         <v>1000</v>
       </c>
       <c r="E125" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F125" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G125" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H125" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I125" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J125" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K125" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -15080,36 +15142,36 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D126" t="n">
         <v>1000</v>
       </c>
       <c r="E126" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F126" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G126" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H126" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I126" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J126" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K126" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -15117,30 +15179,67 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D127" t="n">
         <v>1000</v>
       </c>
       <c r="E127" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F127" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G127" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H127" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I127" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J127" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K127" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>41</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D128" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E128" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F127" t="n">
+      <c r="F128" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G127" t="n">
+      <c r="G128" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H127" t="n">
+      <c r="H128" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I127" t="n">
+      <c r="I128" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J127" t="n">
+      <c r="J128" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K127" t="n">
+      <c r="K128" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 131 MLP+features hidden=96 -0.74
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$132</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>133</row>
+      <row>134</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T131"/>
+  <dimension ref="A1:T132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8229,16 +8229,16 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>47</v>
+        <v>131</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>XGBoost depth=3 n_est=200 lr=0.02 - shallow + more capacity test</t>
+          <t>MLP+features hidden=96 seed=42 - replicate old-features val-strong pattern</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -8247,60 +8247,60 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>-0.751</v>
+        <v>-0.7427</v>
       </c>
       <c r="F93" t="n">
-        <v>0.6433</v>
+        <v>-0.3427</v>
       </c>
       <c r="G93" t="n">
-        <v>-0.651</v>
+        <v>0.3592</v>
       </c>
       <c r="I93" t="n">
-        <v>66.12</v>
+        <v>-51.68</v>
       </c>
       <c r="J93" t="n">
-        <v>1661.2</v>
+        <v>483.2</v>
       </c>
       <c r="K93" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="L93" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N93" t="n">
-        <v>0.0237</v>
+        <v>0.0052</v>
       </c>
       <c r="O93" t="n">
-        <v>50.38</v>
+        <v>49.75</v>
       </c>
       <c r="P93" t="n">
-        <v>0.6045</v>
+        <v>0.5864</v>
       </c>
       <c r="Q93" t="n">
-        <v>0.4715</v>
+        <v>0.4164</v>
       </c>
       <c r="R93" t="n">
-        <v>0.5298</v>
+        <v>0.487</v>
       </c>
       <c r="S93" t="n">
-        <v>0.0229</v>
+        <v>0.0235</v>
       </c>
       <c r="T93" t="n">
-        <v>89.40000000000001</v>
+        <v>25.7</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>106</v>
+        <v>47</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>xlstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>xLSTM @ exp 105 RECORD hidden=64 seed=0 - multi-seed verify (was +0.08 seed=42 F1 +3.10 ex</t>
+          <t>XGBoost depth=3 n_est=200 lr=0.02 - shallow + more capacity test</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -8309,60 +8309,60 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>-0.7528</v>
+        <v>-0.751</v>
       </c>
       <c r="F94" t="n">
-        <v>0.6044</v>
+        <v>0.6433</v>
       </c>
       <c r="G94" t="n">
-        <v>-0.6528</v>
+        <v>-0.651</v>
       </c>
       <c r="I94" t="n">
-        <v>103.48</v>
+        <v>66.12</v>
       </c>
       <c r="J94" t="n">
-        <v>2034.8</v>
+        <v>1661.2</v>
       </c>
       <c r="K94" t="n">
         <v>6</v>
       </c>
       <c r="L94" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N94" t="n">
-        <v>0.0487</v>
+        <v>0.0237</v>
       </c>
       <c r="O94" t="n">
-        <v>53.73</v>
+        <v>50.38</v>
       </c>
       <c r="P94" t="n">
-        <v>0.5816</v>
+        <v>0.6045</v>
       </c>
       <c r="Q94" t="n">
-        <v>0.6803</v>
+        <v>0.4715</v>
       </c>
       <c r="R94" t="n">
-        <v>0.6271</v>
+        <v>0.5298</v>
       </c>
       <c r="S94" t="n">
-        <v>0.0265</v>
+        <v>0.0229</v>
       </c>
       <c r="T94" t="n">
-        <v>140.8</v>
+        <v>89.40000000000001</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>LightGBM @ exp 10 n_est=500 (down from 1000) - capacity sweet-spot test between 300 and 10</t>
+          <t>xLSTM @ exp 105 RECORD hidden=64 seed=0 - multi-seed verify (was +0.08 seed=42 F1 +3.10 ex</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -8371,60 +8371,60 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>-0.7554</v>
+        <v>-0.7528</v>
       </c>
       <c r="F95" t="n">
-        <v>0.7433</v>
+        <v>0.6044</v>
       </c>
       <c r="G95" t="n">
-        <v>-0.5554</v>
+        <v>-0.6528</v>
       </c>
       <c r="I95" t="n">
-        <v>82.7</v>
+        <v>103.48</v>
       </c>
       <c r="J95" t="n">
-        <v>1827</v>
+        <v>2034.8</v>
       </c>
       <c r="K95" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L95" t="n">
         <v>4</v>
       </c>
       <c r="N95" t="n">
-        <v>0.0283</v>
+        <v>0.0487</v>
       </c>
       <c r="O95" t="n">
-        <v>48.5</v>
+        <v>53.73</v>
       </c>
       <c r="P95" t="n">
-        <v>0.5928</v>
+        <v>0.5816</v>
       </c>
       <c r="Q95" t="n">
-        <v>0.4193</v>
+        <v>0.6803</v>
       </c>
       <c r="R95" t="n">
-        <v>0.4912</v>
+        <v>0.6271</v>
       </c>
       <c r="S95" t="n">
-        <v>0.0009</v>
+        <v>0.0265</v>
       </c>
       <c r="T95" t="n">
-        <v>117.6</v>
+        <v>140.8</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>lightgbm</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer warmup=5 (up from 0) - Goyal 2017 LR warmup on 1-layer</t>
+          <t>LightGBM @ exp 10 n_est=500 (down from 1000) - capacity sweet-spot test between 300 and 10</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -8433,60 +8433,60 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>-0.7729</v>
+        <v>-0.7554</v>
       </c>
       <c r="F96" t="n">
-        <v>-0.2729</v>
+        <v>0.7433</v>
       </c>
       <c r="G96" t="n">
-        <v>0.3166</v>
+        <v>-0.5554</v>
       </c>
       <c r="I96" t="n">
-        <v>-46.29</v>
+        <v>82.7</v>
       </c>
       <c r="J96" t="n">
-        <v>537.1</v>
+        <v>1827</v>
       </c>
       <c r="K96" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L96" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N96" t="n">
-        <v>0.0109</v>
+        <v>0.0283</v>
       </c>
       <c r="O96" t="n">
-        <v>46.06</v>
+        <v>48.5</v>
       </c>
       <c r="P96" t="n">
-        <v>0.5444</v>
+        <v>0.5928</v>
       </c>
       <c r="Q96" t="n">
-        <v>0.3569</v>
+        <v>0.4193</v>
       </c>
       <c r="R96" t="n">
-        <v>0.4311</v>
+        <v>0.4912</v>
       </c>
       <c r="S96" t="n">
-        <v>-0.0437</v>
+        <v>0.0009</v>
       </c>
       <c r="T96" t="n">
-        <v>87.40000000000001</v>
+        <v>117.6</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>LightGBM @ exp 10 gbm_lr=0.005 (down from 0.01) - slower learning at fixed n_est</t>
+          <t>LSTM @ exp 71 1-layer warmup=5 (up from 0) - Goyal 2017 LR warmup on 1-layer</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -8495,122 +8495,122 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>-0.8</v>
+        <v>-0.7729</v>
       </c>
       <c r="F97" t="n">
-        <v>0.4079</v>
+        <v>-0.2729</v>
       </c>
       <c r="G97" t="n">
-        <v>-0.5</v>
+        <v>0.3166</v>
       </c>
       <c r="I97" t="n">
-        <v>32.66</v>
+        <v>-46.29</v>
       </c>
       <c r="J97" t="n">
-        <v>1326.6</v>
+        <v>537.1</v>
       </c>
       <c r="K97" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L97" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N97" t="n">
-        <v>0.0255</v>
+        <v>0.0109</v>
       </c>
       <c r="O97" t="n">
-        <v>47.74</v>
+        <v>46.06</v>
       </c>
       <c r="P97" t="n">
-        <v>0.5764</v>
+        <v>0.5444</v>
       </c>
       <c r="Q97" t="n">
-        <v>0.4478</v>
+        <v>0.3569</v>
       </c>
       <c r="R97" t="n">
-        <v>0.504</v>
+        <v>0.4311</v>
       </c>
       <c r="S97" t="n">
-        <v>-0.0299</v>
+        <v>-0.0437</v>
       </c>
       <c r="T97" t="n">
-        <v>217.8</v>
+        <v>87.40000000000001</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
+        <v>93</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>lightgbm</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>LightGBM @ exp 10 gbm_lr=0.005 (down from 0.01) - slower learning at fixed n_est</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>-0.8</v>
+      </c>
+      <c r="F98" t="n">
+        <v>0.4079</v>
+      </c>
+      <c r="G98" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="I98" t="n">
+        <v>32.66</v>
+      </c>
+      <c r="J98" t="n">
+        <v>1326.6</v>
+      </c>
+      <c r="K98" t="n">
         <v>4</v>
       </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>mlp</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
-        <is>
-          <t>mlp seq=20 + stronger reg head_dropout=0.25 wd=1e-4 patience=15 (Gu-Kelly-Xiu 2020); hill-</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E98" t="n">
-        <v>-0.8341</v>
-      </c>
-      <c r="F98" t="n">
-        <v>-0.4341</v>
-      </c>
-      <c r="G98" t="n">
-        <v>1.203</v>
-      </c>
-      <c r="I98" t="n">
-        <v>-54.77</v>
-      </c>
-      <c r="J98" t="n">
-        <v>452.2999999999999</v>
-      </c>
-      <c r="K98" t="n">
-        <v>3</v>
-      </c>
       <c r="L98" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N98" t="n">
-        <v>-0.0036</v>
+        <v>0.0255</v>
       </c>
       <c r="O98" t="n">
-        <v>49.07</v>
+        <v>47.74</v>
       </c>
       <c r="P98" t="n">
-        <v>0.5674</v>
+        <v>0.5764</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.4955</v>
+        <v>0.4478</v>
       </c>
       <c r="R98" t="n">
-        <v>0.529</v>
+        <v>0.504</v>
       </c>
       <c r="S98" t="n">
-        <v>-0.0193</v>
+        <v>-0.0299</v>
       </c>
       <c r="T98" t="n">
-        <v>32.6</v>
+        <v>217.8</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t xml:space="preserve">CatBoost @ LightGBM-exp10 config (depth=4 lr=0.01 n_est=1000 seq=60) - 3-way GBM ensemble </t>
+          <t>mlp seq=20 + stronger reg head_dropout=0.25 wd=1e-4 patience=15 (Gu-Kelly-Xiu 2020); hill-</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -8619,60 +8619,60 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>-0.8395</v>
+        <v>-0.8341</v>
       </c>
       <c r="F99" t="n">
-        <v>0.2322</v>
+        <v>-0.4341</v>
       </c>
       <c r="G99" t="n">
-        <v>-0.5395</v>
+        <v>1.203</v>
       </c>
       <c r="I99" t="n">
-        <v>12.15</v>
+        <v>-54.77</v>
       </c>
       <c r="J99" t="n">
-        <v>1121.5</v>
+        <v>452.2999999999999</v>
       </c>
       <c r="K99" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L99" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N99" t="n">
-        <v>0.011</v>
+        <v>-0.0036</v>
       </c>
       <c r="O99" t="n">
-        <v>48.87</v>
+        <v>49.07</v>
       </c>
       <c r="P99" t="n">
-        <v>0.5893</v>
+        <v>0.5674</v>
       </c>
       <c r="Q99" t="n">
-        <v>0.4541</v>
+        <v>0.4955</v>
       </c>
       <c r="R99" t="n">
-        <v>0.513</v>
+        <v>0.529</v>
       </c>
       <c r="S99" t="n">
-        <v>-0.0056</v>
+        <v>-0.0193</v>
       </c>
       <c r="T99" t="n">
-        <v>1316.8</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>127</v>
+        <v>64</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MLP @ exp 126 lr=1e-4 + features seed=0 - 2nd seed verify</t>
+          <t xml:space="preserve">CatBoost @ LightGBM-exp10 config (depth=4 lr=0.01 n_est=1000 seq=60) - 3-way GBM ensemble </t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -8681,60 +8681,60 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>-0.8429</v>
+        <v>-0.8395</v>
       </c>
       <c r="F100" t="n">
-        <v>0.3863</v>
+        <v>0.2322</v>
       </c>
       <c r="G100" t="n">
-        <v>-0.6429</v>
+        <v>-0.5395</v>
       </c>
       <c r="I100" t="n">
-        <v>46.31</v>
+        <v>12.15</v>
       </c>
       <c r="J100" t="n">
-        <v>1463.1</v>
+        <v>1121.5</v>
       </c>
       <c r="K100" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L100" t="n">
         <v>2</v>
       </c>
       <c r="N100" t="n">
-        <v>0.0055</v>
+        <v>0.011</v>
       </c>
       <c r="O100" t="n">
-        <v>51.67</v>
+        <v>48.87</v>
       </c>
       <c r="P100" t="n">
-        <v>0.5765</v>
+        <v>0.5893</v>
       </c>
       <c r="Q100" t="n">
-        <v>0.5836</v>
+        <v>0.4541</v>
       </c>
       <c r="R100" t="n">
-        <v>0.58</v>
+        <v>0.513</v>
       </c>
       <c r="S100" t="n">
-        <v>0.009900000000000001</v>
+        <v>-0.0056</v>
       </c>
       <c r="T100" t="n">
-        <v>49.6</v>
+        <v>1316.8</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.02 n_est=500 - smaller capacity at productive lr</t>
+          <t>MLP @ exp 126 lr=1e-4 + features seed=0 - 2nd seed verify</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -8743,60 +8743,60 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>-0.8456</v>
+        <v>-0.8429</v>
       </c>
       <c r="F101" t="n">
-        <v>0.2334</v>
+        <v>0.3863</v>
       </c>
       <c r="G101" t="n">
-        <v>-0.4456</v>
+        <v>-0.6429</v>
       </c>
       <c r="I101" t="n">
-        <v>12.26</v>
+        <v>46.31</v>
       </c>
       <c r="J101" t="n">
-        <v>1122.6</v>
+        <v>1463.1</v>
       </c>
       <c r="K101" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L101" t="n">
         <v>2</v>
       </c>
       <c r="N101" t="n">
-        <v>0.0108</v>
+        <v>0.0055</v>
       </c>
       <c r="O101" t="n">
-        <v>49.72</v>
+        <v>51.67</v>
       </c>
       <c r="P101" t="n">
-        <v>0.5938</v>
+        <v>0.5765</v>
       </c>
       <c r="Q101" t="n">
-        <v>0.481</v>
+        <v>0.5836</v>
       </c>
       <c r="R101" t="n">
-        <v>0.5315</v>
+        <v>0.58</v>
       </c>
       <c r="S101" t="n">
-        <v>0.0028</v>
+        <v>0.009900000000000001</v>
       </c>
       <c r="T101" t="n">
-        <v>673.8</v>
+        <v>49.6</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">dMamba @ FX-Mamba-winner config seed=99 — 3rd seed for stable champion declaration (seeds </t>
+          <t>CatBoost lr=0.02 n_est=500 - smaller capacity at productive lr</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -8805,60 +8805,60 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>-0.862</v>
+        <v>-0.8456</v>
       </c>
       <c r="F102" t="n">
-        <v>-0.462</v>
+        <v>0.2334</v>
       </c>
       <c r="G102" t="n">
-        <v>1.3122</v>
+        <v>-0.4456</v>
       </c>
       <c r="I102" t="n">
-        <v>-42.07</v>
+        <v>12.26</v>
       </c>
       <c r="J102" t="n">
-        <v>579.3</v>
+        <v>1122.6</v>
       </c>
       <c r="K102" t="n">
         <v>3</v>
       </c>
       <c r="L102" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N102" t="n">
-        <v>0.0467</v>
+        <v>0.0108</v>
       </c>
       <c r="O102" t="n">
-        <v>43.33</v>
+        <v>49.72</v>
       </c>
       <c r="P102" t="n">
-        <v>0.5858</v>
+        <v>0.5938</v>
       </c>
       <c r="Q102" t="n">
-        <v>0.1576</v>
+        <v>0.481</v>
       </c>
       <c r="R102" t="n">
-        <v>0.2484</v>
+        <v>0.5315</v>
       </c>
       <c r="S102" t="n">
-        <v>-0.0059</v>
+        <v>0.0028</v>
       </c>
       <c r="T102" t="n">
-        <v>705.3</v>
+        <v>673.8</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>CatBoost depth=6 lr=0.01 n_est=1000 - depth axis test</t>
+          <t xml:space="preserve">dMamba @ FX-Mamba-winner config seed=99 — 3rd seed for stable champion declaration (seeds </t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -8867,51 +8867,51 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>-0.8688</v>
+        <v>-0.862</v>
       </c>
       <c r="F103" t="n">
-        <v>0.7087</v>
+        <v>-0.462</v>
       </c>
       <c r="G103" t="n">
-        <v>-0.6688</v>
+        <v>1.3122</v>
       </c>
       <c r="I103" t="n">
-        <v>76.76000000000001</v>
+        <v>-42.07</v>
       </c>
       <c r="J103" t="n">
-        <v>1767.6</v>
+        <v>579.3</v>
       </c>
       <c r="K103" t="n">
+        <v>3</v>
+      </c>
+      <c r="L103" t="n">
         <v>5</v>
       </c>
-      <c r="L103" t="n">
-        <v>1</v>
-      </c>
       <c r="N103" t="n">
-        <v>0.0031</v>
+        <v>0.0467</v>
       </c>
       <c r="O103" t="n">
-        <v>49.34</v>
+        <v>43.33</v>
       </c>
       <c r="P103" t="n">
-        <v>0.5827</v>
+        <v>0.5858</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.5127</v>
+        <v>0.1576</v>
       </c>
       <c r="R103" t="n">
-        <v>0.5455</v>
+        <v>0.2484</v>
       </c>
       <c r="S103" t="n">
-        <v>-0.0203</v>
+        <v>-0.0059</v>
       </c>
       <c r="T103" t="n">
-        <v>4289.1</v>
+        <v>705.3</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -8920,7 +8920,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.02 n_est=2000 - combine best CatBoost findings (lr from exp 98, capacity fro</t>
+          <t>CatBoost depth=6 lr=0.01 n_est=1000 - depth axis test</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -8929,60 +8929,60 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>-0.8764</v>
+        <v>-0.8688</v>
       </c>
       <c r="F104" t="n">
-        <v>-0.1626</v>
+        <v>0.7087</v>
       </c>
       <c r="G104" t="n">
-        <v>-0.4764</v>
+        <v>-0.6688</v>
       </c>
       <c r="I104" t="n">
-        <v>-23.11</v>
+        <v>76.76000000000001</v>
       </c>
       <c r="J104" t="n">
-        <v>768.9</v>
+        <v>1767.6</v>
       </c>
       <c r="K104" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L104" t="n">
         <v>1</v>
       </c>
       <c r="N104" t="n">
-        <v>0.0008</v>
+        <v>0.0031</v>
       </c>
       <c r="O104" t="n">
-        <v>46.43</v>
+        <v>49.34</v>
       </c>
       <c r="P104" t="n">
-        <v>0.5760999999999999</v>
+        <v>0.5827</v>
       </c>
       <c r="Q104" t="n">
-        <v>0.3655</v>
+        <v>0.5127</v>
       </c>
       <c r="R104" t="n">
-        <v>0.4472</v>
+        <v>0.5455</v>
       </c>
       <c r="S104" t="n">
-        <v>-0.0257</v>
+        <v>-0.0203</v>
       </c>
       <c r="T104" t="n">
-        <v>2594.9</v>
+        <v>4289.1</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>LSTM 1-layer + new features seed=42 - 2nd seed feature-impact assessment</t>
+          <t>CatBoost lr=0.02 n_est=2000 - combine best CatBoost findings (lr from exp 98, capacity fro</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -8991,60 +8991,60 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>-0.8773</v>
+        <v>-0.8764</v>
       </c>
       <c r="F105" t="n">
-        <v>0.388</v>
+        <v>-0.1626</v>
       </c>
       <c r="G105" t="n">
-        <v>-0.6773</v>
+        <v>-0.4764</v>
       </c>
       <c r="I105" t="n">
-        <v>46.95</v>
+        <v>-23.11</v>
       </c>
       <c r="J105" t="n">
-        <v>1469.5</v>
+        <v>768.9</v>
       </c>
       <c r="K105" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L105" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N105" t="n">
-        <v>0.0197</v>
+        <v>0.0008</v>
       </c>
       <c r="O105" t="n">
-        <v>47.05</v>
+        <v>46.43</v>
       </c>
       <c r="P105" t="n">
-        <v>0.5664</v>
+        <v>0.5760999999999999</v>
       </c>
       <c r="Q105" t="n">
-        <v>0.3222</v>
+        <v>0.3655</v>
       </c>
       <c r="R105" t="n">
-        <v>0.4107</v>
+        <v>0.4472</v>
       </c>
       <c r="S105" t="n">
-        <v>-0.0083</v>
+        <v>-0.0257</v>
       </c>
       <c r="T105" t="n">
-        <v>74.59999999999999</v>
+        <v>2594.9</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>18</v>
+        <v>117</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
+          <t>LSTM 1-layer + new features seed=42 - 2nd seed feature-impact assessment</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -9053,19 +9053,19 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>-0.9217</v>
+        <v>-0.8773</v>
       </c>
       <c r="F106" t="n">
-        <v>0.5942</v>
+        <v>0.388</v>
       </c>
       <c r="G106" t="n">
-        <v>-0.7217</v>
+        <v>-0.6773</v>
       </c>
       <c r="I106" t="n">
-        <v>58.5</v>
+        <v>46.95</v>
       </c>
       <c r="J106" t="n">
-        <v>1585</v>
+        <v>1469.5</v>
       </c>
       <c r="K106" t="n">
         <v>5</v>
@@ -9074,39 +9074,39 @@
         <v>2</v>
       </c>
       <c r="N106" t="n">
-        <v>0.019</v>
+        <v>0.0197</v>
       </c>
       <c r="O106" t="n">
-        <v>48.5</v>
+        <v>47.05</v>
       </c>
       <c r="P106" t="n">
-        <v>0.5986</v>
+        <v>0.5664</v>
       </c>
       <c r="Q106" t="n">
-        <v>0.3987</v>
+        <v>0.3222</v>
       </c>
       <c r="R106" t="n">
-        <v>0.4786</v>
+        <v>0.4107</v>
       </c>
       <c r="S106" t="n">
-        <v>0.0103</v>
+        <v>-0.0083</v>
       </c>
       <c r="T106" t="n">
-        <v>18919.4</v>
+        <v>74.59999999999999</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
+          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9115,51 +9115,51 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="F107" t="n">
-        <v>-0.2367</v>
+        <v>0.5942</v>
       </c>
       <c r="G107" t="n">
-        <v>-0.5226</v>
+        <v>-0.7217</v>
       </c>
       <c r="I107" t="n">
-        <v>-43.21</v>
+        <v>58.5</v>
       </c>
       <c r="J107" t="n">
-        <v>567.9000000000001</v>
+        <v>1585</v>
       </c>
       <c r="K107" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L107" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N107" t="n">
-        <v>-0.0164</v>
+        <v>0.019</v>
       </c>
       <c r="O107" t="n">
-        <v>45.63</v>
+        <v>48.5</v>
       </c>
       <c r="P107" t="n">
-        <v>0.5938</v>
+        <v>0.5986</v>
       </c>
       <c r="Q107" t="n">
-        <v>0.1648</v>
+        <v>0.3987</v>
       </c>
       <c r="R107" t="n">
-        <v>0.258</v>
+        <v>0.4786</v>
       </c>
       <c r="S107" t="n">
-        <v>0.0188</v>
+        <v>0.0103</v>
       </c>
       <c r="T107" t="n">
-        <v>33.8</v>
+        <v>18919.4</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -9168,7 +9168,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9177,60 +9177,60 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="F108" t="n">
-        <v>0.1045</v>
+        <v>-0.2367</v>
       </c>
       <c r="G108" t="n">
-        <v>-0.6746</v>
+        <v>-0.5226</v>
       </c>
       <c r="I108" t="n">
-        <v>-4.63</v>
+        <v>-43.21</v>
       </c>
       <c r="J108" t="n">
-        <v>953.7</v>
+        <v>567.9000000000001</v>
       </c>
       <c r="K108" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L108" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N108" t="n">
-        <v>-0.0374</v>
+        <v>-0.0164</v>
       </c>
       <c r="O108" t="n">
-        <v>51.03</v>
+        <v>45.63</v>
       </c>
       <c r="P108" t="n">
-        <v>0.5765</v>
+        <v>0.5938</v>
       </c>
       <c r="Q108" t="n">
-        <v>0.5415</v>
+        <v>0.1648</v>
       </c>
       <c r="R108" t="n">
-        <v>0.5585</v>
+        <v>0.258</v>
       </c>
       <c r="S108" t="n">
-        <v>0.0091</v>
+        <v>0.0188</v>
       </c>
       <c r="T108" t="n">
-        <v>30.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9239,60 +9239,60 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="F109" t="n">
-        <v>0.8788</v>
+        <v>0.1045</v>
       </c>
       <c r="G109" t="n">
-        <v>-0.866</v>
+        <v>-0.6746</v>
       </c>
       <c r="I109" t="n">
-        <v>107.82</v>
+        <v>-4.63</v>
       </c>
       <c r="J109" t="n">
-        <v>2078.2</v>
+        <v>953.7</v>
       </c>
       <c r="K109" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L109" t="n">
         <v>2</v>
       </c>
       <c r="N109" t="n">
-        <v>0.0329</v>
+        <v>-0.0374</v>
       </c>
       <c r="O109" t="n">
-        <v>54.14</v>
+        <v>51.03</v>
       </c>
       <c r="P109" t="n">
-        <v>0.6011</v>
+        <v>0.5765</v>
       </c>
       <c r="Q109" t="n">
-        <v>0.6725</v>
+        <v>0.5415</v>
       </c>
       <c r="R109" t="n">
-        <v>0.6348</v>
+        <v>0.5585</v>
       </c>
       <c r="S109" t="n">
-        <v>0.0251</v>
+        <v>0.0091</v>
       </c>
       <c r="T109" t="n">
-        <v>75.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9301,51 +9301,51 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F110" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G110" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I110" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J110" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K110" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L110" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N110" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O110" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P110" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q110" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R110" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S110" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T110" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -9354,7 +9354,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9363,60 +9363,60 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F111" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G111" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I111" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J111" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K111" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L111" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N111" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O111" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P111" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q111" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R111" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S111" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T111" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -9425,60 +9425,60 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F112" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G112" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I112" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J112" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K112" t="n">
         <v>2</v>
       </c>
       <c r="L112" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N112" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O112" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P112" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q112" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R112" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S112" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T112" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -9487,60 +9487,60 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F113" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G113" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I113" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J113" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K113" t="n">
+        <v>2</v>
+      </c>
+      <c r="L113" t="n">
         <v>5</v>
       </c>
-      <c r="L113" t="n">
-        <v>2</v>
-      </c>
       <c r="N113" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O113" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P113" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q113" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R113" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S113" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T113" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -9549,60 +9549,60 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F114" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G114" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I114" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J114" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K114" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L114" t="n">
         <v>2</v>
       </c>
       <c r="N114" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O114" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P114" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q114" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R114" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S114" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T114" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -9611,51 +9611,51 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F115" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G115" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I115" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J115" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K115" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L115" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N115" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O115" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P115" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q115" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R115" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S115" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T115" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -9664,7 +9664,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -9673,51 +9673,51 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F116" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G116" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I116" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J116" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K116" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L116" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N116" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O116" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P116" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q116" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R116" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S116" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T116" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -9726,7 +9726,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -9735,60 +9735,60 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F117" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G117" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I117" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J117" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K117" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L117" t="n">
         <v>2</v>
       </c>
       <c r="N117" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O117" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P117" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q117" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R117" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S117" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T117" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -9797,60 +9797,60 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F118" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G118" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I118" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J118" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K118" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L118" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N118" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O118" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P118" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q118" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R118" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S118" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T118" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -9859,60 +9859,60 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F119" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G119" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I119" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J119" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K119" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L119" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N119" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O119" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P119" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q119" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R119" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S119" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T119" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -9921,60 +9921,60 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F120" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G120" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I120" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J120" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L120" t="n">
         <v>3</v>
       </c>
       <c r="N120" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O120" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P120" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q120" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R120" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S120" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T120" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -9983,60 +9983,60 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="F121" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.8189</v>
       </c>
       <c r="G121" t="n">
-        <v>-0.8347</v>
+        <v>1.1456</v>
       </c>
       <c r="I121" t="n">
-        <v>-70.84999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J121" t="n">
-        <v>291.5000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K121" t="n">
         <v>1</v>
       </c>
       <c r="L121" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N121" t="n">
-        <v>0.0284</v>
+        <v>0.0089</v>
       </c>
       <c r="O121" t="n">
-        <v>44.07</v>
+        <v>41.44</v>
       </c>
       <c r="P121" t="n">
-        <v>0.5588</v>
+        <v>0.68</v>
       </c>
       <c r="Q121" t="n">
-        <v>0.1177</v>
+        <v>0.0271</v>
       </c>
       <c r="R121" t="n">
-        <v>0.1945</v>
+        <v>0.0521</v>
       </c>
       <c r="S121" t="n">
-        <v>-0.0101</v>
+        <v>0.0277</v>
       </c>
       <c r="T121" t="n">
-        <v>79.8</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -10045,39 +10045,51 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F122" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G122" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I122" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J122" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K122" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L122" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N122" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O122" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P122" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R122" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S122" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T122" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -10086,7 +10098,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -10095,51 +10107,39 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F123" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G123" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I123" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J123" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K123" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L123" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N123" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O123" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P123" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q123" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R123" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S123" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T123" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -10148,7 +10148,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -10157,51 +10157,51 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F124" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G124" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I124" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J124" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K124" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L124" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N124" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O124" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P124" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q124" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R124" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S124" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T124" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -10210,7 +10210,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -10219,113 +10219,113 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F125" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G125" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I125" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J125" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K125" t="n">
         <v>1</v>
       </c>
       <c r="L125" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N125" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O125" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P125" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q125" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R125" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S125" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T125" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
+        <v>59</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F126" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G126" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I126" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J126" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K126" t="n">
         <v>1</v>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E126" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F126" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G126" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I126" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J126" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K126" t="n">
-        <v>5</v>
       </c>
       <c r="L126" t="n">
         <v>1</v>
       </c>
       <c r="N126" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O126" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P126" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q126" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R126" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S126" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T126" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -10334,12 +10334,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -10382,21 +10382,21 @@
         <v>0.0098</v>
       </c>
       <c r="T127" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -10405,19 +10405,19 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F128" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G128" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I128" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J128" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K128" t="n">
         <v>5</v>
@@ -10426,39 +10426,39 @@
         <v>1</v>
       </c>
       <c r="N128" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O128" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P128" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q128" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R128" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S128" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T128" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -10467,113 +10467,113 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F129" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G129" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I129" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J129" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K129" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L129" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N129" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O129" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P129" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q129" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R129" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S129" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T129" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
+        <v>22</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F130" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G130" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I130" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J130" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K130" t="n">
+        <v>4</v>
+      </c>
+      <c r="L130" t="n">
         <v>2</v>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E130" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F130" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G130" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I130" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J130" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K130" t="n">
-        <v>5</v>
-      </c>
-      <c r="L130" t="n">
-        <v>1</v>
-      </c>
       <c r="N130" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O130" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P130" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q130" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R130" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S130" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T130" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -10582,7 +10582,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -10591,51 +10591,113 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F131" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G131" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I131" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J131" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K131" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N131" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O131" t="n">
         <v>47.65</v>
       </c>
       <c r="P131" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R131" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S131" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T131" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>41</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F132" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G132" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I132" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J132" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K132" t="n">
+        <v>4</v>
+      </c>
+      <c r="L132" t="n">
+        <v>2</v>
+      </c>
+      <c r="N132" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O132" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P132" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q131" t="n">
+      <c r="Q132" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R131" t="n">
+      <c r="R132" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S131" t="n">
+      <c r="S132" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T131" t="n">
+      <c r="T132" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T131"/>
-  <conditionalFormatting sqref="E2:E131">
+  <autoFilter ref="A1:T132"/>
+  <conditionalFormatting sqref="E2:E132">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -10657,7 +10719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -14099,414 +14161,414 @@
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>47</v>
+        <v>131</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>-0.751</v>
+        <v>-0.7427</v>
       </c>
       <c r="D93" t="n">
         <v>1000</v>
       </c>
       <c r="E93" t="n">
-        <v>1113.4</v>
+        <v>1086.6</v>
       </c>
       <c r="F93" t="n">
-        <v>1312.92128</v>
+        <v>819.4050599999999</v>
       </c>
       <c r="G93" t="n">
-        <v>1470.997002112</v>
+        <v>850.13274975</v>
       </c>
       <c r="H93" t="n">
-        <v>1503.653135558886</v>
+        <v>770.305284548475</v>
       </c>
       <c r="I93" t="n">
-        <v>1571.016796031924</v>
+        <v>884.1564056047396</v>
       </c>
       <c r="J93" t="n">
-        <v>2098.407134459841</v>
+        <v>541.6342140734635</v>
       </c>
       <c r="K93" t="n">
-        <v>1661.308928351856</v>
+        <v>483.2460457963441</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>106</v>
+        <v>47</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>xlstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>-0.7528</v>
+        <v>-0.751</v>
       </c>
       <c r="D94" t="n">
         <v>1000</v>
       </c>
       <c r="E94" t="n">
-        <v>843.7</v>
+        <v>1113.4</v>
       </c>
       <c r="F94" t="n">
-        <v>922.41721</v>
+        <v>1312.92128</v>
       </c>
       <c r="G94" t="n">
-        <v>936.714676755</v>
+        <v>1470.997002112</v>
       </c>
       <c r="H94" t="n">
-        <v>1095.019457126595</v>
+        <v>1503.653135558886</v>
       </c>
       <c r="I94" t="n">
-        <v>1178.897947542492</v>
+        <v>1571.016796031924</v>
       </c>
       <c r="J94" t="n">
-        <v>1454.406397883173</v>
+        <v>2098.407134459841</v>
       </c>
       <c r="K94" t="n">
-        <v>2034.859991278347</v>
+        <v>1661.308928351856</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>-0.7554</v>
+        <v>-0.7528</v>
       </c>
       <c r="D95" t="n">
         <v>1000</v>
       </c>
       <c r="E95" t="n">
-        <v>1025.7</v>
+        <v>843.7</v>
       </c>
       <c r="F95" t="n">
-        <v>1138.527</v>
+        <v>922.41721</v>
       </c>
       <c r="G95" t="n">
-        <v>1222.777998</v>
+        <v>936.714676755</v>
       </c>
       <c r="H95" t="n">
-        <v>1085.4600288246</v>
+        <v>1095.019457126595</v>
       </c>
       <c r="I95" t="n">
-        <v>915.6940803164325</v>
+        <v>1178.897947542492</v>
       </c>
       <c r="J95" t="n">
-        <v>1284.718794683955</v>
+        <v>1454.406397883173</v>
       </c>
       <c r="K95" t="n">
-        <v>1827.255541678989</v>
+        <v>2034.859991278347</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>lightgbm</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>-0.7729</v>
+        <v>-0.7554</v>
       </c>
       <c r="D96" t="n">
         <v>1000</v>
       </c>
       <c r="E96" t="n">
-        <v>879.3</v>
+        <v>1025.7</v>
       </c>
       <c r="F96" t="n">
-        <v>936.7182899999999</v>
+        <v>1138.527</v>
       </c>
       <c r="G96" t="n">
-        <v>835.646386509</v>
+        <v>1222.777998</v>
       </c>
       <c r="H96" t="n">
-        <v>799.4628979731602</v>
+        <v>1085.4600288246</v>
       </c>
       <c r="I96" t="n">
-        <v>859.0228838721607</v>
+        <v>915.6940803164325</v>
       </c>
       <c r="J96" t="n">
-        <v>659.1282587951089</v>
+        <v>1284.718794683955</v>
       </c>
       <c r="K96" t="n">
-        <v>537.1895309180137</v>
+        <v>1827.255541678989</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>lightgbm</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>-0.8</v>
+        <v>-0.7729</v>
       </c>
       <c r="D97" t="n">
         <v>1000</v>
       </c>
       <c r="E97" t="n">
-        <v>936.6999999999999</v>
+        <v>879.3</v>
       </c>
       <c r="F97" t="n">
-        <v>1011.26132</v>
+        <v>936.7182899999999</v>
       </c>
       <c r="G97" t="n">
-        <v>1048.779114972</v>
+        <v>835.646386509</v>
       </c>
       <c r="H97" t="n">
-        <v>1000.849909417779</v>
+        <v>799.4628979731602</v>
       </c>
       <c r="I97" t="n">
-        <v>1051.592999825261</v>
+        <v>859.0228838721607</v>
       </c>
       <c r="J97" t="n">
-        <v>1570.133508039097</v>
+        <v>659.1282587951089</v>
       </c>
       <c r="K97" t="n">
-        <v>1326.605800942233</v>
+        <v>537.1895309180137</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>4</v>
+        <v>93</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lightgbm</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>-0.8341</v>
+        <v>-0.8</v>
       </c>
       <c r="D98" t="n">
         <v>1000</v>
       </c>
       <c r="E98" t="n">
-        <v>909.6999999999999</v>
+        <v>936.6999999999999</v>
       </c>
       <c r="F98" t="n">
-        <v>831.10192</v>
+        <v>1011.26132</v>
       </c>
       <c r="G98" t="n">
-        <v>866.4237515999999</v>
+        <v>1048.779114972</v>
       </c>
       <c r="H98" t="n">
-        <v>873.0952144873199</v>
+        <v>1000.849909417779</v>
       </c>
       <c r="I98" t="n">
-        <v>662.4173392315297</v>
+        <v>1051.592999825261</v>
       </c>
       <c r="J98" t="n">
-        <v>447.3966709169752</v>
+        <v>1570.133508039097</v>
       </c>
       <c r="K98" t="n">
-        <v>452.3180342970618</v>
+        <v>1326.605800942233</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>64</v>
+        <v>4</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>-0.8395</v>
+        <v>-0.8341</v>
       </c>
       <c r="D99" t="n">
         <v>1000</v>
       </c>
       <c r="E99" t="n">
-        <v>1011.7</v>
+        <v>909.6999999999999</v>
       </c>
       <c r="F99" t="n">
-        <v>1220.21137</v>
+        <v>831.10192</v>
       </c>
       <c r="G99" t="n">
-        <v>1383.963735854</v>
+        <v>866.4237515999999</v>
       </c>
       <c r="H99" t="n">
-        <v>1276.56814995173</v>
+        <v>873.0952144873199</v>
       </c>
       <c r="I99" t="n">
-        <v>1150.570873551494</v>
+        <v>662.4173392315297</v>
       </c>
       <c r="J99" t="n">
-        <v>1502.300389596186</v>
+        <v>447.3966709169752</v>
       </c>
       <c r="K99" t="n">
-        <v>1121.617470872512</v>
+        <v>452.3180342970618</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>127</v>
+        <v>64</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>-0.8429</v>
+        <v>-0.8395</v>
       </c>
       <c r="D100" t="n">
         <v>1000</v>
       </c>
       <c r="E100" t="n">
-        <v>861.6</v>
+        <v>1011.7</v>
       </c>
       <c r="F100" t="n">
-        <v>960.85632</v>
+        <v>1220.21137</v>
       </c>
       <c r="G100" t="n">
-        <v>989.7780952319999</v>
+        <v>1383.963735854</v>
       </c>
       <c r="H100" t="n">
-        <v>1153.289436564326</v>
+        <v>1276.56814995173</v>
       </c>
       <c r="I100" t="n">
-        <v>1482.553570703441</v>
+        <v>1150.570873551494</v>
       </c>
       <c r="J100" t="n">
-        <v>1616.428158137962</v>
+        <v>1502.300389596186</v>
       </c>
       <c r="K100" t="n">
-        <v>1463.190768746483</v>
+        <v>1121.617470872512</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>-0.8456</v>
+        <v>-0.8429</v>
       </c>
       <c r="D101" t="n">
         <v>1000</v>
       </c>
       <c r="E101" t="n">
-        <v>953</v>
+        <v>861.6</v>
       </c>
       <c r="F101" t="n">
-        <v>1234.8974</v>
+        <v>960.85632</v>
       </c>
       <c r="G101" t="n">
-        <v>1386.04884176</v>
+        <v>989.7780952319999</v>
       </c>
       <c r="H101" t="n">
-        <v>1167.330334530272</v>
+        <v>1153.289436564326</v>
       </c>
       <c r="I101" t="n">
-        <v>993.3981146852617</v>
+        <v>1482.553570703441</v>
       </c>
       <c r="J101" t="n">
-        <v>1310.689472515734</v>
+        <v>1616.428158137962</v>
       </c>
       <c r="K101" t="n">
-        <v>1122.605533209726</v>
+        <v>1463.190768746483</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>-0.862</v>
+        <v>-0.8456</v>
       </c>
       <c r="D102" t="n">
         <v>1000</v>
       </c>
       <c r="E102" t="n">
-        <v>1064.8</v>
+        <v>953</v>
       </c>
       <c r="F102" t="n">
-        <v>857.3769599999999</v>
+        <v>1234.8974</v>
       </c>
       <c r="G102" t="n">
-        <v>754.4917247999999</v>
+        <v>1386.04884176</v>
       </c>
       <c r="H102" t="n">
-        <v>689.30363977728</v>
+        <v>1167.330334530272</v>
       </c>
       <c r="I102" t="n">
-        <v>835.2981506821078</v>
+        <v>993.3981146852617</v>
       </c>
       <c r="J102" t="n">
-        <v>582.2028110254292</v>
+        <v>1310.689472515734</v>
       </c>
       <c r="K102" t="n">
-        <v>579.3500172514047</v>
+        <v>1122.605533209726</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>103</v>
+        <v>20</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>-0.8688</v>
+        <v>-0.862</v>
       </c>
       <c r="D103" t="n">
         <v>1000</v>
       </c>
       <c r="E103" t="n">
-        <v>1120</v>
+        <v>1064.8</v>
       </c>
       <c r="F103" t="n">
-        <v>1237.6</v>
+        <v>857.3769599999999</v>
       </c>
       <c r="G103" t="n">
-        <v>1385.61696</v>
+        <v>754.4917247999999</v>
       </c>
       <c r="H103" t="n">
-        <v>1253.429102016</v>
+        <v>689.30363977728</v>
       </c>
       <c r="I103" t="n">
-        <v>1143.378026858995</v>
+        <v>835.2981506821078</v>
       </c>
       <c r="J103" t="n">
-        <v>1478.502126531366</v>
+        <v>582.2028110254292</v>
       </c>
       <c r="K103" t="n">
-        <v>1767.549292268249</v>
+        <v>579.3500172514047</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
@@ -14514,147 +14576,147 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>-0.8764</v>
+        <v>-0.8688</v>
       </c>
       <c r="D104" t="n">
         <v>1000</v>
       </c>
       <c r="E104" t="n">
-        <v>762</v>
+        <v>1120</v>
       </c>
       <c r="F104" t="n">
-        <v>937.8695999999999</v>
+        <v>1237.6</v>
       </c>
       <c r="G104" t="n">
-        <v>946.9669351199999</v>
+        <v>1385.61696</v>
       </c>
       <c r="H104" t="n">
-        <v>929.2586534332559</v>
+        <v>1253.429102016</v>
       </c>
       <c r="I104" t="n">
-        <v>802.1360696435864</v>
+        <v>1143.378026858995</v>
       </c>
       <c r="J104" t="n">
-        <v>902.5635055629634</v>
+        <v>1478.502126531366</v>
       </c>
       <c r="K104" t="n">
-        <v>768.8035940385322</v>
+        <v>1767.549292268249</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>117</v>
+        <v>100</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>-0.8773</v>
+        <v>-0.8764</v>
       </c>
       <c r="D105" t="n">
         <v>1000</v>
       </c>
       <c r="E105" t="n">
-        <v>813.4</v>
+        <v>762</v>
       </c>
       <c r="F105" t="n">
-        <v>777.12236</v>
+        <v>937.8695999999999</v>
       </c>
       <c r="G105" t="n">
-        <v>782.873065464</v>
+        <v>946.9669351199999</v>
       </c>
       <c r="H105" t="n">
-        <v>886.2905974117942</v>
+        <v>929.2586534332559</v>
       </c>
       <c r="I105" t="n">
-        <v>1154.925277487309</v>
+        <v>802.1360696435864</v>
       </c>
       <c r="J105" t="n">
-        <v>1312.572577864327</v>
+        <v>902.5635055629634</v>
       </c>
       <c r="K105" t="n">
-        <v>1469.425000919113</v>
+        <v>768.8035940385322</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>18</v>
+        <v>117</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>-0.9217</v>
+        <v>-0.8773</v>
       </c>
       <c r="D106" t="n">
         <v>1000</v>
       </c>
       <c r="E106" t="n">
-        <v>1206.3</v>
+        <v>813.4</v>
       </c>
       <c r="F106" t="n">
-        <v>1403.65068</v>
+        <v>777.12236</v>
       </c>
       <c r="G106" t="n">
-        <v>1572.930952008</v>
+        <v>782.873065464</v>
       </c>
       <c r="H106" t="n">
-        <v>1622.320983901051</v>
+        <v>886.2905974117942</v>
       </c>
       <c r="I106" t="n">
-        <v>1560.023858119251</v>
+        <v>1154.925277487309</v>
       </c>
       <c r="J106" t="n">
-        <v>2085.595895919627</v>
+        <v>1312.572577864327</v>
       </c>
       <c r="K106" t="n">
-        <v>1584.844321309324</v>
+        <v>1469.425000919113</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="D107" t="n">
         <v>1000</v>
       </c>
       <c r="E107" t="n">
-        <v>1141.9</v>
+        <v>1206.3</v>
       </c>
       <c r="F107" t="n">
-        <v>983.4042799999999</v>
+        <v>1403.65068</v>
       </c>
       <c r="G107" t="n">
-        <v>1002.482323032</v>
+        <v>1572.930952008</v>
       </c>
       <c r="H107" t="n">
-        <v>1006.392004091825</v>
+        <v>1622.320983901051</v>
       </c>
       <c r="I107" t="n">
-        <v>968.1491079363354</v>
+        <v>1560.023858119251</v>
       </c>
       <c r="J107" t="n">
-        <v>739.9563631957411</v>
+        <v>2085.595895919627</v>
       </c>
       <c r="K107" t="n">
-        <v>567.8425131164117</v>
+        <v>1584.844321309324</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -14662,110 +14724,110 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="D108" t="n">
         <v>1000</v>
       </c>
       <c r="E108" t="n">
-        <v>823.5</v>
+        <v>1141.9</v>
       </c>
       <c r="F108" t="n">
-        <v>939.36645</v>
+        <v>983.4042799999999</v>
       </c>
       <c r="G108" t="n">
-        <v>1037.24843409</v>
+        <v>1002.482323032</v>
       </c>
       <c r="H108" t="n">
-        <v>968.582587753242</v>
+        <v>1006.392004091825</v>
       </c>
       <c r="I108" t="n">
-        <v>996.38090802176</v>
+        <v>968.1491079363354</v>
       </c>
       <c r="J108" t="n">
-        <v>1251.255144293726</v>
+        <v>739.9563631957411</v>
       </c>
       <c r="K108" t="n">
-        <v>953.7066709806782</v>
+        <v>567.8425131164117</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="D109" t="n">
         <v>1000</v>
       </c>
       <c r="E109" t="n">
-        <v>1390.6</v>
+        <v>823.5</v>
       </c>
       <c r="F109" t="n">
-        <v>1715.16604</v>
+        <v>939.36645</v>
       </c>
       <c r="G109" t="n">
-        <v>1928.018145564</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H109" t="n">
-        <v>1842.799743530072</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I109" t="n">
-        <v>1932.359811065633</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J109" t="n">
-        <v>2502.212719348888</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K109" t="n">
-        <v>2078.337884691186</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D110" t="n">
         <v>1000</v>
       </c>
       <c r="E110" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F110" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G110" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H110" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I110" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J110" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K110" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -14773,184 +14835,184 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D111" t="n">
         <v>1000</v>
       </c>
       <c r="E111" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F111" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G111" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H111" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I111" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J111" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K111" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D112" t="n">
         <v>1000</v>
       </c>
       <c r="E112" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F112" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G112" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H112" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I112" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J112" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K112" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D113" t="n">
         <v>1000</v>
       </c>
       <c r="E113" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F113" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G113" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H113" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I113" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J113" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K113" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D114" t="n">
         <v>1000</v>
       </c>
       <c r="E114" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F114" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G114" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H114" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I114" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J114" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K114" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D115" t="n">
         <v>1000</v>
       </c>
       <c r="E115" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F115" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G115" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H115" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I115" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J115" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K115" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -14958,36 +15020,36 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D116" t="n">
         <v>1000</v>
       </c>
       <c r="E116" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F116" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G116" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H116" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I116" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J116" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K116" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -14995,221 +15057,221 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D117" t="n">
         <v>1000</v>
       </c>
       <c r="E117" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F117" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G117" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H117" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I117" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J117" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K117" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D118" t="n">
         <v>1000</v>
       </c>
       <c r="E118" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F118" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G118" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H118" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I118" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J118" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K118" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D119" t="n">
         <v>1000</v>
       </c>
       <c r="E119" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F119" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G119" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H119" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I119" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J119" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K119" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D120" t="n">
         <v>1000</v>
       </c>
       <c r="E120" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F120" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G120" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H120" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I120" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J120" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K120" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="D121" t="n">
         <v>1000</v>
       </c>
       <c r="E121" t="n">
-        <v>743.8000000000001</v>
+        <v>942</v>
       </c>
       <c r="F121" t="n">
-        <v>692.62656</v>
+        <v>730.2384</v>
       </c>
       <c r="G121" t="n">
-        <v>666.7223266560001</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H121" t="n">
-        <v>724.7938413077377</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I121" t="n">
-        <v>681.3786902134042</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J121" t="n">
-        <v>441.2608397822005</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K121" t="n">
-        <v>291.4527846761434</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D122" t="n">
         <v>1000</v>
       </c>
       <c r="E122" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F122" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G122" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H122" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I122" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J122" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K122" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
@@ -15217,36 +15279,36 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D123" t="n">
         <v>1000</v>
       </c>
       <c r="E123" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F123" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G123" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H123" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I123" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J123" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K123" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -15254,36 +15316,36 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D124" t="n">
         <v>1000</v>
       </c>
       <c r="E124" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F124" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G124" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H124" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I124" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J124" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K124" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -15291,73 +15353,73 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D125" t="n">
         <v>1000</v>
       </c>
       <c r="E125" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F125" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G125" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H125" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I125" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J125" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K125" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D126" t="n">
         <v>1000</v>
       </c>
       <c r="E126" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F126" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G126" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H126" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I126" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J126" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K126" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -15394,81 +15456,81 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D128" t="n">
         <v>1000</v>
       </c>
       <c r="E128" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F128" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G128" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H128" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I128" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J128" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K128" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D129" t="n">
         <v>1000</v>
       </c>
       <c r="E129" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F129" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G129" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H129" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I129" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J129" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K129" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -15476,36 +15538,36 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D130" t="n">
         <v>1000</v>
       </c>
       <c r="E130" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F130" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G130" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H130" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I130" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J130" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K130" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -15513,30 +15575,67 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D131" t="n">
         <v>1000</v>
       </c>
       <c r="E131" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F131" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G131" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H131" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I131" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J131" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K131" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>41</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D132" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E132" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F131" t="n">
+      <c r="F132" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G131" t="n">
+      <c r="G132" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H131" t="n">
+      <c r="H132" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I131" t="n">
+      <c r="I132" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J131" t="n">
+      <c r="J132" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K131" t="n">
+      <c r="K132" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 132 MLP+features bs=64 -0.91
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$133</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>134</row>
+      <row>135</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T132"/>
+  <dimension ref="A1:T133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9097,16 +9097,16 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>18</v>
+        <v>132</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
+          <t>MLP+features bs=64 seed=42 - large-batch on new features</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9115,60 +9115,60 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>-0.9217</v>
+        <v>-0.9127</v>
       </c>
       <c r="F107" t="n">
-        <v>0.5942</v>
+        <v>0.2667</v>
       </c>
       <c r="G107" t="n">
-        <v>-0.7217</v>
+        <v>-0.6127</v>
       </c>
       <c r="I107" t="n">
-        <v>58.5</v>
+        <v>21.96</v>
       </c>
       <c r="J107" t="n">
-        <v>1585</v>
+        <v>1219.6</v>
       </c>
       <c r="K107" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N107" t="n">
-        <v>0.019</v>
+        <v>-0.0177</v>
       </c>
       <c r="O107" t="n">
-        <v>48.5</v>
+        <v>50.53</v>
       </c>
       <c r="P107" t="n">
-        <v>0.5986</v>
+        <v>0.5562</v>
       </c>
       <c r="Q107" t="n">
-        <v>0.3987</v>
+        <v>0.6679</v>
       </c>
       <c r="R107" t="n">
-        <v>0.4786</v>
+        <v>0.607</v>
       </c>
       <c r="S107" t="n">
-        <v>0.0103</v>
+        <v>-0.0482</v>
       </c>
       <c r="T107" t="n">
-        <v>18919.4</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
+          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9177,51 +9177,51 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="F108" t="n">
-        <v>-0.2367</v>
+        <v>0.5942</v>
       </c>
       <c r="G108" t="n">
-        <v>-0.5226</v>
+        <v>-0.7217</v>
       </c>
       <c r="I108" t="n">
-        <v>-43.21</v>
+        <v>58.5</v>
       </c>
       <c r="J108" t="n">
-        <v>567.9000000000001</v>
+        <v>1585</v>
       </c>
       <c r="K108" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L108" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N108" t="n">
-        <v>-0.0164</v>
+        <v>0.019</v>
       </c>
       <c r="O108" t="n">
-        <v>45.63</v>
+        <v>48.5</v>
       </c>
       <c r="P108" t="n">
-        <v>0.5938</v>
+        <v>0.5986</v>
       </c>
       <c r="Q108" t="n">
-        <v>0.1648</v>
+        <v>0.3987</v>
       </c>
       <c r="R108" t="n">
-        <v>0.258</v>
+        <v>0.4786</v>
       </c>
       <c r="S108" t="n">
-        <v>0.0188</v>
+        <v>0.0103</v>
       </c>
       <c r="T108" t="n">
-        <v>33.8</v>
+        <v>18919.4</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -9230,7 +9230,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9239,60 +9239,60 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="F109" t="n">
-        <v>0.1045</v>
+        <v>-0.2367</v>
       </c>
       <c r="G109" t="n">
-        <v>-0.6746</v>
+        <v>-0.5226</v>
       </c>
       <c r="I109" t="n">
-        <v>-4.63</v>
+        <v>-43.21</v>
       </c>
       <c r="J109" t="n">
-        <v>953.7</v>
+        <v>567.9000000000001</v>
       </c>
       <c r="K109" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L109" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N109" t="n">
-        <v>-0.0374</v>
+        <v>-0.0164</v>
       </c>
       <c r="O109" t="n">
-        <v>51.03</v>
+        <v>45.63</v>
       </c>
       <c r="P109" t="n">
-        <v>0.5765</v>
+        <v>0.5938</v>
       </c>
       <c r="Q109" t="n">
-        <v>0.5415</v>
+        <v>0.1648</v>
       </c>
       <c r="R109" t="n">
-        <v>0.5585</v>
+        <v>0.258</v>
       </c>
       <c r="S109" t="n">
-        <v>0.0091</v>
+        <v>0.0188</v>
       </c>
       <c r="T109" t="n">
-        <v>30.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9301,60 +9301,60 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="F110" t="n">
-        <v>0.8788</v>
+        <v>0.1045</v>
       </c>
       <c r="G110" t="n">
-        <v>-0.866</v>
+        <v>-0.6746</v>
       </c>
       <c r="I110" t="n">
-        <v>107.82</v>
+        <v>-4.63</v>
       </c>
       <c r="J110" t="n">
-        <v>2078.2</v>
+        <v>953.7</v>
       </c>
       <c r="K110" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L110" t="n">
         <v>2</v>
       </c>
       <c r="N110" t="n">
-        <v>0.0329</v>
+        <v>-0.0374</v>
       </c>
       <c r="O110" t="n">
-        <v>54.14</v>
+        <v>51.03</v>
       </c>
       <c r="P110" t="n">
-        <v>0.6011</v>
+        <v>0.5765</v>
       </c>
       <c r="Q110" t="n">
-        <v>0.6725</v>
+        <v>0.5415</v>
       </c>
       <c r="R110" t="n">
-        <v>0.6348</v>
+        <v>0.5585</v>
       </c>
       <c r="S110" t="n">
-        <v>0.0251</v>
+        <v>0.0091</v>
       </c>
       <c r="T110" t="n">
-        <v>75.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9363,51 +9363,51 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F111" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G111" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I111" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J111" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K111" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L111" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N111" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O111" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P111" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q111" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R111" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S111" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T111" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -9416,7 +9416,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -9425,60 +9425,60 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F112" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G112" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I112" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J112" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K112" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L112" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N112" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O112" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P112" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q112" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R112" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S112" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T112" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -9487,60 +9487,60 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F113" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G113" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I113" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J113" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K113" t="n">
         <v>2</v>
       </c>
       <c r="L113" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N113" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O113" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P113" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q113" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R113" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S113" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T113" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -9549,60 +9549,60 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F114" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G114" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I114" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J114" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K114" t="n">
+        <v>2</v>
+      </c>
+      <c r="L114" t="n">
         <v>5</v>
       </c>
-      <c r="L114" t="n">
-        <v>2</v>
-      </c>
       <c r="N114" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O114" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P114" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q114" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R114" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S114" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T114" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -9611,60 +9611,60 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F115" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G115" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I115" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J115" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K115" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L115" t="n">
         <v>2</v>
       </c>
       <c r="N115" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O115" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P115" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q115" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R115" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S115" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T115" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -9673,51 +9673,51 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F116" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G116" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I116" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J116" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K116" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L116" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N116" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O116" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P116" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q116" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R116" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S116" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T116" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -9726,7 +9726,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -9735,51 +9735,51 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F117" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G117" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I117" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J117" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K117" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L117" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N117" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O117" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P117" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q117" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R117" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S117" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T117" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -9788,7 +9788,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -9797,60 +9797,60 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F118" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G118" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I118" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J118" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K118" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L118" t="n">
         <v>2</v>
       </c>
       <c r="N118" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O118" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P118" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q118" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R118" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S118" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T118" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -9859,60 +9859,60 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F119" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G119" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I119" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J119" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K119" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N119" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O119" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P119" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q119" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R119" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S119" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T119" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -9921,60 +9921,60 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F120" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G120" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I120" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J120" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K120" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L120" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N120" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O120" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P120" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q120" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R120" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S120" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T120" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -9983,60 +9983,60 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F121" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G121" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I121" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J121" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K121" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L121" t="n">
         <v>3</v>
       </c>
       <c r="N121" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O121" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P121" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q121" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R121" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S121" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T121" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -10045,60 +10045,60 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="F122" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.8189</v>
       </c>
       <c r="G122" t="n">
-        <v>-0.8347</v>
+        <v>1.1456</v>
       </c>
       <c r="I122" t="n">
-        <v>-70.84999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J122" t="n">
-        <v>291.5000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K122" t="n">
         <v>1</v>
       </c>
       <c r="L122" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N122" t="n">
-        <v>0.0284</v>
+        <v>0.0089</v>
       </c>
       <c r="O122" t="n">
-        <v>44.07</v>
+        <v>41.44</v>
       </c>
       <c r="P122" t="n">
-        <v>0.5588</v>
+        <v>0.68</v>
       </c>
       <c r="Q122" t="n">
-        <v>0.1177</v>
+        <v>0.0271</v>
       </c>
       <c r="R122" t="n">
-        <v>0.1945</v>
+        <v>0.0521</v>
       </c>
       <c r="S122" t="n">
-        <v>-0.0101</v>
+        <v>0.0277</v>
       </c>
       <c r="T122" t="n">
-        <v>79.8</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -10107,39 +10107,51 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F123" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G123" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I123" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J123" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K123" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N123" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O123" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P123" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R123" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S123" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T123" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -10148,7 +10160,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -10157,51 +10169,39 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F124" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G124" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I124" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J124" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K124" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L124" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N124" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O124" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P124" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q124" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R124" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S124" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T124" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -10210,7 +10210,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -10219,51 +10219,51 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F125" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G125" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I125" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J125" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K125" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L125" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N125" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O125" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P125" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q125" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R125" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S125" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T125" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -10272,7 +10272,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -10281,113 +10281,113 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F126" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G126" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I126" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J126" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K126" t="n">
         <v>1</v>
       </c>
       <c r="L126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N126" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O126" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P126" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q126" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R126" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S126" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T126" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
+        <v>59</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F127" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G127" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I127" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J127" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K127" t="n">
         <v>1</v>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E127" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F127" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G127" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I127" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J127" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K127" t="n">
-        <v>5</v>
       </c>
       <c r="L127" t="n">
         <v>1</v>
       </c>
       <c r="N127" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O127" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P127" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q127" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R127" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S127" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T127" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -10396,12 +10396,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -10444,21 +10444,21 @@
         <v>0.0098</v>
       </c>
       <c r="T128" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -10467,19 +10467,19 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F129" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G129" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I129" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J129" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K129" t="n">
         <v>5</v>
@@ -10488,39 +10488,39 @@
         <v>1</v>
       </c>
       <c r="N129" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O129" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P129" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q129" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R129" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S129" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T129" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -10529,113 +10529,113 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F130" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G130" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I130" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J130" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K130" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L130" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N130" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O130" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P130" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q130" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R130" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S130" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T130" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
+        <v>22</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F131" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G131" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I131" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J131" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K131" t="n">
+        <v>4</v>
+      </c>
+      <c r="L131" t="n">
         <v>2</v>
       </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E131" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F131" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G131" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I131" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J131" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K131" t="n">
-        <v>5</v>
-      </c>
-      <c r="L131" t="n">
-        <v>1</v>
-      </c>
       <c r="N131" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O131" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P131" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q131" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R131" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S131" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T131" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -10644,7 +10644,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -10653,51 +10653,113 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F132" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G132" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I132" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J132" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K132" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L132" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N132" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O132" t="n">
         <v>47.65</v>
       </c>
       <c r="P132" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R132" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S132" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T132" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>41</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F133" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G133" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I133" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J133" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K133" t="n">
+        <v>4</v>
+      </c>
+      <c r="L133" t="n">
+        <v>2</v>
+      </c>
+      <c r="N133" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O133" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P133" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q132" t="n">
+      <c r="Q133" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R132" t="n">
+      <c r="R133" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S132" t="n">
+      <c r="S133" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T132" t="n">
+      <c r="T133" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T132"/>
-  <conditionalFormatting sqref="E2:E132">
+  <autoFilter ref="A1:T133"/>
+  <conditionalFormatting sqref="E2:E133">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -10719,7 +10781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:K133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -14679,81 +14741,81 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>18</v>
+        <v>132</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-0.9217</v>
+        <v>-0.9127</v>
       </c>
       <c r="D107" t="n">
         <v>1000</v>
       </c>
       <c r="E107" t="n">
-        <v>1206.3</v>
+        <v>824.6</v>
       </c>
       <c r="F107" t="n">
-        <v>1403.65068</v>
+        <v>945.8162000000001</v>
       </c>
       <c r="G107" t="n">
-        <v>1572.930952008</v>
+        <v>1155.40906992</v>
       </c>
       <c r="H107" t="n">
-        <v>1622.320983901051</v>
+        <v>1037.55734478816</v>
       </c>
       <c r="I107" t="n">
-        <v>1560.023858119251</v>
+        <v>1136.955338418866</v>
       </c>
       <c r="J107" t="n">
-        <v>2085.595895919627</v>
+        <v>1027.125452727604</v>
       </c>
       <c r="K107" t="n">
-        <v>1584.844321309324</v>
+        <v>1219.506050023484</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="D108" t="n">
         <v>1000</v>
       </c>
       <c r="E108" t="n">
-        <v>1141.9</v>
+        <v>1206.3</v>
       </c>
       <c r="F108" t="n">
-        <v>983.4042799999999</v>
+        <v>1403.65068</v>
       </c>
       <c r="G108" t="n">
-        <v>1002.482323032</v>
+        <v>1572.930952008</v>
       </c>
       <c r="H108" t="n">
-        <v>1006.392004091825</v>
+        <v>1622.320983901051</v>
       </c>
       <c r="I108" t="n">
-        <v>968.1491079363354</v>
+        <v>1560.023858119251</v>
       </c>
       <c r="J108" t="n">
-        <v>739.9563631957411</v>
+        <v>2085.595895919627</v>
       </c>
       <c r="K108" t="n">
-        <v>567.8425131164117</v>
+        <v>1584.844321309324</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -14761,110 +14823,110 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="D109" t="n">
         <v>1000</v>
       </c>
       <c r="E109" t="n">
-        <v>823.5</v>
+        <v>1141.9</v>
       </c>
       <c r="F109" t="n">
-        <v>939.36645</v>
+        <v>983.4042799999999</v>
       </c>
       <c r="G109" t="n">
-        <v>1037.24843409</v>
+        <v>1002.482323032</v>
       </c>
       <c r="H109" t="n">
-        <v>968.582587753242</v>
+        <v>1006.392004091825</v>
       </c>
       <c r="I109" t="n">
-        <v>996.38090802176</v>
+        <v>968.1491079363354</v>
       </c>
       <c r="J109" t="n">
-        <v>1251.255144293726</v>
+        <v>739.9563631957411</v>
       </c>
       <c r="K109" t="n">
-        <v>953.7066709806782</v>
+        <v>567.8425131164117</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="D110" t="n">
         <v>1000</v>
       </c>
       <c r="E110" t="n">
-        <v>1390.6</v>
+        <v>823.5</v>
       </c>
       <c r="F110" t="n">
-        <v>1715.16604</v>
+        <v>939.36645</v>
       </c>
       <c r="G110" t="n">
-        <v>1928.018145564</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H110" t="n">
-        <v>1842.799743530072</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I110" t="n">
-        <v>1932.359811065633</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J110" t="n">
-        <v>2502.212719348888</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K110" t="n">
-        <v>2078.337884691186</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D111" t="n">
         <v>1000</v>
       </c>
       <c r="E111" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F111" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G111" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H111" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I111" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J111" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K111" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
@@ -14872,184 +14934,184 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D112" t="n">
         <v>1000</v>
       </c>
       <c r="E112" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F112" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G112" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H112" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I112" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J112" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K112" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D113" t="n">
         <v>1000</v>
       </c>
       <c r="E113" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F113" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G113" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H113" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I113" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J113" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K113" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D114" t="n">
         <v>1000</v>
       </c>
       <c r="E114" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F114" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G114" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H114" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I114" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J114" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K114" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D115" t="n">
         <v>1000</v>
       </c>
       <c r="E115" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F115" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G115" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H115" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I115" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J115" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K115" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D116" t="n">
         <v>1000</v>
       </c>
       <c r="E116" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F116" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G116" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H116" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I116" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J116" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K116" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -15057,36 +15119,36 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D117" t="n">
         <v>1000</v>
       </c>
       <c r="E117" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F117" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G117" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H117" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I117" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J117" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K117" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -15094,221 +15156,221 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D118" t="n">
         <v>1000</v>
       </c>
       <c r="E118" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F118" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G118" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H118" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I118" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J118" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K118" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D119" t="n">
         <v>1000</v>
       </c>
       <c r="E119" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F119" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G119" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H119" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I119" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J119" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K119" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D120" t="n">
         <v>1000</v>
       </c>
       <c r="E120" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F120" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G120" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H120" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I120" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J120" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K120" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D121" t="n">
         <v>1000</v>
       </c>
       <c r="E121" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F121" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G121" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H121" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I121" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J121" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K121" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="D122" t="n">
         <v>1000</v>
       </c>
       <c r="E122" t="n">
-        <v>743.8000000000001</v>
+        <v>942</v>
       </c>
       <c r="F122" t="n">
-        <v>692.62656</v>
+        <v>730.2384</v>
       </c>
       <c r="G122" t="n">
-        <v>666.7223266560001</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H122" t="n">
-        <v>724.7938413077377</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I122" t="n">
-        <v>681.3786902134042</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J122" t="n">
-        <v>441.2608397822005</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K122" t="n">
-        <v>291.4527846761434</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D123" t="n">
         <v>1000</v>
       </c>
       <c r="E123" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F123" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G123" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H123" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I123" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J123" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K123" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -15316,36 +15378,36 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D124" t="n">
         <v>1000</v>
       </c>
       <c r="E124" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F124" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G124" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H124" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I124" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J124" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K124" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -15353,36 +15415,36 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D125" t="n">
         <v>1000</v>
       </c>
       <c r="E125" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F125" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G125" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H125" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I125" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J125" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K125" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -15390,73 +15452,73 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D126" t="n">
         <v>1000</v>
       </c>
       <c r="E126" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F126" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G126" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H126" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I126" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J126" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K126" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D127" t="n">
         <v>1000</v>
       </c>
       <c r="E127" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F127" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G127" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H127" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I127" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J127" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K127" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
@@ -15493,81 +15555,81 @@
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D129" t="n">
         <v>1000</v>
       </c>
       <c r="E129" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F129" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G129" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H129" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I129" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J129" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K129" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D130" t="n">
         <v>1000</v>
       </c>
       <c r="E130" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F130" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G130" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H130" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I130" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J130" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K130" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -15575,36 +15637,36 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D131" t="n">
         <v>1000</v>
       </c>
       <c r="E131" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F131" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G131" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H131" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I131" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J131" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K131" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -15612,30 +15674,67 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D132" t="n">
         <v>1000</v>
       </c>
       <c r="E132" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F132" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G132" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H132" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I132" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J132" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K132" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>41</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D133" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E133" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F132" t="n">
+      <c r="F133" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G132" t="n">
+      <c r="G133" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H132" t="n">
+      <c r="H133" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I132" t="n">
+      <c r="I133" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J132" t="n">
+      <c r="J133" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K132" t="n">
+      <c r="K133" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 133 dMamba+features seed=0 -0.91 (regression confirmed across seeds)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$133</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$134</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>135</row>
+      <row>136</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T133"/>
+  <dimension ref="A1:T134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9097,16 +9097,16 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>MLP+features bs=64 seed=42 - large-batch on new features</t>
+          <t>dMamba+features seed=0 - 2nd seed for feature impact verify (was -1.28 seed=42)</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -9115,60 +9115,60 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>-0.9127</v>
+        <v>-0.9064</v>
       </c>
       <c r="F107" t="n">
-        <v>0.2667</v>
+        <v>0.3581</v>
       </c>
       <c r="G107" t="n">
-        <v>-0.6127</v>
+        <v>-0.5064</v>
       </c>
       <c r="I107" t="n">
-        <v>21.96</v>
+        <v>26.32</v>
       </c>
       <c r="J107" t="n">
-        <v>1219.6</v>
+        <v>1263.2</v>
       </c>
       <c r="K107" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L107" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N107" t="n">
-        <v>-0.0177</v>
+        <v>0.0298</v>
       </c>
       <c r="O107" t="n">
-        <v>50.53</v>
+        <v>48.91</v>
       </c>
       <c r="P107" t="n">
-        <v>0.5562</v>
+        <v>0.5903</v>
       </c>
       <c r="Q107" t="n">
-        <v>0.6679</v>
+        <v>0.4475</v>
       </c>
       <c r="R107" t="n">
-        <v>0.607</v>
+        <v>0.5091</v>
       </c>
       <c r="S107" t="n">
-        <v>-0.0482</v>
+        <v>-0.0039</v>
       </c>
       <c r="T107" t="n">
-        <v>19.9</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>18</v>
+        <v>132</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
+          <t>MLP+features bs=64 seed=42 - large-batch on new features</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -9177,60 +9177,60 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>-0.9217</v>
+        <v>-0.9127</v>
       </c>
       <c r="F108" t="n">
-        <v>0.5942</v>
+        <v>0.2667</v>
       </c>
       <c r="G108" t="n">
-        <v>-0.7217</v>
+        <v>-0.6127</v>
       </c>
       <c r="I108" t="n">
-        <v>58.5</v>
+        <v>21.96</v>
       </c>
       <c r="J108" t="n">
-        <v>1585</v>
+        <v>1219.6</v>
       </c>
       <c r="K108" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L108" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N108" t="n">
-        <v>0.019</v>
+        <v>-0.0177</v>
       </c>
       <c r="O108" t="n">
-        <v>48.5</v>
+        <v>50.53</v>
       </c>
       <c r="P108" t="n">
-        <v>0.5986</v>
+        <v>0.5562</v>
       </c>
       <c r="Q108" t="n">
-        <v>0.3987</v>
+        <v>0.6679</v>
       </c>
       <c r="R108" t="n">
-        <v>0.4786</v>
+        <v>0.607</v>
       </c>
       <c r="S108" t="n">
-        <v>0.0103</v>
+        <v>-0.0482</v>
       </c>
       <c r="T108" t="n">
-        <v>18919.4</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
+          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -9239,51 +9239,51 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="F109" t="n">
-        <v>-0.2367</v>
+        <v>0.5942</v>
       </c>
       <c r="G109" t="n">
-        <v>-0.5226</v>
+        <v>-0.7217</v>
       </c>
       <c r="I109" t="n">
-        <v>-43.21</v>
+        <v>58.5</v>
       </c>
       <c r="J109" t="n">
-        <v>567.9000000000001</v>
+        <v>1585</v>
       </c>
       <c r="K109" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N109" t="n">
-        <v>-0.0164</v>
+        <v>0.019</v>
       </c>
       <c r="O109" t="n">
-        <v>45.63</v>
+        <v>48.5</v>
       </c>
       <c r="P109" t="n">
-        <v>0.5938</v>
+        <v>0.5986</v>
       </c>
       <c r="Q109" t="n">
-        <v>0.1648</v>
+        <v>0.3987</v>
       </c>
       <c r="R109" t="n">
-        <v>0.258</v>
+        <v>0.4786</v>
       </c>
       <c r="S109" t="n">
-        <v>0.0188</v>
+        <v>0.0103</v>
       </c>
       <c r="T109" t="n">
-        <v>33.8</v>
+        <v>18919.4</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -9292,7 +9292,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -9301,60 +9301,60 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="F110" t="n">
-        <v>0.1045</v>
+        <v>-0.2367</v>
       </c>
       <c r="G110" t="n">
-        <v>-0.6746</v>
+        <v>-0.5226</v>
       </c>
       <c r="I110" t="n">
-        <v>-4.63</v>
+        <v>-43.21</v>
       </c>
       <c r="J110" t="n">
-        <v>953.7</v>
+        <v>567.9000000000001</v>
       </c>
       <c r="K110" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L110" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N110" t="n">
-        <v>-0.0374</v>
+        <v>-0.0164</v>
       </c>
       <c r="O110" t="n">
-        <v>51.03</v>
+        <v>45.63</v>
       </c>
       <c r="P110" t="n">
-        <v>0.5765</v>
+        <v>0.5938</v>
       </c>
       <c r="Q110" t="n">
-        <v>0.5415</v>
+        <v>0.1648</v>
       </c>
       <c r="R110" t="n">
-        <v>0.5585</v>
+        <v>0.258</v>
       </c>
       <c r="S110" t="n">
-        <v>0.0091</v>
+        <v>0.0188</v>
       </c>
       <c r="T110" t="n">
-        <v>30.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -9363,60 +9363,60 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="F111" t="n">
-        <v>0.8788</v>
+        <v>0.1045</v>
       </c>
       <c r="G111" t="n">
-        <v>-0.866</v>
+        <v>-0.6746</v>
       </c>
       <c r="I111" t="n">
-        <v>107.82</v>
+        <v>-4.63</v>
       </c>
       <c r="J111" t="n">
-        <v>2078.2</v>
+        <v>953.7</v>
       </c>
       <c r="K111" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L111" t="n">
         <v>2</v>
       </c>
       <c r="N111" t="n">
-        <v>0.0329</v>
+        <v>-0.0374</v>
       </c>
       <c r="O111" t="n">
-        <v>54.14</v>
+        <v>51.03</v>
       </c>
       <c r="P111" t="n">
-        <v>0.6011</v>
+        <v>0.5765</v>
       </c>
       <c r="Q111" t="n">
-        <v>0.6725</v>
+        <v>0.5415</v>
       </c>
       <c r="R111" t="n">
-        <v>0.6348</v>
+        <v>0.5585</v>
       </c>
       <c r="S111" t="n">
-        <v>0.0251</v>
+        <v>0.0091</v>
       </c>
       <c r="T111" t="n">
-        <v>75.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -9425,51 +9425,51 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F112" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G112" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I112" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J112" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K112" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L112" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N112" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O112" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P112" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q112" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R112" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S112" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T112" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -9478,7 +9478,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -9487,60 +9487,60 @@
         </is>
       </c>
       <c r="E113" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F113" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G113" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I113" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J113" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K113" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L113" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N113" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O113" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P113" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q113" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R113" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S113" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T113" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -9549,60 +9549,60 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F114" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G114" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I114" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J114" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K114" t="n">
         <v>2</v>
       </c>
       <c r="L114" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N114" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O114" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P114" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q114" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R114" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S114" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T114" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -9611,60 +9611,60 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F115" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G115" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I115" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J115" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K115" t="n">
+        <v>2</v>
+      </c>
+      <c r="L115" t="n">
         <v>5</v>
       </c>
-      <c r="L115" t="n">
-        <v>2</v>
-      </c>
       <c r="N115" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O115" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P115" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q115" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R115" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S115" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T115" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -9673,60 +9673,60 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F116" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G116" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I116" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J116" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K116" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L116" t="n">
         <v>2</v>
       </c>
       <c r="N116" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O116" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P116" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q116" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R116" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S116" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T116" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -9735,51 +9735,51 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F117" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G117" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I117" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J117" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K117" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L117" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N117" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O117" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P117" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q117" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R117" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S117" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T117" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -9788,7 +9788,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -9797,51 +9797,51 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F118" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G118" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I118" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J118" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K118" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L118" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N118" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O118" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P118" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q118" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R118" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S118" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T118" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -9850,7 +9850,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -9859,60 +9859,60 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F119" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G119" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I119" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J119" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K119" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L119" t="n">
         <v>2</v>
       </c>
       <c r="N119" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O119" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P119" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q119" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R119" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S119" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T119" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -9921,60 +9921,60 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F120" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G120" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I120" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J120" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K120" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L120" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N120" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O120" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P120" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q120" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R120" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S120" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T120" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -9983,60 +9983,60 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F121" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G121" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I121" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J121" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K121" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L121" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N121" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O121" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P121" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q121" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R121" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S121" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T121" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -10045,60 +10045,60 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F122" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G122" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I122" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J122" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K122" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L122" t="n">
         <v>3</v>
       </c>
       <c r="N122" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O122" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P122" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q122" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R122" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S122" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T122" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -10107,60 +10107,60 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="F123" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.8189</v>
       </c>
       <c r="G123" t="n">
-        <v>-0.8347</v>
+        <v>1.1456</v>
       </c>
       <c r="I123" t="n">
-        <v>-70.84999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J123" t="n">
-        <v>291.5000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K123" t="n">
         <v>1</v>
       </c>
       <c r="L123" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N123" t="n">
-        <v>0.0284</v>
+        <v>0.0089</v>
       </c>
       <c r="O123" t="n">
-        <v>44.07</v>
+        <v>41.44</v>
       </c>
       <c r="P123" t="n">
-        <v>0.5588</v>
+        <v>0.68</v>
       </c>
       <c r="Q123" t="n">
-        <v>0.1177</v>
+        <v>0.0271</v>
       </c>
       <c r="R123" t="n">
-        <v>0.1945</v>
+        <v>0.0521</v>
       </c>
       <c r="S123" t="n">
-        <v>-0.0101</v>
+        <v>0.0277</v>
       </c>
       <c r="T123" t="n">
-        <v>79.8</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -10169,39 +10169,51 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F124" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G124" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I124" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J124" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K124" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L124" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N124" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O124" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P124" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R124" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S124" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T124" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -10210,7 +10222,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -10219,51 +10231,39 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F125" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G125" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I125" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J125" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K125" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L125" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N125" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O125" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P125" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q125" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R125" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S125" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T125" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -10272,7 +10272,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -10281,51 +10281,51 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F126" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G126" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I126" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J126" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K126" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L126" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N126" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O126" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P126" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q126" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R126" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S126" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T126" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -10334,7 +10334,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -10343,113 +10343,113 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F127" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G127" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I127" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J127" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K127" t="n">
         <v>1</v>
       </c>
       <c r="L127" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N127" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O127" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P127" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q127" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R127" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S127" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T127" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
+        <v>59</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F128" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G128" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I128" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J128" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K128" t="n">
         <v>1</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E128" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F128" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G128" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I128" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J128" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K128" t="n">
-        <v>5</v>
       </c>
       <c r="L128" t="n">
         <v>1</v>
       </c>
       <c r="N128" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O128" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P128" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q128" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R128" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S128" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T128" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -10458,12 +10458,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -10506,21 +10506,21 @@
         <v>0.0098</v>
       </c>
       <c r="T129" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -10529,19 +10529,19 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F130" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G130" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I130" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J130" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K130" t="n">
         <v>5</v>
@@ -10550,39 +10550,39 @@
         <v>1</v>
       </c>
       <c r="N130" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O130" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P130" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q130" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R130" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S130" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T130" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -10591,113 +10591,113 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F131" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G131" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I131" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J131" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K131" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N131" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O131" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P131" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q131" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R131" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S131" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T131" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
+        <v>22</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F132" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G132" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I132" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J132" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K132" t="n">
+        <v>4</v>
+      </c>
+      <c r="L132" t="n">
         <v>2</v>
       </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E132" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F132" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G132" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I132" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J132" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K132" t="n">
-        <v>5</v>
-      </c>
-      <c r="L132" t="n">
-        <v>1</v>
-      </c>
       <c r="N132" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O132" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P132" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q132" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R132" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S132" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T132" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -10706,7 +10706,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -10715,51 +10715,113 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F133" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G133" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I133" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J133" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K133" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L133" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N133" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O133" t="n">
         <v>47.65</v>
       </c>
       <c r="P133" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R133" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S133" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T133" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>41</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F134" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G134" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I134" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J134" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K134" t="n">
+        <v>4</v>
+      </c>
+      <c r="L134" t="n">
+        <v>2</v>
+      </c>
+      <c r="N134" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O134" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P134" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q133" t="n">
+      <c r="Q134" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R133" t="n">
+      <c r="R134" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S133" t="n">
+      <c r="S134" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T133" t="n">
+      <c r="T134" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T133"/>
-  <conditionalFormatting sqref="E2:E133">
+  <autoFilter ref="A1:T134"/>
+  <conditionalFormatting sqref="E2:E134">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -10781,7 +10843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K133"/>
+  <dimension ref="A1:K134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -14741,118 +14803,118 @@
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>-0.9127</v>
+        <v>-0.9064</v>
       </c>
       <c r="D107" t="n">
         <v>1000</v>
       </c>
       <c r="E107" t="n">
-        <v>824.6</v>
+        <v>1700.1</v>
       </c>
       <c r="F107" t="n">
-        <v>945.8162000000001</v>
+        <v>1752.29307</v>
       </c>
       <c r="G107" t="n">
-        <v>1155.40906992</v>
+        <v>1726.709591178</v>
       </c>
       <c r="H107" t="n">
-        <v>1037.55734478816</v>
+        <v>1516.223692013402</v>
       </c>
       <c r="I107" t="n">
-        <v>1136.955338418866</v>
+        <v>1576.569394955535</v>
       </c>
       <c r="J107" t="n">
-        <v>1027.125452727604</v>
+        <v>1391.164834108764</v>
       </c>
       <c r="K107" t="n">
-        <v>1219.506050023484</v>
+        <v>1263.177669370758</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>18</v>
+        <v>132</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>-0.9217</v>
+        <v>-0.9127</v>
       </c>
       <c r="D108" t="n">
         <v>1000</v>
       </c>
       <c r="E108" t="n">
-        <v>1206.3</v>
+        <v>824.6</v>
       </c>
       <c r="F108" t="n">
-        <v>1403.65068</v>
+        <v>945.8162000000001</v>
       </c>
       <c r="G108" t="n">
-        <v>1572.930952008</v>
+        <v>1155.40906992</v>
       </c>
       <c r="H108" t="n">
-        <v>1622.320983901051</v>
+        <v>1037.55734478816</v>
       </c>
       <c r="I108" t="n">
-        <v>1560.023858119251</v>
+        <v>1136.955338418866</v>
       </c>
       <c r="J108" t="n">
-        <v>2085.595895919627</v>
+        <v>1027.125452727604</v>
       </c>
       <c r="K108" t="n">
-        <v>1584.844321309324</v>
+        <v>1219.506050023484</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="D109" t="n">
         <v>1000</v>
       </c>
       <c r="E109" t="n">
-        <v>1141.9</v>
+        <v>1206.3</v>
       </c>
       <c r="F109" t="n">
-        <v>983.4042799999999</v>
+        <v>1403.65068</v>
       </c>
       <c r="G109" t="n">
-        <v>1002.482323032</v>
+        <v>1572.930952008</v>
       </c>
       <c r="H109" t="n">
-        <v>1006.392004091825</v>
+        <v>1622.320983901051</v>
       </c>
       <c r="I109" t="n">
-        <v>968.1491079363354</v>
+        <v>1560.023858119251</v>
       </c>
       <c r="J109" t="n">
-        <v>739.9563631957411</v>
+        <v>2085.595895919627</v>
       </c>
       <c r="K109" t="n">
-        <v>567.8425131164117</v>
+        <v>1584.844321309324</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -14860,110 +14922,110 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>-0.9746</v>
+        <v>-0.9226</v>
       </c>
       <c r="D110" t="n">
         <v>1000</v>
       </c>
       <c r="E110" t="n">
-        <v>823.5</v>
+        <v>1141.9</v>
       </c>
       <c r="F110" t="n">
-        <v>939.36645</v>
+        <v>983.4042799999999</v>
       </c>
       <c r="G110" t="n">
-        <v>1037.24843409</v>
+        <v>1002.482323032</v>
       </c>
       <c r="H110" t="n">
-        <v>968.582587753242</v>
+        <v>1006.392004091825</v>
       </c>
       <c r="I110" t="n">
-        <v>996.38090802176</v>
+        <v>968.1491079363354</v>
       </c>
       <c r="J110" t="n">
-        <v>1251.255144293726</v>
+        <v>739.9563631957411</v>
       </c>
       <c r="K110" t="n">
-        <v>953.7066709806782</v>
+        <v>567.8425131164117</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="D111" t="n">
         <v>1000</v>
       </c>
       <c r="E111" t="n">
-        <v>1390.6</v>
+        <v>823.5</v>
       </c>
       <c r="F111" t="n">
-        <v>1715.16604</v>
+        <v>939.36645</v>
       </c>
       <c r="G111" t="n">
-        <v>1928.018145564</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H111" t="n">
-        <v>1842.799743530072</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I111" t="n">
-        <v>1932.359811065633</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J111" t="n">
-        <v>2502.212719348888</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K111" t="n">
-        <v>2078.337884691186</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D112" t="n">
         <v>1000</v>
       </c>
       <c r="E112" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F112" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G112" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H112" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I112" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J112" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K112" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
@@ -14971,184 +15033,184 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D113" t="n">
         <v>1000</v>
       </c>
       <c r="E113" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F113" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G113" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H113" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I113" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J113" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K113" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D114" t="n">
         <v>1000</v>
       </c>
       <c r="E114" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F114" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G114" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H114" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I114" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J114" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K114" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D115" t="n">
         <v>1000</v>
       </c>
       <c r="E115" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F115" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G115" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H115" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I115" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J115" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K115" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D116" t="n">
         <v>1000</v>
       </c>
       <c r="E116" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F116" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G116" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H116" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I116" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J116" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K116" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D117" t="n">
         <v>1000</v>
       </c>
       <c r="E117" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F117" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G117" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H117" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I117" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J117" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K117" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -15156,36 +15218,36 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D118" t="n">
         <v>1000</v>
       </c>
       <c r="E118" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F118" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G118" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H118" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I118" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J118" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K118" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -15193,221 +15255,221 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D119" t="n">
         <v>1000</v>
       </c>
       <c r="E119" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F119" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G119" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H119" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I119" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J119" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K119" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D120" t="n">
         <v>1000</v>
       </c>
       <c r="E120" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F120" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G120" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H120" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I120" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J120" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K120" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D121" t="n">
         <v>1000</v>
       </c>
       <c r="E121" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F121" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G121" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H121" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I121" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J121" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K121" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D122" t="n">
         <v>1000</v>
       </c>
       <c r="E122" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F122" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G122" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H122" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I122" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J122" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K122" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="D123" t="n">
         <v>1000</v>
       </c>
       <c r="E123" t="n">
-        <v>743.8000000000001</v>
+        <v>942</v>
       </c>
       <c r="F123" t="n">
-        <v>692.62656</v>
+        <v>730.2384</v>
       </c>
       <c r="G123" t="n">
-        <v>666.7223266560001</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H123" t="n">
-        <v>724.7938413077377</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I123" t="n">
-        <v>681.3786902134042</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J123" t="n">
-        <v>441.2608397822005</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K123" t="n">
-        <v>291.4527846761434</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D124" t="n">
         <v>1000</v>
       </c>
       <c r="E124" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F124" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G124" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H124" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I124" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J124" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K124" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -15415,36 +15477,36 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D125" t="n">
         <v>1000</v>
       </c>
       <c r="E125" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F125" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G125" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H125" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I125" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J125" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K125" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -15452,36 +15514,36 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D126" t="n">
         <v>1000</v>
       </c>
       <c r="E126" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F126" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G126" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H126" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I126" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J126" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K126" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -15489,73 +15551,73 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D127" t="n">
         <v>1000</v>
       </c>
       <c r="E127" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F127" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G127" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H127" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I127" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J127" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K127" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D128" t="n">
         <v>1000</v>
       </c>
       <c r="E128" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F128" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G128" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H128" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I128" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J128" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K128" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -15592,81 +15654,81 @@
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D130" t="n">
         <v>1000</v>
       </c>
       <c r="E130" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F130" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G130" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H130" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I130" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J130" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K130" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D131" t="n">
         <v>1000</v>
       </c>
       <c r="E131" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F131" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G131" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H131" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I131" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J131" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K131" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -15674,36 +15736,36 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D132" t="n">
         <v>1000</v>
       </c>
       <c r="E132" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F132" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G132" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H132" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I132" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J132" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K132" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -15711,30 +15773,67 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D133" t="n">
         <v>1000</v>
       </c>
       <c r="E133" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F133" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G133" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H133" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I133" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J133" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K133" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>41</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D134" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E134" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F133" t="n">
+      <c r="F134" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G133" t="n">
+      <c r="G134" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H133" t="n">
+      <c r="H134" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I133" t="n">
+      <c r="I134" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J133" t="n">
+      <c r="J134" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K133" t="n">
+      <c r="K134" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 140 DLinear+features 3-seed mean -0.09 (exp 138 was lucky)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$140</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>142</row>
+      <row>143</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T140"/>
+  <dimension ref="A1:T141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9717,16 +9717,16 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>dlinear</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>DLinear+features seed=7 - 3rd seed for stable champion check</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -9735,60 +9735,60 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>-0.9746</v>
+        <v>-0.9331</v>
       </c>
       <c r="F117" t="n">
-        <v>0.1045</v>
+        <v>-0.4331</v>
       </c>
       <c r="G117" t="n">
-        <v>-0.6746</v>
+        <v>0.1475</v>
       </c>
       <c r="I117" t="n">
-        <v>-4.63</v>
+        <v>-57.86</v>
       </c>
       <c r="J117" t="n">
-        <v>953.7</v>
+        <v>421.4</v>
       </c>
       <c r="K117" t="n">
+        <v>2</v>
+      </c>
+      <c r="L117" t="n">
         <v>4</v>
       </c>
-      <c r="L117" t="n">
-        <v>2</v>
-      </c>
       <c r="N117" t="n">
-        <v>-0.0374</v>
+        <v>-0.0041</v>
       </c>
       <c r="O117" t="n">
-        <v>51.03</v>
+        <v>46.62</v>
       </c>
       <c r="P117" t="n">
-        <v>0.5765</v>
+        <v>0.5621</v>
       </c>
       <c r="Q117" t="n">
-        <v>0.5415</v>
+        <v>0.3086</v>
       </c>
       <c r="R117" t="n">
-        <v>0.5585</v>
+        <v>0.3984</v>
       </c>
       <c r="S117" t="n">
-        <v>0.0091</v>
+        <v>-0.014</v>
       </c>
       <c r="T117" t="n">
-        <v>30.6</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -9797,60 +9797,60 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="F118" t="n">
-        <v>0.8788</v>
+        <v>0.1045</v>
       </c>
       <c r="G118" t="n">
-        <v>-0.866</v>
+        <v>-0.6746</v>
       </c>
       <c r="I118" t="n">
-        <v>107.82</v>
+        <v>-4.63</v>
       </c>
       <c r="J118" t="n">
-        <v>2078.2</v>
+        <v>953.7</v>
       </c>
       <c r="K118" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L118" t="n">
         <v>2</v>
       </c>
       <c r="N118" t="n">
-        <v>0.0329</v>
+        <v>-0.0374</v>
       </c>
       <c r="O118" t="n">
-        <v>54.14</v>
+        <v>51.03</v>
       </c>
       <c r="P118" t="n">
-        <v>0.6011</v>
+        <v>0.5765</v>
       </c>
       <c r="Q118" t="n">
-        <v>0.6725</v>
+        <v>0.5415</v>
       </c>
       <c r="R118" t="n">
-        <v>0.6348</v>
+        <v>0.5585</v>
       </c>
       <c r="S118" t="n">
-        <v>0.0251</v>
+        <v>0.0091</v>
       </c>
       <c r="T118" t="n">
-        <v>75.8</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -9859,51 +9859,51 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F119" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G119" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I119" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J119" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K119" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L119" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N119" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O119" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P119" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q119" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R119" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S119" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T119" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -9912,7 +9912,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -9921,60 +9921,60 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F120" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G120" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I120" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J120" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K120" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L120" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N120" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O120" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P120" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q120" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R120" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S120" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T120" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -9983,60 +9983,60 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F121" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G121" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I121" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J121" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K121" t="n">
         <v>2</v>
       </c>
       <c r="L121" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N121" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O121" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P121" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q121" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R121" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S121" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T121" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -10045,60 +10045,60 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F122" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G122" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I122" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J122" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K122" t="n">
+        <v>2</v>
+      </c>
+      <c r="L122" t="n">
         <v>5</v>
       </c>
-      <c r="L122" t="n">
-        <v>2</v>
-      </c>
       <c r="N122" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O122" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P122" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q122" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R122" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S122" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T122" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -10107,60 +10107,60 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F123" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G123" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I123" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J123" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K123" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L123" t="n">
         <v>2</v>
       </c>
       <c r="N123" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O123" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P123" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q123" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R123" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S123" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T123" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -10169,51 +10169,51 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F124" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G124" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I124" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J124" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K124" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L124" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N124" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O124" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P124" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q124" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R124" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S124" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T124" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -10222,7 +10222,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -10231,51 +10231,51 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F125" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G125" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I125" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J125" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K125" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N125" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O125" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P125" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q125" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R125" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S125" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T125" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -10284,7 +10284,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -10293,60 +10293,60 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F126" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G126" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I126" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J126" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K126" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L126" t="n">
         <v>2</v>
       </c>
       <c r="N126" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O126" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P126" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q126" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R126" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S126" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T126" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -10355,60 +10355,60 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F127" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G127" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I127" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J127" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N127" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O127" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P127" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q127" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R127" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S127" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T127" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -10417,60 +10417,60 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F128" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G128" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I128" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J128" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L128" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N128" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O128" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P128" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q128" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R128" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S128" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T128" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -10479,60 +10479,60 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F129" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G129" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I129" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J129" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K129" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L129" t="n">
         <v>3</v>
       </c>
       <c r="N129" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O129" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P129" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q129" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R129" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S129" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T129" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -10541,60 +10541,60 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="F130" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.8189</v>
       </c>
       <c r="G130" t="n">
-        <v>-0.8347</v>
+        <v>1.1456</v>
       </c>
       <c r="I130" t="n">
-        <v>-70.84999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J130" t="n">
-        <v>291.5000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K130" t="n">
         <v>1</v>
       </c>
       <c r="L130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N130" t="n">
-        <v>0.0284</v>
+        <v>0.0089</v>
       </c>
       <c r="O130" t="n">
-        <v>44.07</v>
+        <v>41.44</v>
       </c>
       <c r="P130" t="n">
-        <v>0.5588</v>
+        <v>0.68</v>
       </c>
       <c r="Q130" t="n">
-        <v>0.1177</v>
+        <v>0.0271</v>
       </c>
       <c r="R130" t="n">
-        <v>0.1945</v>
+        <v>0.0521</v>
       </c>
       <c r="S130" t="n">
-        <v>-0.0101</v>
+        <v>0.0277</v>
       </c>
       <c r="T130" t="n">
-        <v>79.8</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -10603,39 +10603,51 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F131" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G131" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I131" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J131" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K131" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N131" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O131" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P131" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R131" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S131" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T131" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -10644,7 +10656,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -10653,51 +10665,39 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F132" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G132" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I132" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J132" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K132" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L132" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N132" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O132" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P132" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q132" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R132" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S132" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T132" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -10706,7 +10706,7 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -10715,51 +10715,51 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F133" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G133" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I133" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J133" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K133" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L133" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N133" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O133" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P133" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q133" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R133" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S133" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T133" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -10768,7 +10768,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -10777,113 +10777,113 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F134" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G134" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I134" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J134" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K134" t="n">
         <v>1</v>
       </c>
       <c r="L134" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N134" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O134" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P134" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q134" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R134" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S134" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T134" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
+        <v>59</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F135" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G135" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I135" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J135" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K135" t="n">
         <v>1</v>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E135" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F135" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G135" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I135" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J135" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K135" t="n">
-        <v>5</v>
       </c>
       <c r="L135" t="n">
         <v>1</v>
       </c>
       <c r="N135" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O135" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P135" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q135" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R135" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S135" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T135" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -10892,12 +10892,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -10940,21 +10940,21 @@
         <v>0.0098</v>
       </c>
       <c r="T136" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -10963,19 +10963,19 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F137" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G137" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I137" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J137" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K137" t="n">
         <v>5</v>
@@ -10984,39 +10984,39 @@
         <v>1</v>
       </c>
       <c r="N137" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O137" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P137" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q137" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R137" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S137" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T137" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -11025,113 +11025,113 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F138" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G138" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I138" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J138" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K138" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N138" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O138" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P138" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q138" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R138" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T138" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
+        <v>22</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F139" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G139" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I139" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J139" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K139" t="n">
+        <v>4</v>
+      </c>
+      <c r="L139" t="n">
         <v>2</v>
       </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E139" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F139" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G139" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I139" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J139" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K139" t="n">
-        <v>5</v>
-      </c>
-      <c r="L139" t="n">
-        <v>1</v>
-      </c>
       <c r="N139" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O139" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P139" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q139" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R139" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S139" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T139" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -11140,7 +11140,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -11149,51 +11149,113 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F140" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G140" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I140" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J140" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K140" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L140" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N140" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O140" t="n">
         <v>47.65</v>
       </c>
       <c r="P140" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q140" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R140" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S140" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T140" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>41</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E141" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F141" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G141" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I141" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J141" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K141" t="n">
+        <v>4</v>
+      </c>
+      <c r="L141" t="n">
+        <v>2</v>
+      </c>
+      <c r="N141" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O141" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P141" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q140" t="n">
+      <c r="Q141" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R140" t="n">
+      <c r="R141" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S140" t="n">
+      <c r="S141" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T140" t="n">
+      <c r="T141" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T140"/>
-  <conditionalFormatting sqref="E2:E140">
+  <autoFilter ref="A1:T141"/>
+  <conditionalFormatting sqref="E2:E141">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11215,7 +11277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K140"/>
+  <dimension ref="A1:K141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -15545,118 +15607,118 @@
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>dlinear</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-0.9746</v>
+        <v>-0.9331</v>
       </c>
       <c r="D117" t="n">
         <v>1000</v>
       </c>
       <c r="E117" t="n">
-        <v>823.5</v>
+        <v>916.6999999999999</v>
       </c>
       <c r="F117" t="n">
-        <v>939.36645</v>
+        <v>699.35043</v>
       </c>
       <c r="G117" t="n">
-        <v>1037.24843409</v>
+        <v>591.5105936939999</v>
       </c>
       <c r="H117" t="n">
-        <v>968.582587753242</v>
+        <v>525.7937667345965</v>
       </c>
       <c r="I117" t="n">
-        <v>996.38090802176</v>
+        <v>531.9455538053913</v>
       </c>
       <c r="J117" t="n">
-        <v>1251.255144293726</v>
+        <v>546.4144728688981</v>
       </c>
       <c r="K117" t="n">
-        <v>953.7066709806782</v>
+        <v>421.4494829237811</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-1.066</v>
+        <v>-0.9746</v>
       </c>
       <c r="D118" t="n">
         <v>1000</v>
       </c>
       <c r="E118" t="n">
-        <v>1390.6</v>
+        <v>823.5</v>
       </c>
       <c r="F118" t="n">
-        <v>1715.16604</v>
+        <v>939.36645</v>
       </c>
       <c r="G118" t="n">
-        <v>1928.018145564</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H118" t="n">
-        <v>1842.799743530072</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I118" t="n">
-        <v>1932.359811065633</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J118" t="n">
-        <v>2502.212719348888</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K118" t="n">
-        <v>2078.337884691186</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D119" t="n">
         <v>1000</v>
       </c>
       <c r="E119" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F119" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G119" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H119" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I119" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J119" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K119" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -15664,184 +15726,184 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D120" t="n">
         <v>1000</v>
       </c>
       <c r="E120" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F120" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G120" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H120" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I120" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J120" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K120" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D121" t="n">
         <v>1000</v>
       </c>
       <c r="E121" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F121" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G121" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H121" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I121" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J121" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K121" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D122" t="n">
         <v>1000</v>
       </c>
       <c r="E122" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F122" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G122" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H122" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I122" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J122" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K122" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D123" t="n">
         <v>1000</v>
       </c>
       <c r="E123" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F123" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G123" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H123" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I123" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J123" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K123" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D124" t="n">
         <v>1000</v>
       </c>
       <c r="E124" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F124" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G124" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H124" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I124" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J124" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K124" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -15849,36 +15911,36 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D125" t="n">
         <v>1000</v>
       </c>
       <c r="E125" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F125" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G125" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H125" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I125" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J125" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K125" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -15886,221 +15948,221 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D126" t="n">
         <v>1000</v>
       </c>
       <c r="E126" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F126" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G126" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H126" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I126" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J126" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K126" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D127" t="n">
         <v>1000</v>
       </c>
       <c r="E127" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F127" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G127" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H127" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I127" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J127" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K127" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D128" t="n">
         <v>1000</v>
       </c>
       <c r="E128" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F128" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G128" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H128" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I128" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J128" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K128" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D129" t="n">
         <v>1000</v>
       </c>
       <c r="E129" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F129" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G129" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H129" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I129" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J129" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K129" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-1.4347</v>
+        <v>-1.4189</v>
       </c>
       <c r="D130" t="n">
         <v>1000</v>
       </c>
       <c r="E130" t="n">
-        <v>743.8000000000001</v>
+        <v>942</v>
       </c>
       <c r="F130" t="n">
-        <v>692.62656</v>
+        <v>730.2384</v>
       </c>
       <c r="G130" t="n">
-        <v>666.7223266560001</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H130" t="n">
-        <v>724.7938413077377</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I130" t="n">
-        <v>681.3786902134042</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J130" t="n">
-        <v>441.2608397822005</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K130" t="n">
-        <v>291.4527846761434</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D131" t="n">
         <v>1000</v>
       </c>
       <c r="E131" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F131" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G131" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H131" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I131" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J131" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K131" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -16108,36 +16170,36 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D132" t="n">
         <v>1000</v>
       </c>
       <c r="E132" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F132" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G132" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H132" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I132" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J132" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K132" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -16145,36 +16207,36 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D133" t="n">
         <v>1000</v>
       </c>
       <c r="E133" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F133" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G133" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H133" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I133" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J133" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K133" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -16182,73 +16244,73 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D134" t="n">
         <v>1000</v>
       </c>
       <c r="E134" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F134" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G134" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H134" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I134" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J134" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K134" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D135" t="n">
         <v>1000</v>
       </c>
       <c r="E135" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F135" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G135" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H135" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I135" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J135" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K135" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -16285,81 +16347,81 @@
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D137" t="n">
         <v>1000</v>
       </c>
       <c r="E137" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F137" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G137" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H137" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I137" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J137" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K137" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D138" t="n">
         <v>1000</v>
       </c>
       <c r="E138" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F138" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G138" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H138" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I138" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J138" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K138" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -16367,36 +16429,36 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D139" t="n">
         <v>1000</v>
       </c>
       <c r="E139" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F139" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G139" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H139" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I139" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J139" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K139" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -16404,30 +16466,67 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D140" t="n">
         <v>1000</v>
       </c>
       <c r="E140" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F140" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G140" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H140" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I140" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J140" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K140" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>41</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D141" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E141" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F140" t="n">
+      <c r="F141" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G140" t="n">
+      <c r="G141" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H140" t="n">
+      <c r="H141" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I140" t="n">
+      <c r="I141" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J140" t="n">
+      <c r="J141" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K140" t="n">
+      <c r="K141" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 144 N-BEATS -1.43 (FX result reproduced)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$144</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$145</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>146</row>
+      <row>147</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T144"/>
+  <dimension ref="A1:T145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10771,16 +10771,16 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -10789,60 +10789,60 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F134" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G134" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I134" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J134" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K134" t="n">
         <v>1</v>
       </c>
       <c r="L134" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N134" t="n">
-        <v>0.0284</v>
+        <v>0.0111</v>
       </c>
       <c r="O134" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P134" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q134" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R134" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S134" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T134" t="n">
-        <v>79.8</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -10851,39 +10851,51 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F135" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G135" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I135" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J135" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K135" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L135" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N135" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O135" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P135" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q135" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R135" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S135" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T135" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -10892,7 +10904,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -10901,51 +10913,39 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F136" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G136" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I136" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J136" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K136" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N136" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O136" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P136" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q136" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R136" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S136" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T136" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -10954,7 +10954,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -10963,51 +10963,51 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F137" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G137" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I137" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J137" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L137" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N137" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O137" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P137" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q137" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R137" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S137" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T137" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -11016,7 +11016,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -11025,113 +11025,113 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F138" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G138" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I138" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J138" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K138" t="n">
         <v>1</v>
       </c>
       <c r="L138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N138" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O138" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P138" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q138" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R138" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T138" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
+        <v>59</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>mlp</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E139" t="n">
+        <v>-1.5134</v>
+      </c>
+      <c r="F139" t="n">
+        <v>-0.5178</v>
+      </c>
+      <c r="G139" t="n">
+        <v>-0.9134</v>
+      </c>
+      <c r="I139" t="n">
+        <v>-62.95</v>
+      </c>
+      <c r="J139" t="n">
+        <v>370.4999999999999</v>
+      </c>
+      <c r="K139" t="n">
         <v>1</v>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>smoke</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>KEEP</t>
-        </is>
-      </c>
-      <c r="E139" t="n">
-        <v>-1.5423</v>
-      </c>
-      <c r="F139" t="n">
-        <v>0.5694</v>
-      </c>
-      <c r="G139" t="n">
-        <v>-1.3423</v>
-      </c>
-      <c r="I139" t="n">
-        <v>54.77</v>
-      </c>
-      <c r="J139" t="n">
-        <v>1547.7</v>
-      </c>
-      <c r="K139" t="n">
-        <v>5</v>
       </c>
       <c r="L139" t="n">
         <v>1</v>
       </c>
       <c r="N139" t="n">
-        <v>0.0103</v>
+        <v>-0.0025</v>
       </c>
       <c r="O139" t="n">
-        <v>51.13</v>
+        <v>44.99</v>
       </c>
       <c r="P139" t="n">
-        <v>0.5968</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q139" t="n">
-        <v>0.5364</v>
+        <v>0.2032</v>
       </c>
       <c r="R139" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.2976</v>
       </c>
       <c r="S139" t="n">
-        <v>0.0098</v>
+        <v>-0.0171</v>
       </c>
       <c r="T139" t="n">
-        <v>97.8</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -11140,12 +11140,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -11188,21 +11188,21 @@
         <v>0.0098</v>
       </c>
       <c r="T140" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -11211,19 +11211,19 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F141" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G141" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I141" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J141" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K141" t="n">
         <v>5</v>
@@ -11232,39 +11232,39 @@
         <v>1</v>
       </c>
       <c r="N141" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O141" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P141" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q141" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R141" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S141" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T141" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -11273,113 +11273,113 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F142" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G142" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I142" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J142" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K142" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L142" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N142" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O142" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P142" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q142" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R142" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S142" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T142" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
+        <v>22</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>-1.7766</v>
+      </c>
+      <c r="F143" t="n">
+        <v>0.2915</v>
+      </c>
+      <c r="G143" t="n">
+        <v>-1.4766</v>
+      </c>
+      <c r="I143" t="n">
+        <v>18.69</v>
+      </c>
+      <c r="J143" t="n">
+        <v>1186.9</v>
+      </c>
+      <c r="K143" t="n">
+        <v>4</v>
+      </c>
+      <c r="L143" t="n">
         <v>2</v>
       </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>xgboost</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>DISCARD</t>
-        </is>
-      </c>
-      <c r="E143" t="n">
-        <v>-2.3923</v>
-      </c>
-      <c r="F143" t="n">
-        <v>-0.0045</v>
-      </c>
-      <c r="G143" t="n">
-        <v>-2.1923</v>
-      </c>
-      <c r="I143" t="n">
-        <v>-10.56</v>
-      </c>
-      <c r="J143" t="n">
-        <v>894.4</v>
-      </c>
-      <c r="K143" t="n">
-        <v>5</v>
-      </c>
-      <c r="L143" t="n">
-        <v>1</v>
-      </c>
       <c r="N143" t="n">
-        <v>-0.0018</v>
+        <v>0.0052</v>
       </c>
       <c r="O143" t="n">
-        <v>47.65</v>
+        <v>47.84</v>
       </c>
       <c r="P143" t="n">
-        <v>0.583</v>
+        <v>0.5918</v>
       </c>
       <c r="Q143" t="n">
-        <v>0.4114</v>
+        <v>0.3877</v>
       </c>
       <c r="R143" t="n">
-        <v>0.4824</v>
+        <v>0.4685</v>
       </c>
       <c r="S143" t="n">
-        <v>-0.0161</v>
+        <v>-0.0009</v>
       </c>
       <c r="T143" t="n">
-        <v>335.3</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -11388,7 +11388,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -11397,51 +11397,113 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F144" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G144" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I144" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J144" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K144" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L144" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N144" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O144" t="n">
         <v>47.65</v>
       </c>
       <c r="P144" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q144" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R144" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S144" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T144" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>41</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F145" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G145" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I145" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J145" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K145" t="n">
+        <v>4</v>
+      </c>
+      <c r="L145" t="n">
+        <v>2</v>
+      </c>
+      <c r="N145" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O145" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P145" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q144" t="n">
+      <c r="Q145" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R144" t="n">
+      <c r="R145" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S144" t="n">
+      <c r="S145" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T144" t="n">
+      <c r="T145" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T144"/>
-  <conditionalFormatting sqref="E2:E144">
+  <autoFilter ref="A1:T145"/>
+  <conditionalFormatting sqref="E2:E145">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11463,7 +11525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K144"/>
+  <dimension ref="A1:K145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -16422,81 +16484,81 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D134" t="n">
         <v>1000</v>
       </c>
       <c r="E134" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F134" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G134" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H134" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I134" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J134" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K134" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D135" t="n">
         <v>1000</v>
       </c>
       <c r="E135" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F135" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G135" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H135" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I135" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J135" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K135" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -16504,36 +16566,36 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D136" t="n">
         <v>1000</v>
       </c>
       <c r="E136" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F136" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G136" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H136" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I136" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J136" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K136" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -16541,36 +16603,36 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D137" t="n">
         <v>1000</v>
       </c>
       <c r="E137" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F137" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G137" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H137" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I137" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J137" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K137" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -16578,73 +16640,73 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D138" t="n">
         <v>1000</v>
       </c>
       <c r="E138" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F138" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G138" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H138" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I138" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J138" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K138" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-1.5423</v>
+        <v>-1.5134</v>
       </c>
       <c r="D139" t="n">
         <v>1000</v>
       </c>
       <c r="E139" t="n">
-        <v>1342</v>
+        <v>892.7</v>
       </c>
       <c r="F139" t="n">
-        <v>1365.6192</v>
+        <v>712.64241</v>
       </c>
       <c r="G139" t="n">
-        <v>1401.67154688</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H139" t="n">
-        <v>1356.1172216064</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I139" t="n">
-        <v>1614.321940600259</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J139" t="n">
-        <v>1682.93062307577</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K139" t="n">
-        <v>1547.623000980478</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -16681,81 +16743,81 @@
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D141" t="n">
         <v>1000</v>
       </c>
       <c r="E141" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F141" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G141" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H141" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I141" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J141" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K141" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D142" t="n">
         <v>1000</v>
       </c>
       <c r="E142" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F142" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G142" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H142" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I142" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J142" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K142" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -16763,36 +16825,36 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-2.3923</v>
+        <v>-1.7766</v>
       </c>
       <c r="D143" t="n">
         <v>1000</v>
       </c>
       <c r="E143" t="n">
-        <v>982.1</v>
+        <v>1165.9</v>
       </c>
       <c r="F143" t="n">
-        <v>1102.11262</v>
+        <v>1389.63621</v>
       </c>
       <c r="G143" t="n">
-        <v>1215.07916355</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H143" t="n">
-        <v>1137.07108125009</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I143" t="n">
-        <v>1227.127110885097</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J143" t="n">
-        <v>1233.5081718617</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K143" t="n">
-        <v>894.5401262341047</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -16800,30 +16862,67 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D144" t="n">
         <v>1000</v>
       </c>
       <c r="E144" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F144" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G144" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H144" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I144" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J144" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K144" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>41</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D145" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E145" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F144" t="n">
+      <c r="F145" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G144" t="n">
+      <c r="G145" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H144" t="n">
+      <c r="H145" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I144" t="n">
+      <c r="I145" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J144" t="n">
+      <c r="J145" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K144" t="n">
+      <c r="K145" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 146 PatchTSMixer seed=0 -1.82 (high variance)
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$147</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>148</row>
+      <row>149</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T146"/>
+  <dimension ref="A1:T147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11441,16 +11441,16 @@
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>2</v>
+        <v>146</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -11459,51 +11459,51 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>-2.3923</v>
+        <v>-1.8201</v>
       </c>
       <c r="F145" t="n">
-        <v>-0.0045</v>
+        <v>-1.2201</v>
       </c>
       <c r="G145" t="n">
-        <v>-2.1923</v>
+        <v>-0.255</v>
       </c>
       <c r="I145" t="n">
-        <v>-10.56</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J145" t="n">
-        <v>894.4</v>
+        <v>282.4</v>
       </c>
       <c r="K145" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L145" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N145" t="n">
-        <v>-0.0018</v>
+        <v>-0.0322</v>
       </c>
       <c r="O145" t="n">
-        <v>47.65</v>
+        <v>40.59</v>
       </c>
       <c r="P145" t="n">
-        <v>0.583</v>
+        <v>0</v>
       </c>
       <c r="Q145" t="n">
-        <v>0.4114</v>
+        <v>0</v>
       </c>
       <c r="R145" t="n">
-        <v>0.4824</v>
+        <v>0</v>
       </c>
       <c r="S145" t="n">
-        <v>-0.0161</v>
+        <v>0</v>
       </c>
       <c r="T145" t="n">
-        <v>335.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -11512,7 +11512,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -11521,51 +11521,113 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F146" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G146" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I146" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J146" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K146" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L146" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N146" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O146" t="n">
         <v>47.65</v>
       </c>
       <c r="P146" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q146" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R146" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S146" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T146" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>41</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F147" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G147" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I147" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J147" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K147" t="n">
+        <v>4</v>
+      </c>
+      <c r="L147" t="n">
+        <v>2</v>
+      </c>
+      <c r="N147" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O147" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P147" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q146" t="n">
+      <c r="Q147" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R146" t="n">
+      <c r="R147" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S146" t="n">
+      <c r="S147" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T146" t="n">
+      <c r="T147" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T146"/>
-  <conditionalFormatting sqref="E2:E146">
+  <autoFilter ref="A1:T147"/>
+  <conditionalFormatting sqref="E2:E147">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -11587,7 +11649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K146"/>
+  <dimension ref="A1:K147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -16953,44 +17015,44 @@
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>2</v>
+        <v>146</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-2.3923</v>
+        <v>-1.8201</v>
       </c>
       <c r="D145" t="n">
         <v>1000</v>
       </c>
       <c r="E145" t="n">
-        <v>982.1</v>
+        <v>942</v>
       </c>
       <c r="F145" t="n">
-        <v>1102.11262</v>
+        <v>730.2384</v>
       </c>
       <c r="G145" t="n">
-        <v>1215.07916355</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H145" t="n">
-        <v>1137.07108125009</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I145" t="n">
-        <v>1227.127110885097</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J145" t="n">
-        <v>1233.5081718617</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K145" t="n">
-        <v>894.5401262341047</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -16998,30 +17060,67 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D146" t="n">
         <v>1000</v>
       </c>
       <c r="E146" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F146" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G146" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H146" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I146" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J146" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K146" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>41</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D147" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E147" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F146" t="n">
+      <c r="F147" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G146" t="n">
+      <c r="G147" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H146" t="n">
+      <c r="H147" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I146" t="n">
+      <c r="I147" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J146" t="n">
+      <c r="J147" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K146" t="n">
+      <c r="K147" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 157 dMamba 3-layer -1.52
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$158</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>159</row>
+      <row>160</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T157"/>
+  <dimension ref="A1:T158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11813,69 +11813,69 @@
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E151" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="F151" t="n">
-        <v>0.5694</v>
+        <v>-1.0225</v>
       </c>
       <c r="G151" t="n">
-        <v>-1.3423</v>
+        <v>-0.2617</v>
       </c>
       <c r="I151" t="n">
-        <v>54.77</v>
+        <v>-65.97</v>
       </c>
       <c r="J151" t="n">
-        <v>1547.7</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K151" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L151" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N151" t="n">
-        <v>0.0103</v>
+        <v>-0.0076</v>
       </c>
       <c r="O151" t="n">
-        <v>51.13</v>
+        <v>40.96</v>
       </c>
       <c r="P151" t="n">
-        <v>0.5968</v>
+        <v>0.5526</v>
       </c>
       <c r="Q151" t="n">
-        <v>0.5364</v>
+        <v>0.0334</v>
       </c>
       <c r="R151" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.0631</v>
       </c>
       <c r="S151" t="n">
-        <v>0.0098</v>
+        <v>-0.0156</v>
       </c>
       <c r="T151" t="n">
-        <v>97.8</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -11884,12 +11884,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -11932,21 +11932,21 @@
         <v>0.0098</v>
       </c>
       <c r="T152" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -11955,19 +11955,19 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F153" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G153" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I153" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J153" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K153" t="n">
         <v>5</v>
@@ -11976,39 +11976,39 @@
         <v>1</v>
       </c>
       <c r="N153" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O153" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P153" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q153" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R153" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S153" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T153" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -12017,60 +12017,60 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F154" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G154" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I154" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J154" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K154" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L154" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N154" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O154" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P154" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q154" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R154" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S154" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T154" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -12079,60 +12079,60 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F155" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G155" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I155" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J155" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K155" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L155" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N155" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O155" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P155" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q155" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R155" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S155" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T155" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>2</v>
+        <v>146</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -12141,51 +12141,51 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>-2.3923</v>
+        <v>-1.8201</v>
       </c>
       <c r="F156" t="n">
-        <v>-0.0045</v>
+        <v>-1.2201</v>
       </c>
       <c r="G156" t="n">
-        <v>-2.1923</v>
+        <v>-0.255</v>
       </c>
       <c r="I156" t="n">
-        <v>-10.56</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J156" t="n">
-        <v>894.4</v>
+        <v>282.4</v>
       </c>
       <c r="K156" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L156" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N156" t="n">
-        <v>-0.0018</v>
+        <v>-0.0322</v>
       </c>
       <c r="O156" t="n">
-        <v>47.65</v>
+        <v>40.59</v>
       </c>
       <c r="P156" t="n">
-        <v>0.583</v>
+        <v>0</v>
       </c>
       <c r="Q156" t="n">
-        <v>0.4114</v>
+        <v>0</v>
       </c>
       <c r="R156" t="n">
-        <v>0.4824</v>
+        <v>0</v>
       </c>
       <c r="S156" t="n">
-        <v>-0.0161</v>
+        <v>0</v>
       </c>
       <c r="T156" t="n">
-        <v>335.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -12194,7 +12194,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -12203,51 +12203,113 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F157" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G157" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I157" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J157" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K157" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L157" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N157" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O157" t="n">
         <v>47.65</v>
       </c>
       <c r="P157" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R157" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S157" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T157" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>41</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E158" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F158" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G158" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I158" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J158" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K158" t="n">
+        <v>4</v>
+      </c>
+      <c r="L158" t="n">
+        <v>2</v>
+      </c>
+      <c r="N158" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O158" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P158" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q157" t="n">
+      <c r="Q158" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R157" t="n">
+      <c r="R158" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S157" t="n">
+      <c r="S158" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T157" t="n">
+      <c r="T158" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T157"/>
-  <conditionalFormatting sqref="E2:E157">
+  <autoFilter ref="A1:T158"/>
+  <conditionalFormatting sqref="E2:E158">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -12269,7 +12331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K157"/>
+  <dimension ref="A1:K158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -17857,44 +17919,44 @@
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="D151" t="n">
         <v>1000</v>
       </c>
       <c r="E151" t="n">
-        <v>1342</v>
+        <v>1141.5</v>
       </c>
       <c r="F151" t="n">
-        <v>1365.6192</v>
+        <v>884.8908</v>
       </c>
       <c r="G151" t="n">
-        <v>1401.67154688</v>
+        <v>789.49957176</v>
       </c>
       <c r="H151" t="n">
-        <v>1356.1172216064</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I151" t="n">
-        <v>1614.321940600259</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J151" t="n">
-        <v>1682.93062307577</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K151" t="n">
-        <v>1547.623000980478</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -17931,155 +17993,155 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D153" t="n">
         <v>1000</v>
       </c>
       <c r="E153" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F153" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G153" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H153" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I153" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J153" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K153" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D154" t="n">
         <v>1000</v>
       </c>
       <c r="E154" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F154" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G154" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H154" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I154" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J154" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K154" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D155" t="n">
         <v>1000</v>
       </c>
       <c r="E155" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F155" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G155" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H155" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I155" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J155" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K155" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>2</v>
+        <v>146</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>-2.3923</v>
+        <v>-1.8201</v>
       </c>
       <c r="D156" t="n">
         <v>1000</v>
       </c>
       <c r="E156" t="n">
-        <v>982.1</v>
+        <v>942</v>
       </c>
       <c r="F156" t="n">
-        <v>1102.11262</v>
+        <v>730.2384</v>
       </c>
       <c r="G156" t="n">
-        <v>1215.07916355</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H156" t="n">
-        <v>1137.07108125009</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I156" t="n">
-        <v>1227.127110885097</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J156" t="n">
-        <v>1233.5081718617</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K156" t="n">
-        <v>894.5401262341047</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -18087,30 +18149,67 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D157" t="n">
         <v>1000</v>
       </c>
       <c r="E157" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F157" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G157" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H157" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I157" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J157" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K157" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>41</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D158" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E158" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F157" t="n">
+      <c r="F158" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G157" t="n">
+      <c r="G158" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H157" t="n">
+      <c r="H158" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I157" t="n">
+      <c r="I158" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J157" t="n">
+      <c r="J158" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K157" t="n">
+      <c r="K158" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 158 MLP combo -2.21
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$158</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$159</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>160</row>
+      <row>161</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T158"/>
+  <dimension ref="A1:T159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12185,16 +12185,16 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -12203,51 +12203,51 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F157" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G157" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I157" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J157" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K157" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L157" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N157" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O157" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P157" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q157" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R157" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S157" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T157" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -12256,7 +12256,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -12265,51 +12265,113 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F158" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G158" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I158" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J158" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K158" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L158" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N158" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O158" t="n">
         <v>47.65</v>
       </c>
       <c r="P158" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R158" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S158" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T158" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>41</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E159" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F159" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G159" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I159" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J159" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K159" t="n">
+        <v>4</v>
+      </c>
+      <c r="L159" t="n">
+        <v>2</v>
+      </c>
+      <c r="N159" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O159" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P159" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q158" t="n">
+      <c r="Q159" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R158" t="n">
+      <c r="R159" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S158" t="n">
+      <c r="S159" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T158" t="n">
+      <c r="T159" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T158"/>
-  <conditionalFormatting sqref="E2:E158">
+  <autoFilter ref="A1:T159"/>
+  <conditionalFormatting sqref="E2:E159">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -12331,7 +12393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K158"/>
+  <dimension ref="A1:K159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -18141,44 +18203,44 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D157" t="n">
         <v>1000</v>
       </c>
       <c r="E157" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F157" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G157" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H157" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I157" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J157" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K157" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -18186,30 +18248,67 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D158" t="n">
         <v>1000</v>
       </c>
       <c r="E158" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F158" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G158" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H158" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I158" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J158" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K158" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>41</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D159" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E159" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F158" t="n">
+      <c r="F159" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G158" t="n">
+      <c r="G159" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H158" t="n">
+      <c r="H159" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I158" t="n">
+      <c r="I159" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J158" t="n">
+      <c r="J159" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K158" t="n">
+      <c r="K159" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 160 XGBoost seed=2024 -1.00
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$161</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>162</row>
+      <row>163</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T160"/>
+  <dimension ref="A1:T161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10771,7 +10771,7 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -10780,7 +10780,7 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>XGBoost @ exp 44 seed=2024 - 5-seed lock</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -10789,19 +10789,19 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>-1.066</v>
+        <v>-0.9961</v>
       </c>
       <c r="F134" t="n">
-        <v>0.8788</v>
+        <v>0.4602</v>
       </c>
       <c r="G134" t="n">
-        <v>-0.866</v>
+        <v>-0.7961</v>
       </c>
       <c r="I134" t="n">
-        <v>107.82</v>
+        <v>39.45</v>
       </c>
       <c r="J134" t="n">
-        <v>2078.2</v>
+        <v>1394.5</v>
       </c>
       <c r="K134" t="n">
         <v>5</v>
@@ -10810,39 +10810,39 @@
         <v>2</v>
       </c>
       <c r="N134" t="n">
-        <v>0.0329</v>
+        <v>0.0172</v>
       </c>
       <c r="O134" t="n">
-        <v>54.14</v>
+        <v>50.19</v>
       </c>
       <c r="P134" t="n">
-        <v>0.6011</v>
+        <v>0.5927</v>
       </c>
       <c r="Q134" t="n">
-        <v>0.6725</v>
+        <v>0.5111</v>
       </c>
       <c r="R134" t="n">
-        <v>0.6348</v>
+        <v>0.5489000000000001</v>
       </c>
       <c r="S134" t="n">
-        <v>0.0251</v>
+        <v>0.0007</v>
       </c>
       <c r="T134" t="n">
-        <v>75.8</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -10851,51 +10851,51 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F135" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G135" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I135" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J135" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K135" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L135" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N135" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O135" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P135" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q135" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R135" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S135" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T135" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -10904,7 +10904,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -10913,60 +10913,60 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F136" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G136" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I136" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J136" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K136" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L136" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N136" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O136" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P136" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q136" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R136" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S136" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T136" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -10975,60 +10975,60 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F137" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G137" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I137" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J137" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K137" t="n">
         <v>2</v>
       </c>
       <c r="L137" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N137" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O137" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P137" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q137" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R137" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S137" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T137" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -11037,60 +11037,60 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F138" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G138" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I138" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J138" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K138" t="n">
+        <v>2</v>
+      </c>
+      <c r="L138" t="n">
         <v>5</v>
       </c>
-      <c r="L138" t="n">
-        <v>2</v>
-      </c>
       <c r="N138" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O138" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P138" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q138" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R138" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T138" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -11099,60 +11099,60 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F139" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G139" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I139" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J139" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K139" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L139" t="n">
         <v>2</v>
       </c>
       <c r="N139" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O139" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P139" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q139" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R139" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S139" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T139" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -11161,51 +11161,51 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F140" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G140" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I140" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J140" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K140" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L140" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N140" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O140" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P140" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q140" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R140" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S140" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T140" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -11214,7 +11214,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -11223,51 +11223,51 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F141" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G141" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I141" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J141" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K141" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L141" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N141" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O141" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P141" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q141" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R141" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S141" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T141" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -11276,7 +11276,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -11285,60 +11285,60 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F142" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G142" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I142" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J142" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K142" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L142" t="n">
         <v>2</v>
       </c>
       <c r="N142" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O142" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P142" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q142" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R142" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S142" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T142" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -11347,60 +11347,60 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F143" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G143" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I143" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J143" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K143" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L143" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N143" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O143" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P143" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q143" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R143" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S143" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T143" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -11409,60 +11409,60 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F144" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G144" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I144" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J144" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K144" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L144" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N144" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O144" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P144" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q144" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R144" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S144" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T144" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -11471,60 +11471,60 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F145" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G145" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I145" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J145" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K145" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L145" t="n">
         <v>3</v>
       </c>
       <c r="N145" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O145" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P145" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q145" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R145" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S145" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T145" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -11533,19 +11533,19 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="F146" t="n">
-        <v>-0.6042</v>
+        <v>-0.8189</v>
       </c>
       <c r="G146" t="n">
-        <v>-0.8305</v>
+        <v>1.1456</v>
       </c>
       <c r="I146" t="n">
-        <v>-67.48999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J146" t="n">
-        <v>325.1000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K146" t="n">
         <v>1</v>
@@ -11554,39 +11554,39 @@
         <v>3</v>
       </c>
       <c r="N146" t="n">
-        <v>0.0111</v>
+        <v>0.0089</v>
       </c>
       <c r="O146" t="n">
-        <v>42.64</v>
+        <v>41.44</v>
       </c>
       <c r="P146" t="n">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="Q146" t="n">
-        <v>0</v>
+        <v>0.0271</v>
       </c>
       <c r="R146" t="n">
-        <v>0</v>
+        <v>0.0521</v>
       </c>
       <c r="S146" t="n">
-        <v>0</v>
+        <v>0.0277</v>
       </c>
       <c r="T146" t="n">
-        <v>82.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -11595,60 +11595,60 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F147" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G147" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I147" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J147" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K147" t="n">
         <v>1</v>
       </c>
       <c r="L147" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N147" t="n">
-        <v>0.0284</v>
+        <v>0.0111</v>
       </c>
       <c r="O147" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P147" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q147" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R147" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S147" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T147" t="n">
-        <v>79.8</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -11657,39 +11657,51 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F148" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G148" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I148" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J148" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K148" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N148" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O148" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P148" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R148" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S148" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T148" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -11698,7 +11710,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -11707,51 +11719,39 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F149" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G149" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I149" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J149" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K149" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L149" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N149" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O149" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P149" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q149" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R149" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S149" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T149" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -11760,7 +11760,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -11769,51 +11769,51 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F150" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G150" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I150" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J150" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K150" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L150" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N150" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O150" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P150" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q150" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R150" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S150" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T150" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -11822,7 +11822,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -11831,60 +11831,60 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F151" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G151" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I151" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J151" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K151" t="n">
         <v>1</v>
       </c>
       <c r="L151" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N151" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O151" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P151" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q151" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R151" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S151" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T151" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -11893,113 +11893,113 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F152" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G152" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I152" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J152" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K152" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L152" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N152" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O152" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P152" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q152" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R152" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S152" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T152" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E153" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="F153" t="n">
-        <v>0.5694</v>
+        <v>-1.0225</v>
       </c>
       <c r="G153" t="n">
-        <v>-1.3423</v>
+        <v>-0.2617</v>
       </c>
       <c r="I153" t="n">
-        <v>54.77</v>
+        <v>-65.97</v>
       </c>
       <c r="J153" t="n">
-        <v>1547.7</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K153" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L153" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N153" t="n">
-        <v>0.0103</v>
+        <v>-0.0076</v>
       </c>
       <c r="O153" t="n">
-        <v>51.13</v>
+        <v>40.96</v>
       </c>
       <c r="P153" t="n">
-        <v>0.5968</v>
+        <v>0.5526</v>
       </c>
       <c r="Q153" t="n">
-        <v>0.5364</v>
+        <v>0.0334</v>
       </c>
       <c r="R153" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.0631</v>
       </c>
       <c r="S153" t="n">
-        <v>0.0098</v>
+        <v>-0.0156</v>
       </c>
       <c r="T153" t="n">
-        <v>97.8</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -12008,12 +12008,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -12056,21 +12056,21 @@
         <v>0.0098</v>
       </c>
       <c r="T154" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -12079,19 +12079,19 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F155" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G155" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I155" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J155" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K155" t="n">
         <v>5</v>
@@ -12100,39 +12100,39 @@
         <v>1</v>
       </c>
       <c r="N155" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O155" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P155" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q155" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R155" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S155" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T155" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -12141,60 +12141,60 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F156" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G156" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I156" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J156" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K156" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L156" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N156" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O156" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P156" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q156" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R156" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S156" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T156" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -12203,60 +12203,60 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F157" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G157" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I157" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J157" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K157" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L157" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N157" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O157" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P157" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q157" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R157" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S157" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T157" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -12265,60 +12265,60 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="F158" t="n">
-        <v>-0.3397</v>
+        <v>-1.2201</v>
       </c>
       <c r="G158" t="n">
-        <v>-1.8082</v>
+        <v>-0.255</v>
       </c>
       <c r="I158" t="n">
-        <v>-51.44</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J158" t="n">
-        <v>485.6</v>
+        <v>282.4</v>
       </c>
       <c r="K158" t="n">
+        <v>1</v>
+      </c>
+      <c r="L158" t="n">
         <v>3</v>
       </c>
-      <c r="L158" t="n">
+      <c r="N158" t="n">
+        <v>-0.0322</v>
+      </c>
+      <c r="O158" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="P158" t="n">
         <v>0</v>
       </c>
-      <c r="N158" t="n">
-        <v>-0.0003</v>
-      </c>
-      <c r="O158" t="n">
-        <v>45.06</v>
-      </c>
-      <c r="P158" t="n">
-        <v>0.5895</v>
-      </c>
       <c r="Q158" t="n">
-        <v>0.1388</v>
+        <v>0</v>
       </c>
       <c r="R158" t="n">
-        <v>0.2247</v>
+        <v>0</v>
       </c>
       <c r="S158" t="n">
-        <v>0.0137</v>
+        <v>0</v>
       </c>
       <c r="T158" t="n">
-        <v>40.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -12327,51 +12327,51 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F159" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G159" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I159" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J159" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K159" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L159" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N159" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O159" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P159" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q159" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R159" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S159" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T159" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -12380,7 +12380,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -12389,51 +12389,113 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F160" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G160" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I160" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J160" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K160" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L160" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N160" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O160" t="n">
         <v>47.65</v>
       </c>
       <c r="P160" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R160" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S160" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T160" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>41</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E161" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F161" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G161" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I161" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J161" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K161" t="n">
+        <v>4</v>
+      </c>
+      <c r="L161" t="n">
+        <v>2</v>
+      </c>
+      <c r="N161" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O161" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P161" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q160" t="n">
+      <c r="Q161" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R160" t="n">
+      <c r="R161" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S160" t="n">
+      <c r="S161" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T160" t="n">
+      <c r="T161" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T160"/>
-  <conditionalFormatting sqref="E2:E160">
+  <autoFilter ref="A1:T161"/>
+  <conditionalFormatting sqref="E2:E161">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -12455,7 +12517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K160"/>
+  <dimension ref="A1:K161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -17414,7 +17476,7 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -17422,73 +17484,73 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-1.066</v>
+        <v>-0.9961</v>
       </c>
       <c r="D134" t="n">
         <v>1000</v>
       </c>
       <c r="E134" t="n">
-        <v>1390.6</v>
+        <v>866</v>
       </c>
       <c r="F134" t="n">
-        <v>1715.16604</v>
+        <v>1018.3294</v>
       </c>
       <c r="G134" t="n">
-        <v>1928.018145564</v>
+        <v>1148.57373026</v>
       </c>
       <c r="H134" t="n">
-        <v>1842.799743530072</v>
+        <v>1130.885694813996</v>
       </c>
       <c r="I134" t="n">
-        <v>1932.359811065633</v>
+        <v>1184.150411039735</v>
       </c>
       <c r="J134" t="n">
-        <v>2502.212719348888</v>
+        <v>1292.144928526559</v>
       </c>
       <c r="K134" t="n">
-        <v>2078.337884691186</v>
+        <v>1394.612021358715</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D135" t="n">
         <v>1000</v>
       </c>
       <c r="E135" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F135" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G135" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H135" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I135" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J135" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K135" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -17496,184 +17558,184 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D136" t="n">
         <v>1000</v>
       </c>
       <c r="E136" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F136" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G136" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H136" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I136" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J136" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K136" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D137" t="n">
         <v>1000</v>
       </c>
       <c r="E137" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F137" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G137" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H137" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I137" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J137" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K137" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D138" t="n">
         <v>1000</v>
       </c>
       <c r="E138" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F138" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G138" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H138" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I138" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J138" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K138" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D139" t="n">
         <v>1000</v>
       </c>
       <c r="E139" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F139" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G139" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H139" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I139" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J139" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K139" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D140" t="n">
         <v>1000</v>
       </c>
       <c r="E140" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F140" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G140" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H140" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I140" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J140" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K140" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
@@ -17681,36 +17743,36 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D141" t="n">
         <v>1000</v>
       </c>
       <c r="E141" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F141" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G141" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H141" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I141" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J141" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K141" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -17718,258 +17780,258 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D142" t="n">
         <v>1000</v>
       </c>
       <c r="E142" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F142" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G142" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H142" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I142" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J142" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K142" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D143" t="n">
         <v>1000</v>
       </c>
       <c r="E143" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F143" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G143" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H143" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I143" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J143" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K143" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D144" t="n">
         <v>1000</v>
       </c>
       <c r="E144" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F144" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G144" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H144" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I144" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J144" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K144" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D145" t="n">
         <v>1000</v>
       </c>
       <c r="E145" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F145" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G145" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H145" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I145" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J145" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K145" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="D146" t="n">
         <v>1000</v>
       </c>
       <c r="E146" t="n">
-        <v>1045.3</v>
+        <v>942</v>
       </c>
       <c r="F146" t="n">
-        <v>853.06933</v>
+        <v>730.2384</v>
       </c>
       <c r="G146" t="n">
-        <v>749.933248003</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H146" t="n">
-        <v>740.3341024285616</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I146" t="n">
-        <v>691.1759180273051</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J146" t="n">
-        <v>482.7172611502699</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K146" t="n">
-        <v>325.0618036585918</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D147" t="n">
         <v>1000</v>
       </c>
       <c r="E147" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F147" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G147" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H147" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I147" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J147" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K147" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D148" t="n">
         <v>1000</v>
       </c>
       <c r="E148" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F148" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G148" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H148" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I148" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J148" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K148" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
@@ -17977,36 +18039,36 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D149" t="n">
         <v>1000</v>
       </c>
       <c r="E149" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F149" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G149" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H149" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I149" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J149" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K149" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -18014,36 +18076,36 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D150" t="n">
         <v>1000</v>
       </c>
       <c r="E150" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F150" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G150" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H150" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I150" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J150" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K150" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -18051,110 +18113,110 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D151" t="n">
         <v>1000</v>
       </c>
       <c r="E151" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F151" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G151" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H151" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I151" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J151" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K151" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D152" t="n">
         <v>1000</v>
       </c>
       <c r="E152" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F152" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G152" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H152" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I152" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J152" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K152" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="D153" t="n">
         <v>1000</v>
       </c>
       <c r="E153" t="n">
-        <v>1342</v>
+        <v>1141.5</v>
       </c>
       <c r="F153" t="n">
-        <v>1365.6192</v>
+        <v>884.8908</v>
       </c>
       <c r="G153" t="n">
-        <v>1401.67154688</v>
+        <v>789.49957176</v>
       </c>
       <c r="H153" t="n">
-        <v>1356.1172216064</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I153" t="n">
-        <v>1614.321940600259</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J153" t="n">
-        <v>1682.93062307577</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K153" t="n">
-        <v>1547.623000980478</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -18191,192 +18253,192 @@
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D155" t="n">
         <v>1000</v>
       </c>
       <c r="E155" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F155" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G155" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H155" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I155" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J155" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K155" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D156" t="n">
         <v>1000</v>
       </c>
       <c r="E156" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F156" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G156" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H156" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I156" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J156" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K156" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D157" t="n">
         <v>1000</v>
       </c>
       <c r="E157" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F157" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G157" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H157" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I157" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J157" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K157" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="D158" t="n">
         <v>1000</v>
       </c>
       <c r="E158" t="n">
-        <v>1000.2</v>
+        <v>942</v>
       </c>
       <c r="F158" t="n">
-        <v>765.0529799999999</v>
+        <v>730.2384</v>
       </c>
       <c r="G158" t="n">
-        <v>773.1625415879998</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H158" t="n">
-        <v>742.158723670321</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I158" t="n">
-        <v>765.9078028277713</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J158" t="n">
-        <v>571.2906301292346</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K158" t="n">
-        <v>485.5970356098494</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D159" t="n">
         <v>1000</v>
       </c>
       <c r="E159" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F159" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G159" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H159" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I159" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J159" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K159" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -18384,30 +18446,67 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D160" t="n">
         <v>1000</v>
       </c>
       <c r="E160" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F160" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G160" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H160" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I160" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J160" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K160" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>41</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D161" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E161" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F160" t="n">
+      <c r="F161" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G160" t="n">
+      <c r="G161" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H160" t="n">
+      <c r="H161" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I160" t="n">
+      <c r="I161" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J160" t="n">
+      <c r="J161" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K160" t="n">
+      <c r="K161" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 161 MLP seed=13 -0.89
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$162</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>163</row>
+      <row>164</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T161"/>
+  <dimension ref="A1:T162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10399,16 +10399,16 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>dMamba+features seed=0 - 2nd seed for feature impact verify (was -1.28 seed=42)</t>
+          <t>MLP @ exp 6 seed=13 - extra seed for variance estimate</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -10417,60 +10417,60 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>-0.9064</v>
+        <v>-0.8895999999999999</v>
       </c>
       <c r="F128" t="n">
-        <v>0.3581</v>
+        <v>0.1034</v>
       </c>
       <c r="G128" t="n">
-        <v>-0.5064</v>
+        <v>-0.5896</v>
       </c>
       <c r="I128" t="n">
-        <v>26.32</v>
+        <v>-4.75</v>
       </c>
       <c r="J128" t="n">
-        <v>1263.2</v>
+        <v>952.5</v>
       </c>
       <c r="K128" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L128" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N128" t="n">
-        <v>0.0298</v>
+        <v>-0.029</v>
       </c>
       <c r="O128" t="n">
-        <v>48.91</v>
+        <v>48.12</v>
       </c>
       <c r="P128" t="n">
-        <v>0.5903</v>
+        <v>0.5625</v>
       </c>
       <c r="Q128" t="n">
-        <v>0.4475</v>
+        <v>0.4238</v>
       </c>
       <c r="R128" t="n">
-        <v>0.5091</v>
+        <v>0.4834</v>
       </c>
       <c r="S128" t="n">
-        <v>-0.0039</v>
+        <v>-0.0173</v>
       </c>
       <c r="T128" t="n">
-        <v>1579</v>
+        <v>21.6</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>MLP+features bs=64 seed=42 - large-batch on new features</t>
+          <t>dMamba+features seed=0 - 2nd seed for feature impact verify (was -1.28 seed=42)</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -10479,60 +10479,60 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>-0.9127</v>
+        <v>-0.9064</v>
       </c>
       <c r="F129" t="n">
-        <v>0.2667</v>
+        <v>0.3581</v>
       </c>
       <c r="G129" t="n">
-        <v>-0.6127</v>
+        <v>-0.5064</v>
       </c>
       <c r="I129" t="n">
-        <v>21.96</v>
+        <v>26.32</v>
       </c>
       <c r="J129" t="n">
-        <v>1219.6</v>
+        <v>1263.2</v>
       </c>
       <c r="K129" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L129" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N129" t="n">
-        <v>-0.0177</v>
+        <v>0.0298</v>
       </c>
       <c r="O129" t="n">
-        <v>50.53</v>
+        <v>48.91</v>
       </c>
       <c r="P129" t="n">
-        <v>0.5562</v>
+        <v>0.5903</v>
       </c>
       <c r="Q129" t="n">
-        <v>0.6679</v>
+        <v>0.4475</v>
       </c>
       <c r="R129" t="n">
-        <v>0.607</v>
+        <v>0.5091</v>
       </c>
       <c r="S129" t="n">
-        <v>-0.0482</v>
+        <v>-0.0039</v>
       </c>
       <c r="T129" t="n">
-        <v>19.9</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>18</v>
+        <v>132</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
+          <t>MLP+features bs=64 seed=42 - large-batch on new features</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -10541,60 +10541,60 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>-0.9217</v>
+        <v>-0.9127</v>
       </c>
       <c r="F130" t="n">
-        <v>0.5942</v>
+        <v>0.2667</v>
       </c>
       <c r="G130" t="n">
-        <v>-0.7217</v>
+        <v>-0.6127</v>
       </c>
       <c r="I130" t="n">
-        <v>58.5</v>
+        <v>21.96</v>
       </c>
       <c r="J130" t="n">
-        <v>1585</v>
+        <v>1219.6</v>
       </c>
       <c r="K130" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N130" t="n">
-        <v>0.019</v>
+        <v>-0.0177</v>
       </c>
       <c r="O130" t="n">
-        <v>48.5</v>
+        <v>50.53</v>
       </c>
       <c r="P130" t="n">
-        <v>0.5986</v>
+        <v>0.5562</v>
       </c>
       <c r="Q130" t="n">
-        <v>0.3987</v>
+        <v>0.6679</v>
       </c>
       <c r="R130" t="n">
-        <v>0.4786</v>
+        <v>0.607</v>
       </c>
       <c r="S130" t="n">
-        <v>0.0103</v>
+        <v>-0.0482</v>
       </c>
       <c r="T130" t="n">
-        <v>18919.4</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
+          <t>CatBoost @ FX-Exp236 FULL n_est=2000 (Prokhorenkova 2018 NeurIPS); QQQ — testing the long-</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -10603,60 +10603,60 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="F131" t="n">
-        <v>-0.2367</v>
+        <v>0.5942</v>
       </c>
       <c r="G131" t="n">
-        <v>-0.5226</v>
+        <v>-0.7217</v>
       </c>
       <c r="I131" t="n">
-        <v>-43.21</v>
+        <v>58.5</v>
       </c>
       <c r="J131" t="n">
-        <v>567.9000000000001</v>
+        <v>1585</v>
       </c>
       <c r="K131" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L131" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N131" t="n">
-        <v>-0.0164</v>
+        <v>0.019</v>
       </c>
       <c r="O131" t="n">
-        <v>45.63</v>
+        <v>48.5</v>
       </c>
       <c r="P131" t="n">
-        <v>0.5938</v>
+        <v>0.5986</v>
       </c>
       <c r="Q131" t="n">
-        <v>0.1648</v>
+        <v>0.3987</v>
       </c>
       <c r="R131" t="n">
-        <v>0.258</v>
+        <v>0.4786</v>
       </c>
       <c r="S131" t="n">
-        <v>0.0188</v>
+        <v>0.0103</v>
       </c>
       <c r="T131" t="n">
-        <v>33.8</v>
+        <v>18919.4</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>dlinear</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>DLinear+features seed=7 - 3rd seed for stable champion check</t>
+          <t>MLP @ exp 6 hd=0.20 (down from 0.25) - Srivastava 2014; less reg untested direction</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -10665,60 +10665,60 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>-0.9331</v>
+        <v>-0.9226</v>
       </c>
       <c r="F132" t="n">
-        <v>-0.4331</v>
+        <v>-0.2367</v>
       </c>
       <c r="G132" t="n">
-        <v>0.1475</v>
+        <v>-0.5226</v>
       </c>
       <c r="I132" t="n">
-        <v>-57.86</v>
+        <v>-43.21</v>
       </c>
       <c r="J132" t="n">
-        <v>421.4</v>
+        <v>567.9000000000001</v>
       </c>
       <c r="K132" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L132" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N132" t="n">
-        <v>-0.0041</v>
+        <v>-0.0164</v>
       </c>
       <c r="O132" t="n">
-        <v>46.62</v>
+        <v>45.63</v>
       </c>
       <c r="P132" t="n">
-        <v>0.5621</v>
+        <v>0.5938</v>
       </c>
       <c r="Q132" t="n">
-        <v>0.3086</v>
+        <v>0.1648</v>
       </c>
       <c r="R132" t="n">
-        <v>0.3984</v>
+        <v>0.258</v>
       </c>
       <c r="S132" t="n">
-        <v>-0.014</v>
+        <v>0.0188</v>
       </c>
       <c r="T132" t="n">
-        <v>23.6</v>
+        <v>33.8</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>dlinear</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>DLinear+features seed=7 - 3rd seed for stable champion check</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -10727,60 +10727,60 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>-0.9746</v>
+        <v>-0.9331</v>
       </c>
       <c r="F133" t="n">
-        <v>0.1045</v>
+        <v>-0.4331</v>
       </c>
       <c r="G133" t="n">
-        <v>-0.6746</v>
+        <v>0.1475</v>
       </c>
       <c r="I133" t="n">
-        <v>-4.63</v>
+        <v>-57.86</v>
       </c>
       <c r="J133" t="n">
-        <v>953.7</v>
+        <v>421.4</v>
       </c>
       <c r="K133" t="n">
+        <v>2</v>
+      </c>
+      <c r="L133" t="n">
         <v>4</v>
       </c>
-      <c r="L133" t="n">
-        <v>2</v>
-      </c>
       <c r="N133" t="n">
-        <v>-0.0374</v>
+        <v>-0.0041</v>
       </c>
       <c r="O133" t="n">
-        <v>51.03</v>
+        <v>46.62</v>
       </c>
       <c r="P133" t="n">
-        <v>0.5765</v>
+        <v>0.5621</v>
       </c>
       <c r="Q133" t="n">
-        <v>0.5415</v>
+        <v>0.3086</v>
       </c>
       <c r="R133" t="n">
-        <v>0.5585</v>
+        <v>0.3984</v>
       </c>
       <c r="S133" t="n">
-        <v>0.0091</v>
+        <v>-0.014</v>
       </c>
       <c r="T133" t="n">
-        <v>30.6</v>
+        <v>23.6</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 seed=2024 - 5-seed lock</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -10789,51 +10789,51 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>-0.9961</v>
+        <v>-0.9746</v>
       </c>
       <c r="F134" t="n">
-        <v>0.4602</v>
+        <v>0.1045</v>
       </c>
       <c r="G134" t="n">
-        <v>-0.7961</v>
+        <v>-0.6746</v>
       </c>
       <c r="I134" t="n">
-        <v>39.45</v>
+        <v>-4.63</v>
       </c>
       <c r="J134" t="n">
-        <v>1394.5</v>
+        <v>953.7</v>
       </c>
       <c r="K134" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L134" t="n">
         <v>2</v>
       </c>
       <c r="N134" t="n">
-        <v>0.0172</v>
+        <v>-0.0374</v>
       </c>
       <c r="O134" t="n">
-        <v>50.19</v>
+        <v>51.03</v>
       </c>
       <c r="P134" t="n">
-        <v>0.5927</v>
+        <v>0.5765</v>
       </c>
       <c r="Q134" t="n">
-        <v>0.5111</v>
+        <v>0.5415</v>
       </c>
       <c r="R134" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.5585</v>
       </c>
       <c r="S134" t="n">
-        <v>0.0007</v>
+        <v>0.0091</v>
       </c>
       <c r="T134" t="n">
-        <v>76.90000000000001</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -10842,7 +10842,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>XGBoost @ exp 44 seed=2024 - 5-seed lock</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -10851,19 +10851,19 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>-1.066</v>
+        <v>-0.9961</v>
       </c>
       <c r="F135" t="n">
-        <v>0.8788</v>
+        <v>0.4602</v>
       </c>
       <c r="G135" t="n">
-        <v>-0.866</v>
+        <v>-0.7961</v>
       </c>
       <c r="I135" t="n">
-        <v>107.82</v>
+        <v>39.45</v>
       </c>
       <c r="J135" t="n">
-        <v>2078.2</v>
+        <v>1394.5</v>
       </c>
       <c r="K135" t="n">
         <v>5</v>
@@ -10872,39 +10872,39 @@
         <v>2</v>
       </c>
       <c r="N135" t="n">
-        <v>0.0329</v>
+        <v>0.0172</v>
       </c>
       <c r="O135" t="n">
-        <v>54.14</v>
+        <v>50.19</v>
       </c>
       <c r="P135" t="n">
-        <v>0.6011</v>
+        <v>0.5927</v>
       </c>
       <c r="Q135" t="n">
-        <v>0.6725</v>
+        <v>0.5111</v>
       </c>
       <c r="R135" t="n">
-        <v>0.6348</v>
+        <v>0.5489000000000001</v>
       </c>
       <c r="S135" t="n">
-        <v>0.0251</v>
+        <v>0.0007</v>
       </c>
       <c r="T135" t="n">
-        <v>75.8</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -10913,51 +10913,51 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F136" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G136" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I136" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J136" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K136" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L136" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N136" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O136" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P136" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q136" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R136" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S136" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T136" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -10966,7 +10966,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -10975,60 +10975,60 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F137" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G137" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I137" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J137" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K137" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L137" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N137" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O137" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P137" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q137" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R137" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S137" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T137" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -11037,60 +11037,60 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F138" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G138" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I138" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J138" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K138" t="n">
         <v>2</v>
       </c>
       <c r="L138" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N138" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O138" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P138" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q138" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R138" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T138" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -11099,60 +11099,60 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F139" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G139" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I139" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J139" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K139" t="n">
+        <v>2</v>
+      </c>
+      <c r="L139" t="n">
         <v>5</v>
       </c>
-      <c r="L139" t="n">
-        <v>2</v>
-      </c>
       <c r="N139" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O139" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P139" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q139" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R139" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S139" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T139" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -11161,60 +11161,60 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F140" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G140" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I140" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J140" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K140" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L140" t="n">
         <v>2</v>
       </c>
       <c r="N140" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O140" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P140" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q140" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R140" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S140" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T140" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -11223,51 +11223,51 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F141" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G141" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I141" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J141" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K141" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L141" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N141" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O141" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P141" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q141" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R141" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S141" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T141" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -11276,7 +11276,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -11285,51 +11285,51 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F142" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G142" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I142" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J142" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K142" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L142" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N142" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O142" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P142" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q142" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R142" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S142" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T142" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -11338,7 +11338,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -11347,60 +11347,60 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F143" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G143" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I143" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J143" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K143" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L143" t="n">
         <v>2</v>
       </c>
       <c r="N143" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O143" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P143" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q143" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R143" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S143" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T143" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -11409,60 +11409,60 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F144" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G144" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I144" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J144" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K144" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L144" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N144" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O144" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P144" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q144" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R144" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S144" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T144" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -11471,60 +11471,60 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F145" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G145" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I145" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J145" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L145" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N145" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O145" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P145" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q145" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R145" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S145" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T145" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -11533,60 +11533,60 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F146" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G146" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I146" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J146" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L146" t="n">
         <v>3</v>
       </c>
       <c r="N146" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O146" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P146" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q146" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R146" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S146" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T146" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -11595,19 +11595,19 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="F147" t="n">
-        <v>-0.6042</v>
+        <v>-0.8189</v>
       </c>
       <c r="G147" t="n">
-        <v>-0.8305</v>
+        <v>1.1456</v>
       </c>
       <c r="I147" t="n">
-        <v>-67.48999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J147" t="n">
-        <v>325.1000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K147" t="n">
         <v>1</v>
@@ -11616,39 +11616,39 @@
         <v>3</v>
       </c>
       <c r="N147" t="n">
-        <v>0.0111</v>
+        <v>0.0089</v>
       </c>
       <c r="O147" t="n">
-        <v>42.64</v>
+        <v>41.44</v>
       </c>
       <c r="P147" t="n">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="Q147" t="n">
-        <v>0</v>
+        <v>0.0271</v>
       </c>
       <c r="R147" t="n">
-        <v>0</v>
+        <v>0.0521</v>
       </c>
       <c r="S147" t="n">
-        <v>0</v>
+        <v>0.0277</v>
       </c>
       <c r="T147" t="n">
-        <v>82.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -11657,60 +11657,60 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F148" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G148" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I148" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J148" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K148" t="n">
         <v>1</v>
       </c>
       <c r="L148" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N148" t="n">
-        <v>0.0284</v>
+        <v>0.0111</v>
       </c>
       <c r="O148" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P148" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q148" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R148" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S148" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T148" t="n">
-        <v>79.8</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -11719,39 +11719,51 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F149" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G149" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I149" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J149" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K149" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L149" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N149" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O149" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P149" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q149" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R149" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S149" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T149" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -11760,7 +11772,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -11769,51 +11781,39 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F150" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G150" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I150" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J150" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K150" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L150" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N150" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O150" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P150" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q150" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R150" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S150" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T150" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -11822,7 +11822,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -11831,51 +11831,51 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F151" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G151" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I151" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J151" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K151" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L151" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N151" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O151" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P151" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q151" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R151" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S151" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T151" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -11884,7 +11884,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -11893,60 +11893,60 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F152" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G152" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I152" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J152" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K152" t="n">
         <v>1</v>
       </c>
       <c r="L152" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N152" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O152" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P152" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q152" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R152" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S152" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T152" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -11955,113 +11955,113 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F153" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G153" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I153" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J153" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K153" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L153" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N153" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O153" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P153" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q153" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R153" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S153" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T153" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E154" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="F154" t="n">
-        <v>0.5694</v>
+        <v>-1.0225</v>
       </c>
       <c r="G154" t="n">
-        <v>-1.3423</v>
+        <v>-0.2617</v>
       </c>
       <c r="I154" t="n">
-        <v>54.77</v>
+        <v>-65.97</v>
       </c>
       <c r="J154" t="n">
-        <v>1547.7</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K154" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L154" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N154" t="n">
-        <v>0.0103</v>
+        <v>-0.0076</v>
       </c>
       <c r="O154" t="n">
-        <v>51.13</v>
+        <v>40.96</v>
       </c>
       <c r="P154" t="n">
-        <v>0.5968</v>
+        <v>0.5526</v>
       </c>
       <c r="Q154" t="n">
-        <v>0.5364</v>
+        <v>0.0334</v>
       </c>
       <c r="R154" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.0631</v>
       </c>
       <c r="S154" t="n">
-        <v>0.0098</v>
+        <v>-0.0156</v>
       </c>
       <c r="T154" t="n">
-        <v>97.8</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -12070,12 +12070,12 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -12118,21 +12118,21 @@
         <v>0.0098</v>
       </c>
       <c r="T155" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -12141,19 +12141,19 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F156" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G156" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I156" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J156" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K156" t="n">
         <v>5</v>
@@ -12162,39 +12162,39 @@
         <v>1</v>
       </c>
       <c r="N156" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O156" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P156" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q156" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R156" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S156" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T156" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -12203,60 +12203,60 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F157" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G157" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I157" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J157" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K157" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L157" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N157" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O157" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P157" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q157" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R157" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S157" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T157" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -12265,60 +12265,60 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F158" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G158" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I158" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J158" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K158" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L158" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N158" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O158" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P158" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q158" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R158" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S158" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T158" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -12327,60 +12327,60 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="F159" t="n">
-        <v>-0.3397</v>
+        <v>-1.2201</v>
       </c>
       <c r="G159" t="n">
-        <v>-1.8082</v>
+        <v>-0.255</v>
       </c>
       <c r="I159" t="n">
-        <v>-51.44</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J159" t="n">
-        <v>485.6</v>
+        <v>282.4</v>
       </c>
       <c r="K159" t="n">
+        <v>1</v>
+      </c>
+      <c r="L159" t="n">
         <v>3</v>
       </c>
-      <c r="L159" t="n">
+      <c r="N159" t="n">
+        <v>-0.0322</v>
+      </c>
+      <c r="O159" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="P159" t="n">
         <v>0</v>
       </c>
-      <c r="N159" t="n">
-        <v>-0.0003</v>
-      </c>
-      <c r="O159" t="n">
-        <v>45.06</v>
-      </c>
-      <c r="P159" t="n">
-        <v>0.5895</v>
-      </c>
       <c r="Q159" t="n">
-        <v>0.1388</v>
+        <v>0</v>
       </c>
       <c r="R159" t="n">
-        <v>0.2247</v>
+        <v>0</v>
       </c>
       <c r="S159" t="n">
-        <v>0.0137</v>
+        <v>0</v>
       </c>
       <c r="T159" t="n">
-        <v>40.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -12389,51 +12389,51 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F160" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G160" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I160" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J160" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K160" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L160" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N160" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O160" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P160" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q160" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R160" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S160" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T160" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -12442,7 +12442,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -12451,51 +12451,113 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F161" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G161" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I161" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J161" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K161" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L161" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N161" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O161" t="n">
         <v>47.65</v>
       </c>
       <c r="P161" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R161" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S161" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T161" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>41</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E162" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F162" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G162" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I162" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J162" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K162" t="n">
+        <v>4</v>
+      </c>
+      <c r="L162" t="n">
+        <v>2</v>
+      </c>
+      <c r="N162" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O162" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P162" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q161" t="n">
+      <c r="Q162" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R161" t="n">
+      <c r="R162" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S161" t="n">
+      <c r="S162" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T161" t="n">
+      <c r="T162" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T161"/>
-  <conditionalFormatting sqref="E2:E161">
+  <autoFilter ref="A1:T162"/>
+  <conditionalFormatting sqref="E2:E162">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -12517,7 +12579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K161"/>
+  <dimension ref="A1:K162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -17254,266 +17316,266 @@
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>-0.9064</v>
+        <v>-0.8895999999999999</v>
       </c>
       <c r="D128" t="n">
         <v>1000</v>
       </c>
       <c r="E128" t="n">
-        <v>1700.1</v>
+        <v>1222</v>
       </c>
       <c r="F128" t="n">
-        <v>1752.29307</v>
+        <v>1174.8308</v>
       </c>
       <c r="G128" t="n">
-        <v>1726.709591178</v>
+        <v>1304.29715416</v>
       </c>
       <c r="H128" t="n">
-        <v>1516.223692013402</v>
+        <v>1198.518654957624</v>
       </c>
       <c r="I128" t="n">
-        <v>1576.569394955535</v>
+        <v>896.9713613702858</v>
       </c>
       <c r="J128" t="n">
-        <v>1391.164834108764</v>
+        <v>944.1520549783628</v>
       </c>
       <c r="K128" t="n">
-        <v>1263.177669370758</v>
+        <v>952.649423473168</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>-0.9127</v>
+        <v>-0.9064</v>
       </c>
       <c r="D129" t="n">
         <v>1000</v>
       </c>
       <c r="E129" t="n">
-        <v>824.6</v>
+        <v>1700.1</v>
       </c>
       <c r="F129" t="n">
-        <v>945.8162000000001</v>
+        <v>1752.29307</v>
       </c>
       <c r="G129" t="n">
-        <v>1155.40906992</v>
+        <v>1726.709591178</v>
       </c>
       <c r="H129" t="n">
-        <v>1037.55734478816</v>
+        <v>1516.223692013402</v>
       </c>
       <c r="I129" t="n">
-        <v>1136.955338418866</v>
+        <v>1576.569394955535</v>
       </c>
       <c r="J129" t="n">
-        <v>1027.125452727604</v>
+        <v>1391.164834108764</v>
       </c>
       <c r="K129" t="n">
-        <v>1219.506050023484</v>
+        <v>1263.177669370758</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>18</v>
+        <v>132</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-0.9217</v>
+        <v>-0.9127</v>
       </c>
       <c r="D130" t="n">
         <v>1000</v>
       </c>
       <c r="E130" t="n">
-        <v>1206.3</v>
+        <v>824.6</v>
       </c>
       <c r="F130" t="n">
-        <v>1403.65068</v>
+        <v>945.8162000000001</v>
       </c>
       <c r="G130" t="n">
-        <v>1572.930952008</v>
+        <v>1155.40906992</v>
       </c>
       <c r="H130" t="n">
-        <v>1622.320983901051</v>
+        <v>1037.55734478816</v>
       </c>
       <c r="I130" t="n">
-        <v>1560.023858119251</v>
+        <v>1136.955338418866</v>
       </c>
       <c r="J130" t="n">
-        <v>2085.595895919627</v>
+        <v>1027.125452727604</v>
       </c>
       <c r="K130" t="n">
-        <v>1584.844321309324</v>
+        <v>1219.506050023484</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-0.9226</v>
+        <v>-0.9217</v>
       </c>
       <c r="D131" t="n">
         <v>1000</v>
       </c>
       <c r="E131" t="n">
-        <v>1141.9</v>
+        <v>1206.3</v>
       </c>
       <c r="F131" t="n">
-        <v>983.4042799999999</v>
+        <v>1403.65068</v>
       </c>
       <c r="G131" t="n">
-        <v>1002.482323032</v>
+        <v>1572.930952008</v>
       </c>
       <c r="H131" t="n">
-        <v>1006.392004091825</v>
+        <v>1622.320983901051</v>
       </c>
       <c r="I131" t="n">
-        <v>968.1491079363354</v>
+        <v>1560.023858119251</v>
       </c>
       <c r="J131" t="n">
-        <v>739.9563631957411</v>
+        <v>2085.595895919627</v>
       </c>
       <c r="K131" t="n">
-        <v>567.8425131164117</v>
+        <v>1584.844321309324</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>140</v>
+        <v>60</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>dlinear</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-0.9331</v>
+        <v>-0.9226</v>
       </c>
       <c r="D132" t="n">
         <v>1000</v>
       </c>
       <c r="E132" t="n">
-        <v>916.6999999999999</v>
+        <v>1141.9</v>
       </c>
       <c r="F132" t="n">
-        <v>699.35043</v>
+        <v>983.4042799999999</v>
       </c>
       <c r="G132" t="n">
-        <v>591.5105936939999</v>
+        <v>1002.482323032</v>
       </c>
       <c r="H132" t="n">
-        <v>525.7937667345965</v>
+        <v>1006.392004091825</v>
       </c>
       <c r="I132" t="n">
-        <v>531.9455538053913</v>
+        <v>968.1491079363354</v>
       </c>
       <c r="J132" t="n">
-        <v>546.4144728688981</v>
+        <v>739.9563631957411</v>
       </c>
       <c r="K132" t="n">
-        <v>421.4494829237811</v>
+        <v>567.8425131164117</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>dlinear</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-0.9746</v>
+        <v>-0.9331</v>
       </c>
       <c r="D133" t="n">
         <v>1000</v>
       </c>
       <c r="E133" t="n">
-        <v>823.5</v>
+        <v>916.6999999999999</v>
       </c>
       <c r="F133" t="n">
-        <v>939.36645</v>
+        <v>699.35043</v>
       </c>
       <c r="G133" t="n">
-        <v>1037.24843409</v>
+        <v>591.5105936939999</v>
       </c>
       <c r="H133" t="n">
-        <v>968.582587753242</v>
+        <v>525.7937667345965</v>
       </c>
       <c r="I133" t="n">
-        <v>996.38090802176</v>
+        <v>531.9455538053913</v>
       </c>
       <c r="J133" t="n">
-        <v>1251.255144293726</v>
+        <v>546.4144728688981</v>
       </c>
       <c r="K133" t="n">
-        <v>953.7066709806782</v>
+        <v>421.4494829237811</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-0.9961</v>
+        <v>-0.9746</v>
       </c>
       <c r="D134" t="n">
         <v>1000</v>
       </c>
       <c r="E134" t="n">
-        <v>866</v>
+        <v>823.5</v>
       </c>
       <c r="F134" t="n">
-        <v>1018.3294</v>
+        <v>939.36645</v>
       </c>
       <c r="G134" t="n">
-        <v>1148.57373026</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H134" t="n">
-        <v>1130.885694813996</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I134" t="n">
-        <v>1184.150411039735</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J134" t="n">
-        <v>1292.144928526559</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K134" t="n">
-        <v>1394.612021358715</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -17521,73 +17583,73 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-1.066</v>
+        <v>-0.9961</v>
       </c>
       <c r="D135" t="n">
         <v>1000</v>
       </c>
       <c r="E135" t="n">
-        <v>1390.6</v>
+        <v>866</v>
       </c>
       <c r="F135" t="n">
-        <v>1715.16604</v>
+        <v>1018.3294</v>
       </c>
       <c r="G135" t="n">
-        <v>1928.018145564</v>
+        <v>1148.57373026</v>
       </c>
       <c r="H135" t="n">
-        <v>1842.799743530072</v>
+        <v>1130.885694813996</v>
       </c>
       <c r="I135" t="n">
-        <v>1932.359811065633</v>
+        <v>1184.150411039735</v>
       </c>
       <c r="J135" t="n">
-        <v>2502.212719348888</v>
+        <v>1292.144928526559</v>
       </c>
       <c r="K135" t="n">
-        <v>2078.337884691186</v>
+        <v>1394.612021358715</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D136" t="n">
         <v>1000</v>
       </c>
       <c r="E136" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F136" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G136" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H136" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I136" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J136" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K136" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -17595,184 +17657,184 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D137" t="n">
         <v>1000</v>
       </c>
       <c r="E137" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F137" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G137" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H137" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I137" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J137" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K137" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D138" t="n">
         <v>1000</v>
       </c>
       <c r="E138" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F138" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G138" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H138" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I138" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J138" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K138" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D139" t="n">
         <v>1000</v>
       </c>
       <c r="E139" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F139" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G139" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H139" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I139" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J139" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K139" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D140" t="n">
         <v>1000</v>
       </c>
       <c r="E140" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F140" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G140" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H140" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I140" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J140" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K140" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D141" t="n">
         <v>1000</v>
       </c>
       <c r="E141" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F141" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G141" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H141" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I141" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J141" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K141" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
@@ -17780,36 +17842,36 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D142" t="n">
         <v>1000</v>
       </c>
       <c r="E142" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F142" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G142" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H142" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I142" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J142" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K142" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -17817,258 +17879,258 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D143" t="n">
         <v>1000</v>
       </c>
       <c r="E143" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F143" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G143" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H143" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I143" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J143" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K143" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D144" t="n">
         <v>1000</v>
       </c>
       <c r="E144" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F144" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G144" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H144" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I144" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J144" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K144" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D145" t="n">
         <v>1000</v>
       </c>
       <c r="E145" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F145" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G145" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H145" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I145" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J145" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K145" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D146" t="n">
         <v>1000</v>
       </c>
       <c r="E146" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F146" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G146" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H146" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I146" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J146" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K146" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="D147" t="n">
         <v>1000</v>
       </c>
       <c r="E147" t="n">
-        <v>1045.3</v>
+        <v>942</v>
       </c>
       <c r="F147" t="n">
-        <v>853.06933</v>
+        <v>730.2384</v>
       </c>
       <c r="G147" t="n">
-        <v>749.933248003</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H147" t="n">
-        <v>740.3341024285616</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I147" t="n">
-        <v>691.1759180273051</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J147" t="n">
-        <v>482.7172611502699</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K147" t="n">
-        <v>325.0618036585918</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D148" t="n">
         <v>1000</v>
       </c>
       <c r="E148" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F148" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G148" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H148" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I148" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J148" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K148" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D149" t="n">
         <v>1000</v>
       </c>
       <c r="E149" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F149" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G149" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H149" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I149" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J149" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K149" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -18076,36 +18138,36 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D150" t="n">
         <v>1000</v>
       </c>
       <c r="E150" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F150" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G150" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H150" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I150" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J150" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K150" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -18113,36 +18175,36 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D151" t="n">
         <v>1000</v>
       </c>
       <c r="E151" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F151" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G151" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H151" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I151" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J151" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K151" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -18150,110 +18212,110 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D152" t="n">
         <v>1000</v>
       </c>
       <c r="E152" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F152" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G152" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H152" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I152" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J152" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K152" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D153" t="n">
         <v>1000</v>
       </c>
       <c r="E153" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F153" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G153" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H153" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I153" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J153" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K153" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="D154" t="n">
         <v>1000</v>
       </c>
       <c r="E154" t="n">
-        <v>1342</v>
+        <v>1141.5</v>
       </c>
       <c r="F154" t="n">
-        <v>1365.6192</v>
+        <v>884.8908</v>
       </c>
       <c r="G154" t="n">
-        <v>1401.67154688</v>
+        <v>789.49957176</v>
       </c>
       <c r="H154" t="n">
-        <v>1356.1172216064</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I154" t="n">
-        <v>1614.321940600259</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J154" t="n">
-        <v>1682.93062307577</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K154" t="n">
-        <v>1547.623000980478</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -18290,192 +18352,192 @@
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D156" t="n">
         <v>1000</v>
       </c>
       <c r="E156" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F156" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G156" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H156" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I156" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J156" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K156" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D157" t="n">
         <v>1000</v>
       </c>
       <c r="E157" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F157" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G157" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H157" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I157" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J157" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K157" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D158" t="n">
         <v>1000</v>
       </c>
       <c r="E158" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F158" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G158" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H158" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I158" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J158" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K158" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="D159" t="n">
         <v>1000</v>
       </c>
       <c r="E159" t="n">
-        <v>1000.2</v>
+        <v>942</v>
       </c>
       <c r="F159" t="n">
-        <v>765.0529799999999</v>
+        <v>730.2384</v>
       </c>
       <c r="G159" t="n">
-        <v>773.1625415879998</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H159" t="n">
-        <v>742.158723670321</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I159" t="n">
-        <v>765.9078028277713</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J159" t="n">
-        <v>571.2906301292346</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K159" t="n">
-        <v>485.5970356098494</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D160" t="n">
         <v>1000</v>
       </c>
       <c r="E160" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F160" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G160" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H160" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I160" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J160" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K160" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -18483,30 +18545,67 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D161" t="n">
         <v>1000</v>
       </c>
       <c r="E161" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F161" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G161" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H161" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I161" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J161" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K161" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>41</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D162" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E162" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F161" t="n">
+      <c r="F162" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G161" t="n">
+      <c r="G162" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H161" t="n">
+      <c r="H162" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I161" t="n">
+      <c r="I162" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J161" t="n">
+      <c r="J162" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K161" t="n">
+      <c r="K162" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 162 LSTM seed=13 -0.97
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$163</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>164</row>
+      <row>165</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T162"/>
+  <dimension ref="A1:T163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -10771,16 +10771,16 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>70</v>
+        <v>162</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
+          <t>LSTM 1-layer seed=13 - extra seed for variance</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -10789,60 +10789,60 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>-0.9746</v>
+        <v>-0.9699</v>
       </c>
       <c r="F134" t="n">
-        <v>0.1045</v>
+        <v>-0.3593</v>
       </c>
       <c r="G134" t="n">
-        <v>-0.6746</v>
+        <v>-0.4699</v>
       </c>
       <c r="I134" t="n">
-        <v>-4.63</v>
+        <v>-52.86</v>
       </c>
       <c r="J134" t="n">
-        <v>953.7</v>
+        <v>471.4</v>
       </c>
       <c r="K134" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L134" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N134" t="n">
-        <v>-0.0374</v>
+        <v>0.0046</v>
       </c>
       <c r="O134" t="n">
-        <v>51.03</v>
+        <v>44.14</v>
       </c>
       <c r="P134" t="n">
-        <v>0.5765</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Q134" t="n">
-        <v>0.5415</v>
+        <v>0.1041</v>
       </c>
       <c r="R134" t="n">
-        <v>0.5585</v>
+        <v>0.1755</v>
       </c>
       <c r="S134" t="n">
-        <v>0.0091</v>
+        <v>-0.0086</v>
       </c>
       <c r="T134" t="n">
-        <v>30.6</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 seed=2024 - 5-seed lock</t>
+          <t>MLP @ exp 6 hidden=64 (further narrower from 96) - val regime fit hill-climb</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -10851,51 +10851,51 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>-0.9961</v>
+        <v>-0.9746</v>
       </c>
       <c r="F135" t="n">
-        <v>0.4602</v>
+        <v>0.1045</v>
       </c>
       <c r="G135" t="n">
-        <v>-0.7961</v>
+        <v>-0.6746</v>
       </c>
       <c r="I135" t="n">
-        <v>39.45</v>
+        <v>-4.63</v>
       </c>
       <c r="J135" t="n">
-        <v>1394.5</v>
+        <v>953.7</v>
       </c>
       <c r="K135" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L135" t="n">
         <v>2</v>
       </c>
       <c r="N135" t="n">
-        <v>0.0172</v>
+        <v>-0.0374</v>
       </c>
       <c r="O135" t="n">
-        <v>50.19</v>
+        <v>51.03</v>
       </c>
       <c r="P135" t="n">
-        <v>0.5927</v>
+        <v>0.5765</v>
       </c>
       <c r="Q135" t="n">
-        <v>0.5111</v>
+        <v>0.5415</v>
       </c>
       <c r="R135" t="n">
-        <v>0.5489000000000001</v>
+        <v>0.5585</v>
       </c>
       <c r="S135" t="n">
-        <v>0.0007</v>
+        <v>0.0091</v>
       </c>
       <c r="T135" t="n">
-        <v>76.90000000000001</v>
+        <v>30.6</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -10904,7 +10904,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>XGBoost @ exp 44 seed=2024 - 5-seed lock</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -10913,19 +10913,19 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>-1.066</v>
+        <v>-0.9961</v>
       </c>
       <c r="F136" t="n">
-        <v>0.8788</v>
+        <v>0.4602</v>
       </c>
       <c r="G136" t="n">
-        <v>-0.866</v>
+        <v>-0.7961</v>
       </c>
       <c r="I136" t="n">
-        <v>107.82</v>
+        <v>39.45</v>
       </c>
       <c r="J136" t="n">
-        <v>2078.2</v>
+        <v>1394.5</v>
       </c>
       <c r="K136" t="n">
         <v>5</v>
@@ -10934,39 +10934,39 @@
         <v>2</v>
       </c>
       <c r="N136" t="n">
-        <v>0.0329</v>
+        <v>0.0172</v>
       </c>
       <c r="O136" t="n">
-        <v>54.14</v>
+        <v>50.19</v>
       </c>
       <c r="P136" t="n">
-        <v>0.6011</v>
+        <v>0.5927</v>
       </c>
       <c r="Q136" t="n">
-        <v>0.6725</v>
+        <v>0.5111</v>
       </c>
       <c r="R136" t="n">
-        <v>0.6348</v>
+        <v>0.5489000000000001</v>
       </c>
       <c r="S136" t="n">
-        <v>0.0251</v>
+        <v>0.0007</v>
       </c>
       <c r="T136" t="n">
-        <v>75.8</v>
+        <v>76.90000000000001</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -10975,51 +10975,51 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F137" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G137" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I137" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J137" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K137" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L137" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N137" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O137" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P137" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q137" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R137" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S137" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T137" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -11028,7 +11028,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -11037,60 +11037,60 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F138" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G138" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I138" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J138" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L138" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N138" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O138" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P138" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q138" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R138" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S138" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T138" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -11099,60 +11099,60 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F139" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G139" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I139" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J139" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K139" t="n">
         <v>2</v>
       </c>
       <c r="L139" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N139" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O139" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P139" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q139" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R139" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S139" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T139" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -11161,60 +11161,60 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F140" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G140" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I140" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J140" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K140" t="n">
+        <v>2</v>
+      </c>
+      <c r="L140" t="n">
         <v>5</v>
       </c>
-      <c r="L140" t="n">
-        <v>2</v>
-      </c>
       <c r="N140" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O140" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P140" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q140" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R140" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S140" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T140" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -11223,60 +11223,60 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F141" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G141" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I141" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J141" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K141" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L141" t="n">
         <v>2</v>
       </c>
       <c r="N141" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O141" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P141" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q141" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R141" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S141" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T141" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -11285,51 +11285,51 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F142" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G142" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I142" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J142" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K142" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L142" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N142" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O142" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P142" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q142" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R142" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S142" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T142" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -11338,7 +11338,7 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -11347,51 +11347,51 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F143" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G143" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I143" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J143" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K143" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L143" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N143" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O143" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P143" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q143" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R143" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S143" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T143" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -11400,7 +11400,7 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -11409,60 +11409,60 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F144" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G144" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I144" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J144" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K144" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L144" t="n">
         <v>2</v>
       </c>
       <c r="N144" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O144" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P144" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q144" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R144" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S144" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T144" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -11471,60 +11471,60 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F145" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G145" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I145" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J145" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K145" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L145" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N145" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O145" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P145" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q145" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R145" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S145" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T145" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -11533,60 +11533,60 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F146" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G146" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I146" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J146" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K146" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L146" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N146" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O146" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P146" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q146" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R146" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S146" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T146" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -11595,60 +11595,60 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F147" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G147" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I147" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J147" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L147" t="n">
         <v>3</v>
       </c>
       <c r="N147" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O147" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P147" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q147" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R147" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S147" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T147" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -11657,19 +11657,19 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="F148" t="n">
-        <v>-0.6042</v>
+        <v>-0.8189</v>
       </c>
       <c r="G148" t="n">
-        <v>-0.8305</v>
+        <v>1.1456</v>
       </c>
       <c r="I148" t="n">
-        <v>-67.48999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J148" t="n">
-        <v>325.1000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K148" t="n">
         <v>1</v>
@@ -11678,39 +11678,39 @@
         <v>3</v>
       </c>
       <c r="N148" t="n">
-        <v>0.0111</v>
+        <v>0.0089</v>
       </c>
       <c r="O148" t="n">
-        <v>42.64</v>
+        <v>41.44</v>
       </c>
       <c r="P148" t="n">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="Q148" t="n">
-        <v>0</v>
+        <v>0.0271</v>
       </c>
       <c r="R148" t="n">
-        <v>0</v>
+        <v>0.0521</v>
       </c>
       <c r="S148" t="n">
-        <v>0</v>
+        <v>0.0277</v>
       </c>
       <c r="T148" t="n">
-        <v>82.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -11719,60 +11719,60 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F149" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G149" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I149" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J149" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K149" t="n">
         <v>1</v>
       </c>
       <c r="L149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N149" t="n">
-        <v>0.0284</v>
+        <v>0.0111</v>
       </c>
       <c r="O149" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P149" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q149" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R149" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S149" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T149" t="n">
-        <v>79.8</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -11781,39 +11781,51 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F150" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G150" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I150" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J150" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K150" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L150" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N150" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O150" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P150" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R150" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S150" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T150" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -11822,7 +11834,7 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -11831,51 +11843,39 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F151" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G151" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I151" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J151" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K151" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L151" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N151" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O151" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P151" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q151" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R151" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S151" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T151" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -11884,7 +11884,7 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -11893,51 +11893,51 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F152" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G152" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I152" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J152" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K152" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L152" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N152" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O152" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P152" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q152" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R152" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S152" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T152" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -11946,7 +11946,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -11955,60 +11955,60 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F153" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G153" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I153" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J153" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K153" t="n">
         <v>1</v>
       </c>
       <c r="L153" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N153" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O153" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P153" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q153" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R153" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S153" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T153" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -12017,113 +12017,113 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F154" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G154" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I154" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J154" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K154" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L154" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N154" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O154" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P154" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q154" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R154" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S154" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T154" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E155" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="F155" t="n">
-        <v>0.5694</v>
+        <v>-1.0225</v>
       </c>
       <c r="G155" t="n">
-        <v>-1.3423</v>
+        <v>-0.2617</v>
       </c>
       <c r="I155" t="n">
-        <v>54.77</v>
+        <v>-65.97</v>
       </c>
       <c r="J155" t="n">
-        <v>1547.7</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K155" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L155" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N155" t="n">
-        <v>0.0103</v>
+        <v>-0.0076</v>
       </c>
       <c r="O155" t="n">
-        <v>51.13</v>
+        <v>40.96</v>
       </c>
       <c r="P155" t="n">
-        <v>0.5968</v>
+        <v>0.5526</v>
       </c>
       <c r="Q155" t="n">
-        <v>0.5364</v>
+        <v>0.0334</v>
       </c>
       <c r="R155" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.0631</v>
       </c>
       <c r="S155" t="n">
-        <v>0.0098</v>
+        <v>-0.0156</v>
       </c>
       <c r="T155" t="n">
-        <v>97.8</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -12132,12 +12132,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -12180,21 +12180,21 @@
         <v>0.0098</v>
       </c>
       <c r="T156" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -12203,19 +12203,19 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F157" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G157" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I157" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J157" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K157" t="n">
         <v>5</v>
@@ -12224,39 +12224,39 @@
         <v>1</v>
       </c>
       <c r="N157" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O157" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P157" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q157" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R157" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S157" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T157" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -12265,60 +12265,60 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F158" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G158" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I158" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J158" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K158" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L158" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N158" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O158" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P158" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q158" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R158" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S158" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T158" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -12327,60 +12327,60 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F159" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G159" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I159" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J159" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K159" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L159" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N159" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O159" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P159" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q159" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R159" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S159" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T159" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -12389,60 +12389,60 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="F160" t="n">
-        <v>-0.3397</v>
+        <v>-1.2201</v>
       </c>
       <c r="G160" t="n">
-        <v>-1.8082</v>
+        <v>-0.255</v>
       </c>
       <c r="I160" t="n">
-        <v>-51.44</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J160" t="n">
-        <v>485.6</v>
+        <v>282.4</v>
       </c>
       <c r="K160" t="n">
+        <v>1</v>
+      </c>
+      <c r="L160" t="n">
         <v>3</v>
       </c>
-      <c r="L160" t="n">
+      <c r="N160" t="n">
+        <v>-0.0322</v>
+      </c>
+      <c r="O160" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="P160" t="n">
         <v>0</v>
       </c>
-      <c r="N160" t="n">
-        <v>-0.0003</v>
-      </c>
-      <c r="O160" t="n">
-        <v>45.06</v>
-      </c>
-      <c r="P160" t="n">
-        <v>0.5895</v>
-      </c>
       <c r="Q160" t="n">
-        <v>0.1388</v>
+        <v>0</v>
       </c>
       <c r="R160" t="n">
-        <v>0.2247</v>
+        <v>0</v>
       </c>
       <c r="S160" t="n">
-        <v>0.0137</v>
+        <v>0</v>
       </c>
       <c r="T160" t="n">
-        <v>40.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -12451,51 +12451,51 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F161" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G161" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I161" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J161" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K161" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N161" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O161" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P161" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q161" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R161" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S161" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T161" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -12504,7 +12504,7 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -12513,51 +12513,113 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F162" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G162" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I162" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J162" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K162" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L162" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N162" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O162" t="n">
         <v>47.65</v>
       </c>
       <c r="P162" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R162" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S162" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T162" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>41</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E163" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F163" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G163" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I163" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J163" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K163" t="n">
+        <v>4</v>
+      </c>
+      <c r="L163" t="n">
+        <v>2</v>
+      </c>
+      <c r="N163" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O163" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P163" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q162" t="n">
+      <c r="Q163" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R162" t="n">
+      <c r="R163" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S162" t="n">
+      <c r="S163" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T162" t="n">
+      <c r="T163" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T162"/>
-  <conditionalFormatting sqref="E2:E162">
+  <autoFilter ref="A1:T163"/>
+  <conditionalFormatting sqref="E2:E163">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -12579,7 +12641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K162"/>
+  <dimension ref="A1:K163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -17538,81 +17600,81 @@
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>70</v>
+        <v>162</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-0.9746</v>
+        <v>-0.9699</v>
       </c>
       <c r="D134" t="n">
         <v>1000</v>
       </c>
       <c r="E134" t="n">
-        <v>823.5</v>
+        <v>1140.1</v>
       </c>
       <c r="F134" t="n">
-        <v>939.36645</v>
+        <v>1015.25905</v>
       </c>
       <c r="G134" t="n">
-        <v>1037.24843409</v>
+        <v>925.5101499799999</v>
       </c>
       <c r="H134" t="n">
-        <v>968.582587753242</v>
+        <v>879.8824995859859</v>
       </c>
       <c r="I134" t="n">
-        <v>996.38090802176</v>
+        <v>935.4910735598202</v>
       </c>
       <c r="J134" t="n">
-        <v>1251.255144293726</v>
+        <v>644.0856041459361</v>
       </c>
       <c r="K134" t="n">
-        <v>953.7066709806782</v>
+        <v>471.4062536744107</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-0.9961</v>
+        <v>-0.9746</v>
       </c>
       <c r="D135" t="n">
         <v>1000</v>
       </c>
       <c r="E135" t="n">
-        <v>866</v>
+        <v>823.5</v>
       </c>
       <c r="F135" t="n">
-        <v>1018.3294</v>
+        <v>939.36645</v>
       </c>
       <c r="G135" t="n">
-        <v>1148.57373026</v>
+        <v>1037.24843409</v>
       </c>
       <c r="H135" t="n">
-        <v>1130.885694813996</v>
+        <v>968.582587753242</v>
       </c>
       <c r="I135" t="n">
-        <v>1184.150411039735</v>
+        <v>996.38090802176</v>
       </c>
       <c r="J135" t="n">
-        <v>1292.144928526559</v>
+        <v>1251.255144293726</v>
       </c>
       <c r="K135" t="n">
-        <v>1394.612021358715</v>
+        <v>953.7066709806782</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -17620,73 +17682,73 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.066</v>
+        <v>-0.9961</v>
       </c>
       <c r="D136" t="n">
         <v>1000</v>
       </c>
       <c r="E136" t="n">
-        <v>1390.6</v>
+        <v>866</v>
       </c>
       <c r="F136" t="n">
-        <v>1715.16604</v>
+        <v>1018.3294</v>
       </c>
       <c r="G136" t="n">
-        <v>1928.018145564</v>
+        <v>1148.57373026</v>
       </c>
       <c r="H136" t="n">
-        <v>1842.799743530072</v>
+        <v>1130.885694813996</v>
       </c>
       <c r="I136" t="n">
-        <v>1932.359811065633</v>
+        <v>1184.150411039735</v>
       </c>
       <c r="J136" t="n">
-        <v>2502.212719348888</v>
+        <v>1292.144928526559</v>
       </c>
       <c r="K136" t="n">
-        <v>2078.337884691186</v>
+        <v>1394.612021358715</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D137" t="n">
         <v>1000</v>
       </c>
       <c r="E137" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F137" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G137" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H137" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I137" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J137" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K137" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -17694,184 +17756,184 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D138" t="n">
         <v>1000</v>
       </c>
       <c r="E138" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F138" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G138" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H138" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I138" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J138" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K138" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D139" t="n">
         <v>1000</v>
       </c>
       <c r="E139" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F139" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G139" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H139" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I139" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J139" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K139" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D140" t="n">
         <v>1000</v>
       </c>
       <c r="E140" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F140" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G140" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H140" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I140" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J140" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K140" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D141" t="n">
         <v>1000</v>
       </c>
       <c r="E141" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F141" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G141" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H141" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I141" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J141" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K141" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D142" t="n">
         <v>1000</v>
       </c>
       <c r="E142" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F142" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G142" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H142" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I142" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J142" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K142" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
@@ -17879,36 +17941,36 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D143" t="n">
         <v>1000</v>
       </c>
       <c r="E143" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F143" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G143" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H143" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I143" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J143" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K143" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
@@ -17916,258 +17978,258 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D144" t="n">
         <v>1000</v>
       </c>
       <c r="E144" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F144" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G144" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H144" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I144" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J144" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K144" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D145" t="n">
         <v>1000</v>
       </c>
       <c r="E145" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F145" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G145" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H145" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I145" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J145" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K145" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D146" t="n">
         <v>1000</v>
       </c>
       <c r="E146" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F146" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G146" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H146" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I146" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J146" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K146" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D147" t="n">
         <v>1000</v>
       </c>
       <c r="E147" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F147" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G147" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H147" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I147" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J147" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K147" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="D148" t="n">
         <v>1000</v>
       </c>
       <c r="E148" t="n">
-        <v>1045.3</v>
+        <v>942</v>
       </c>
       <c r="F148" t="n">
-        <v>853.06933</v>
+        <v>730.2384</v>
       </c>
       <c r="G148" t="n">
-        <v>749.933248003</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H148" t="n">
-        <v>740.3341024285616</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I148" t="n">
-        <v>691.1759180273051</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J148" t="n">
-        <v>482.7172611502699</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K148" t="n">
-        <v>325.0618036585918</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D149" t="n">
         <v>1000</v>
       </c>
       <c r="E149" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F149" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G149" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H149" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I149" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J149" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K149" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D150" t="n">
         <v>1000</v>
       </c>
       <c r="E150" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F150" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G150" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H150" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I150" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J150" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K150" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -18175,36 +18237,36 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D151" t="n">
         <v>1000</v>
       </c>
       <c r="E151" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F151" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G151" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H151" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I151" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J151" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K151" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -18212,36 +18274,36 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D152" t="n">
         <v>1000</v>
       </c>
       <c r="E152" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F152" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G152" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H152" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I152" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J152" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K152" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -18249,110 +18311,110 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D153" t="n">
         <v>1000</v>
       </c>
       <c r="E153" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F153" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G153" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H153" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I153" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J153" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K153" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D154" t="n">
         <v>1000</v>
       </c>
       <c r="E154" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F154" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G154" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H154" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I154" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J154" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K154" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="D155" t="n">
         <v>1000</v>
       </c>
       <c r="E155" t="n">
-        <v>1342</v>
+        <v>1141.5</v>
       </c>
       <c r="F155" t="n">
-        <v>1365.6192</v>
+        <v>884.8908</v>
       </c>
       <c r="G155" t="n">
-        <v>1401.67154688</v>
+        <v>789.49957176</v>
       </c>
       <c r="H155" t="n">
-        <v>1356.1172216064</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I155" t="n">
-        <v>1614.321940600259</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J155" t="n">
-        <v>1682.93062307577</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K155" t="n">
-        <v>1547.623000980478</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -18389,192 +18451,192 @@
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D157" t="n">
         <v>1000</v>
       </c>
       <c r="E157" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F157" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G157" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H157" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I157" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J157" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K157" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D158" t="n">
         <v>1000</v>
       </c>
       <c r="E158" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F158" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G158" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H158" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I158" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J158" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K158" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D159" t="n">
         <v>1000</v>
       </c>
       <c r="E159" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F159" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G159" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H159" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I159" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J159" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K159" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="D160" t="n">
         <v>1000</v>
       </c>
       <c r="E160" t="n">
-        <v>1000.2</v>
+        <v>942</v>
       </c>
       <c r="F160" t="n">
-        <v>765.0529799999999</v>
+        <v>730.2384</v>
       </c>
       <c r="G160" t="n">
-        <v>773.1625415879998</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H160" t="n">
-        <v>742.158723670321</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I160" t="n">
-        <v>765.9078028277713</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J160" t="n">
-        <v>571.2906301292346</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K160" t="n">
-        <v>485.5970356098494</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D161" t="n">
         <v>1000</v>
       </c>
       <c r="E161" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F161" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G161" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H161" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I161" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J161" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K161" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
@@ -18582,30 +18644,67 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D162" t="n">
         <v>1000</v>
       </c>
       <c r="E162" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F162" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G162" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H162" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I162" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J162" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K162" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>41</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E163" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F162" t="n">
+      <c r="F163" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G162" t="n">
+      <c r="G163" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H162" t="n">
+      <c r="H163" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I162" t="n">
+      <c r="I163" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J162" t="n">
+      <c r="J163" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K162" t="n">
+      <c r="K163" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 164 LSTM ep=50 -1.01
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$164</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$165</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>166</row>
+      <row>167</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T164"/>
+  <dimension ref="A1:T165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11019,16 +11019,16 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>45</v>
+        <v>164</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
+          <t>LSTM 1-layer epochs=50 pat=8 - faster training axis</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -11037,60 +11037,60 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-1.066</v>
+        <v>-1.0099</v>
       </c>
       <c r="F138" t="n">
-        <v>0.8788</v>
+        <v>0.376</v>
       </c>
       <c r="G138" t="n">
-        <v>-0.866</v>
+        <v>-0.8099</v>
       </c>
       <c r="I138" t="n">
-        <v>107.82</v>
+        <v>44.25</v>
       </c>
       <c r="J138" t="n">
-        <v>2078.2</v>
+        <v>1442.5</v>
       </c>
       <c r="K138" t="n">
         <v>5</v>
       </c>
       <c r="L138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N138" t="n">
-        <v>0.0329</v>
+        <v>0.0352</v>
       </c>
       <c r="O138" t="n">
-        <v>54.14</v>
+        <v>46.62</v>
       </c>
       <c r="P138" t="n">
-        <v>0.6011</v>
+        <v>0.5726</v>
       </c>
       <c r="Q138" t="n">
-        <v>0.6725</v>
+        <v>0.2689</v>
       </c>
       <c r="R138" t="n">
-        <v>0.6348</v>
+        <v>0.3659</v>
       </c>
       <c r="S138" t="n">
-        <v>0.0251</v>
+        <v>0.0003</v>
       </c>
       <c r="T138" t="n">
-        <v>75.8</v>
+        <v>35</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>XGBoost @ exp 44 lr=0.01 (down from 0.02) - extending lower-lr trend</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -11099,51 +11099,51 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="F139" t="n">
-        <v>-0.5057</v>
+        <v>0.8788</v>
       </c>
       <c r="G139" t="n">
-        <v>-0.5119</v>
+        <v>-0.866</v>
       </c>
       <c r="I139" t="n">
-        <v>-62.25</v>
+        <v>107.82</v>
       </c>
       <c r="J139" t="n">
-        <v>377.4999999999999</v>
+        <v>2078.2</v>
       </c>
       <c r="K139" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L139" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N139" t="n">
-        <v>0.0032</v>
+        <v>0.0329</v>
       </c>
       <c r="O139" t="n">
-        <v>44.56</v>
+        <v>54.14</v>
       </c>
       <c r="P139" t="n">
-        <v>0.6421</v>
+        <v>0.6011</v>
       </c>
       <c r="Q139" t="n">
-        <v>0.0756</v>
+        <v>0.6725</v>
       </c>
       <c r="R139" t="n">
-        <v>0.1353</v>
+        <v>0.6348</v>
       </c>
       <c r="S139" t="n">
-        <v>0.0379</v>
+        <v>0.0251</v>
       </c>
       <c r="T139" t="n">
-        <v>53.3</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -11152,7 +11152,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -11161,60 +11161,60 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F140" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G140" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I140" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J140" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K140" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L140" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N140" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O140" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P140" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q140" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R140" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S140" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T140" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -11223,60 +11223,60 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="F141" t="n">
-        <v>-0.6484</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G141" t="n">
-        <v>1.8519</v>
+        <v>-0.0276</v>
       </c>
       <c r="I141" t="n">
-        <v>-51.47</v>
+        <v>-67.98</v>
       </c>
       <c r="J141" t="n">
-        <v>485.3000000000001</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K141" t="n">
         <v>2</v>
       </c>
       <c r="L141" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N141" t="n">
-        <v>0.008200000000000001</v>
+        <v>-0.0254</v>
       </c>
       <c r="O141" t="n">
-        <v>43.33</v>
+        <v>44.42</v>
       </c>
       <c r="P141" t="n">
-        <v>0.5736</v>
+        <v>0.5676</v>
       </c>
       <c r="Q141" t="n">
-        <v>0.1799</v>
+        <v>0.1301</v>
       </c>
       <c r="R141" t="n">
-        <v>0.2739</v>
+        <v>0.2117</v>
       </c>
       <c r="S141" t="n">
-        <v>-0.0183</v>
+        <v>-0.0037</v>
       </c>
       <c r="T141" t="n">
-        <v>823.8</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -11285,60 +11285,60 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F142" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G142" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I142" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J142" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K142" t="n">
+        <v>2</v>
+      </c>
+      <c r="L142" t="n">
         <v>5</v>
       </c>
-      <c r="L142" t="n">
-        <v>2</v>
-      </c>
       <c r="N142" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O142" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P142" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q142" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R142" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S142" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T142" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -11347,60 +11347,60 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F143" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G143" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I143" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J143" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K143" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L143" t="n">
         <v>2</v>
       </c>
       <c r="N143" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O143" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P143" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q143" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R143" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S143" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T143" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -11409,51 +11409,51 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F144" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G144" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I144" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J144" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K144" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L144" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N144" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O144" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P144" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q144" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R144" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S144" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T144" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -11462,7 +11462,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -11471,51 +11471,51 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F145" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G145" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I145" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J145" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K145" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L145" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N145" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O145" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P145" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q145" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R145" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S145" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T145" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -11524,7 +11524,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -11533,60 +11533,60 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F146" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G146" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I146" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J146" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K146" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L146" t="n">
         <v>2</v>
       </c>
       <c r="N146" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O146" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P146" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q146" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R146" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S146" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T146" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -11595,60 +11595,60 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F147" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G147" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I147" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J147" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K147" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N147" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O147" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P147" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q147" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R147" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S147" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T147" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
@@ -11657,60 +11657,60 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F148" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G148" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I148" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J148" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K148" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L148" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N148" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O148" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P148" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q148" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R148" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S148" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T148" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -11719,60 +11719,60 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F149" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G149" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I149" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J149" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K149" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L149" t="n">
         <v>3</v>
       </c>
       <c r="N149" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O149" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P149" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q149" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R149" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S149" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T149" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -11781,19 +11781,19 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="F150" t="n">
-        <v>-0.6042</v>
+        <v>-0.8189</v>
       </c>
       <c r="G150" t="n">
-        <v>-0.8305</v>
+        <v>1.1456</v>
       </c>
       <c r="I150" t="n">
-        <v>-67.48999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J150" t="n">
-        <v>325.1000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K150" t="n">
         <v>1</v>
@@ -11802,39 +11802,39 @@
         <v>3</v>
       </c>
       <c r="N150" t="n">
-        <v>0.0111</v>
+        <v>0.0089</v>
       </c>
       <c r="O150" t="n">
-        <v>42.64</v>
+        <v>41.44</v>
       </c>
       <c r="P150" t="n">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="Q150" t="n">
-        <v>0</v>
+        <v>0.0271</v>
       </c>
       <c r="R150" t="n">
-        <v>0</v>
+        <v>0.0521</v>
       </c>
       <c r="S150" t="n">
-        <v>0</v>
+        <v>0.0277</v>
       </c>
       <c r="T150" t="n">
-        <v>82.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -11843,60 +11843,60 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F151" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G151" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I151" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J151" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K151" t="n">
         <v>1</v>
       </c>
       <c r="L151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N151" t="n">
-        <v>0.0284</v>
+        <v>0.0111</v>
       </c>
       <c r="O151" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P151" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q151" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R151" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S151" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T151" t="n">
-        <v>79.8</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -11905,39 +11905,51 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="F152" t="n">
-        <v>-0.0343</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G152" t="n">
-        <v>-1.2001</v>
+        <v>-0.8347</v>
       </c>
       <c r="I152" t="n">
-        <v>-22.74</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J152" t="n">
-        <v>772.5999999999999</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K152" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L152" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N152" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0284</v>
       </c>
       <c r="O152" t="n">
-        <v>47.05</v>
+        <v>44.07</v>
+      </c>
+      <c r="P152" t="n">
+        <v>0.5588</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>0.1177</v>
+      </c>
+      <c r="R152" t="n">
+        <v>0.1945</v>
+      </c>
+      <c r="S152" t="n">
+        <v>-0.0101</v>
       </c>
       <c r="T152" t="n">
-        <v>38.6</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -11946,7 +11958,7 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -11955,51 +11967,39 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F153" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G153" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I153" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J153" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K153" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L153" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N153" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O153" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P153" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q153" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R153" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S153" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T153" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -12008,7 +12008,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -12017,51 +12017,51 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F154" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G154" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I154" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J154" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K154" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L154" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N154" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O154" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P154" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q154" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R154" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S154" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T154" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -12070,7 +12070,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -12079,60 +12079,60 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F155" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G155" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I155" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J155" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K155" t="n">
         <v>1</v>
       </c>
       <c r="L155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N155" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O155" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P155" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q155" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R155" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S155" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T155" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -12141,113 +12141,113 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F156" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G156" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I156" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J156" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K156" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L156" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N156" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O156" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P156" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q156" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R156" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S156" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T156" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E157" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="F157" t="n">
-        <v>0.5694</v>
+        <v>-1.0225</v>
       </c>
       <c r="G157" t="n">
-        <v>-1.3423</v>
+        <v>-0.2617</v>
       </c>
       <c r="I157" t="n">
-        <v>54.77</v>
+        <v>-65.97</v>
       </c>
       <c r="J157" t="n">
-        <v>1547.7</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K157" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L157" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N157" t="n">
-        <v>0.0103</v>
+        <v>-0.0076</v>
       </c>
       <c r="O157" t="n">
-        <v>51.13</v>
+        <v>40.96</v>
       </c>
       <c r="P157" t="n">
-        <v>0.5968</v>
+        <v>0.5526</v>
       </c>
       <c r="Q157" t="n">
-        <v>0.5364</v>
+        <v>0.0334</v>
       </c>
       <c r="R157" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.0631</v>
       </c>
       <c r="S157" t="n">
-        <v>0.0098</v>
+        <v>-0.0156</v>
       </c>
       <c r="T157" t="n">
-        <v>97.8</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -12256,12 +12256,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -12304,21 +12304,21 @@
         <v>0.0098</v>
       </c>
       <c r="T158" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -12327,19 +12327,19 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F159" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G159" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I159" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J159" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K159" t="n">
         <v>5</v>
@@ -12348,39 +12348,39 @@
         <v>1</v>
       </c>
       <c r="N159" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O159" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P159" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q159" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R159" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S159" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T159" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -12389,60 +12389,60 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F160" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G160" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I160" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J160" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K160" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L160" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N160" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O160" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P160" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q160" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R160" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S160" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T160" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -12451,60 +12451,60 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F161" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G161" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I161" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J161" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K161" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L161" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N161" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O161" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P161" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q161" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R161" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S161" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T161" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -12513,60 +12513,60 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="F162" t="n">
-        <v>-0.3397</v>
+        <v>-1.2201</v>
       </c>
       <c r="G162" t="n">
-        <v>-1.8082</v>
+        <v>-0.255</v>
       </c>
       <c r="I162" t="n">
-        <v>-51.44</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J162" t="n">
-        <v>485.6</v>
+        <v>282.4</v>
       </c>
       <c r="K162" t="n">
+        <v>1</v>
+      </c>
+      <c r="L162" t="n">
         <v>3</v>
       </c>
-      <c r="L162" t="n">
+      <c r="N162" t="n">
+        <v>-0.0322</v>
+      </c>
+      <c r="O162" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="P162" t="n">
         <v>0</v>
       </c>
-      <c r="N162" t="n">
-        <v>-0.0003</v>
-      </c>
-      <c r="O162" t="n">
-        <v>45.06</v>
-      </c>
-      <c r="P162" t="n">
-        <v>0.5895</v>
-      </c>
       <c r="Q162" t="n">
-        <v>0.1388</v>
+        <v>0</v>
       </c>
       <c r="R162" t="n">
-        <v>0.2247</v>
+        <v>0</v>
       </c>
       <c r="S162" t="n">
-        <v>0.0137</v>
+        <v>0</v>
       </c>
       <c r="T162" t="n">
-        <v>40.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -12575,51 +12575,51 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F163" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G163" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I163" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J163" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K163" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L163" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N163" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O163" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P163" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q163" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R163" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S163" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T163" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -12628,7 +12628,7 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -12637,51 +12637,113 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F164" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G164" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I164" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J164" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K164" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L164" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N164" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O164" t="n">
         <v>47.65</v>
       </c>
       <c r="P164" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R164" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S164" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T164" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>41</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E165" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F165" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G165" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I165" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J165" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K165" t="n">
+        <v>4</v>
+      </c>
+      <c r="L165" t="n">
+        <v>2</v>
+      </c>
+      <c r="N165" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O165" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P165" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q164" t="n">
+      <c r="Q165" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R164" t="n">
+      <c r="R165" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S164" t="n">
+      <c r="S165" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T164" t="n">
+      <c r="T165" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T164"/>
-  <conditionalFormatting sqref="E2:E164">
+  <autoFilter ref="A1:T165"/>
+  <conditionalFormatting sqref="E2:E165">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -12703,7 +12765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K164"/>
+  <dimension ref="A1:K165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -17810,81 +17872,81 @@
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>45</v>
+        <v>164</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.066</v>
+        <v>-1.0099</v>
       </c>
       <c r="D138" t="n">
         <v>1000</v>
       </c>
       <c r="E138" t="n">
-        <v>1390.6</v>
+        <v>1364.2</v>
       </c>
       <c r="F138" t="n">
-        <v>1715.16604</v>
+        <v>1215.36578</v>
       </c>
       <c r="G138" t="n">
-        <v>1928.018145564</v>
+        <v>961.718941714</v>
       </c>
       <c r="H138" t="n">
-        <v>1842.799743530072</v>
+        <v>997.2063706632466</v>
       </c>
       <c r="I138" t="n">
-        <v>1932.359811065633</v>
+        <v>1106.400468250872</v>
       </c>
       <c r="J138" t="n">
-        <v>2502.212719348888</v>
+        <v>1469.742382024458</v>
       </c>
       <c r="K138" t="n">
-        <v>2078.337884691186</v>
+        <v>1442.405173718804</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>23</v>
+        <v>45</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-1.1119</v>
+        <v>-1.066</v>
       </c>
       <c r="D139" t="n">
         <v>1000</v>
       </c>
       <c r="E139" t="n">
-        <v>1045.3</v>
+        <v>1390.6</v>
       </c>
       <c r="F139" t="n">
-        <v>853.06933</v>
+        <v>1715.16604</v>
       </c>
       <c r="G139" t="n">
-        <v>732.018792073</v>
+        <v>1928.018145564</v>
       </c>
       <c r="H139" t="n">
-        <v>707.34975878014</v>
+        <v>1842.799743530072</v>
       </c>
       <c r="I139" t="n">
-        <v>660.5939397247727</v>
+        <v>1932.359811065633</v>
       </c>
       <c r="J139" t="n">
-        <v>432.6229711257536</v>
+        <v>2502.212719348888</v>
       </c>
       <c r="K139" t="n">
-        <v>377.4635423072201</v>
+        <v>2078.337884691186</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
@@ -17892,184 +17954,184 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D140" t="n">
         <v>1000</v>
       </c>
       <c r="E140" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F140" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G140" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H140" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I140" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J140" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K140" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.1484</v>
+        <v>-1.1144</v>
       </c>
       <c r="D141" t="n">
         <v>1000</v>
       </c>
       <c r="E141" t="n">
-        <v>953.5</v>
+        <v>759.5</v>
       </c>
       <c r="F141" t="n">
-        <v>734.5763999999999</v>
+        <v>825.34865</v>
       </c>
       <c r="G141" t="n">
-        <v>658.4742849599999</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H141" t="n">
-        <v>766.3323728364478</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I141" t="n">
-        <v>828.0987620870656</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J141" t="n">
-        <v>590.5172272442865</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K141" t="n">
-        <v>485.3461090720791</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D142" t="n">
         <v>1000</v>
       </c>
       <c r="E142" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F142" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G142" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H142" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I142" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J142" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K142" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D143" t="n">
         <v>1000</v>
       </c>
       <c r="E143" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F143" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G143" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H143" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I143" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J143" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K143" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D144" t="n">
         <v>1000</v>
       </c>
       <c r="E144" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F144" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G144" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H144" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I144" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J144" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K144" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
@@ -18077,36 +18139,36 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D145" t="n">
         <v>1000</v>
       </c>
       <c r="E145" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F145" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G145" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H145" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I145" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J145" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K145" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
@@ -18114,258 +18176,258 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D146" t="n">
         <v>1000</v>
       </c>
       <c r="E146" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F146" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G146" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H146" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I146" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J146" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K146" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D147" t="n">
         <v>1000</v>
       </c>
       <c r="E147" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F147" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G147" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H147" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I147" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J147" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K147" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D148" t="n">
         <v>1000</v>
       </c>
       <c r="E148" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F148" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G148" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H148" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I148" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J148" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K148" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D149" t="n">
         <v>1000</v>
       </c>
       <c r="E149" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F149" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G149" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H149" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I149" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J149" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K149" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="D150" t="n">
         <v>1000</v>
       </c>
       <c r="E150" t="n">
-        <v>1045.3</v>
+        <v>942</v>
       </c>
       <c r="F150" t="n">
-        <v>853.06933</v>
+        <v>730.2384</v>
       </c>
       <c r="G150" t="n">
-        <v>749.933248003</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H150" t="n">
-        <v>740.3341024285616</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I150" t="n">
-        <v>691.1759180273051</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J150" t="n">
-        <v>482.7172611502699</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K150" t="n">
-        <v>325.0618036585918</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D151" t="n">
         <v>1000</v>
       </c>
       <c r="E151" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F151" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G151" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H151" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I151" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J151" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K151" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>-1.5001</v>
+        <v>-1.4347</v>
       </c>
       <c r="D152" t="n">
         <v>1000</v>
       </c>
       <c r="E152" t="n">
-        <v>969.0999999999999</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F152" t="n">
-        <v>872.5776399999999</v>
+        <v>692.62656</v>
       </c>
       <c r="G152" t="n">
-        <v>1116.724863672</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H152" t="n">
-        <v>1199.809193529197</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I152" t="n">
-        <v>1246.001847480071</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J152" t="n">
-        <v>1151.804107810577</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K152" t="n">
-        <v>772.5150151085543</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -18373,36 +18435,36 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D153" t="n">
         <v>1000</v>
       </c>
       <c r="E153" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F153" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G153" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H153" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I153" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J153" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K153" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -18410,36 +18472,36 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D154" t="n">
         <v>1000</v>
       </c>
       <c r="E154" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F154" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G154" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H154" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I154" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J154" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K154" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -18447,110 +18509,110 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D155" t="n">
         <v>1000</v>
       </c>
       <c r="E155" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F155" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G155" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H155" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I155" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J155" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K155" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D156" t="n">
         <v>1000</v>
       </c>
       <c r="E156" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F156" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G156" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H156" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I156" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J156" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K156" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="D157" t="n">
         <v>1000</v>
       </c>
       <c r="E157" t="n">
-        <v>1342</v>
+        <v>1141.5</v>
       </c>
       <c r="F157" t="n">
-        <v>1365.6192</v>
+        <v>884.8908</v>
       </c>
       <c r="G157" t="n">
-        <v>1401.67154688</v>
+        <v>789.49957176</v>
       </c>
       <c r="H157" t="n">
-        <v>1356.1172216064</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I157" t="n">
-        <v>1614.321940600259</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J157" t="n">
-        <v>1682.93062307577</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K157" t="n">
-        <v>1547.623000980478</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -18587,192 +18649,192 @@
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D159" t="n">
         <v>1000</v>
       </c>
       <c r="E159" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F159" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G159" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H159" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I159" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J159" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K159" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D160" t="n">
         <v>1000</v>
       </c>
       <c r="E160" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F160" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G160" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H160" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I160" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J160" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K160" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D161" t="n">
         <v>1000</v>
       </c>
       <c r="E161" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F161" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G161" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H161" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I161" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J161" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K161" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="D162" t="n">
         <v>1000</v>
       </c>
       <c r="E162" t="n">
-        <v>1000.2</v>
+        <v>942</v>
       </c>
       <c r="F162" t="n">
-        <v>765.0529799999999</v>
+        <v>730.2384</v>
       </c>
       <c r="G162" t="n">
-        <v>773.1625415879998</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H162" t="n">
-        <v>742.158723670321</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I162" t="n">
-        <v>765.9078028277713</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J162" t="n">
-        <v>571.2906301292346</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K162" t="n">
-        <v>485.5970356098494</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D163" t="n">
         <v>1000</v>
       </c>
       <c r="E163" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F163" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G163" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H163" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I163" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J163" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K163" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -18780,30 +18842,67 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D164" t="n">
         <v>1000</v>
       </c>
       <c r="E164" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F164" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G164" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H164" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I164" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J164" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K164" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>41</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D165" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E165" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F164" t="n">
+      <c r="F165" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G164" t="n">
+      <c r="G165" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H164" t="n">
+      <c r="H165" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I164" t="n">
+      <c r="I165" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J164" t="n">
+      <c r="J165" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K164" t="n">
+      <c r="K165" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 170 — CatBoost seed=99 val crash -1.4536; 3-seed median +0.07
Major seed-variance insight on CatBoost lr=0.05 + n_est=1000:
- A_sharpe stable: +0.20 / +0.49 / +0.47 across seeds 42/0/99
- val_sharpe WILD: +0.64 / +1.49 / -1.15
- composite punished by min(test,val)-0.1*n_neg formula

3-seed median composite +0.0728 (= exp 167 result). Lift IS real but
marginal — much weaker than 2-seed mean +0.23 suggested.

Notable: exp 170 produced RECORD per-fold test alpha (F2=+3.74, F1=+2.38)
yet val crashed. Ordered-boosting permutation seed-dependence is more
extreme than expected (Prokhorenkova 2018 §3.2).

Exp 171 pre-auth: seed=7 4-seed median lock per Lakshminarayanan 2017 §3.2
+ Picard 2021. Then deploy-vs-abandon decision.
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$170</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$171</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>172</row>
+      <row>173</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T170"/>
+  <dimension ref="A1:T171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12259,16 +12259,16 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -12277,39 +12277,51 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F158" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G158" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I158" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J158" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K158" t="n">
         <v>4</v>
       </c>
       <c r="L158" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N158" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O158" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P158" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R158" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S158" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T158" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -12318,7 +12330,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -12327,51 +12339,39 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F159" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G159" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I159" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J159" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K159" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L159" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N159" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O159" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P159" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q159" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R159" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S159" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T159" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -12380,7 +12380,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -12389,51 +12389,51 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F160" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G160" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I160" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J160" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K160" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L160" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N160" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O160" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P160" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q160" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R160" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S160" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T160" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -12442,7 +12442,7 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -12451,60 +12451,60 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F161" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G161" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I161" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J161" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K161" t="n">
         <v>1</v>
       </c>
       <c r="L161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N161" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O161" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P161" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q161" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R161" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S161" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T161" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -12513,113 +12513,113 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F162" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G162" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I162" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J162" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K162" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L162" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N162" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O162" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P162" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q162" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R162" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S162" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T162" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="F163" t="n">
-        <v>0.5694</v>
+        <v>-1.0225</v>
       </c>
       <c r="G163" t="n">
-        <v>-1.3423</v>
+        <v>-0.2617</v>
       </c>
       <c r="I163" t="n">
-        <v>54.77</v>
+        <v>-65.97</v>
       </c>
       <c r="J163" t="n">
-        <v>1547.7</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K163" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L163" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N163" t="n">
-        <v>0.0103</v>
+        <v>-0.0076</v>
       </c>
       <c r="O163" t="n">
-        <v>51.13</v>
+        <v>40.96</v>
       </c>
       <c r="P163" t="n">
-        <v>0.5968</v>
+        <v>0.5526</v>
       </c>
       <c r="Q163" t="n">
-        <v>0.5364</v>
+        <v>0.0334</v>
       </c>
       <c r="R163" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.0631</v>
       </c>
       <c r="S163" t="n">
-        <v>0.0098</v>
+        <v>-0.0156</v>
       </c>
       <c r="T163" t="n">
-        <v>97.8</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -12628,12 +12628,12 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E164" t="n">
@@ -12676,21 +12676,21 @@
         <v>0.0098</v>
       </c>
       <c r="T164" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -12699,19 +12699,19 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F165" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G165" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I165" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J165" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K165" t="n">
         <v>5</v>
@@ -12720,39 +12720,39 @@
         <v>1</v>
       </c>
       <c r="N165" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O165" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P165" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q165" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R165" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S165" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T165" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -12761,60 +12761,60 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F166" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G166" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I166" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J166" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K166" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N166" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O166" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P166" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q166" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R166" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S166" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T166" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -12823,60 +12823,60 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F167" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G167" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I167" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J167" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K167" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L167" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N167" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O167" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P167" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q167" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R167" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S167" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T167" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -12885,60 +12885,60 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="F168" t="n">
-        <v>-0.3397</v>
+        <v>-1.2201</v>
       </c>
       <c r="G168" t="n">
-        <v>-1.8082</v>
+        <v>-0.255</v>
       </c>
       <c r="I168" t="n">
-        <v>-51.44</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J168" t="n">
-        <v>485.6</v>
+        <v>282.4</v>
       </c>
       <c r="K168" t="n">
+        <v>1</v>
+      </c>
+      <c r="L168" t="n">
         <v>3</v>
       </c>
-      <c r="L168" t="n">
+      <c r="N168" t="n">
+        <v>-0.0322</v>
+      </c>
+      <c r="O168" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="P168" t="n">
         <v>0</v>
       </c>
-      <c r="N168" t="n">
-        <v>-0.0003</v>
-      </c>
-      <c r="O168" t="n">
-        <v>45.06</v>
-      </c>
-      <c r="P168" t="n">
-        <v>0.5895</v>
-      </c>
       <c r="Q168" t="n">
-        <v>0.1388</v>
+        <v>0</v>
       </c>
       <c r="R168" t="n">
-        <v>0.2247</v>
+        <v>0</v>
       </c>
       <c r="S168" t="n">
-        <v>0.0137</v>
+        <v>0</v>
       </c>
       <c r="T168" t="n">
-        <v>40.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -12947,51 +12947,51 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F169" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G169" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I169" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J169" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K169" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L169" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N169" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O169" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P169" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q169" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R169" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S169" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T169" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -13000,7 +13000,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -13009,51 +13009,113 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F170" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G170" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I170" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J170" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K170" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L170" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N170" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O170" t="n">
         <v>47.65</v>
       </c>
       <c r="P170" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R170" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S170" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T170" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>41</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E171" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F171" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G171" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I171" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J171" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K171" t="n">
+        <v>4</v>
+      </c>
+      <c r="L171" t="n">
+        <v>2</v>
+      </c>
+      <c r="N171" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O171" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P171" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q170" t="n">
+      <c r="Q171" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R170" t="n">
+      <c r="R171" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S170" t="n">
+      <c r="S171" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T170" t="n">
+      <c r="T171" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T170"/>
-  <conditionalFormatting sqref="E2:E170">
+  <autoFilter ref="A1:T171"/>
+  <conditionalFormatting sqref="E2:E171">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -13075,7 +13137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K170"/>
+  <dimension ref="A1:K171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -18922,44 +18984,44 @@
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D158" t="n">
         <v>1000</v>
       </c>
       <c r="E158" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F158" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G158" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H158" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I158" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J158" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K158" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -18967,36 +19029,36 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D159" t="n">
         <v>1000</v>
       </c>
       <c r="E159" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F159" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G159" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H159" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I159" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J159" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K159" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -19004,36 +19066,36 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D160" t="n">
         <v>1000</v>
       </c>
       <c r="E160" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F160" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G160" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H160" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I160" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J160" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K160" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
@@ -19041,110 +19103,110 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D161" t="n">
         <v>1000</v>
       </c>
       <c r="E161" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F161" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G161" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H161" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I161" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J161" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K161" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D162" t="n">
         <v>1000</v>
       </c>
       <c r="E162" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F162" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G162" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H162" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I162" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J162" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K162" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="D163" t="n">
         <v>1000</v>
       </c>
       <c r="E163" t="n">
-        <v>1342</v>
+        <v>1141.5</v>
       </c>
       <c r="F163" t="n">
-        <v>1365.6192</v>
+        <v>884.8908</v>
       </c>
       <c r="G163" t="n">
-        <v>1401.67154688</v>
+        <v>789.49957176</v>
       </c>
       <c r="H163" t="n">
-        <v>1356.1172216064</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I163" t="n">
-        <v>1614.321940600259</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J163" t="n">
-        <v>1682.93062307577</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K163" t="n">
-        <v>1547.623000980478</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
@@ -19181,192 +19243,192 @@
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D165" t="n">
         <v>1000</v>
       </c>
       <c r="E165" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F165" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G165" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H165" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I165" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J165" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K165" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D166" t="n">
         <v>1000</v>
       </c>
       <c r="E166" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F166" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G166" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H166" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I166" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J166" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K166" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D167" t="n">
         <v>1000</v>
       </c>
       <c r="E167" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F167" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G167" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H167" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I167" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J167" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K167" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="D168" t="n">
         <v>1000</v>
       </c>
       <c r="E168" t="n">
-        <v>1000.2</v>
+        <v>942</v>
       </c>
       <c r="F168" t="n">
-        <v>765.0529799999999</v>
+        <v>730.2384</v>
       </c>
       <c r="G168" t="n">
-        <v>773.1625415879998</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H168" t="n">
-        <v>742.158723670321</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I168" t="n">
-        <v>765.9078028277713</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J168" t="n">
-        <v>571.2906301292346</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K168" t="n">
-        <v>485.5970356098494</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D169" t="n">
         <v>1000</v>
       </c>
       <c r="E169" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F169" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G169" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H169" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I169" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J169" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K169" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
@@ -19374,30 +19436,67 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D170" t="n">
         <v>1000</v>
       </c>
       <c r="E170" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F170" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G170" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H170" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I170" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J170" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K170" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>41</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D171" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E171" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F170" t="n">
+      <c r="F171" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G170" t="n">
+      <c r="G171" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H170" t="n">
+      <c r="H171" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I170" t="n">
+      <c r="I171" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J170" t="n">
+      <c r="J171" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K170" t="n">
+      <c r="K171" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 177 — LSTM lr=2e-3 destabilized -1.12; HP-only axes EXHAUSTED
6 consecutive LSTM DISCARDs (172-177): hidden=128, seq=10, bs=16, lr=1e-3,
wd=7e-4, hd=0.1 all confirmed champions; no single-knob HP improvement.
Per CLAUDE.md structural-change rule.

PIVOT to Mamba (21/25 budget; global champion +1.32). mambats variant
(Cai et al. 2024 NeurIPS arXiv:2405.16440) NEVER tested on QQQ — only
dmamba and vanilla. mambats adds season-trend decomposition which may
capture FOMC/EOM/quad-witching patterns dmamba misses.

Exp 178: mambats with dMamba champion HPs (expand=2 d_state=32 seed=42).
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$177</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$178</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>179</row>
+      <row>180</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T177"/>
+  <dimension ref="A1:T178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -11949,16 +11949,16 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>51</v>
+        <v>177</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM lr=2e-3 (Smith 2017 highest-leverage axis untested) - one knob from exp 74 lr=1e-3</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -11967,60 +11967,60 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>-1.1484</v>
+        <v>-1.1172</v>
       </c>
       <c r="F153" t="n">
-        <v>-0.6484</v>
+        <v>0.0506</v>
       </c>
       <c r="G153" t="n">
-        <v>1.8519</v>
+        <v>-0.7171999999999999</v>
       </c>
       <c r="I153" t="n">
-        <v>-51.47</v>
+        <v>-11.99</v>
       </c>
       <c r="J153" t="n">
-        <v>485.3000000000001</v>
+        <v>880.1</v>
       </c>
       <c r="K153" t="n">
+        <v>3</v>
+      </c>
+      <c r="L153" t="n">
         <v>2</v>
       </c>
-      <c r="L153" t="n">
-        <v>5</v>
-      </c>
       <c r="N153" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0322</v>
       </c>
       <c r="O153" t="n">
-        <v>43.33</v>
+        <v>46.2</v>
       </c>
       <c r="P153" t="n">
-        <v>0.5736</v>
+        <v>0.5585</v>
       </c>
       <c r="Q153" t="n">
-        <v>0.1799</v>
+        <v>0.29</v>
       </c>
       <c r="R153" t="n">
-        <v>0.2739</v>
+        <v>0.3817</v>
       </c>
       <c r="S153" t="n">
-        <v>-0.0183</v>
+        <v>-0.0182</v>
       </c>
       <c r="T153" t="n">
-        <v>823.8</v>
+        <v>52.2</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -12029,60 +12029,60 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F154" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G154" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I154" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J154" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K154" t="n">
+        <v>2</v>
+      </c>
+      <c r="L154" t="n">
         <v>5</v>
       </c>
-      <c r="L154" t="n">
-        <v>2</v>
-      </c>
       <c r="N154" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O154" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P154" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q154" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R154" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S154" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T154" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -12091,60 +12091,60 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F155" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G155" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I155" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J155" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K155" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L155" t="n">
         <v>2</v>
       </c>
       <c r="N155" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O155" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P155" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q155" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R155" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S155" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T155" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -12153,51 +12153,51 @@
         </is>
       </c>
       <c r="E156" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F156" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G156" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I156" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J156" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K156" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L156" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N156" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O156" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P156" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q156" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R156" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S156" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T156" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -12206,7 +12206,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
@@ -12215,51 +12215,51 @@
         </is>
       </c>
       <c r="E157" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F157" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G157" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I157" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J157" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K157" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L157" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N157" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O157" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P157" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q157" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R157" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S157" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T157" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -12268,7 +12268,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -12277,60 +12277,60 @@
         </is>
       </c>
       <c r="E158" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F158" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G158" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I158" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J158" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K158" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L158" t="n">
         <v>2</v>
       </c>
       <c r="N158" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O158" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P158" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q158" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R158" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S158" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T158" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -12339,60 +12339,60 @@
         </is>
       </c>
       <c r="E159" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F159" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G159" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I159" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J159" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K159" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L159" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N159" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O159" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P159" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q159" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R159" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S159" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T159" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -12401,60 +12401,60 @@
         </is>
       </c>
       <c r="E160" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F160" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G160" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I160" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J160" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K160" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L160" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N160" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O160" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P160" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q160" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R160" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S160" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T160" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
@@ -12463,60 +12463,60 @@
         </is>
       </c>
       <c r="E161" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F161" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G161" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I161" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J161" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K161" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L161" t="n">
         <v>3</v>
       </c>
       <c r="N161" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O161" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P161" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q161" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R161" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S161" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T161" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D162" t="inlineStr">
@@ -12525,19 +12525,19 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="F162" t="n">
-        <v>-0.6042</v>
+        <v>-0.8189</v>
       </c>
       <c r="G162" t="n">
-        <v>-0.8305</v>
+        <v>1.1456</v>
       </c>
       <c r="I162" t="n">
-        <v>-67.48999999999999</v>
+        <v>-58.71</v>
       </c>
       <c r="J162" t="n">
-        <v>325.1000000000001</v>
+        <v>412.9</v>
       </c>
       <c r="K162" t="n">
         <v>1</v>
@@ -12546,39 +12546,39 @@
         <v>3</v>
       </c>
       <c r="N162" t="n">
-        <v>0.0111</v>
+        <v>0.0089</v>
       </c>
       <c r="O162" t="n">
-        <v>42.64</v>
+        <v>41.44</v>
       </c>
       <c r="P162" t="n">
-        <v>0</v>
+        <v>0.68</v>
       </c>
       <c r="Q162" t="n">
-        <v>0</v>
+        <v>0.0271</v>
       </c>
       <c r="R162" t="n">
-        <v>0</v>
+        <v>0.0521</v>
       </c>
       <c r="S162" t="n">
-        <v>0</v>
+        <v>0.0277</v>
       </c>
       <c r="T162" t="n">
-        <v>82.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D163" t="inlineStr">
@@ -12587,60 +12587,60 @@
         </is>
       </c>
       <c r="E163" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F163" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G163" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I163" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J163" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K163" t="n">
         <v>1</v>
       </c>
       <c r="L163" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N163" t="n">
-        <v>0.0284</v>
+        <v>0.0111</v>
       </c>
       <c r="O163" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P163" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q163" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R163" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S163" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T163" t="n">
-        <v>79.8</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D164" t="inlineStr">
@@ -12649,60 +12649,60 @@
         </is>
       </c>
       <c r="E164" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="F164" t="n">
-        <v>0.4732</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G164" t="n">
-        <v>-1.1536</v>
+        <v>-0.8347</v>
       </c>
       <c r="I164" t="n">
-        <v>41.21</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J164" t="n">
-        <v>1412.1</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K164" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L164" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N164" t="n">
-        <v>0.0231</v>
+        <v>0.0284</v>
       </c>
       <c r="O164" t="n">
-        <v>48.31</v>
+        <v>44.07</v>
       </c>
       <c r="P164" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.5588</v>
       </c>
       <c r="Q164" t="n">
-        <v>0.3418</v>
+        <v>0.1177</v>
       </c>
       <c r="R164" t="n">
-        <v>0.4395</v>
+        <v>0.1945</v>
       </c>
       <c r="S164" t="n">
-        <v>0.0329</v>
+        <v>-0.0101</v>
       </c>
       <c r="T164" t="n">
-        <v>1311.2</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
@@ -12711,39 +12711,51 @@
         </is>
       </c>
       <c r="E165" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F165" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G165" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I165" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J165" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K165" t="n">
         <v>4</v>
       </c>
       <c r="L165" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N165" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O165" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P165" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R165" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S165" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T165" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -12752,7 +12764,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -12761,51 +12773,39 @@
         </is>
       </c>
       <c r="E166" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F166" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G166" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I166" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J166" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K166" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N166" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O166" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P166" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q166" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R166" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S166" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T166" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -12814,7 +12814,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -12823,51 +12823,51 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F167" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G167" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I167" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J167" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K167" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L167" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N167" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O167" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P167" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q167" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R167" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S167" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T167" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -12876,7 +12876,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -12885,60 +12885,60 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F168" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G168" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I168" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J168" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K168" t="n">
         <v>1</v>
       </c>
       <c r="L168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N168" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O168" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P168" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q168" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R168" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S168" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T168" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -12947,113 +12947,113 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F169" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G169" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I169" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J169" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K169" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L169" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N169" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O169" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P169" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q169" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R169" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S169" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T169" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E170" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="F170" t="n">
-        <v>0.5694</v>
+        <v>-1.0225</v>
       </c>
       <c r="G170" t="n">
-        <v>-1.3423</v>
+        <v>-0.2617</v>
       </c>
       <c r="I170" t="n">
-        <v>54.77</v>
+        <v>-65.97</v>
       </c>
       <c r="J170" t="n">
-        <v>1547.7</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K170" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L170" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N170" t="n">
-        <v>0.0103</v>
+        <v>-0.0076</v>
       </c>
       <c r="O170" t="n">
-        <v>51.13</v>
+        <v>40.96</v>
       </c>
       <c r="P170" t="n">
-        <v>0.5968</v>
+        <v>0.5526</v>
       </c>
       <c r="Q170" t="n">
-        <v>0.5364</v>
+        <v>0.0334</v>
       </c>
       <c r="R170" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.0631</v>
       </c>
       <c r="S170" t="n">
-        <v>0.0098</v>
+        <v>-0.0156</v>
       </c>
       <c r="T170" t="n">
-        <v>97.8</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -13062,12 +13062,12 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -13110,21 +13110,21 @@
         <v>0.0098</v>
       </c>
       <c r="T171" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -13133,19 +13133,19 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F172" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G172" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I172" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J172" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K172" t="n">
         <v>5</v>
@@ -13154,39 +13154,39 @@
         <v>1</v>
       </c>
       <c r="N172" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O172" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P172" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q172" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R172" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S172" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T172" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -13195,60 +13195,60 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F173" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G173" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I173" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J173" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K173" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L173" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N173" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O173" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P173" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q173" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R173" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S173" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T173" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -13257,60 +13257,60 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F174" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G174" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I174" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J174" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K174" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L174" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N174" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O174" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P174" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q174" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R174" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S174" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T174" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -13319,60 +13319,60 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="F175" t="n">
-        <v>-0.3397</v>
+        <v>-1.2201</v>
       </c>
       <c r="G175" t="n">
-        <v>-1.8082</v>
+        <v>-0.255</v>
       </c>
       <c r="I175" t="n">
-        <v>-51.44</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J175" t="n">
-        <v>485.6</v>
+        <v>282.4</v>
       </c>
       <c r="K175" t="n">
+        <v>1</v>
+      </c>
+      <c r="L175" t="n">
         <v>3</v>
       </c>
-      <c r="L175" t="n">
+      <c r="N175" t="n">
+        <v>-0.0322</v>
+      </c>
+      <c r="O175" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="P175" t="n">
         <v>0</v>
       </c>
-      <c r="N175" t="n">
-        <v>-0.0003</v>
-      </c>
-      <c r="O175" t="n">
-        <v>45.06</v>
-      </c>
-      <c r="P175" t="n">
-        <v>0.5895</v>
-      </c>
       <c r="Q175" t="n">
-        <v>0.1388</v>
+        <v>0</v>
       </c>
       <c r="R175" t="n">
-        <v>0.2247</v>
+        <v>0</v>
       </c>
       <c r="S175" t="n">
-        <v>0.0137</v>
+        <v>0</v>
       </c>
       <c r="T175" t="n">
-        <v>40.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -13381,51 +13381,51 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F176" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G176" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I176" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J176" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K176" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L176" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N176" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O176" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P176" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q176" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R176" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S176" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T176" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -13434,7 +13434,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -13443,51 +13443,113 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F177" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G177" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I177" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J177" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K177" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L177" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N177" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O177" t="n">
         <v>47.65</v>
       </c>
       <c r="P177" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R177" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S177" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T177" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>41</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E178" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F178" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G178" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I178" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J178" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K178" t="n">
+        <v>4</v>
+      </c>
+      <c r="L178" t="n">
+        <v>2</v>
+      </c>
+      <c r="N178" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O178" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P178" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q177" t="n">
+      <c r="Q178" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R177" t="n">
+      <c r="R178" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S177" t="n">
+      <c r="S178" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T177" t="n">
+      <c r="T178" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T177"/>
-  <conditionalFormatting sqref="E2:E177">
+  <autoFilter ref="A1:T178"/>
+  <conditionalFormatting sqref="E2:E178">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -13509,7 +13571,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K177"/>
+  <dimension ref="A1:K178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -19171,155 +19233,155 @@
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>51</v>
+        <v>177</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>-1.1484</v>
+        <v>-1.1172</v>
       </c>
       <c r="D153" t="n">
         <v>1000</v>
       </c>
       <c r="E153" t="n">
-        <v>953.5</v>
+        <v>1207.8</v>
       </c>
       <c r="F153" t="n">
-        <v>734.5763999999999</v>
+        <v>1063.22634</v>
       </c>
       <c r="G153" t="n">
-        <v>658.4742849599999</v>
+        <v>1012.829411484</v>
       </c>
       <c r="H153" t="n">
-        <v>766.3323728364478</v>
+        <v>978.899626199286</v>
       </c>
       <c r="I153" t="n">
-        <v>828.0987620870656</v>
+        <v>1221.373063608849</v>
       </c>
       <c r="J153" t="n">
-        <v>590.5172272442865</v>
+        <v>1413.861458433604</v>
       </c>
       <c r="K153" t="n">
-        <v>485.3461090720791</v>
+        <v>880.1287578749184</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D154" t="n">
         <v>1000</v>
       </c>
       <c r="E154" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F154" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G154" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H154" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I154" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J154" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K154" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D155" t="n">
         <v>1000</v>
       </c>
       <c r="E155" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F155" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G155" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H155" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I155" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J155" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K155" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D156" t="n">
         <v>1000</v>
       </c>
       <c r="E156" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F156" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G156" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H156" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I156" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J156" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K156" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -19327,36 +19389,36 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D157" t="n">
         <v>1000</v>
       </c>
       <c r="E157" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F157" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G157" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H157" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I157" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J157" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K157" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -19364,295 +19426,295 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D158" t="n">
         <v>1000</v>
       </c>
       <c r="E158" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F158" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G158" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H158" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I158" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J158" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K158" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D159" t="n">
         <v>1000</v>
       </c>
       <c r="E159" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F159" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G159" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H159" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I159" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J159" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K159" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D160" t="n">
         <v>1000</v>
       </c>
       <c r="E160" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F160" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G160" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H160" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I160" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J160" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K160" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D161" t="n">
         <v>1000</v>
       </c>
       <c r="E161" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F161" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G161" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H161" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I161" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J161" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K161" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>144</v>
+        <v>110</v>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>-1.4305</v>
+        <v>-1.4189</v>
       </c>
       <c r="D162" t="n">
         <v>1000</v>
       </c>
       <c r="E162" t="n">
-        <v>1045.3</v>
+        <v>942</v>
       </c>
       <c r="F162" t="n">
-        <v>853.06933</v>
+        <v>730.2384</v>
       </c>
       <c r="G162" t="n">
-        <v>749.933248003</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H162" t="n">
-        <v>740.3341024285616</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I162" t="n">
-        <v>691.1759180273051</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J162" t="n">
-        <v>482.7172611502699</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K162" t="n">
-        <v>325.0618036585918</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D163" t="n">
         <v>1000</v>
       </c>
       <c r="E163" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F163" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G163" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H163" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I163" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J163" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K163" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="D164" t="n">
         <v>1000</v>
       </c>
       <c r="E164" t="n">
-        <v>1236.4</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F164" t="n">
-        <v>1500.74232</v>
+        <v>692.62656</v>
       </c>
       <c r="G164" t="n">
-        <v>1734.708047688</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H164" t="n">
-        <v>1677.809623723833</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I164" t="n">
-        <v>1544.088196713044</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J164" t="n">
-        <v>1750.069562154564</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K164" t="n">
-        <v>1412.131129702517</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D165" t="n">
         <v>1000</v>
       </c>
       <c r="E165" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F165" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G165" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H165" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I165" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J165" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K165" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B166" t="inlineStr">
         <is>
@@ -19660,36 +19722,36 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D166" t="n">
         <v>1000</v>
       </c>
       <c r="E166" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F166" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G166" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H166" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I166" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J166" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K166" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
@@ -19697,36 +19759,36 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D167" t="n">
         <v>1000</v>
       </c>
       <c r="E167" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F167" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G167" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H167" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I167" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J167" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K167" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -19734,110 +19796,110 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D168" t="n">
         <v>1000</v>
       </c>
       <c r="E168" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F168" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G168" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H168" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I168" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J168" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K168" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D169" t="n">
         <v>1000</v>
       </c>
       <c r="E169" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F169" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G169" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H169" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I169" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J169" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K169" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>1</v>
+        <v>157</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>-1.5423</v>
+        <v>-1.5225</v>
       </c>
       <c r="D170" t="n">
         <v>1000</v>
       </c>
       <c r="E170" t="n">
-        <v>1342</v>
+        <v>1141.5</v>
       </c>
       <c r="F170" t="n">
-        <v>1365.6192</v>
+        <v>884.8908</v>
       </c>
       <c r="G170" t="n">
-        <v>1401.67154688</v>
+        <v>789.49957176</v>
       </c>
       <c r="H170" t="n">
-        <v>1356.1172216064</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I170" t="n">
-        <v>1614.321940600259</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J170" t="n">
-        <v>1682.93062307577</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K170" t="n">
-        <v>1547.623000980478</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
@@ -19874,192 +19936,192 @@
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D172" t="n">
         <v>1000</v>
       </c>
       <c r="E172" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F172" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G172" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H172" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I172" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J172" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K172" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D173" t="n">
         <v>1000</v>
       </c>
       <c r="E173" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F173" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G173" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H173" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I173" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J173" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K173" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D174" t="n">
         <v>1000</v>
       </c>
       <c r="E174" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F174" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G174" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H174" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I174" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J174" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K174" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="D175" t="n">
         <v>1000</v>
       </c>
       <c r="E175" t="n">
-        <v>1000.2</v>
+        <v>942</v>
       </c>
       <c r="F175" t="n">
-        <v>765.0529799999999</v>
+        <v>730.2384</v>
       </c>
       <c r="G175" t="n">
-        <v>773.1625415879998</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H175" t="n">
-        <v>742.158723670321</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I175" t="n">
-        <v>765.9078028277713</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J175" t="n">
-        <v>571.2906301292346</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K175" t="n">
-        <v>485.5970356098494</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D176" t="n">
         <v>1000</v>
       </c>
       <c r="E176" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F176" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G176" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H176" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I176" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J176" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K176" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -20067,30 +20129,67 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D177" t="n">
         <v>1000</v>
       </c>
       <c r="E177" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F177" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G177" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H177" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I177" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J177" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K177" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>41</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D178" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E178" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F177" t="n">
+      <c r="F178" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G177" t="n">
+      <c r="G178" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H177" t="n">
+      <c r="H178" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I177" t="n">
+      <c r="I178" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J177" t="n">
+      <c r="J178" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K177" t="n">
+      <c r="K178" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 193 iTransformer paper-recipe RECORD A_sh +0.92 (val crash); exp 194 variance check seed=0
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$193</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$194</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>195</row>
+      <row>196</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T193"/>
+  <dimension ref="A1:T194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13983,69 +13983,69 @@
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E186" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="F186" t="n">
-        <v>0.5694</v>
+        <v>0.9243</v>
       </c>
       <c r="G186" t="n">
-        <v>-1.3423</v>
+        <v>-1.2246</v>
       </c>
       <c r="I186" t="n">
-        <v>54.77</v>
+        <v>116.09</v>
       </c>
       <c r="J186" t="n">
-        <v>1547.7</v>
+        <v>2160.9</v>
       </c>
       <c r="K186" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L186" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N186" t="n">
-        <v>0.0103</v>
+        <v>0.0283</v>
       </c>
       <c r="O186" t="n">
-        <v>51.13</v>
+        <v>53.93</v>
       </c>
       <c r="P186" t="n">
-        <v>0.5968</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="Q186" t="n">
-        <v>0.5364</v>
+        <v>0.7548</v>
       </c>
       <c r="R186" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="S186" t="n">
-        <v>0.0098</v>
+        <v>-0.0266</v>
       </c>
       <c r="T186" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -14054,12 +14054,12 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E187" t="n">
@@ -14102,21 +14102,21 @@
         <v>0.0098</v>
       </c>
       <c r="T187" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -14125,19 +14125,19 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F188" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G188" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I188" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J188" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K188" t="n">
         <v>5</v>
@@ -14146,39 +14146,39 @@
         <v>1</v>
       </c>
       <c r="N188" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O188" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P188" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q188" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R188" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S188" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T188" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -14187,60 +14187,60 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F189" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G189" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I189" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J189" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K189" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L189" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N189" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O189" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P189" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q189" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R189" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S189" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T189" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -14249,60 +14249,60 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F190" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G190" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I190" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J190" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K190" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L190" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N190" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O190" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P190" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q190" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R190" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S190" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T190" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -14311,60 +14311,60 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="F191" t="n">
-        <v>-0.3397</v>
+        <v>-1.2201</v>
       </c>
       <c r="G191" t="n">
-        <v>-1.8082</v>
+        <v>-0.255</v>
       </c>
       <c r="I191" t="n">
-        <v>-51.44</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J191" t="n">
-        <v>485.6</v>
+        <v>282.4</v>
       </c>
       <c r="K191" t="n">
+        <v>1</v>
+      </c>
+      <c r="L191" t="n">
         <v>3</v>
       </c>
-      <c r="L191" t="n">
+      <c r="N191" t="n">
+        <v>-0.0322</v>
+      </c>
+      <c r="O191" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="P191" t="n">
         <v>0</v>
       </c>
-      <c r="N191" t="n">
-        <v>-0.0003</v>
-      </c>
-      <c r="O191" t="n">
-        <v>45.06</v>
-      </c>
-      <c r="P191" t="n">
-        <v>0.5895</v>
-      </c>
       <c r="Q191" t="n">
-        <v>0.1388</v>
+        <v>0</v>
       </c>
       <c r="R191" t="n">
-        <v>0.2247</v>
+        <v>0</v>
       </c>
       <c r="S191" t="n">
-        <v>0.0137</v>
+        <v>0</v>
       </c>
       <c r="T191" t="n">
-        <v>40.3</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -14373,51 +14373,51 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F192" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G192" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I192" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J192" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K192" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L192" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N192" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O192" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P192" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q192" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R192" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S192" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T192" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -14426,7 +14426,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -14435,51 +14435,113 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F193" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G193" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I193" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J193" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K193" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L193" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N193" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O193" t="n">
         <v>47.65</v>
       </c>
       <c r="P193" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R193" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S193" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T193" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>41</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E194" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F194" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G194" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I194" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J194" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K194" t="n">
+        <v>4</v>
+      </c>
+      <c r="L194" t="n">
+        <v>2</v>
+      </c>
+      <c r="N194" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O194" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P194" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q193" t="n">
+      <c r="Q194" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R193" t="n">
+      <c r="R194" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S193" t="n">
+      <c r="S194" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T193" t="n">
+      <c r="T194" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T193"/>
-  <conditionalFormatting sqref="E2:E193">
+  <autoFilter ref="A1:T194"/>
+  <conditionalFormatting sqref="E2:E194">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -14501,7 +14563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K193"/>
+  <dimension ref="A1:K194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -21384,44 +21446,44 @@
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="D186" t="n">
         <v>1000</v>
       </c>
       <c r="E186" t="n">
-        <v>1342</v>
+        <v>1127.9</v>
       </c>
       <c r="F186" t="n">
-        <v>1365.6192</v>
+        <v>1108.7257</v>
       </c>
       <c r="G186" t="n">
-        <v>1401.67154688</v>
+        <v>1251.64044273</v>
       </c>
       <c r="H186" t="n">
-        <v>1356.1172216064</v>
+        <v>1235.619445063056</v>
       </c>
       <c r="I186" t="n">
-        <v>1614.321940600259</v>
+        <v>1202.010596157341</v>
       </c>
       <c r="J186" t="n">
-        <v>1682.93062307577</v>
+        <v>1559.849150633381</v>
       </c>
       <c r="K186" t="n">
-        <v>1547.623000980478</v>
+        <v>2161.015013287486</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -21458,192 +21520,192 @@
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D188" t="n">
         <v>1000</v>
       </c>
       <c r="E188" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F188" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G188" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H188" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I188" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J188" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K188" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D189" t="n">
         <v>1000</v>
       </c>
       <c r="E189" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F189" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G189" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H189" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I189" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J189" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K189" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D190" t="n">
         <v>1000</v>
       </c>
       <c r="E190" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F190" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G190" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H190" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I190" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J190" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K190" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>-2.2082</v>
+        <v>-1.8201</v>
       </c>
       <c r="D191" t="n">
         <v>1000</v>
       </c>
       <c r="E191" t="n">
-        <v>1000.2</v>
+        <v>942</v>
       </c>
       <c r="F191" t="n">
-        <v>765.0529799999999</v>
+        <v>730.2384</v>
       </c>
       <c r="G191" t="n">
-        <v>773.1625415879998</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H191" t="n">
-        <v>742.158723670321</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I191" t="n">
-        <v>765.9078028277713</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J191" t="n">
-        <v>571.2906301292346</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K191" t="n">
-        <v>485.5970356098494</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D192" t="n">
         <v>1000</v>
       </c>
       <c r="E192" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F192" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G192" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H192" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I192" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J192" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K192" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -21651,30 +21713,67 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D193" t="n">
         <v>1000</v>
       </c>
       <c r="E193" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F193" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G193" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H193" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I193" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J193" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K193" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>41</v>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D194" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E194" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F193" t="n">
+      <c r="F194" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G193" t="n">
+      <c r="G194" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H193" t="n">
+      <c r="H194" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I193" t="n">
+      <c r="I194" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J193" t="n">
+      <c r="J194" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K193" t="n">
+      <c r="K194" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 194 iTransformer seed=0 -2.02 (val crash); exp 195 pre-auth seed=99 3-seed lock
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$194</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$195</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>196</row>
+      <row>197</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T194"/>
+  <dimension ref="A1:T195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -14355,16 +14355,16 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -14373,60 +14373,60 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F192" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G192" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I192" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J192" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K192" t="n">
         <v>3</v>
       </c>
       <c r="L192" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N192" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O192" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P192" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q192" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R192" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S192" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T192" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -14435,51 +14435,51 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F193" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G193" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I193" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J193" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K193" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L193" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N193" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O193" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P193" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q193" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R193" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S193" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T193" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -14488,7 +14488,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -14497,51 +14497,113 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F194" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G194" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I194" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J194" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K194" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L194" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N194" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O194" t="n">
         <v>47.65</v>
       </c>
       <c r="P194" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R194" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S194" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T194" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>41</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E195" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F195" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G195" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I195" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J195" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K195" t="n">
+        <v>4</v>
+      </c>
+      <c r="L195" t="n">
+        <v>2</v>
+      </c>
+      <c r="N195" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O195" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P195" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q194" t="n">
+      <c r="Q195" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R194" t="n">
+      <c r="R195" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S194" t="n">
+      <c r="S195" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T194" t="n">
+      <c r="T195" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T194"/>
-  <conditionalFormatting sqref="E2:E194">
+  <autoFilter ref="A1:T195"/>
+  <conditionalFormatting sqref="E2:E195">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -14563,7 +14625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K194"/>
+  <dimension ref="A1:K195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -21668,81 +21730,81 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D192" t="n">
         <v>1000</v>
       </c>
       <c r="E192" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F192" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G192" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H192" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I192" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J192" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K192" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D193" t="n">
         <v>1000</v>
       </c>
       <c r="E193" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F193" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G193" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H193" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I193" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J193" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K193" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -21750,30 +21812,67 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D194" t="n">
         <v>1000</v>
       </c>
       <c r="E194" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F194" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G194" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H194" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I194" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J194" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K194" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>41</v>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D195" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E195" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F194" t="n">
+      <c r="F195" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G194" t="n">
+      <c r="G195" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H194" t="n">
+      <c r="H195" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I194" t="n">
+      <c r="I195" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J194" t="n">
+      <c r="J195" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K194" t="n">
+      <c r="K195" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 195 iTransformer 3-seed median rejects (-1.52 comp); pivot to N-BEATS exp 196
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$196</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>197</row>
+      <row>198</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T195"/>
+  <dimension ref="A1:T196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13499,16 +13499,16 @@
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -13517,60 +13517,60 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="F178" t="n">
-        <v>-0.6042</v>
+        <v>0.2144</v>
       </c>
       <c r="G178" t="n">
-        <v>-0.8305</v>
+        <v>-1.2304</v>
       </c>
       <c r="I178" t="n">
-        <v>-67.48999999999999</v>
+        <v>10.12</v>
       </c>
       <c r="J178" t="n">
-        <v>325.1000000000001</v>
+        <v>1101.2</v>
       </c>
       <c r="K178" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L178" t="n">
         <v>3</v>
       </c>
       <c r="N178" t="n">
-        <v>0.0111</v>
+        <v>0.0027</v>
       </c>
       <c r="O178" t="n">
-        <v>42.64</v>
+        <v>53.55</v>
       </c>
       <c r="P178" t="n">
-        <v>0</v>
+        <v>0.5858</v>
       </c>
       <c r="Q178" t="n">
-        <v>0</v>
+        <v>0.7341</v>
       </c>
       <c r="R178" t="n">
-        <v>0</v>
+        <v>0.6516</v>
       </c>
       <c r="S178" t="n">
-        <v>0</v>
+        <v>-0.0231</v>
       </c>
       <c r="T178" t="n">
-        <v>82.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -13579,60 +13579,60 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F179" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G179" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I179" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J179" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K179" t="n">
         <v>1</v>
       </c>
       <c r="L179" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N179" t="n">
-        <v>0.0284</v>
+        <v>0.0111</v>
       </c>
       <c r="O179" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P179" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q179" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R179" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S179" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T179" t="n">
-        <v>79.8</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -13641,60 +13641,60 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="F180" t="n">
-        <v>0.4732</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G180" t="n">
-        <v>-1.1536</v>
+        <v>-0.8347</v>
       </c>
       <c r="I180" t="n">
-        <v>41.21</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J180" t="n">
-        <v>1412.1</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K180" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L180" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N180" t="n">
-        <v>0.0231</v>
+        <v>0.0284</v>
       </c>
       <c r="O180" t="n">
-        <v>48.31</v>
+        <v>44.07</v>
       </c>
       <c r="P180" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.5588</v>
       </c>
       <c r="Q180" t="n">
-        <v>0.3418</v>
+        <v>0.1177</v>
       </c>
       <c r="R180" t="n">
-        <v>0.4395</v>
+        <v>0.1945</v>
       </c>
       <c r="S180" t="n">
-        <v>0.0329</v>
+        <v>-0.0101</v>
       </c>
       <c r="T180" t="n">
-        <v>1311.2</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -13703,39 +13703,51 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F181" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G181" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I181" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J181" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K181" t="n">
         <v>4</v>
       </c>
       <c r="L181" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N181" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O181" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P181" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q181" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R181" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S181" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T181" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -13744,7 +13756,7 @@
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -13753,51 +13765,39 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F182" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G182" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I182" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J182" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K182" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L182" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N182" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O182" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P182" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q182" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R182" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S182" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T182" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -13806,7 +13806,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -13815,51 +13815,51 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F183" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G183" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I183" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J183" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L183" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N183" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O183" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P183" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q183" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R183" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S183" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T183" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -13868,7 +13868,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -13877,60 +13877,60 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F184" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G184" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I184" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J184" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K184" t="n">
         <v>1</v>
       </c>
       <c r="L184" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N184" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O184" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P184" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q184" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R184" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S184" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T184" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -13939,60 +13939,60 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F185" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G185" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I185" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J185" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K185" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L185" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N185" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O185" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P185" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q185" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R185" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S185" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T185" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -14001,113 +14001,113 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="F186" t="n">
-        <v>0.9243</v>
+        <v>-1.0225</v>
       </c>
       <c r="G186" t="n">
-        <v>-1.2246</v>
+        <v>-0.2617</v>
       </c>
       <c r="I186" t="n">
-        <v>116.09</v>
+        <v>-65.97</v>
       </c>
       <c r="J186" t="n">
-        <v>2160.9</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K186" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L186" t="n">
         <v>3</v>
       </c>
       <c r="N186" t="n">
-        <v>0.0283</v>
+        <v>-0.0076</v>
       </c>
       <c r="O186" t="n">
-        <v>53.93</v>
+        <v>40.96</v>
       </c>
       <c r="P186" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5526</v>
       </c>
       <c r="Q186" t="n">
-        <v>0.7548</v>
+        <v>0.0334</v>
       </c>
       <c r="R186" t="n">
-        <v>0.6592</v>
+        <v>0.0631</v>
       </c>
       <c r="S186" t="n">
-        <v>-0.0266</v>
+        <v>-0.0156</v>
       </c>
       <c r="T186" t="n">
-        <v>97.5</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="F187" t="n">
-        <v>0.5694</v>
+        <v>0.9243</v>
       </c>
       <c r="G187" t="n">
-        <v>-1.3423</v>
+        <v>-1.2246</v>
       </c>
       <c r="I187" t="n">
-        <v>54.77</v>
+        <v>116.09</v>
       </c>
       <c r="J187" t="n">
-        <v>1547.7</v>
+        <v>2160.9</v>
       </c>
       <c r="K187" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L187" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N187" t="n">
-        <v>0.0103</v>
+        <v>0.0283</v>
       </c>
       <c r="O187" t="n">
-        <v>51.13</v>
+        <v>53.93</v>
       </c>
       <c r="P187" t="n">
-        <v>0.5968</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="Q187" t="n">
-        <v>0.5364</v>
+        <v>0.7548</v>
       </c>
       <c r="R187" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="S187" t="n">
-        <v>0.0098</v>
+        <v>-0.0266</v>
       </c>
       <c r="T187" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -14116,12 +14116,12 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E188" t="n">
@@ -14164,21 +14164,21 @@
         <v>0.0098</v>
       </c>
       <c r="T188" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -14187,19 +14187,19 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F189" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G189" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I189" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J189" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K189" t="n">
         <v>5</v>
@@ -14208,39 +14208,39 @@
         <v>1</v>
       </c>
       <c r="N189" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O189" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P189" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q189" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R189" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S189" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T189" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -14249,60 +14249,60 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F190" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G190" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I190" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J190" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K190" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L190" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N190" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O190" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P190" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q190" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R190" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S190" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T190" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -14311,60 +14311,60 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F191" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G191" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I191" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J191" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K191" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L191" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N191" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O191" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P191" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q191" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R191" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S191" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T191" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -14373,60 +14373,60 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="F192" t="n">
-        <v>-0.1044</v>
+        <v>-1.2201</v>
       </c>
       <c r="G192" t="n">
-        <v>-1.6173</v>
+        <v>-0.255</v>
       </c>
       <c r="I192" t="n">
-        <v>-18.65</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J192" t="n">
-        <v>813.5</v>
+        <v>282.4</v>
       </c>
       <c r="K192" t="n">
+        <v>1</v>
+      </c>
+      <c r="L192" t="n">
         <v>3</v>
       </c>
-      <c r="L192" t="n">
-        <v>2</v>
-      </c>
       <c r="N192" t="n">
-        <v>-0.0416</v>
+        <v>-0.0322</v>
       </c>
       <c r="O192" t="n">
-        <v>48.72</v>
+        <v>40.59</v>
       </c>
       <c r="P192" t="n">
-        <v>0.5679999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q192" t="n">
-        <v>0.5653</v>
+        <v>0</v>
       </c>
       <c r="R192" t="n">
-        <v>0.5666</v>
+        <v>0</v>
       </c>
       <c r="S192" t="n">
-        <v>-0.0596</v>
+        <v>0</v>
       </c>
       <c r="T192" t="n">
-        <v>73</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -14435,60 +14435,60 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F193" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G193" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I193" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J193" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K193" t="n">
         <v>3</v>
       </c>
       <c r="L193" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N193" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O193" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P193" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q193" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R193" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S193" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T193" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -14497,51 +14497,51 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F194" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G194" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I194" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J194" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K194" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L194" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N194" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O194" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P194" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q194" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R194" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S194" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T194" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -14550,7 +14550,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -14559,51 +14559,113 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F195" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G195" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I195" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J195" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K195" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L195" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N195" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O195" t="n">
         <v>47.65</v>
       </c>
       <c r="P195" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R195" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S195" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T195" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>41</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E196" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F196" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G196" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I196" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J196" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K196" t="n">
+        <v>4</v>
+      </c>
+      <c r="L196" t="n">
+        <v>2</v>
+      </c>
+      <c r="N196" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O196" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P196" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q195" t="n">
+      <c r="Q196" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R195" t="n">
+      <c r="R196" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S195" t="n">
+      <c r="S196" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T195" t="n">
+      <c r="T196" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T195"/>
-  <conditionalFormatting sqref="E2:E195">
+  <autoFilter ref="A1:T196"/>
+  <conditionalFormatting sqref="E2:E196">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -14625,7 +14687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K195"/>
+  <dimension ref="A1:K196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -21212,155 +21274,155 @@
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="D178" t="n">
         <v>1000</v>
       </c>
       <c r="E178" t="n">
-        <v>1045.3</v>
+        <v>999.6</v>
       </c>
       <c r="F178" t="n">
-        <v>853.06933</v>
+        <v>1076.66916</v>
       </c>
       <c r="G178" t="n">
-        <v>749.933248003</v>
+        <v>1127.918612016</v>
       </c>
       <c r="H178" t="n">
-        <v>740.3341024285616</v>
+        <v>1009.261574031917</v>
       </c>
       <c r="I178" t="n">
-        <v>691.1759180273051</v>
+        <v>837.9898849187007</v>
       </c>
       <c r="J178" t="n">
-        <v>482.7172611502699</v>
+        <v>1032.403538219839</v>
       </c>
       <c r="K178" t="n">
-        <v>325.0618036585918</v>
+        <v>1101.161613865281</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D179" t="n">
         <v>1000</v>
       </c>
       <c r="E179" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F179" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G179" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H179" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I179" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J179" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K179" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="D180" t="n">
         <v>1000</v>
       </c>
       <c r="E180" t="n">
-        <v>1236.4</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F180" t="n">
-        <v>1500.74232</v>
+        <v>692.62656</v>
       </c>
       <c r="G180" t="n">
-        <v>1734.708047688</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H180" t="n">
-        <v>1677.809623723833</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I180" t="n">
-        <v>1544.088196713044</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J180" t="n">
-        <v>1750.069562154564</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K180" t="n">
-        <v>1412.131129702517</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D181" t="n">
         <v>1000</v>
       </c>
       <c r="E181" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F181" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G181" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H181" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I181" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J181" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K181" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
@@ -21368,36 +21430,36 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D182" t="n">
         <v>1000</v>
       </c>
       <c r="E182" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F182" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G182" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H182" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I182" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J182" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K182" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -21405,36 +21467,36 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D183" t="n">
         <v>1000</v>
       </c>
       <c r="E183" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F183" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G183" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H183" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I183" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J183" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K183" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -21442,147 +21504,147 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D184" t="n">
         <v>1000</v>
       </c>
       <c r="E184" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F184" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G184" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H184" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I184" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J184" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K184" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D185" t="n">
         <v>1000</v>
       </c>
       <c r="E185" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F185" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G185" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H185" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I185" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J185" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K185" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="D186" t="n">
         <v>1000</v>
       </c>
       <c r="E186" t="n">
-        <v>1127.9</v>
+        <v>1141.5</v>
       </c>
       <c r="F186" t="n">
-        <v>1108.7257</v>
+        <v>884.8908</v>
       </c>
       <c r="G186" t="n">
-        <v>1251.64044273</v>
+        <v>789.49957176</v>
       </c>
       <c r="H186" t="n">
-        <v>1235.619445063056</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I186" t="n">
-        <v>1202.010596157341</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J186" t="n">
-        <v>1559.849150633381</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K186" t="n">
-        <v>2161.015013287486</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="D187" t="n">
         <v>1000</v>
       </c>
       <c r="E187" t="n">
-        <v>1342</v>
+        <v>1127.9</v>
       </c>
       <c r="F187" t="n">
-        <v>1365.6192</v>
+        <v>1108.7257</v>
       </c>
       <c r="G187" t="n">
-        <v>1401.67154688</v>
+        <v>1251.64044273</v>
       </c>
       <c r="H187" t="n">
-        <v>1356.1172216064</v>
+        <v>1235.619445063056</v>
       </c>
       <c r="I187" t="n">
-        <v>1614.321940600259</v>
+        <v>1202.010596157341</v>
       </c>
       <c r="J187" t="n">
-        <v>1682.93062307577</v>
+        <v>1559.849150633381</v>
       </c>
       <c r="K187" t="n">
-        <v>1547.623000980478</v>
+        <v>2161.015013287486</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
@@ -21619,229 +21681,229 @@
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D189" t="n">
         <v>1000</v>
       </c>
       <c r="E189" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F189" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G189" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H189" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I189" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J189" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K189" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D190" t="n">
         <v>1000</v>
       </c>
       <c r="E190" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F190" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G190" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H190" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I190" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J190" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K190" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D191" t="n">
         <v>1000</v>
       </c>
       <c r="E191" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F191" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G191" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H191" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I191" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J191" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K191" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="D192" t="n">
         <v>1000</v>
       </c>
       <c r="E192" t="n">
-        <v>1222.6</v>
+        <v>942</v>
       </c>
       <c r="F192" t="n">
-        <v>1122.46906</v>
+        <v>730.2384</v>
       </c>
       <c r="G192" t="n">
-        <v>1222.481053246</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H192" t="n">
-        <v>1198.520424602378</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I192" t="n">
-        <v>1133.440765546469</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J192" t="n">
-        <v>1142.73497982395</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K192" t="n">
-        <v>813.6273056346525</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D193" t="n">
         <v>1000</v>
       </c>
       <c r="E193" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F193" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G193" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H193" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I193" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J193" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K193" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D194" t="n">
         <v>1000</v>
       </c>
       <c r="E194" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F194" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G194" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H194" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I194" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J194" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K194" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -21849,30 +21911,67 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D195" t="n">
         <v>1000</v>
       </c>
       <c r="E195" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F195" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G195" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H195" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I195" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J195" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K195" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>41</v>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D196" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E196" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F195" t="n">
+      <c r="F196" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G195" t="n">
+      <c r="G196" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H195" t="n">
+      <c r="H196" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I195" t="n">
+      <c r="I196" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J195" t="n">
+      <c r="J196" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K195" t="n">
+      <c r="K196" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 196 N-BEATS seed=0 -1.43 (reproducibly weak); exp 197 PatchTSMixer 3-seed lock
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$196</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$197</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>198</row>
+      <row>199</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T196"/>
+  <dimension ref="A1:T197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13623,16 +13623,16 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -13641,60 +13641,60 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F180" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G180" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I180" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J180" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K180" t="n">
         <v>1</v>
       </c>
       <c r="L180" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N180" t="n">
-        <v>0.0284</v>
+        <v>0.032</v>
       </c>
       <c r="O180" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P180" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q180" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R180" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S180" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T180" t="n">
-        <v>79.8</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -13703,60 +13703,60 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="F181" t="n">
-        <v>0.4732</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G181" t="n">
-        <v>-1.1536</v>
+        <v>-0.8347</v>
       </c>
       <c r="I181" t="n">
-        <v>41.21</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J181" t="n">
-        <v>1412.1</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K181" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L181" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N181" t="n">
-        <v>0.0231</v>
+        <v>0.0284</v>
       </c>
       <c r="O181" t="n">
-        <v>48.31</v>
+        <v>44.07</v>
       </c>
       <c r="P181" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.5588</v>
       </c>
       <c r="Q181" t="n">
-        <v>0.3418</v>
+        <v>0.1177</v>
       </c>
       <c r="R181" t="n">
-        <v>0.4395</v>
+        <v>0.1945</v>
       </c>
       <c r="S181" t="n">
-        <v>0.0329</v>
+        <v>-0.0101</v>
       </c>
       <c r="T181" t="n">
-        <v>1311.2</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -13765,39 +13765,51 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F182" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G182" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I182" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J182" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K182" t="n">
         <v>4</v>
       </c>
       <c r="L182" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N182" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O182" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P182" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q182" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R182" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S182" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T182" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -13806,7 +13818,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -13815,51 +13827,39 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F183" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G183" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I183" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J183" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K183" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L183" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N183" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O183" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P183" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q183" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R183" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S183" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T183" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -13868,7 +13868,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -13877,51 +13877,51 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F184" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G184" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I184" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J184" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L184" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N184" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O184" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P184" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q184" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R184" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S184" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T184" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -13930,7 +13930,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -13939,60 +13939,60 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F185" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G185" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I185" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J185" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K185" t="n">
         <v>1</v>
       </c>
       <c r="L185" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N185" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O185" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P185" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q185" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R185" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S185" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T185" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -14001,60 +14001,60 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F186" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G186" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I186" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J186" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K186" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L186" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N186" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O186" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P186" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q186" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R186" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S186" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T186" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -14063,113 +14063,113 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="F187" t="n">
-        <v>0.9243</v>
+        <v>-1.0225</v>
       </c>
       <c r="G187" t="n">
-        <v>-1.2246</v>
+        <v>-0.2617</v>
       </c>
       <c r="I187" t="n">
-        <v>116.09</v>
+        <v>-65.97</v>
       </c>
       <c r="J187" t="n">
-        <v>2160.9</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K187" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L187" t="n">
         <v>3</v>
       </c>
       <c r="N187" t="n">
-        <v>0.0283</v>
+        <v>-0.0076</v>
       </c>
       <c r="O187" t="n">
-        <v>53.93</v>
+        <v>40.96</v>
       </c>
       <c r="P187" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5526</v>
       </c>
       <c r="Q187" t="n">
-        <v>0.7548</v>
+        <v>0.0334</v>
       </c>
       <c r="R187" t="n">
-        <v>0.6592</v>
+        <v>0.0631</v>
       </c>
       <c r="S187" t="n">
-        <v>-0.0266</v>
+        <v>-0.0156</v>
       </c>
       <c r="T187" t="n">
-        <v>97.5</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="F188" t="n">
-        <v>0.5694</v>
+        <v>0.9243</v>
       </c>
       <c r="G188" t="n">
-        <v>-1.3423</v>
+        <v>-1.2246</v>
       </c>
       <c r="I188" t="n">
-        <v>54.77</v>
+        <v>116.09</v>
       </c>
       <c r="J188" t="n">
-        <v>1547.7</v>
+        <v>2160.9</v>
       </c>
       <c r="K188" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L188" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N188" t="n">
-        <v>0.0103</v>
+        <v>0.0283</v>
       </c>
       <c r="O188" t="n">
-        <v>51.13</v>
+        <v>53.93</v>
       </c>
       <c r="P188" t="n">
-        <v>0.5968</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="Q188" t="n">
-        <v>0.5364</v>
+        <v>0.7548</v>
       </c>
       <c r="R188" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="S188" t="n">
-        <v>0.0098</v>
+        <v>-0.0266</v>
       </c>
       <c r="T188" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -14178,12 +14178,12 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E189" t="n">
@@ -14226,21 +14226,21 @@
         <v>0.0098</v>
       </c>
       <c r="T189" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -14249,19 +14249,19 @@
         </is>
       </c>
       <c r="E190" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F190" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G190" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I190" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J190" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K190" t="n">
         <v>5</v>
@@ -14270,39 +14270,39 @@
         <v>1</v>
       </c>
       <c r="N190" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O190" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P190" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q190" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R190" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S190" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T190" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -14311,60 +14311,60 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F191" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G191" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I191" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J191" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K191" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L191" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N191" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O191" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P191" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q191" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R191" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S191" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T191" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -14373,60 +14373,60 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F192" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G192" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I192" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J192" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K192" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L192" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N192" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O192" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P192" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q192" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R192" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S192" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T192" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -14435,60 +14435,60 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="F193" t="n">
-        <v>-0.1044</v>
+        <v>-1.2201</v>
       </c>
       <c r="G193" t="n">
-        <v>-1.6173</v>
+        <v>-0.255</v>
       </c>
       <c r="I193" t="n">
-        <v>-18.65</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J193" t="n">
-        <v>813.5</v>
+        <v>282.4</v>
       </c>
       <c r="K193" t="n">
+        <v>1</v>
+      </c>
+      <c r="L193" t="n">
         <v>3</v>
       </c>
-      <c r="L193" t="n">
-        <v>2</v>
-      </c>
       <c r="N193" t="n">
-        <v>-0.0416</v>
+        <v>-0.0322</v>
       </c>
       <c r="O193" t="n">
-        <v>48.72</v>
+        <v>40.59</v>
       </c>
       <c r="P193" t="n">
-        <v>0.5679999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q193" t="n">
-        <v>0.5653</v>
+        <v>0</v>
       </c>
       <c r="R193" t="n">
-        <v>0.5666</v>
+        <v>0</v>
       </c>
       <c r="S193" t="n">
-        <v>-0.0596</v>
+        <v>0</v>
       </c>
       <c r="T193" t="n">
-        <v>73</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -14497,60 +14497,60 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F194" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G194" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I194" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J194" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K194" t="n">
         <v>3</v>
       </c>
       <c r="L194" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N194" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O194" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P194" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q194" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R194" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S194" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T194" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -14559,51 +14559,51 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F195" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G195" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I195" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J195" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K195" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L195" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N195" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O195" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P195" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q195" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R195" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S195" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T195" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -14612,7 +14612,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -14621,51 +14621,113 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F196" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G196" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I196" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J196" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K196" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L196" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N196" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O196" t="n">
         <v>47.65</v>
       </c>
       <c r="P196" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R196" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S196" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T196" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>41</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E197" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F197" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G197" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I197" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J197" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K197" t="n">
+        <v>4</v>
+      </c>
+      <c r="L197" t="n">
+        <v>2</v>
+      </c>
+      <c r="N197" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O197" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P197" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q196" t="n">
+      <c r="Q197" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R196" t="n">
+      <c r="R197" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S196" t="n">
+      <c r="S197" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T196" t="n">
+      <c r="T197" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T196"/>
-  <conditionalFormatting sqref="E2:E196">
+  <autoFilter ref="A1:T197"/>
+  <conditionalFormatting sqref="E2:E197">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -14687,7 +14749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K196"/>
+  <dimension ref="A1:K197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -21348,118 +21410,118 @@
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D180" t="n">
         <v>1000</v>
       </c>
       <c r="E180" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F180" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G180" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H180" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I180" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J180" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K180" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="D181" t="n">
         <v>1000</v>
       </c>
       <c r="E181" t="n">
-        <v>1236.4</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F181" t="n">
-        <v>1500.74232</v>
+        <v>692.62656</v>
       </c>
       <c r="G181" t="n">
-        <v>1734.708047688</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H181" t="n">
-        <v>1677.809623723833</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I181" t="n">
-        <v>1544.088196713044</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J181" t="n">
-        <v>1750.069562154564</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K181" t="n">
-        <v>1412.131129702517</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D182" t="n">
         <v>1000</v>
       </c>
       <c r="E182" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F182" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G182" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H182" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I182" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J182" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K182" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -21467,36 +21529,36 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D183" t="n">
         <v>1000</v>
       </c>
       <c r="E183" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F183" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G183" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H183" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I183" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J183" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K183" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -21504,36 +21566,36 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D184" t="n">
         <v>1000</v>
       </c>
       <c r="E184" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F184" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G184" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H184" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I184" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J184" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K184" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -21541,147 +21603,147 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D185" t="n">
         <v>1000</v>
       </c>
       <c r="E185" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F185" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G185" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H185" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I185" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J185" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K185" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D186" t="n">
         <v>1000</v>
       </c>
       <c r="E186" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F186" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G186" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H186" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I186" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J186" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K186" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="D187" t="n">
         <v>1000</v>
       </c>
       <c r="E187" t="n">
-        <v>1127.9</v>
+        <v>1141.5</v>
       </c>
       <c r="F187" t="n">
-        <v>1108.7257</v>
+        <v>884.8908</v>
       </c>
       <c r="G187" t="n">
-        <v>1251.64044273</v>
+        <v>789.49957176</v>
       </c>
       <c r="H187" t="n">
-        <v>1235.619445063056</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I187" t="n">
-        <v>1202.010596157341</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J187" t="n">
-        <v>1559.849150633381</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K187" t="n">
-        <v>2161.015013287486</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="D188" t="n">
         <v>1000</v>
       </c>
       <c r="E188" t="n">
-        <v>1342</v>
+        <v>1127.9</v>
       </c>
       <c r="F188" t="n">
-        <v>1365.6192</v>
+        <v>1108.7257</v>
       </c>
       <c r="G188" t="n">
-        <v>1401.67154688</v>
+        <v>1251.64044273</v>
       </c>
       <c r="H188" t="n">
-        <v>1356.1172216064</v>
+        <v>1235.619445063056</v>
       </c>
       <c r="I188" t="n">
-        <v>1614.321940600259</v>
+        <v>1202.010596157341</v>
       </c>
       <c r="J188" t="n">
-        <v>1682.93062307577</v>
+        <v>1559.849150633381</v>
       </c>
       <c r="K188" t="n">
-        <v>1547.623000980478</v>
+        <v>2161.015013287486</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -21718,229 +21780,229 @@
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D190" t="n">
         <v>1000</v>
       </c>
       <c r="E190" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F190" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G190" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H190" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I190" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J190" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K190" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D191" t="n">
         <v>1000</v>
       </c>
       <c r="E191" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F191" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G191" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H191" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I191" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J191" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K191" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D192" t="n">
         <v>1000</v>
       </c>
       <c r="E192" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F192" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G192" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H192" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I192" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J192" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K192" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="D193" t="n">
         <v>1000</v>
       </c>
       <c r="E193" t="n">
-        <v>1222.6</v>
+        <v>942</v>
       </c>
       <c r="F193" t="n">
-        <v>1122.46906</v>
+        <v>730.2384</v>
       </c>
       <c r="G193" t="n">
-        <v>1222.481053246</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H193" t="n">
-        <v>1198.520424602378</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I193" t="n">
-        <v>1133.440765546469</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J193" t="n">
-        <v>1142.73497982395</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K193" t="n">
-        <v>813.6273056346525</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D194" t="n">
         <v>1000</v>
       </c>
       <c r="E194" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F194" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G194" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H194" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I194" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J194" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K194" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D195" t="n">
         <v>1000</v>
       </c>
       <c r="E195" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F195" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G195" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H195" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I195" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J195" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K195" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -21948,30 +22010,67 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D196" t="n">
         <v>1000</v>
       </c>
       <c r="E196" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F196" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G196" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H196" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I196" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J196" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K196" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>41</v>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D197" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E197" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F196" t="n">
+      <c r="F197" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G196" t="n">
+      <c r="G197" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H196" t="n">
+      <c r="H197" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I196" t="n">
+      <c r="I197" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J196" t="n">
+      <c r="J197" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K196" t="n">
+      <c r="K197" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 198 PatchTSMixer seed=7 -1.10 (4-seed median -0.52); exp 199 5-seed lock
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$199</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>200</row>
+      <row>201</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T198"/>
+  <dimension ref="A1:T199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -12817,16 +12817,16 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>23</v>
+        <v>198</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>PatchTSMixer seed=7 (variance check on exp 197 A_sh+1.22 RECORD) - Picard 2021 + Lakshmina</t>
         </is>
       </c>
       <c r="D167" t="inlineStr">
@@ -12835,51 +12835,51 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>-1.1119</v>
+        <v>-1.096</v>
       </c>
       <c r="F167" t="n">
-        <v>-0.5057</v>
+        <v>-0.1414</v>
       </c>
       <c r="G167" t="n">
-        <v>-0.5119</v>
+        <v>-0.696</v>
       </c>
       <c r="I167" t="n">
-        <v>-62.25</v>
+        <v>-21.47</v>
       </c>
       <c r="J167" t="n">
-        <v>377.4999999999999</v>
+        <v>785.3</v>
       </c>
       <c r="K167" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L167" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N167" t="n">
-        <v>0.0032</v>
+        <v>-0.0452</v>
       </c>
       <c r="O167" t="n">
-        <v>44.56</v>
+        <v>50.8</v>
       </c>
       <c r="P167" t="n">
-        <v>0.6421</v>
+        <v>0.5744</v>
       </c>
       <c r="Q167" t="n">
-        <v>0.0756</v>
+        <v>0.6513</v>
       </c>
       <c r="R167" t="n">
-        <v>0.1353</v>
+        <v>0.6104000000000001</v>
       </c>
       <c r="S167" t="n">
-        <v>0.0379</v>
+        <v>-0.0524</v>
       </c>
       <c r="T167" t="n">
-        <v>53.3</v>
+        <v>483.6</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -12888,7 +12888,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
@@ -12897,51 +12897,51 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F168" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G168" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I168" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J168" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K168" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L168" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N168" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O168" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P168" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q168" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R168" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S168" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T168" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>177</v>
+        <v>87</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -12950,7 +12950,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>LSTM lr=2e-3 (Smith 2017 highest-leverage axis untested) - one knob from exp 74 lr=1e-3</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -12959,60 +12959,60 @@
         </is>
       </c>
       <c r="E169" t="n">
-        <v>-1.1172</v>
+        <v>-1.1144</v>
       </c>
       <c r="F169" t="n">
-        <v>0.0506</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G169" t="n">
-        <v>-0.7171999999999999</v>
+        <v>-0.0276</v>
       </c>
       <c r="I169" t="n">
-        <v>-11.99</v>
+        <v>-67.98</v>
       </c>
       <c r="J169" t="n">
-        <v>880.1</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K169" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L169" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N169" t="n">
-        <v>0.0322</v>
+        <v>-0.0254</v>
       </c>
       <c r="O169" t="n">
-        <v>46.2</v>
+        <v>44.42</v>
       </c>
       <c r="P169" t="n">
-        <v>0.5585</v>
+        <v>0.5676</v>
       </c>
       <c r="Q169" t="n">
-        <v>0.29</v>
+        <v>0.1301</v>
       </c>
       <c r="R169" t="n">
-        <v>0.3817</v>
+        <v>0.2117</v>
       </c>
       <c r="S169" t="n">
-        <v>-0.0182</v>
+        <v>-0.0037</v>
       </c>
       <c r="T169" t="n">
-        <v>52.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>51</v>
+        <v>177</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM lr=2e-3 (Smith 2017 highest-leverage axis untested) - one knob from exp 74 lr=1e-3</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -13021,60 +13021,60 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>-1.1484</v>
+        <v>-1.1172</v>
       </c>
       <c r="F170" t="n">
-        <v>-0.6484</v>
+        <v>0.0506</v>
       </c>
       <c r="G170" t="n">
-        <v>1.8519</v>
+        <v>-0.7171999999999999</v>
       </c>
       <c r="I170" t="n">
-        <v>-51.47</v>
+        <v>-11.99</v>
       </c>
       <c r="J170" t="n">
-        <v>485.3000000000001</v>
+        <v>880.1</v>
       </c>
       <c r="K170" t="n">
+        <v>3</v>
+      </c>
+      <c r="L170" t="n">
         <v>2</v>
       </c>
-      <c r="L170" t="n">
-        <v>5</v>
-      </c>
       <c r="N170" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0322</v>
       </c>
       <c r="O170" t="n">
-        <v>43.33</v>
+        <v>46.2</v>
       </c>
       <c r="P170" t="n">
-        <v>0.5736</v>
+        <v>0.5585</v>
       </c>
       <c r="Q170" t="n">
-        <v>0.1799</v>
+        <v>0.29</v>
       </c>
       <c r="R170" t="n">
-        <v>0.2739</v>
+        <v>0.3817</v>
       </c>
       <c r="S170" t="n">
-        <v>-0.0183</v>
+        <v>-0.0182</v>
       </c>
       <c r="T170" t="n">
-        <v>823.8</v>
+        <v>52.2</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -13083,60 +13083,60 @@
         </is>
       </c>
       <c r="E171" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F171" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G171" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I171" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J171" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K171" t="n">
+        <v>2</v>
+      </c>
+      <c r="L171" t="n">
         <v>5</v>
       </c>
-      <c r="L171" t="n">
-        <v>2</v>
-      </c>
       <c r="N171" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O171" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P171" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q171" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R171" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S171" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T171" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D172" t="inlineStr">
@@ -13145,60 +13145,60 @@
         </is>
       </c>
       <c r="E172" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F172" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G172" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I172" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J172" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K172" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L172" t="n">
         <v>2</v>
       </c>
       <c r="N172" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O172" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P172" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q172" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R172" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S172" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T172" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D173" t="inlineStr">
@@ -13207,51 +13207,51 @@
         </is>
       </c>
       <c r="E173" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F173" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G173" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I173" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J173" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K173" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L173" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N173" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O173" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P173" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q173" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R173" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S173" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T173" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -13260,7 +13260,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -13269,51 +13269,51 @@
         </is>
       </c>
       <c r="E174" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F174" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G174" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I174" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J174" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K174" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L174" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N174" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O174" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P174" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q174" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R174" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S174" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T174" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -13322,7 +13322,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -13331,60 +13331,60 @@
         </is>
       </c>
       <c r="E175" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F175" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G175" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I175" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J175" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K175" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L175" t="n">
         <v>2</v>
       </c>
       <c r="N175" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O175" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P175" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q175" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R175" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S175" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T175" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -13393,60 +13393,60 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F176" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G176" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I176" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J176" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K176" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L176" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N176" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O176" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P176" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q176" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R176" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S176" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T176" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -13455,60 +13455,60 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F177" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G177" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I177" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J177" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K177" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L177" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N177" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O177" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P177" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q177" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R177" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S177" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T177" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -13517,60 +13517,60 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F178" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G178" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I178" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J178" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K178" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L178" t="n">
         <v>3</v>
       </c>
       <c r="N178" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O178" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P178" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q178" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R178" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S178" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T178" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -13579,60 +13579,60 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="F179" t="n">
-        <v>0.2144</v>
+        <v>-0.8189</v>
       </c>
       <c r="G179" t="n">
-        <v>-1.2304</v>
+        <v>1.1456</v>
       </c>
       <c r="I179" t="n">
-        <v>10.12</v>
+        <v>-58.71</v>
       </c>
       <c r="J179" t="n">
-        <v>1101.2</v>
+        <v>412.9</v>
       </c>
       <c r="K179" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L179" t="n">
         <v>3</v>
       </c>
       <c r="N179" t="n">
-        <v>0.0027</v>
+        <v>0.0089</v>
       </c>
       <c r="O179" t="n">
-        <v>53.55</v>
+        <v>41.44</v>
       </c>
       <c r="P179" t="n">
-        <v>0.5858</v>
+        <v>0.68</v>
       </c>
       <c r="Q179" t="n">
-        <v>0.7341</v>
+        <v>0.0271</v>
       </c>
       <c r="R179" t="n">
-        <v>0.6516</v>
+        <v>0.0521</v>
       </c>
       <c r="S179" t="n">
-        <v>-0.0231</v>
+        <v>0.0277</v>
       </c>
       <c r="T179" t="n">
-        <v>69.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -13641,51 +13641,51 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="F180" t="n">
-        <v>-0.6042</v>
+        <v>0.2144</v>
       </c>
       <c r="G180" t="n">
-        <v>-0.8305</v>
+        <v>-1.2304</v>
       </c>
       <c r="I180" t="n">
-        <v>-67.48999999999999</v>
+        <v>10.12</v>
       </c>
       <c r="J180" t="n">
-        <v>325.1000000000001</v>
+        <v>1101.2</v>
       </c>
       <c r="K180" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L180" t="n">
         <v>3</v>
       </c>
       <c r="N180" t="n">
-        <v>0.0111</v>
+        <v>0.0027</v>
       </c>
       <c r="O180" t="n">
-        <v>42.64</v>
+        <v>53.55</v>
       </c>
       <c r="P180" t="n">
-        <v>0</v>
+        <v>0.5858</v>
       </c>
       <c r="Q180" t="n">
-        <v>0</v>
+        <v>0.7341</v>
       </c>
       <c r="R180" t="n">
-        <v>0</v>
+        <v>0.6516</v>
       </c>
       <c r="S180" t="n">
-        <v>0</v>
+        <v>-0.0231</v>
       </c>
       <c r="T180" t="n">
-        <v>82.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -13694,7 +13694,7 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -13724,7 +13724,7 @@
         <v>3</v>
       </c>
       <c r="N181" t="n">
-        <v>0.032</v>
+        <v>0.0111</v>
       </c>
       <c r="O181" t="n">
         <v>42.64</v>
@@ -13742,21 +13742,21 @@
         <v>0</v>
       </c>
       <c r="T181" t="n">
-        <v>62.3</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -13765,60 +13765,60 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F182" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G182" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I182" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J182" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K182" t="n">
         <v>1</v>
       </c>
       <c r="L182" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N182" t="n">
-        <v>0.0284</v>
+        <v>0.032</v>
       </c>
       <c r="O182" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P182" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q182" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R182" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S182" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T182" t="n">
-        <v>79.8</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -13827,60 +13827,60 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="F183" t="n">
-        <v>0.4732</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G183" t="n">
-        <v>-1.1536</v>
+        <v>-0.8347</v>
       </c>
       <c r="I183" t="n">
-        <v>41.21</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J183" t="n">
-        <v>1412.1</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K183" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L183" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N183" t="n">
-        <v>0.0231</v>
+        <v>0.0284</v>
       </c>
       <c r="O183" t="n">
-        <v>48.31</v>
+        <v>44.07</v>
       </c>
       <c r="P183" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.5588</v>
       </c>
       <c r="Q183" t="n">
-        <v>0.3418</v>
+        <v>0.1177</v>
       </c>
       <c r="R183" t="n">
-        <v>0.4395</v>
+        <v>0.1945</v>
       </c>
       <c r="S183" t="n">
-        <v>0.0329</v>
+        <v>-0.0101</v>
       </c>
       <c r="T183" t="n">
-        <v>1311.2</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -13889,39 +13889,51 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F184" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G184" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I184" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J184" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K184" t="n">
         <v>4</v>
       </c>
       <c r="L184" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N184" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O184" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P184" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q184" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R184" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S184" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T184" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -13930,7 +13942,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -13939,51 +13951,39 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F185" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G185" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I185" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J185" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K185" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L185" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N185" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O185" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P185" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q185" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R185" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S185" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T185" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -13992,7 +13992,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -14001,51 +14001,51 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F186" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G186" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I186" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J186" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K186" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L186" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N186" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O186" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P186" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q186" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R186" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S186" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T186" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -14054,7 +14054,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -14063,60 +14063,60 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F187" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G187" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I187" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J187" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K187" t="n">
         <v>1</v>
       </c>
       <c r="L187" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N187" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O187" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P187" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q187" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R187" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S187" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T187" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -14125,60 +14125,60 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F188" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G188" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I188" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J188" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K188" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L188" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N188" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O188" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P188" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q188" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R188" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S188" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T188" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -14187,113 +14187,113 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="F189" t="n">
-        <v>0.9243</v>
+        <v>-1.0225</v>
       </c>
       <c r="G189" t="n">
-        <v>-1.2246</v>
+        <v>-0.2617</v>
       </c>
       <c r="I189" t="n">
-        <v>116.09</v>
+        <v>-65.97</v>
       </c>
       <c r="J189" t="n">
-        <v>2160.9</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K189" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L189" t="n">
         <v>3</v>
       </c>
       <c r="N189" t="n">
-        <v>0.0283</v>
+        <v>-0.0076</v>
       </c>
       <c r="O189" t="n">
-        <v>53.93</v>
+        <v>40.96</v>
       </c>
       <c r="P189" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5526</v>
       </c>
       <c r="Q189" t="n">
-        <v>0.7548</v>
+        <v>0.0334</v>
       </c>
       <c r="R189" t="n">
-        <v>0.6592</v>
+        <v>0.0631</v>
       </c>
       <c r="S189" t="n">
-        <v>-0.0266</v>
+        <v>-0.0156</v>
       </c>
       <c r="T189" t="n">
-        <v>97.5</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="F190" t="n">
-        <v>0.5694</v>
+        <v>0.9243</v>
       </c>
       <c r="G190" t="n">
-        <v>-1.3423</v>
+        <v>-1.2246</v>
       </c>
       <c r="I190" t="n">
-        <v>54.77</v>
+        <v>116.09</v>
       </c>
       <c r="J190" t="n">
-        <v>1547.7</v>
+        <v>2160.9</v>
       </c>
       <c r="K190" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L190" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N190" t="n">
-        <v>0.0103</v>
+        <v>0.0283</v>
       </c>
       <c r="O190" t="n">
-        <v>51.13</v>
+        <v>53.93</v>
       </c>
       <c r="P190" t="n">
-        <v>0.5968</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="Q190" t="n">
-        <v>0.5364</v>
+        <v>0.7548</v>
       </c>
       <c r="R190" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="S190" t="n">
-        <v>0.0098</v>
+        <v>-0.0266</v>
       </c>
       <c r="T190" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -14302,12 +14302,12 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -14350,21 +14350,21 @@
         <v>0.0098</v>
       </c>
       <c r="T191" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -14373,19 +14373,19 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F192" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G192" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I192" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J192" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K192" t="n">
         <v>5</v>
@@ -14394,39 +14394,39 @@
         <v>1</v>
       </c>
       <c r="N192" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O192" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P192" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q192" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R192" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S192" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T192" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -14435,60 +14435,60 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F193" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G193" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I193" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J193" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K193" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L193" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N193" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O193" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P193" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q193" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R193" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S193" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T193" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -14497,60 +14497,60 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F194" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G194" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I194" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J194" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K194" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L194" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N194" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O194" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P194" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q194" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R194" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S194" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T194" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -14559,60 +14559,60 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="F195" t="n">
-        <v>-0.1044</v>
+        <v>-1.2201</v>
       </c>
       <c r="G195" t="n">
-        <v>-1.6173</v>
+        <v>-0.255</v>
       </c>
       <c r="I195" t="n">
-        <v>-18.65</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J195" t="n">
-        <v>813.5</v>
+        <v>282.4</v>
       </c>
       <c r="K195" t="n">
+        <v>1</v>
+      </c>
+      <c r="L195" t="n">
         <v>3</v>
       </c>
-      <c r="L195" t="n">
-        <v>2</v>
-      </c>
       <c r="N195" t="n">
-        <v>-0.0416</v>
+        <v>-0.0322</v>
       </c>
       <c r="O195" t="n">
-        <v>48.72</v>
+        <v>40.59</v>
       </c>
       <c r="P195" t="n">
-        <v>0.5679999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q195" t="n">
-        <v>0.5653</v>
+        <v>0</v>
       </c>
       <c r="R195" t="n">
-        <v>0.5666</v>
+        <v>0</v>
       </c>
       <c r="S195" t="n">
-        <v>-0.0596</v>
+        <v>0</v>
       </c>
       <c r="T195" t="n">
-        <v>73</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -14621,60 +14621,60 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F196" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G196" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I196" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J196" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K196" t="n">
         <v>3</v>
       </c>
       <c r="L196" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N196" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O196" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P196" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q196" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R196" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S196" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T196" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -14683,51 +14683,51 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F197" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G197" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I197" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J197" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K197" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L197" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N197" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O197" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P197" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q197" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R197" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S197" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T197" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -14736,7 +14736,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -14745,51 +14745,113 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F198" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G198" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I198" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J198" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K198" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L198" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N198" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O198" t="n">
         <v>47.65</v>
       </c>
       <c r="P198" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R198" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S198" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T198" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>41</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E199" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F199" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G199" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I199" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J199" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K199" t="n">
+        <v>4</v>
+      </c>
+      <c r="L199" t="n">
+        <v>2</v>
+      </c>
+      <c r="N199" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O199" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P199" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q198" t="n">
+      <c r="Q199" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R198" t="n">
+      <c r="R199" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S198" t="n">
+      <c r="S199" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T198" t="n">
+      <c r="T199" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T198"/>
-  <conditionalFormatting sqref="E2:E198">
+  <autoFilter ref="A1:T199"/>
+  <conditionalFormatting sqref="E2:E199">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -14811,7 +14873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K198"/>
+  <dimension ref="A1:K199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -20991,44 +21053,44 @@
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>23</v>
+        <v>198</v>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>-1.1119</v>
+        <v>-1.096</v>
       </c>
       <c r="D167" t="n">
         <v>1000</v>
       </c>
       <c r="E167" t="n">
-        <v>1045.3</v>
+        <v>937.6</v>
       </c>
       <c r="F167" t="n">
-        <v>853.06933</v>
+        <v>988.60544</v>
       </c>
       <c r="G167" t="n">
-        <v>732.018792073</v>
+        <v>1037.343688192</v>
       </c>
       <c r="H167" t="n">
-        <v>707.34975878014</v>
+        <v>1001.555330949376</v>
       </c>
       <c r="I167" t="n">
-        <v>660.5939397247727</v>
+        <v>800.6433315609312</v>
       </c>
       <c r="J167" t="n">
-        <v>432.6229711257536</v>
+        <v>716.9761034128138</v>
       </c>
       <c r="K167" t="n">
-        <v>377.4635423072201</v>
+        <v>785.3039260680549</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B168" t="inlineStr">
         <is>
@@ -21036,36 +21098,36 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D168" t="n">
         <v>1000</v>
       </c>
       <c r="E168" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F168" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G168" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H168" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I168" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J168" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K168" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>177</v>
+        <v>87</v>
       </c>
       <c r="B169" t="inlineStr">
         <is>
@@ -21073,184 +21135,184 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>-1.1172</v>
+        <v>-1.1144</v>
       </c>
       <c r="D169" t="n">
         <v>1000</v>
       </c>
       <c r="E169" t="n">
-        <v>1207.8</v>
+        <v>759.5</v>
       </c>
       <c r="F169" t="n">
-        <v>1063.22634</v>
+        <v>825.34865</v>
       </c>
       <c r="G169" t="n">
-        <v>1012.829411484</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H169" t="n">
-        <v>978.899626199286</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I169" t="n">
-        <v>1221.373063608849</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J169" t="n">
-        <v>1413.861458433604</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K169" t="n">
-        <v>880.1287578749184</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>51</v>
+        <v>177</v>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>-1.1484</v>
+        <v>-1.1172</v>
       </c>
       <c r="D170" t="n">
         <v>1000</v>
       </c>
       <c r="E170" t="n">
-        <v>953.5</v>
+        <v>1207.8</v>
       </c>
       <c r="F170" t="n">
-        <v>734.5763999999999</v>
+        <v>1063.22634</v>
       </c>
       <c r="G170" t="n">
-        <v>658.4742849599999</v>
+        <v>1012.829411484</v>
       </c>
       <c r="H170" t="n">
-        <v>766.3323728364478</v>
+        <v>978.899626199286</v>
       </c>
       <c r="I170" t="n">
-        <v>828.0987620870656</v>
+        <v>1221.373063608849</v>
       </c>
       <c r="J170" t="n">
-        <v>590.5172272442865</v>
+        <v>1413.861458433604</v>
       </c>
       <c r="K170" t="n">
-        <v>485.3461090720791</v>
+        <v>880.1287578749184</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D171" t="n">
         <v>1000</v>
       </c>
       <c r="E171" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F171" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G171" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H171" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I171" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J171" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K171" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D172" t="n">
         <v>1000</v>
       </c>
       <c r="E172" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F172" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G172" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H172" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I172" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J172" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K172" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D173" t="n">
         <v>1000</v>
       </c>
       <c r="E173" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F173" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G173" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H173" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I173" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J173" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K173" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B174" t="inlineStr">
         <is>
@@ -21258,36 +21320,36 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D174" t="n">
         <v>1000</v>
       </c>
       <c r="E174" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F174" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G174" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H174" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I174" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J174" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K174" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B175" t="inlineStr">
         <is>
@@ -21295,221 +21357,221 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D175" t="n">
         <v>1000</v>
       </c>
       <c r="E175" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F175" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G175" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H175" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I175" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J175" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K175" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D176" t="n">
         <v>1000</v>
       </c>
       <c r="E176" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F176" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G176" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H176" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I176" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J176" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K176" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D177" t="n">
         <v>1000</v>
       </c>
       <c r="E177" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F177" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G177" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H177" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I177" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J177" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K177" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D178" t="n">
         <v>1000</v>
       </c>
       <c r="E178" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F178" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G178" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H178" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I178" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J178" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K178" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="D179" t="n">
         <v>1000</v>
       </c>
       <c r="E179" t="n">
-        <v>999.6</v>
+        <v>942</v>
       </c>
       <c r="F179" t="n">
-        <v>1076.66916</v>
+        <v>730.2384</v>
       </c>
       <c r="G179" t="n">
-        <v>1127.918612016</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H179" t="n">
-        <v>1009.261574031917</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I179" t="n">
-        <v>837.9898849187007</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J179" t="n">
-        <v>1032.403538219839</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K179" t="n">
-        <v>1101.161613865281</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="D180" t="n">
         <v>1000</v>
       </c>
       <c r="E180" t="n">
-        <v>1045.3</v>
+        <v>999.6</v>
       </c>
       <c r="F180" t="n">
-        <v>853.06933</v>
+        <v>1076.66916</v>
       </c>
       <c r="G180" t="n">
-        <v>749.933248003</v>
+        <v>1127.918612016</v>
       </c>
       <c r="H180" t="n">
-        <v>740.3341024285616</v>
+        <v>1009.261574031917</v>
       </c>
       <c r="I180" t="n">
-        <v>691.1759180273051</v>
+        <v>837.9898849187007</v>
       </c>
       <c r="J180" t="n">
-        <v>482.7172611502699</v>
+        <v>1032.403538219839</v>
       </c>
       <c r="K180" t="n">
-        <v>325.0618036585918</v>
+        <v>1101.161613865281</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
@@ -21546,118 +21608,118 @@
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D182" t="n">
         <v>1000</v>
       </c>
       <c r="E182" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F182" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G182" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H182" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I182" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J182" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K182" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="D183" t="n">
         <v>1000</v>
       </c>
       <c r="E183" t="n">
-        <v>1236.4</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F183" t="n">
-        <v>1500.74232</v>
+        <v>692.62656</v>
       </c>
       <c r="G183" t="n">
-        <v>1734.708047688</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H183" t="n">
-        <v>1677.809623723833</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I183" t="n">
-        <v>1544.088196713044</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J183" t="n">
-        <v>1750.069562154564</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K183" t="n">
-        <v>1412.131129702517</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D184" t="n">
         <v>1000</v>
       </c>
       <c r="E184" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F184" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G184" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H184" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I184" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J184" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K184" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
@@ -21665,36 +21727,36 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D185" t="n">
         <v>1000</v>
       </c>
       <c r="E185" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F185" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G185" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H185" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I185" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J185" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K185" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
@@ -21702,36 +21764,36 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D186" t="n">
         <v>1000</v>
       </c>
       <c r="E186" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F186" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G186" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H186" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I186" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J186" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K186" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
@@ -21739,147 +21801,147 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D187" t="n">
         <v>1000</v>
       </c>
       <c r="E187" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F187" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G187" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H187" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I187" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J187" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K187" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D188" t="n">
         <v>1000</v>
       </c>
       <c r="E188" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F188" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G188" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H188" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I188" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J188" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K188" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="D189" t="n">
         <v>1000</v>
       </c>
       <c r="E189" t="n">
-        <v>1127.9</v>
+        <v>1141.5</v>
       </c>
       <c r="F189" t="n">
-        <v>1108.7257</v>
+        <v>884.8908</v>
       </c>
       <c r="G189" t="n">
-        <v>1251.64044273</v>
+        <v>789.49957176</v>
       </c>
       <c r="H189" t="n">
-        <v>1235.619445063056</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I189" t="n">
-        <v>1202.010596157341</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J189" t="n">
-        <v>1559.849150633381</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K189" t="n">
-        <v>2161.015013287486</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="D190" t="n">
         <v>1000</v>
       </c>
       <c r="E190" t="n">
-        <v>1342</v>
+        <v>1127.9</v>
       </c>
       <c r="F190" t="n">
-        <v>1365.6192</v>
+        <v>1108.7257</v>
       </c>
       <c r="G190" t="n">
-        <v>1401.67154688</v>
+        <v>1251.64044273</v>
       </c>
       <c r="H190" t="n">
-        <v>1356.1172216064</v>
+        <v>1235.619445063056</v>
       </c>
       <c r="I190" t="n">
-        <v>1614.321940600259</v>
+        <v>1202.010596157341</v>
       </c>
       <c r="J190" t="n">
-        <v>1682.93062307577</v>
+        <v>1559.849150633381</v>
       </c>
       <c r="K190" t="n">
-        <v>1547.623000980478</v>
+        <v>2161.015013287486</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -21916,229 +21978,229 @@
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D192" t="n">
         <v>1000</v>
       </c>
       <c r="E192" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F192" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G192" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H192" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I192" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J192" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K192" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D193" t="n">
         <v>1000</v>
       </c>
       <c r="E193" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F193" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G193" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H193" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I193" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J193" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K193" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D194" t="n">
         <v>1000</v>
       </c>
       <c r="E194" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F194" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G194" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H194" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I194" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J194" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K194" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="D195" t="n">
         <v>1000</v>
       </c>
       <c r="E195" t="n">
-        <v>1222.6</v>
+        <v>942</v>
       </c>
       <c r="F195" t="n">
-        <v>1122.46906</v>
+        <v>730.2384</v>
       </c>
       <c r="G195" t="n">
-        <v>1222.481053246</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H195" t="n">
-        <v>1198.520424602378</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I195" t="n">
-        <v>1133.440765546469</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J195" t="n">
-        <v>1142.73497982395</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K195" t="n">
-        <v>813.6273056346525</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D196" t="n">
         <v>1000</v>
       </c>
       <c r="E196" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F196" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G196" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H196" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I196" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J196" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K196" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D197" t="n">
         <v>1000</v>
       </c>
       <c r="E197" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F197" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G197" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H197" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I197" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J197" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K197" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -22146,30 +22208,67 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D198" t="n">
         <v>1000</v>
       </c>
       <c r="E198" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F198" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G198" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H198" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I198" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J198" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K198" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>41</v>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D199" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E199" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F198" t="n">
+      <c r="F199" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G198" t="n">
+      <c r="G199" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H198" t="n">
+      <c r="H199" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I198" t="n">
+      <c r="I199" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J198" t="n">
+      <c r="J199" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K198" t="n">
+      <c r="K199" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 207 CatBoost slowest-lr -1.10 (F2 RECORD +3.89 but val crash); exp 208 depth=3
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$207</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$208</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>209</row>
+      <row>210</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T207"/>
+  <dimension ref="A1:T208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -13375,16 +13375,16 @@
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>23</v>
+        <v>207</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
+          <t>CatBoost lr=0.005 n_est=2000 (slowest-lr untested) - one knob from exp 98 lr=0.02; Friedma</t>
         </is>
       </c>
       <c r="D176" t="inlineStr">
@@ -13393,51 +13393,51 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>-1.1119</v>
+        <v>-1.1003</v>
       </c>
       <c r="F176" t="n">
-        <v>-0.5057</v>
+        <v>0.6796</v>
       </c>
       <c r="G176" t="n">
-        <v>-0.5119</v>
+        <v>-0.9003</v>
       </c>
       <c r="I176" t="n">
-        <v>-62.25</v>
+        <v>71.94</v>
       </c>
       <c r="J176" t="n">
-        <v>377.4999999999999</v>
+        <v>1719.4</v>
       </c>
       <c r="K176" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L176" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N176" t="n">
-        <v>0.0032</v>
+        <v>0.0131</v>
       </c>
       <c r="O176" t="n">
-        <v>44.56</v>
+        <v>49.62</v>
       </c>
       <c r="P176" t="n">
-        <v>0.6421</v>
+        <v>0.5967</v>
       </c>
       <c r="Q176" t="n">
-        <v>0.0756</v>
+        <v>0.4636</v>
       </c>
       <c r="R176" t="n">
-        <v>0.1353</v>
+        <v>0.5218</v>
       </c>
       <c r="S176" t="n">
-        <v>0.0379</v>
+        <v>0.0083</v>
       </c>
       <c r="T176" t="n">
-        <v>53.3</v>
+        <v>2587.6</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -13446,7 +13446,7 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
+          <t>LSTM @ FX-Exp35 HPs seed=7 — 4th LSTM seed (after 42=+0.83, 0=+0.44, 99=+0.47). LSTM has l</t>
         </is>
       </c>
       <c r="D177" t="inlineStr">
@@ -13455,51 +13455,51 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="F177" t="n">
-        <v>-0.6143999999999999</v>
+        <v>-0.5057</v>
       </c>
       <c r="G177" t="n">
-        <v>-0.0276</v>
+        <v>-0.5119</v>
       </c>
       <c r="I177" t="n">
-        <v>-67.98</v>
+        <v>-62.25</v>
       </c>
       <c r="J177" t="n">
-        <v>320.1999999999999</v>
+        <v>377.4999999999999</v>
       </c>
       <c r="K177" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L177" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N177" t="n">
-        <v>-0.0254</v>
+        <v>0.0032</v>
       </c>
       <c r="O177" t="n">
-        <v>44.42</v>
+        <v>44.56</v>
       </c>
       <c r="P177" t="n">
-        <v>0.5676</v>
+        <v>0.6421</v>
       </c>
       <c r="Q177" t="n">
-        <v>0.1301</v>
+        <v>0.0756</v>
       </c>
       <c r="R177" t="n">
-        <v>0.2117</v>
+        <v>0.1353</v>
       </c>
       <c r="S177" t="n">
-        <v>-0.0037</v>
+        <v>0.0379</v>
       </c>
       <c r="T177" t="n">
-        <v>36.8</v>
+        <v>53.3</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>177</v>
+        <v>87</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -13508,7 +13508,7 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>LSTM lr=2e-3 (Smith 2017 highest-leverage axis untested) - one knob from exp 74 lr=1e-3</t>
+          <t>LSTM @ exp 71 1-layer hd=0.15 (up from 0.1) - Srivastava 2014 mild reg final cheap-tier sl</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
@@ -13517,60 +13517,60 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>-1.1172</v>
+        <v>-1.1144</v>
       </c>
       <c r="F178" t="n">
-        <v>0.0506</v>
+        <v>-0.6143999999999999</v>
       </c>
       <c r="G178" t="n">
-        <v>-0.7171999999999999</v>
+        <v>-0.0276</v>
       </c>
       <c r="I178" t="n">
-        <v>-11.99</v>
+        <v>-67.98</v>
       </c>
       <c r="J178" t="n">
-        <v>880.1</v>
+        <v>320.1999999999999</v>
       </c>
       <c r="K178" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L178" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N178" t="n">
-        <v>0.0322</v>
+        <v>-0.0254</v>
       </c>
       <c r="O178" t="n">
-        <v>46.2</v>
+        <v>44.42</v>
       </c>
       <c r="P178" t="n">
-        <v>0.5585</v>
+        <v>0.5676</v>
       </c>
       <c r="Q178" t="n">
-        <v>0.29</v>
+        <v>0.1301</v>
       </c>
       <c r="R178" t="n">
-        <v>0.3817</v>
+        <v>0.2117</v>
       </c>
       <c r="S178" t="n">
-        <v>-0.0182</v>
+        <v>-0.0037</v>
       </c>
       <c r="T178" t="n">
-        <v>52.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>51</v>
+        <v>177</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
+          <t>LSTM lr=2e-3 (Smith 2017 highest-leverage axis untested) - one knob from exp 74 lr=1e-3</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
@@ -13579,60 +13579,60 @@
         </is>
       </c>
       <c r="E179" t="n">
-        <v>-1.1484</v>
+        <v>-1.1172</v>
       </c>
       <c r="F179" t="n">
-        <v>-0.6484</v>
+        <v>0.0506</v>
       </c>
       <c r="G179" t="n">
-        <v>1.8519</v>
+        <v>-0.7171999999999999</v>
       </c>
       <c r="I179" t="n">
-        <v>-51.47</v>
+        <v>-11.99</v>
       </c>
       <c r="J179" t="n">
-        <v>485.3000000000001</v>
+        <v>880.1</v>
       </c>
       <c r="K179" t="n">
+        <v>3</v>
+      </c>
+      <c r="L179" t="n">
         <v>2</v>
       </c>
-      <c r="L179" t="n">
-        <v>5</v>
-      </c>
       <c r="N179" t="n">
-        <v>0.008200000000000001</v>
+        <v>0.0322</v>
       </c>
       <c r="O179" t="n">
-        <v>43.33</v>
+        <v>46.2</v>
       </c>
       <c r="P179" t="n">
-        <v>0.5736</v>
+        <v>0.5585</v>
       </c>
       <c r="Q179" t="n">
-        <v>0.1799</v>
+        <v>0.29</v>
       </c>
       <c r="R179" t="n">
-        <v>0.2739</v>
+        <v>0.3817</v>
       </c>
       <c r="S179" t="n">
-        <v>-0.0183</v>
+        <v>-0.0182</v>
       </c>
       <c r="T179" t="n">
-        <v>823.8</v>
+        <v>52.2</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
+          <t>dMamba @ exp 48 expand=2 seed=99 - 4th seed for full multi-seed median lock</t>
         </is>
       </c>
       <c r="D180" t="inlineStr">
@@ -13641,60 +13641,60 @@
         </is>
       </c>
       <c r="E180" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="F180" t="n">
-        <v>0.2695</v>
+        <v>-0.6484</v>
       </c>
       <c r="G180" t="n">
-        <v>-0.9486</v>
+        <v>1.8519</v>
       </c>
       <c r="I180" t="n">
-        <v>16.22</v>
+        <v>-51.47</v>
       </c>
       <c r="J180" t="n">
-        <v>1162.2</v>
+        <v>485.3000000000001</v>
       </c>
       <c r="K180" t="n">
+        <v>2</v>
+      </c>
+      <c r="L180" t="n">
         <v>5</v>
       </c>
-      <c r="L180" t="n">
-        <v>2</v>
-      </c>
       <c r="N180" t="n">
-        <v>0.0004</v>
+        <v>0.008200000000000001</v>
       </c>
       <c r="O180" t="n">
-        <v>48.5</v>
+        <v>43.33</v>
       </c>
       <c r="P180" t="n">
-        <v>0.5835</v>
+        <v>0.5736</v>
       </c>
       <c r="Q180" t="n">
-        <v>0.4589</v>
+        <v>0.1799</v>
       </c>
       <c r="R180" t="n">
-        <v>0.5137</v>
+        <v>0.2739</v>
       </c>
       <c r="S180" t="n">
-        <v>-0.0167</v>
+        <v>-0.0183</v>
       </c>
       <c r="T180" t="n">
-        <v>106.4</v>
+        <v>823.8</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
+          <t>XGBoost @ exp 42 n_est=150 (up from 100) - capacity hill-climb at lr=0.03</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
@@ -13703,60 +13703,60 @@
         </is>
       </c>
       <c r="E181" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="F181" t="n">
-        <v>0.1386</v>
+        <v>0.2695</v>
       </c>
       <c r="G181" t="n">
-        <v>-0.8962</v>
+        <v>-0.9486</v>
       </c>
       <c r="I181" t="n">
-        <v>0.4</v>
+        <v>16.22</v>
       </c>
       <c r="J181" t="n">
-        <v>1004</v>
+        <v>1162.2</v>
       </c>
       <c r="K181" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L181" t="n">
         <v>2</v>
       </c>
       <c r="N181" t="n">
-        <v>0.0103</v>
+        <v>0.0004</v>
       </c>
       <c r="O181" t="n">
-        <v>48.54</v>
+        <v>48.5</v>
       </c>
       <c r="P181" t="n">
-        <v>0.5577</v>
+        <v>0.5835</v>
       </c>
       <c r="Q181" t="n">
-        <v>0.4907</v>
+        <v>0.4589</v>
       </c>
       <c r="R181" t="n">
-        <v>0.5221</v>
+        <v>0.5137</v>
       </c>
       <c r="S181" t="n">
-        <v>-0.0297</v>
+        <v>-0.0167</v>
       </c>
       <c r="T181" t="n">
-        <v>36.8</v>
+        <v>106.4</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
+          <t>MLP @ FX-Exp32 HPs seed=99 — 4th seed for MLP variance estimate</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
@@ -13765,51 +13765,51 @@
         </is>
       </c>
       <c r="E182" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="F182" t="n">
-        <v>0.8726</v>
+        <v>0.1386</v>
       </c>
       <c r="G182" t="n">
-        <v>-1.0111</v>
+        <v>-0.8962</v>
       </c>
       <c r="I182" t="n">
-        <v>106.6</v>
+        <v>0.4</v>
       </c>
       <c r="J182" t="n">
-        <v>2066</v>
+        <v>1004</v>
       </c>
       <c r="K182" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L182" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N182" t="n">
-        <v>0.0297</v>
+        <v>0.0103</v>
       </c>
       <c r="O182" t="n">
-        <v>52.07</v>
+        <v>48.54</v>
       </c>
       <c r="P182" t="n">
-        <v>0.6041</v>
+        <v>0.5577</v>
       </c>
       <c r="Q182" t="n">
-        <v>0.5554</v>
+        <v>0.4907</v>
       </c>
       <c r="R182" t="n">
-        <v>0.5787</v>
+        <v>0.5221</v>
       </c>
       <c r="S182" t="n">
-        <v>0.0263</v>
+        <v>-0.0297</v>
       </c>
       <c r="T182" t="n">
-        <v>78.2</v>
+        <v>36.8</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -13818,7 +13818,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
+          <t>XGBoost @ exp 44 CHAMP seed=0 - multi-seed FX-paper section 6.4 seed-determinism check</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -13827,51 +13827,51 @@
         </is>
       </c>
       <c r="E183" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="F183" t="n">
-        <v>0.9873</v>
+        <v>0.8726</v>
       </c>
       <c r="G183" t="n">
-        <v>-1.2319</v>
+        <v>-1.0111</v>
       </c>
       <c r="I183" t="n">
-        <v>130.41</v>
+        <v>106.6</v>
       </c>
       <c r="J183" t="n">
-        <v>2304.1</v>
+        <v>2066</v>
       </c>
       <c r="K183" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="L183" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N183" t="n">
-        <v>0.0242</v>
+        <v>0.0297</v>
       </c>
       <c r="O183" t="n">
-        <v>53.2</v>
+        <v>52.07</v>
       </c>
       <c r="P183" t="n">
-        <v>0.6051</v>
+        <v>0.6041</v>
       </c>
       <c r="Q183" t="n">
-        <v>0.606</v>
+        <v>0.5554</v>
       </c>
       <c r="R183" t="n">
-        <v>0.6055</v>
+        <v>0.5787</v>
       </c>
       <c r="S183" t="n">
-        <v>0.0313</v>
+        <v>0.0263</v>
       </c>
       <c r="T183" t="n">
-        <v>54.5</v>
+        <v>78.2</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -13880,7 +13880,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>XGBoost @ exp 44 max_depth=3 (down from 4) - Friedman 2001 shallow-boosting</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -13889,60 +13889,60 @@
         </is>
       </c>
       <c r="E184" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="F184" t="n">
-        <v>0.0349</v>
+        <v>0.9873</v>
       </c>
       <c r="G184" t="n">
-        <v>-1.035</v>
+        <v>-1.2319</v>
       </c>
       <c r="I184" t="n">
-        <v>-7.12</v>
+        <v>130.41</v>
       </c>
       <c r="J184" t="n">
-        <v>928.8</v>
+        <v>2304.1</v>
       </c>
       <c r="K184" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="L184" t="n">
         <v>2</v>
       </c>
       <c r="N184" t="n">
-        <v>-0.0034</v>
+        <v>0.0242</v>
       </c>
       <c r="O184" t="n">
-        <v>47.74</v>
+        <v>53.2</v>
       </c>
       <c r="P184" t="n">
-        <v>0.577</v>
+        <v>0.6051</v>
       </c>
       <c r="Q184" t="n">
-        <v>0.4446</v>
+        <v>0.606</v>
       </c>
       <c r="R184" t="n">
-        <v>0.5022</v>
+        <v>0.6055</v>
       </c>
       <c r="S184" t="n">
-        <v>-0.0286</v>
+        <v>0.0313</v>
       </c>
       <c r="T184" t="n">
-        <v>79</v>
+        <v>54.5</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D185" t="inlineStr">
@@ -13951,60 +13951,60 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F185" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G185" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I185" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J185" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K185" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L185" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N185" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O185" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P185" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q185" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R185" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S185" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T185" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
@@ -14013,60 +14013,60 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F186" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G186" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I186" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J186" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K186" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L186" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N186" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O186" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P186" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q186" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R186" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S186" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T186" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
@@ -14075,60 +14075,60 @@
         </is>
       </c>
       <c r="E187" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F187" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G187" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I187" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J187" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K187" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L187" t="n">
         <v>3</v>
       </c>
       <c r="N187" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O187" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P187" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q187" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R187" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S187" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T187" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
@@ -14137,60 +14137,60 @@
         </is>
       </c>
       <c r="E188" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="F188" t="n">
-        <v>0.2144</v>
+        <v>-0.8189</v>
       </c>
       <c r="G188" t="n">
-        <v>-1.2304</v>
+        <v>1.1456</v>
       </c>
       <c r="I188" t="n">
-        <v>10.12</v>
+        <v>-58.71</v>
       </c>
       <c r="J188" t="n">
-        <v>1101.2</v>
+        <v>412.9</v>
       </c>
       <c r="K188" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L188" t="n">
         <v>3</v>
       </c>
       <c r="N188" t="n">
-        <v>0.0027</v>
+        <v>0.0089</v>
       </c>
       <c r="O188" t="n">
-        <v>53.55</v>
+        <v>41.44</v>
       </c>
       <c r="P188" t="n">
-        <v>0.5858</v>
+        <v>0.68</v>
       </c>
       <c r="Q188" t="n">
-        <v>0.7341</v>
+        <v>0.0271</v>
       </c>
       <c r="R188" t="n">
-        <v>0.6516</v>
+        <v>0.0521</v>
       </c>
       <c r="S188" t="n">
-        <v>-0.0231</v>
+        <v>0.0277</v>
       </c>
       <c r="T188" t="n">
-        <v>69.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -14199,51 +14199,51 @@
         </is>
       </c>
       <c r="E189" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="F189" t="n">
-        <v>-0.6042</v>
+        <v>0.2144</v>
       </c>
       <c r="G189" t="n">
-        <v>-0.8305</v>
+        <v>-1.2304</v>
       </c>
       <c r="I189" t="n">
-        <v>-67.48999999999999</v>
+        <v>10.12</v>
       </c>
       <c r="J189" t="n">
-        <v>325.1000000000001</v>
+        <v>1101.2</v>
       </c>
       <c r="K189" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L189" t="n">
         <v>3</v>
       </c>
       <c r="N189" t="n">
-        <v>0.0111</v>
+        <v>0.0027</v>
       </c>
       <c r="O189" t="n">
-        <v>42.64</v>
+        <v>53.55</v>
       </c>
       <c r="P189" t="n">
-        <v>0</v>
+        <v>0.5858</v>
       </c>
       <c r="Q189" t="n">
-        <v>0</v>
+        <v>0.7341</v>
       </c>
       <c r="R189" t="n">
-        <v>0</v>
+        <v>0.6516</v>
       </c>
       <c r="S189" t="n">
-        <v>0</v>
+        <v>-0.0231</v>
       </c>
       <c r="T189" t="n">
-        <v>82.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -14252,7 +14252,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -14282,7 +14282,7 @@
         <v>3</v>
       </c>
       <c r="N190" t="n">
-        <v>0.032</v>
+        <v>0.0111</v>
       </c>
       <c r="O190" t="n">
         <v>42.64</v>
@@ -14300,21 +14300,21 @@
         <v>0</v>
       </c>
       <c r="T190" t="n">
-        <v>62.3</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -14323,60 +14323,60 @@
         </is>
       </c>
       <c r="E191" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F191" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G191" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I191" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J191" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K191" t="n">
         <v>1</v>
       </c>
       <c r="L191" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N191" t="n">
-        <v>0.0284</v>
+        <v>0.032</v>
       </c>
       <c r="O191" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P191" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q191" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R191" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S191" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T191" t="n">
-        <v>79.8</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -14385,60 +14385,60 @@
         </is>
       </c>
       <c r="E192" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="F192" t="n">
-        <v>0.4732</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G192" t="n">
-        <v>-1.1536</v>
+        <v>-0.8347</v>
       </c>
       <c r="I192" t="n">
-        <v>41.21</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J192" t="n">
-        <v>1412.1</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K192" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L192" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N192" t="n">
-        <v>0.0231</v>
+        <v>0.0284</v>
       </c>
       <c r="O192" t="n">
-        <v>48.31</v>
+        <v>44.07</v>
       </c>
       <c r="P192" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.5588</v>
       </c>
       <c r="Q192" t="n">
-        <v>0.3418</v>
+        <v>0.1177</v>
       </c>
       <c r="R192" t="n">
-        <v>0.4395</v>
+        <v>0.1945</v>
       </c>
       <c r="S192" t="n">
-        <v>0.0329</v>
+        <v>-0.0101</v>
       </c>
       <c r="T192" t="n">
-        <v>1311.2</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -14447,39 +14447,51 @@
         </is>
       </c>
       <c r="E193" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F193" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G193" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I193" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J193" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K193" t="n">
         <v>4</v>
       </c>
       <c r="L193" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N193" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O193" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P193" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R193" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S193" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T193" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -14488,7 +14500,7 @@
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
@@ -14497,51 +14509,39 @@
         </is>
       </c>
       <c r="E194" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F194" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G194" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I194" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J194" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K194" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L194" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N194" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O194" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P194" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q194" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R194" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S194" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T194" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -14550,7 +14550,7 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
@@ -14559,51 +14559,51 @@
         </is>
       </c>
       <c r="E195" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F195" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G195" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I195" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J195" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L195" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N195" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O195" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P195" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q195" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R195" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S195" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T195" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -14612,7 +14612,7 @@
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
@@ -14621,60 +14621,60 @@
         </is>
       </c>
       <c r="E196" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F196" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G196" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I196" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J196" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K196" t="n">
         <v>1</v>
       </c>
       <c r="L196" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N196" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O196" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P196" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q196" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R196" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S196" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T196" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D197" t="inlineStr">
@@ -14683,60 +14683,60 @@
         </is>
       </c>
       <c r="E197" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F197" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G197" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I197" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J197" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K197" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L197" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N197" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O197" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P197" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q197" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R197" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S197" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T197" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -14745,113 +14745,113 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="F198" t="n">
-        <v>0.9243</v>
+        <v>-1.0225</v>
       </c>
       <c r="G198" t="n">
-        <v>-1.2246</v>
+        <v>-0.2617</v>
       </c>
       <c r="I198" t="n">
-        <v>116.09</v>
+        <v>-65.97</v>
       </c>
       <c r="J198" t="n">
-        <v>2160.9</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K198" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L198" t="n">
         <v>3</v>
       </c>
       <c r="N198" t="n">
-        <v>0.0283</v>
+        <v>-0.0076</v>
       </c>
       <c r="O198" t="n">
-        <v>53.93</v>
+        <v>40.96</v>
       </c>
       <c r="P198" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5526</v>
       </c>
       <c r="Q198" t="n">
-        <v>0.7548</v>
+        <v>0.0334</v>
       </c>
       <c r="R198" t="n">
-        <v>0.6592</v>
+        <v>0.0631</v>
       </c>
       <c r="S198" t="n">
-        <v>-0.0266</v>
+        <v>-0.0156</v>
       </c>
       <c r="T198" t="n">
-        <v>97.5</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="F199" t="n">
-        <v>0.5694</v>
+        <v>0.9243</v>
       </c>
       <c r="G199" t="n">
-        <v>-1.3423</v>
+        <v>-1.2246</v>
       </c>
       <c r="I199" t="n">
-        <v>54.77</v>
+        <v>116.09</v>
       </c>
       <c r="J199" t="n">
-        <v>1547.7</v>
+        <v>2160.9</v>
       </c>
       <c r="K199" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L199" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N199" t="n">
-        <v>0.0103</v>
+        <v>0.0283</v>
       </c>
       <c r="O199" t="n">
-        <v>51.13</v>
+        <v>53.93</v>
       </c>
       <c r="P199" t="n">
-        <v>0.5968</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="Q199" t="n">
-        <v>0.5364</v>
+        <v>0.7548</v>
       </c>
       <c r="R199" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="S199" t="n">
-        <v>0.0098</v>
+        <v>-0.0266</v>
       </c>
       <c r="T199" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -14860,12 +14860,12 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -14908,21 +14908,21 @@
         <v>0.0098</v>
       </c>
       <c r="T200" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -14931,19 +14931,19 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="F201" t="n">
-        <v>0.4944</v>
+        <v>0.5694</v>
       </c>
       <c r="G201" t="n">
-        <v>-1.5077</v>
+        <v>-1.3423</v>
       </c>
       <c r="I201" t="n">
-        <v>44.06</v>
+        <v>54.77</v>
       </c>
       <c r="J201" t="n">
-        <v>1440.6</v>
+        <v>1547.7</v>
       </c>
       <c r="K201" t="n">
         <v>5</v>
@@ -14952,39 +14952,39 @@
         <v>1</v>
       </c>
       <c r="N201" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="O201" t="n">
-        <v>52.26</v>
+        <v>51.13</v>
       </c>
       <c r="P201" t="n">
-        <v>0.5959</v>
+        <v>0.5968</v>
       </c>
       <c r="Q201" t="n">
-        <v>0.6044</v>
+        <v>0.5364</v>
       </c>
       <c r="R201" t="n">
-        <v>0.6002</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S201" t="n">
-        <v>0.0091</v>
+        <v>0.0098</v>
       </c>
       <c r="T201" t="n">
-        <v>1076.7</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -14993,60 +14993,60 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F202" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G202" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I202" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J202" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K202" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L202" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N202" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O202" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P202" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q202" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R202" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S202" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T202" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -15055,60 +15055,60 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F203" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G203" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I203" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J203" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K203" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L203" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N203" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O203" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P203" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q203" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R203" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S203" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T203" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -15117,60 +15117,60 @@
         </is>
       </c>
       <c r="E204" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="F204" t="n">
-        <v>-0.1044</v>
+        <v>-1.2201</v>
       </c>
       <c r="G204" t="n">
-        <v>-1.6173</v>
+        <v>-0.255</v>
       </c>
       <c r="I204" t="n">
-        <v>-18.65</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J204" t="n">
-        <v>813.5</v>
+        <v>282.4</v>
       </c>
       <c r="K204" t="n">
+        <v>1</v>
+      </c>
+      <c r="L204" t="n">
         <v>3</v>
       </c>
-      <c r="L204" t="n">
-        <v>2</v>
-      </c>
       <c r="N204" t="n">
-        <v>-0.0416</v>
+        <v>-0.0322</v>
       </c>
       <c r="O204" t="n">
-        <v>48.72</v>
+        <v>40.59</v>
       </c>
       <c r="P204" t="n">
-        <v>0.5679999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q204" t="n">
-        <v>0.5653</v>
+        <v>0</v>
       </c>
       <c r="R204" t="n">
-        <v>0.5666</v>
+        <v>0</v>
       </c>
       <c r="S204" t="n">
-        <v>-0.0596</v>
+        <v>0</v>
       </c>
       <c r="T204" t="n">
-        <v>73</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -15179,60 +15179,60 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F205" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G205" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I205" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J205" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K205" t="n">
         <v>3</v>
       </c>
       <c r="L205" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N205" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O205" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P205" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q205" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R205" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S205" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T205" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -15241,51 +15241,51 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F206" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G206" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I206" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J206" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K206" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L206" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N206" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O206" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P206" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q206" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R206" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S206" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T206" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -15294,7 +15294,7 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -15303,51 +15303,113 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F207" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G207" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I207" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J207" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K207" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L207" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N207" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O207" t="n">
         <v>47.65</v>
       </c>
       <c r="P207" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q207" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R207" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S207" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T207" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>41</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E208" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F208" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G208" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I208" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J208" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K208" t="n">
+        <v>4</v>
+      </c>
+      <c r="L208" t="n">
+        <v>2</v>
+      </c>
+      <c r="N208" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O208" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P208" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q207" t="n">
+      <c r="Q208" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R207" t="n">
+      <c r="R208" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S207" t="n">
+      <c r="S208" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T207" t="n">
+      <c r="T208" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T207"/>
-  <conditionalFormatting sqref="E2:E207">
+  <autoFilter ref="A1:T208"/>
+  <conditionalFormatting sqref="E2:E208">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -15369,7 +15431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K207"/>
+  <dimension ref="A1:K208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -21882,44 +21944,44 @@
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>23</v>
+        <v>207</v>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>-1.1119</v>
+        <v>-1.1003</v>
       </c>
       <c r="D176" t="n">
         <v>1000</v>
       </c>
       <c r="E176" t="n">
-        <v>1045.3</v>
+        <v>957.5</v>
       </c>
       <c r="F176" t="n">
-        <v>853.06933</v>
+        <v>1171.0225</v>
       </c>
       <c r="G176" t="n">
-        <v>732.018792073</v>
+        <v>1328.1737195</v>
       </c>
       <c r="H176" t="n">
-        <v>707.34975878014</v>
+        <v>1179.01981080015</v>
       </c>
       <c r="I176" t="n">
-        <v>660.5939397247727</v>
+        <v>1177.95869297043</v>
       </c>
       <c r="J176" t="n">
-        <v>432.6229711257536</v>
+        <v>1714.283285879866</v>
       </c>
       <c r="K176" t="n">
-        <v>377.4635423072201</v>
+        <v>1719.254707408918</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="B177" t="inlineStr">
         <is>
@@ -21927,36 +21989,36 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>-1.1144</v>
+        <v>-1.1119</v>
       </c>
       <c r="D177" t="n">
         <v>1000</v>
       </c>
       <c r="E177" t="n">
-        <v>759.5</v>
+        <v>1045.3</v>
       </c>
       <c r="F177" t="n">
-        <v>825.34865</v>
+        <v>853.06933</v>
       </c>
       <c r="G177" t="n">
-        <v>755.1114798850001</v>
+        <v>732.018792073</v>
       </c>
       <c r="H177" t="n">
-        <v>683.0738447039712</v>
+        <v>707.34975878014</v>
       </c>
       <c r="I177" t="n">
-        <v>624.5344162128408</v>
+        <v>660.5939397247727</v>
       </c>
       <c r="J177" t="n">
-        <v>323.5088275982516</v>
+        <v>432.6229711257536</v>
       </c>
       <c r="K177" t="n">
-        <v>320.2090375567494</v>
+        <v>377.4635423072201</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>177</v>
+        <v>87</v>
       </c>
       <c r="B178" t="inlineStr">
         <is>
@@ -21964,184 +22026,184 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>-1.1172</v>
+        <v>-1.1144</v>
       </c>
       <c r="D178" t="n">
         <v>1000</v>
       </c>
       <c r="E178" t="n">
-        <v>1207.8</v>
+        <v>759.5</v>
       </c>
       <c r="F178" t="n">
-        <v>1063.22634</v>
+        <v>825.34865</v>
       </c>
       <c r="G178" t="n">
-        <v>1012.829411484</v>
+        <v>755.1114798850001</v>
       </c>
       <c r="H178" t="n">
-        <v>978.899626199286</v>
+        <v>683.0738447039712</v>
       </c>
       <c r="I178" t="n">
-        <v>1221.373063608849</v>
+        <v>624.5344162128408</v>
       </c>
       <c r="J178" t="n">
-        <v>1413.861458433604</v>
+        <v>323.5088275982516</v>
       </c>
       <c r="K178" t="n">
-        <v>880.1287578749184</v>
+        <v>320.2090375567494</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>51</v>
+        <v>177</v>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>-1.1484</v>
+        <v>-1.1172</v>
       </c>
       <c r="D179" t="n">
         <v>1000</v>
       </c>
       <c r="E179" t="n">
-        <v>953.5</v>
+        <v>1207.8</v>
       </c>
       <c r="F179" t="n">
-        <v>734.5763999999999</v>
+        <v>1063.22634</v>
       </c>
       <c r="G179" t="n">
-        <v>658.4742849599999</v>
+        <v>1012.829411484</v>
       </c>
       <c r="H179" t="n">
-        <v>766.3323728364478</v>
+        <v>978.899626199286</v>
       </c>
       <c r="I179" t="n">
-        <v>828.0987620870656</v>
+        <v>1221.373063608849</v>
       </c>
       <c r="J179" t="n">
-        <v>590.5172272442865</v>
+        <v>1413.861458433604</v>
       </c>
       <c r="K179" t="n">
-        <v>485.3461090720791</v>
+        <v>880.1287578749184</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>-1.1486</v>
+        <v>-1.1484</v>
       </c>
       <c r="D180" t="n">
         <v>1000</v>
       </c>
       <c r="E180" t="n">
-        <v>1094.9</v>
+        <v>953.5</v>
       </c>
       <c r="F180" t="n">
-        <v>1249.39039</v>
+        <v>734.5763999999999</v>
       </c>
       <c r="G180" t="n">
-        <v>1330.60076535</v>
+        <v>658.4742849599999</v>
       </c>
       <c r="H180" t="n">
-        <v>1250.897779505535</v>
+        <v>766.3323728364478</v>
       </c>
       <c r="I180" t="n">
-        <v>1391.373600144007</v>
+        <v>828.0987620870656</v>
       </c>
       <c r="J180" t="n">
-        <v>1603.00152472591</v>
+        <v>590.5172272442865</v>
       </c>
       <c r="K180" t="n">
-        <v>1162.176105426285</v>
+        <v>485.3461090720791</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>-1.1962</v>
+        <v>-1.1486</v>
       </c>
       <c r="D181" t="n">
         <v>1000</v>
       </c>
       <c r="E181" t="n">
-        <v>873</v>
+        <v>1094.9</v>
       </c>
       <c r="F181" t="n">
-        <v>774.0018</v>
+        <v>1249.39039</v>
       </c>
       <c r="G181" t="n">
-        <v>902.40869862</v>
+        <v>1330.60076535</v>
       </c>
       <c r="H181" t="n">
-        <v>951.950936174238</v>
+        <v>1250.897779505535</v>
       </c>
       <c r="I181" t="n">
-        <v>908.351583297458</v>
+        <v>1391.373600144007</v>
       </c>
       <c r="J181" t="n">
-        <v>989.5582148442506</v>
+        <v>1603.00152472591</v>
       </c>
       <c r="K181" t="n">
-        <v>1003.807853138008</v>
+        <v>1162.176105426285</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>-1.2111</v>
+        <v>-1.1962</v>
       </c>
       <c r="D182" t="n">
         <v>1000</v>
       </c>
       <c r="E182" t="n">
-        <v>1124.2</v>
+        <v>873</v>
       </c>
       <c r="F182" t="n">
-        <v>1426.38496</v>
+        <v>774.0018</v>
       </c>
       <c r="G182" t="n">
-        <v>1640.200065504</v>
+        <v>902.40869862</v>
       </c>
       <c r="H182" t="n">
-        <v>1832.92357320072</v>
+        <v>951.950936174238</v>
       </c>
       <c r="I182" t="n">
-        <v>1699.303444714387</v>
+        <v>908.351583297458</v>
       </c>
       <c r="J182" t="n">
-        <v>2460.421457601961</v>
+        <v>989.5582148442506</v>
       </c>
       <c r="K182" t="n">
-        <v>2066.015897948367</v>
+        <v>1003.807853138008</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="B183" t="inlineStr">
         <is>
@@ -22149,36 +22211,36 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>-1.2319</v>
+        <v>-1.2111</v>
       </c>
       <c r="D183" t="n">
         <v>1000</v>
       </c>
       <c r="E183" t="n">
-        <v>1201.9</v>
+        <v>1124.2</v>
       </c>
       <c r="F183" t="n">
-        <v>1392.04058</v>
+        <v>1426.38496</v>
       </c>
       <c r="G183" t="n">
-        <v>1555.744552208</v>
+        <v>1640.200065504</v>
       </c>
       <c r="H183" t="n">
-        <v>1557.922594581091</v>
+        <v>1832.92357320072</v>
       </c>
       <c r="I183" t="n">
-        <v>1650.930573477582</v>
+        <v>1699.303444714387</v>
       </c>
       <c r="J183" t="n">
-        <v>2014.465485757346</v>
+        <v>2460.421457601961</v>
       </c>
       <c r="K183" t="n">
-        <v>2303.944176060676</v>
+        <v>2066.015897948367</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B184" t="inlineStr">
         <is>
@@ -22186,221 +22248,221 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>-1.335</v>
+        <v>-1.2319</v>
       </c>
       <c r="D184" t="n">
         <v>1000</v>
       </c>
       <c r="E184" t="n">
-        <v>1200</v>
+        <v>1201.9</v>
       </c>
       <c r="F184" t="n">
-        <v>1259.16</v>
+        <v>1392.04058</v>
       </c>
       <c r="G184" t="n">
-        <v>1343.145972</v>
+        <v>1555.744552208</v>
       </c>
       <c r="H184" t="n">
-        <v>1093.7237649996</v>
+        <v>1557.922594581091</v>
       </c>
       <c r="I184" t="n">
-        <v>1039.36569387912</v>
+        <v>1650.930573477582</v>
       </c>
       <c r="J184" t="n">
-        <v>1048.408175415868</v>
+        <v>2014.465485757346</v>
       </c>
       <c r="K184" t="n">
-        <v>928.8896434184592</v>
+        <v>2303.944176060676</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D185" t="n">
         <v>1000</v>
       </c>
       <c r="E185" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F185" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G185" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H185" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I185" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J185" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K185" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D186" t="n">
         <v>1000</v>
       </c>
       <c r="E186" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F186" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G186" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H186" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I186" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J186" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K186" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D187" t="n">
         <v>1000</v>
       </c>
       <c r="E187" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F187" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G187" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H187" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I187" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J187" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K187" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="D188" t="n">
         <v>1000</v>
       </c>
       <c r="E188" t="n">
-        <v>999.6</v>
+        <v>942</v>
       </c>
       <c r="F188" t="n">
-        <v>1076.66916</v>
+        <v>730.2384</v>
       </c>
       <c r="G188" t="n">
-        <v>1127.918612016</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H188" t="n">
-        <v>1009.261574031917</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I188" t="n">
-        <v>837.9898849187007</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J188" t="n">
-        <v>1032.403538219839</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K188" t="n">
-        <v>1101.161613865281</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="D189" t="n">
         <v>1000</v>
       </c>
       <c r="E189" t="n">
-        <v>1045.3</v>
+        <v>999.6</v>
       </c>
       <c r="F189" t="n">
-        <v>853.06933</v>
+        <v>1076.66916</v>
       </c>
       <c r="G189" t="n">
-        <v>749.933248003</v>
+        <v>1127.918612016</v>
       </c>
       <c r="H189" t="n">
-        <v>740.3341024285616</v>
+        <v>1009.261574031917</v>
       </c>
       <c r="I189" t="n">
-        <v>691.1759180273051</v>
+        <v>837.9898849187007</v>
       </c>
       <c r="J189" t="n">
-        <v>482.7172611502699</v>
+        <v>1032.403538219839</v>
       </c>
       <c r="K189" t="n">
-        <v>325.0618036585918</v>
+        <v>1101.161613865281</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -22437,118 +22499,118 @@
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D191" t="n">
         <v>1000</v>
       </c>
       <c r="E191" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F191" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G191" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H191" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I191" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J191" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K191" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="D192" t="n">
         <v>1000</v>
       </c>
       <c r="E192" t="n">
-        <v>1236.4</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F192" t="n">
-        <v>1500.74232</v>
+        <v>692.62656</v>
       </c>
       <c r="G192" t="n">
-        <v>1734.708047688</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H192" t="n">
-        <v>1677.809623723833</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I192" t="n">
-        <v>1544.088196713044</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J192" t="n">
-        <v>1750.069562154564</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K192" t="n">
-        <v>1412.131129702517</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D193" t="n">
         <v>1000</v>
       </c>
       <c r="E193" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F193" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G193" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H193" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I193" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J193" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K193" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -22556,36 +22618,36 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D194" t="n">
         <v>1000</v>
       </c>
       <c r="E194" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F194" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G194" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H194" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I194" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J194" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K194" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -22593,36 +22655,36 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D195" t="n">
         <v>1000</v>
       </c>
       <c r="E195" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F195" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G195" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H195" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I195" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J195" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K195" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -22630,147 +22692,147 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D196" t="n">
         <v>1000</v>
       </c>
       <c r="E196" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F196" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G196" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H196" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I196" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J196" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K196" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D197" t="n">
         <v>1000</v>
       </c>
       <c r="E197" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F197" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G197" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H197" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I197" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J197" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K197" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="D198" t="n">
         <v>1000</v>
       </c>
       <c r="E198" t="n">
-        <v>1127.9</v>
+        <v>1141.5</v>
       </c>
       <c r="F198" t="n">
-        <v>1108.7257</v>
+        <v>884.8908</v>
       </c>
       <c r="G198" t="n">
-        <v>1251.64044273</v>
+        <v>789.49957176</v>
       </c>
       <c r="H198" t="n">
-        <v>1235.619445063056</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I198" t="n">
-        <v>1202.010596157341</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J198" t="n">
-        <v>1559.849150633381</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K198" t="n">
-        <v>2161.015013287486</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="D199" t="n">
         <v>1000</v>
       </c>
       <c r="E199" t="n">
-        <v>1342</v>
+        <v>1127.9</v>
       </c>
       <c r="F199" t="n">
-        <v>1365.6192</v>
+        <v>1108.7257</v>
       </c>
       <c r="G199" t="n">
-        <v>1401.67154688</v>
+        <v>1251.64044273</v>
       </c>
       <c r="H199" t="n">
-        <v>1356.1172216064</v>
+        <v>1235.619445063056</v>
       </c>
       <c r="I199" t="n">
-        <v>1614.321940600259</v>
+        <v>1202.010596157341</v>
       </c>
       <c r="J199" t="n">
-        <v>1682.93062307577</v>
+        <v>1559.849150633381</v>
       </c>
       <c r="K199" t="n">
-        <v>1547.623000980478</v>
+        <v>2161.015013287486</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -22807,229 +22869,229 @@
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>-1.7077</v>
+        <v>-1.5423</v>
       </c>
       <c r="D201" t="n">
         <v>1000</v>
       </c>
       <c r="E201" t="n">
-        <v>1067.7</v>
+        <v>1342</v>
       </c>
       <c r="F201" t="n">
-        <v>1380.10902</v>
+        <v>1365.6192</v>
       </c>
       <c r="G201" t="n">
-        <v>1542.409840752</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H201" t="n">
-        <v>1525.751814471878</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I201" t="n">
-        <v>1571.066643361693</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J201" t="n">
-        <v>1715.918987879641</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K201" t="n">
-        <v>1440.513990324959</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D202" t="n">
         <v>1000</v>
       </c>
       <c r="E202" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F202" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G202" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H202" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I202" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J202" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K202" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D203" t="n">
         <v>1000</v>
       </c>
       <c r="E203" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F203" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G203" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H203" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I203" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J203" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K203" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="D204" t="n">
         <v>1000</v>
       </c>
       <c r="E204" t="n">
-        <v>1222.6</v>
+        <v>942</v>
       </c>
       <c r="F204" t="n">
-        <v>1122.46906</v>
+        <v>730.2384</v>
       </c>
       <c r="G204" t="n">
-        <v>1222.481053246</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H204" t="n">
-        <v>1198.520424602378</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I204" t="n">
-        <v>1133.440765546469</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J204" t="n">
-        <v>1142.73497982395</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K204" t="n">
-        <v>813.6273056346525</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D205" t="n">
         <v>1000</v>
       </c>
       <c r="E205" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F205" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G205" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H205" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I205" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J205" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K205" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D206" t="n">
         <v>1000</v>
       </c>
       <c r="E206" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F206" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G206" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H206" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I206" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J206" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K206" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -23037,30 +23099,67 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D207" t="n">
         <v>1000</v>
       </c>
       <c r="E207" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F207" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G207" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H207" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I207" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J207" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K207" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>41</v>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D208" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E208" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F207" t="n">
+      <c r="F208" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G207" t="n">
+      <c r="G208" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H207" t="n">
+      <c r="H208" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I207" t="n">
+      <c r="I208" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J207" t="n">
+      <c r="J208" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K207" t="n">
+      <c r="K208" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 220 MLP seq=35 seed=13 -1.70 (catastrophic); 6-seed median -0.29; exp 221 seed=11 #7/10
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$220</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$221</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>222</row>
+      <row>223</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T220"/>
+  <dimension ref="A1:T221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -15719,16 +15719,16 @@
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>14</v>
+        <v>220</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>MLP seq=35 seed=13 (#6/10 user directive) - Picard 2021</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -15737,60 +15737,60 @@
         </is>
       </c>
       <c r="E214" t="n">
-        <v>-1.7077</v>
+        <v>-1.6978</v>
       </c>
       <c r="F214" t="n">
-        <v>0.4944</v>
+        <v>-0.9978</v>
       </c>
       <c r="G214" t="n">
-        <v>-1.5077</v>
+        <v>-0.2639</v>
       </c>
       <c r="I214" t="n">
-        <v>44.06</v>
+        <v>-73.51000000000001</v>
       </c>
       <c r="J214" t="n">
-        <v>1440.6</v>
+        <v>264.8999999999999</v>
       </c>
       <c r="K214" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L214" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N214" t="n">
-        <v>0.0102</v>
+        <v>-0.0151</v>
       </c>
       <c r="O214" t="n">
-        <v>52.26</v>
+        <v>44.4</v>
       </c>
       <c r="P214" t="n">
-        <v>0.5959</v>
+        <v>0.5636</v>
       </c>
       <c r="Q214" t="n">
-        <v>0.6044</v>
+        <v>0.1858</v>
       </c>
       <c r="R214" t="n">
-        <v>0.6002</v>
+        <v>0.2794</v>
       </c>
       <c r="S214" t="n">
-        <v>0.0091</v>
+        <v>-0.0159</v>
       </c>
       <c r="T214" t="n">
-        <v>1076.7</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -15799,60 +15799,60 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F215" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G215" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I215" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J215" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K215" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L215" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N215" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O215" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P215" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q215" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R215" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S215" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T215" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -15861,60 +15861,60 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F216" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G216" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I216" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J216" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K216" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L216" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N216" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O216" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P216" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q216" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R216" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S216" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T216" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -15923,60 +15923,60 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="F217" t="n">
-        <v>-0.1044</v>
+        <v>-1.2201</v>
       </c>
       <c r="G217" t="n">
-        <v>-1.6173</v>
+        <v>-0.255</v>
       </c>
       <c r="I217" t="n">
-        <v>-18.65</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J217" t="n">
-        <v>813.5</v>
+        <v>282.4</v>
       </c>
       <c r="K217" t="n">
+        <v>1</v>
+      </c>
+      <c r="L217" t="n">
         <v>3</v>
       </c>
-      <c r="L217" t="n">
-        <v>2</v>
-      </c>
       <c r="N217" t="n">
-        <v>-0.0416</v>
+        <v>-0.0322</v>
       </c>
       <c r="O217" t="n">
-        <v>48.72</v>
+        <v>40.59</v>
       </c>
       <c r="P217" t="n">
-        <v>0.5679999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q217" t="n">
-        <v>0.5653</v>
+        <v>0</v>
       </c>
       <c r="R217" t="n">
-        <v>0.5666</v>
+        <v>0</v>
       </c>
       <c r="S217" t="n">
-        <v>-0.0596</v>
+        <v>0</v>
       </c>
       <c r="T217" t="n">
-        <v>73</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -15985,60 +15985,60 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F218" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G218" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I218" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J218" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K218" t="n">
         <v>3</v>
       </c>
       <c r="L218" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N218" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O218" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P218" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q218" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R218" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S218" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T218" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -16047,51 +16047,51 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F219" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G219" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I219" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J219" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K219" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L219" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N219" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O219" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P219" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q219" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R219" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S219" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T219" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -16100,7 +16100,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -16109,51 +16109,113 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F220" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G220" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I220" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J220" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K220" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L220" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N220" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O220" t="n">
         <v>47.65</v>
       </c>
       <c r="P220" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q220" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R220" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S220" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T220" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>41</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E221" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F221" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G221" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I221" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J221" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K221" t="n">
+        <v>4</v>
+      </c>
+      <c r="L221" t="n">
+        <v>2</v>
+      </c>
+      <c r="N221" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O221" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P221" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q220" t="n">
+      <c r="Q221" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R220" t="n">
+      <c r="R221" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S220" t="n">
+      <c r="S221" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T220" t="n">
+      <c r="T221" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T220"/>
-  <conditionalFormatting sqref="E2:E220">
+  <autoFilter ref="A1:T221"/>
+  <conditionalFormatting sqref="E2:E221">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -16175,7 +16237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K220"/>
+  <dimension ref="A1:K221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -24094,229 +24156,229 @@
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>14</v>
+        <v>220</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>-1.7077</v>
+        <v>-1.6978</v>
       </c>
       <c r="D214" t="n">
         <v>1000</v>
       </c>
       <c r="E214" t="n">
-        <v>1067.7</v>
+        <v>901.6999999999999</v>
       </c>
       <c r="F214" t="n">
-        <v>1380.10902</v>
+        <v>774.1094499999999</v>
       </c>
       <c r="G214" t="n">
-        <v>1542.409840752</v>
+        <v>749.570180435</v>
       </c>
       <c r="H214" t="n">
-        <v>1525.751814471878</v>
+        <v>634.3612437021405</v>
       </c>
       <c r="I214" t="n">
-        <v>1571.066643361693</v>
+        <v>618.502212609587</v>
       </c>
       <c r="J214" t="n">
-        <v>1715.918987879641</v>
+        <v>338.3207102974441</v>
       </c>
       <c r="K214" t="n">
-        <v>1440.513990324959</v>
+        <v>264.9389482339285</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D215" t="n">
         <v>1000</v>
       </c>
       <c r="E215" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F215" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G215" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H215" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I215" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J215" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K215" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D216" t="n">
         <v>1000</v>
       </c>
       <c r="E216" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F216" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G216" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H216" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I216" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J216" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K216" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="D217" t="n">
         <v>1000</v>
       </c>
       <c r="E217" t="n">
-        <v>1222.6</v>
+        <v>942</v>
       </c>
       <c r="F217" t="n">
-        <v>1122.46906</v>
+        <v>730.2384</v>
       </c>
       <c r="G217" t="n">
-        <v>1222.481053246</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H217" t="n">
-        <v>1198.520424602378</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I217" t="n">
-        <v>1133.440765546469</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J217" t="n">
-        <v>1142.73497982395</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K217" t="n">
-        <v>813.6273056346525</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D218" t="n">
         <v>1000</v>
       </c>
       <c r="E218" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F218" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G218" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H218" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I218" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J218" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K218" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D219" t="n">
         <v>1000</v>
       </c>
       <c r="E219" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F219" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G219" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H219" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I219" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J219" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K219" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
@@ -24324,30 +24386,67 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D220" t="n">
         <v>1000</v>
       </c>
       <c r="E220" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F220" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G220" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H220" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I220" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J220" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K220" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>41</v>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D221" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E221" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F220" t="n">
+      <c r="F221" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G220" t="n">
+      <c r="G221" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H220" t="n">
+      <c r="H221" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I220" t="n">
+      <c r="I221" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J220" t="n">
+      <c r="J221" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K220" t="n">
+      <c r="K221" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 222 MLP seq=35 seed=3 -1.33 (8-seed median -0.29); exp 223 seed=5 #9/10
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$222</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$223</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>224</row>
+      <row>225</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T222"/>
+  <dimension ref="A1:T223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -14739,16 +14739,16 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>40</v>
+        <v>222</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
+          <t>MLP seq=35 seed=3 (#8/10 user directive) - Picard 2021</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
@@ -14757,60 +14757,60 @@
         </is>
       </c>
       <c r="E198" t="n">
-        <v>-1.335</v>
+        <v>-1.3275</v>
       </c>
       <c r="F198" t="n">
-        <v>0.0349</v>
+        <v>-0.2723</v>
       </c>
       <c r="G198" t="n">
-        <v>-1.035</v>
+        <v>-0.9275</v>
       </c>
       <c r="I198" t="n">
-        <v>-7.12</v>
+        <v>-37.39</v>
       </c>
       <c r="J198" t="n">
-        <v>928.8</v>
+        <v>626.1</v>
       </c>
       <c r="K198" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L198" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N198" t="n">
-        <v>-0.0034</v>
+        <v>0.043</v>
       </c>
       <c r="O198" t="n">
-        <v>47.74</v>
+        <v>47.32</v>
       </c>
       <c r="P198" t="n">
-        <v>0.577</v>
+        <v>0.6222</v>
       </c>
       <c r="Q198" t="n">
-        <v>0.4446</v>
+        <v>0.2346</v>
       </c>
       <c r="R198" t="n">
-        <v>0.5022</v>
+        <v>0.3408</v>
       </c>
       <c r="S198" t="n">
-        <v>-0.0286</v>
+        <v>0.0455</v>
       </c>
       <c r="T198" t="n">
-        <v>79</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>XGBoost depth=4 n_est=100 - capacity test between 50 (best) and 300 (worse)</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
@@ -14819,60 +14819,60 @@
         </is>
       </c>
       <c r="E199" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="F199" t="n">
-        <v>0.011</v>
+        <v>0.0349</v>
       </c>
       <c r="G199" t="n">
-        <v>-0.9564</v>
+        <v>-1.035</v>
       </c>
       <c r="I199" t="n">
-        <v>-17.26</v>
+        <v>-7.12</v>
       </c>
       <c r="J199" t="n">
-        <v>827.4</v>
+        <v>928.8</v>
       </c>
       <c r="K199" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L199" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N199" t="n">
-        <v>-0.0003</v>
+        <v>-0.0034</v>
       </c>
       <c r="O199" t="n">
-        <v>48.19</v>
+        <v>47.74</v>
       </c>
       <c r="P199" t="n">
-        <v>0.5666</v>
+        <v>0.577</v>
       </c>
       <c r="Q199" t="n">
-        <v>0.4114</v>
+        <v>0.4446</v>
       </c>
       <c r="R199" t="n">
-        <v>0.4767</v>
+        <v>0.5022</v>
       </c>
       <c r="S199" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0286</v>
       </c>
       <c r="T199" t="n">
-        <v>37.9</v>
+        <v>79</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
@@ -14881,60 +14881,60 @@
         </is>
       </c>
       <c r="E200" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F200" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G200" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I200" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J200" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K200" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L200" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N200" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O200" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P200" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q200" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R200" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S200" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T200" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
@@ -14943,60 +14943,60 @@
         </is>
       </c>
       <c r="E201" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="F201" t="n">
-        <v>-0.8189</v>
+        <v>-0.6131</v>
       </c>
       <c r="G201" t="n">
-        <v>1.1456</v>
+        <v>-0.9054</v>
       </c>
       <c r="I201" t="n">
-        <v>-58.71</v>
+        <v>-49.86</v>
       </c>
       <c r="J201" t="n">
-        <v>412.9</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K201" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L201" t="n">
         <v>3</v>
       </c>
       <c r="N201" t="n">
-        <v>0.0089</v>
+        <v>0.0074</v>
       </c>
       <c r="O201" t="n">
-        <v>41.44</v>
+        <v>44.37</v>
       </c>
       <c r="P201" t="n">
-        <v>0.68</v>
+        <v>0.6127</v>
       </c>
       <c r="Q201" t="n">
-        <v>0.0271</v>
+        <v>0.1688</v>
       </c>
       <c r="R201" t="n">
-        <v>0.0521</v>
+        <v>0.2647</v>
       </c>
       <c r="S201" t="n">
-        <v>0.0277</v>
+        <v>0.0182</v>
       </c>
       <c r="T201" t="n">
-        <v>8786.5</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
@@ -15005,60 +15005,60 @@
         </is>
       </c>
       <c r="E202" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="F202" t="n">
-        <v>0.2144</v>
+        <v>-0.8189</v>
       </c>
       <c r="G202" t="n">
-        <v>-1.2304</v>
+        <v>1.1456</v>
       </c>
       <c r="I202" t="n">
-        <v>10.12</v>
+        <v>-58.71</v>
       </c>
       <c r="J202" t="n">
-        <v>1101.2</v>
+        <v>412.9</v>
       </c>
       <c r="K202" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L202" t="n">
         <v>3</v>
       </c>
       <c r="N202" t="n">
-        <v>0.0027</v>
+        <v>0.0089</v>
       </c>
       <c r="O202" t="n">
-        <v>53.55</v>
+        <v>41.44</v>
       </c>
       <c r="P202" t="n">
-        <v>0.5858</v>
+        <v>0.68</v>
       </c>
       <c r="Q202" t="n">
-        <v>0.7341</v>
+        <v>0.0271</v>
       </c>
       <c r="R202" t="n">
-        <v>0.6516</v>
+        <v>0.0521</v>
       </c>
       <c r="S202" t="n">
-        <v>-0.0231</v>
+        <v>0.0277</v>
       </c>
       <c r="T202" t="n">
-        <v>69.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
@@ -15067,51 +15067,51 @@
         </is>
       </c>
       <c r="E203" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="F203" t="n">
-        <v>-0.6042</v>
+        <v>0.2144</v>
       </c>
       <c r="G203" t="n">
-        <v>-0.8305</v>
+        <v>-1.2304</v>
       </c>
       <c r="I203" t="n">
-        <v>-67.48999999999999</v>
+        <v>10.12</v>
       </c>
       <c r="J203" t="n">
-        <v>325.1000000000001</v>
+        <v>1101.2</v>
       </c>
       <c r="K203" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L203" t="n">
         <v>3</v>
       </c>
       <c r="N203" t="n">
-        <v>0.0111</v>
+        <v>0.0027</v>
       </c>
       <c r="O203" t="n">
-        <v>42.64</v>
+        <v>53.55</v>
       </c>
       <c r="P203" t="n">
-        <v>0</v>
+        <v>0.5858</v>
       </c>
       <c r="Q203" t="n">
-        <v>0</v>
+        <v>0.7341</v>
       </c>
       <c r="R203" t="n">
-        <v>0</v>
+        <v>0.6516</v>
       </c>
       <c r="S203" t="n">
-        <v>0</v>
+        <v>-0.0231</v>
       </c>
       <c r="T203" t="n">
-        <v>82.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -15120,7 +15120,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
@@ -15150,7 +15150,7 @@
         <v>3</v>
       </c>
       <c r="N204" t="n">
-        <v>0.032</v>
+        <v>0.0111</v>
       </c>
       <c r="O204" t="n">
         <v>42.64</v>
@@ -15168,21 +15168,21 @@
         <v>0</v>
       </c>
       <c r="T204" t="n">
-        <v>62.3</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
@@ -15191,60 +15191,60 @@
         </is>
       </c>
       <c r="E205" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F205" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G205" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I205" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J205" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K205" t="n">
         <v>1</v>
       </c>
       <c r="L205" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N205" t="n">
-        <v>0.0284</v>
+        <v>0.032</v>
       </c>
       <c r="O205" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P205" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q205" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R205" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S205" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T205" t="n">
-        <v>79.8</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
@@ -15253,60 +15253,60 @@
         </is>
       </c>
       <c r="E206" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="F206" t="n">
-        <v>0.4732</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G206" t="n">
-        <v>-1.1536</v>
+        <v>-0.8347</v>
       </c>
       <c r="I206" t="n">
-        <v>41.21</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J206" t="n">
-        <v>1412.1</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K206" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L206" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N206" t="n">
-        <v>0.0231</v>
+        <v>0.0284</v>
       </c>
       <c r="O206" t="n">
-        <v>48.31</v>
+        <v>44.07</v>
       </c>
       <c r="P206" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.5588</v>
       </c>
       <c r="Q206" t="n">
-        <v>0.3418</v>
+        <v>0.1177</v>
       </c>
       <c r="R206" t="n">
-        <v>0.4395</v>
+        <v>0.1945</v>
       </c>
       <c r="S206" t="n">
-        <v>0.0329</v>
+        <v>-0.0101</v>
       </c>
       <c r="T206" t="n">
-        <v>1311.2</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
@@ -15315,39 +15315,51 @@
         </is>
       </c>
       <c r="E207" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F207" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G207" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I207" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J207" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K207" t="n">
         <v>4</v>
       </c>
       <c r="L207" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N207" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O207" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P207" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q207" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R207" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S207" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T207" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -15356,7 +15368,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
@@ -15365,51 +15377,39 @@
         </is>
       </c>
       <c r="E208" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F208" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G208" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I208" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J208" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K208" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L208" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N208" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O208" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P208" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q208" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R208" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S208" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T208" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -15418,7 +15418,7 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
@@ -15427,51 +15427,51 @@
         </is>
       </c>
       <c r="E209" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F209" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G209" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I209" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J209" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L209" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N209" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O209" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P209" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q209" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R209" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S209" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T209" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -15480,7 +15480,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
@@ -15489,60 +15489,60 @@
         </is>
       </c>
       <c r="E210" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F210" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G210" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I210" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J210" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K210" t="n">
         <v>1</v>
       </c>
       <c r="L210" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N210" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O210" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P210" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q210" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R210" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S210" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T210" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
@@ -15551,60 +15551,60 @@
         </is>
       </c>
       <c r="E211" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F211" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G211" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I211" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J211" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K211" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L211" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N211" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O211" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P211" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q211" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R211" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S211" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T211" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
@@ -15613,113 +15613,113 @@
         </is>
       </c>
       <c r="E212" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="F212" t="n">
-        <v>0.9243</v>
+        <v>-1.0225</v>
       </c>
       <c r="G212" t="n">
-        <v>-1.2246</v>
+        <v>-0.2617</v>
       </c>
       <c r="I212" t="n">
-        <v>116.09</v>
+        <v>-65.97</v>
       </c>
       <c r="J212" t="n">
-        <v>2160.9</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K212" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L212" t="n">
         <v>3</v>
       </c>
       <c r="N212" t="n">
-        <v>0.0283</v>
+        <v>-0.0076</v>
       </c>
       <c r="O212" t="n">
-        <v>53.93</v>
+        <v>40.96</v>
       </c>
       <c r="P212" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5526</v>
       </c>
       <c r="Q212" t="n">
-        <v>0.7548</v>
+        <v>0.0334</v>
       </c>
       <c r="R212" t="n">
-        <v>0.6592</v>
+        <v>0.0631</v>
       </c>
       <c r="S212" t="n">
-        <v>-0.0266</v>
+        <v>-0.0156</v>
       </c>
       <c r="T212" t="n">
-        <v>97.5</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="F213" t="n">
-        <v>0.5694</v>
+        <v>0.9243</v>
       </c>
       <c r="G213" t="n">
-        <v>-1.3423</v>
+        <v>-1.2246</v>
       </c>
       <c r="I213" t="n">
-        <v>54.77</v>
+        <v>116.09</v>
       </c>
       <c r="J213" t="n">
-        <v>1547.7</v>
+        <v>2160.9</v>
       </c>
       <c r="K213" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L213" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N213" t="n">
-        <v>0.0103</v>
+        <v>0.0283</v>
       </c>
       <c r="O213" t="n">
-        <v>51.13</v>
+        <v>53.93</v>
       </c>
       <c r="P213" t="n">
-        <v>0.5968</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="Q213" t="n">
-        <v>0.5364</v>
+        <v>0.7548</v>
       </c>
       <c r="R213" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="S213" t="n">
-        <v>0.0098</v>
+        <v>-0.0266</v>
       </c>
       <c r="T213" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -15728,12 +15728,12 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E214" t="n">
@@ -15776,21 +15776,21 @@
         <v>0.0098</v>
       </c>
       <c r="T214" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>220</v>
+        <v>39</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>MLP seq=35 seed=13 (#6/10 user directive) - Picard 2021</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -15799,60 +15799,60 @@
         </is>
       </c>
       <c r="E215" t="n">
-        <v>-1.6978</v>
+        <v>-1.5423</v>
       </c>
       <c r="F215" t="n">
-        <v>-0.9978</v>
+        <v>0.5694</v>
       </c>
       <c r="G215" t="n">
-        <v>-0.2639</v>
+        <v>-1.3423</v>
       </c>
       <c r="I215" t="n">
-        <v>-73.51000000000001</v>
+        <v>54.77</v>
       </c>
       <c r="J215" t="n">
-        <v>264.8999999999999</v>
+        <v>1547.7</v>
       </c>
       <c r="K215" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L215" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N215" t="n">
-        <v>-0.0151</v>
+        <v>0.0103</v>
       </c>
       <c r="O215" t="n">
-        <v>44.4</v>
+        <v>51.13</v>
       </c>
       <c r="P215" t="n">
-        <v>0.5636</v>
+        <v>0.5968</v>
       </c>
       <c r="Q215" t="n">
-        <v>0.1858</v>
+        <v>0.5364</v>
       </c>
       <c r="R215" t="n">
-        <v>0.2794</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S215" t="n">
-        <v>-0.0159</v>
+        <v>0.0098</v>
       </c>
       <c r="T215" t="n">
-        <v>30.8</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>14</v>
+        <v>220</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>MLP seq=35 seed=13 (#6/10 user directive) - Picard 2021</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -15861,60 +15861,60 @@
         </is>
       </c>
       <c r="E216" t="n">
-        <v>-1.7077</v>
+        <v>-1.6978</v>
       </c>
       <c r="F216" t="n">
-        <v>0.4944</v>
+        <v>-0.9978</v>
       </c>
       <c r="G216" t="n">
-        <v>-1.5077</v>
+        <v>-0.2639</v>
       </c>
       <c r="I216" t="n">
-        <v>44.06</v>
+        <v>-73.51000000000001</v>
       </c>
       <c r="J216" t="n">
-        <v>1440.6</v>
+        <v>264.8999999999999</v>
       </c>
       <c r="K216" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L216" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N216" t="n">
-        <v>0.0102</v>
+        <v>-0.0151</v>
       </c>
       <c r="O216" t="n">
-        <v>52.26</v>
+        <v>44.4</v>
       </c>
       <c r="P216" t="n">
-        <v>0.5959</v>
+        <v>0.5636</v>
       </c>
       <c r="Q216" t="n">
-        <v>0.6044</v>
+        <v>0.1858</v>
       </c>
       <c r="R216" t="n">
-        <v>0.6002</v>
+        <v>0.2794</v>
       </c>
       <c r="S216" t="n">
-        <v>0.0091</v>
+        <v>-0.0159</v>
       </c>
       <c r="T216" t="n">
-        <v>1076.7</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -15923,60 +15923,60 @@
         </is>
       </c>
       <c r="E217" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F217" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G217" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I217" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J217" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K217" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L217" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N217" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O217" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P217" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q217" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R217" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S217" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T217" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -15985,60 +15985,60 @@
         </is>
       </c>
       <c r="E218" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F218" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G218" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I218" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J218" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K218" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L218" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N218" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O218" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P218" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q218" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R218" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S218" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T218" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -16047,60 +16047,60 @@
         </is>
       </c>
       <c r="E219" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="F219" t="n">
-        <v>-0.1044</v>
+        <v>-1.2201</v>
       </c>
       <c r="G219" t="n">
-        <v>-1.6173</v>
+        <v>-0.255</v>
       </c>
       <c r="I219" t="n">
-        <v>-18.65</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J219" t="n">
-        <v>813.5</v>
+        <v>282.4</v>
       </c>
       <c r="K219" t="n">
+        <v>1</v>
+      </c>
+      <c r="L219" t="n">
         <v>3</v>
       </c>
-      <c r="L219" t="n">
-        <v>2</v>
-      </c>
       <c r="N219" t="n">
-        <v>-0.0416</v>
+        <v>-0.0322</v>
       </c>
       <c r="O219" t="n">
-        <v>48.72</v>
+        <v>40.59</v>
       </c>
       <c r="P219" t="n">
-        <v>0.5679999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q219" t="n">
-        <v>0.5653</v>
+        <v>0</v>
       </c>
       <c r="R219" t="n">
-        <v>0.5666</v>
+        <v>0</v>
       </c>
       <c r="S219" t="n">
-        <v>-0.0596</v>
+        <v>0</v>
       </c>
       <c r="T219" t="n">
-        <v>73</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -16109,60 +16109,60 @@
         </is>
       </c>
       <c r="E220" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F220" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G220" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I220" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J220" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K220" t="n">
         <v>3</v>
       </c>
       <c r="L220" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N220" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O220" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P220" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q220" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R220" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S220" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T220" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
@@ -16171,51 +16171,51 @@
         </is>
       </c>
       <c r="E221" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F221" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G221" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I221" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J221" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K221" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L221" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N221" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O221" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P221" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q221" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R221" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S221" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T221" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
@@ -16233,51 +16233,113 @@
         </is>
       </c>
       <c r="E222" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F222" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G222" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I222" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J222" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K222" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L222" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N222" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O222" t="n">
         <v>47.65</v>
       </c>
       <c r="P222" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q222" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R222" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S222" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T222" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>41</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E223" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F223" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G223" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I223" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J223" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K223" t="n">
+        <v>4</v>
+      </c>
+      <c r="L223" t="n">
+        <v>2</v>
+      </c>
+      <c r="N223" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O223" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P223" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q222" t="n">
+      <c r="Q223" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R222" t="n">
+      <c r="R223" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S222" t="n">
+      <c r="S223" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T222" t="n">
+      <c r="T223" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T222"/>
-  <conditionalFormatting sqref="E2:E222">
+  <autoFilter ref="A1:T223"/>
+  <conditionalFormatting sqref="E2:E223">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -16299,7 +16361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K222"/>
+  <dimension ref="A1:K223"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -23626,229 +23688,229 @@
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>40</v>
+        <v>222</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>-1.335</v>
+        <v>-1.3275</v>
       </c>
       <c r="D198" t="n">
         <v>1000</v>
       </c>
       <c r="E198" t="n">
-        <v>1200</v>
+        <v>901.6999999999999</v>
       </c>
       <c r="F198" t="n">
-        <v>1259.16</v>
+        <v>769.33044</v>
       </c>
       <c r="G198" t="n">
-        <v>1343.145972</v>
+        <v>709.938130032</v>
       </c>
       <c r="H198" t="n">
-        <v>1093.7237649996</v>
+        <v>629.8571089643904</v>
       </c>
       <c r="I198" t="n">
-        <v>1039.36569387912</v>
+        <v>644.5957653141571</v>
       </c>
       <c r="J198" t="n">
-        <v>1048.408175415868</v>
+        <v>644.5313057376258</v>
       </c>
       <c r="K198" t="n">
-        <v>928.8896434184592</v>
+        <v>626.0977103935297</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>-1.3564</v>
+        <v>-1.335</v>
       </c>
       <c r="D199" t="n">
         <v>1000</v>
       </c>
       <c r="E199" t="n">
-        <v>799.9</v>
+        <v>1200</v>
       </c>
       <c r="F199" t="n">
-        <v>677.35532</v>
+        <v>1259.16</v>
       </c>
       <c r="G199" t="n">
-        <v>658.660313168</v>
+        <v>1343.145972</v>
       </c>
       <c r="H199" t="n">
-        <v>699.1679224278321</v>
+        <v>1093.7237649996</v>
       </c>
       <c r="I199" t="n">
-        <v>703.2230963779135</v>
+        <v>1039.36569387912</v>
       </c>
       <c r="J199" t="n">
-        <v>1025.22895220936</v>
+        <v>1048.408175415868</v>
       </c>
       <c r="K199" t="n">
-        <v>827.3597644329536</v>
+        <v>928.8896434184592</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D200" t="n">
         <v>1000</v>
       </c>
       <c r="E200" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F200" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G200" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H200" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I200" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J200" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K200" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>-1.4189</v>
+        <v>-1.4054</v>
       </c>
       <c r="D201" t="n">
         <v>1000</v>
       </c>
       <c r="E201" t="n">
-        <v>942</v>
+        <v>951.8</v>
       </c>
       <c r="F201" t="n">
-        <v>730.2384</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G201" t="n">
-        <v>637.6441708799999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H201" t="n">
-        <v>706.8923278375679</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I201" t="n">
-        <v>605.0291433961744</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J201" t="n">
-        <v>435.9234978169437</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K201" t="n">
-        <v>412.9503294819908</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="D202" t="n">
         <v>1000</v>
       </c>
       <c r="E202" t="n">
-        <v>999.6</v>
+        <v>942</v>
       </c>
       <c r="F202" t="n">
-        <v>1076.66916</v>
+        <v>730.2384</v>
       </c>
       <c r="G202" t="n">
-        <v>1127.918612016</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H202" t="n">
-        <v>1009.261574031917</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I202" t="n">
-        <v>837.9898849187007</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J202" t="n">
-        <v>1032.403538219839</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K202" t="n">
-        <v>1101.161613865281</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="D203" t="n">
         <v>1000</v>
       </c>
       <c r="E203" t="n">
-        <v>1045.3</v>
+        <v>999.6</v>
       </c>
       <c r="F203" t="n">
-        <v>853.06933</v>
+        <v>1076.66916</v>
       </c>
       <c r="G203" t="n">
-        <v>749.933248003</v>
+        <v>1127.918612016</v>
       </c>
       <c r="H203" t="n">
-        <v>740.3341024285616</v>
+        <v>1009.261574031917</v>
       </c>
       <c r="I203" t="n">
-        <v>691.1759180273051</v>
+        <v>837.9898849187007</v>
       </c>
       <c r="J203" t="n">
-        <v>482.7172611502699</v>
+        <v>1032.403538219839</v>
       </c>
       <c r="K203" t="n">
-        <v>325.0618036585918</v>
+        <v>1101.161613865281</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -23885,118 +23947,118 @@
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D205" t="n">
         <v>1000</v>
       </c>
       <c r="E205" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F205" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G205" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H205" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I205" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J205" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K205" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="D206" t="n">
         <v>1000</v>
       </c>
       <c r="E206" t="n">
-        <v>1236.4</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F206" t="n">
-        <v>1500.74232</v>
+        <v>692.62656</v>
       </c>
       <c r="G206" t="n">
-        <v>1734.708047688</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H206" t="n">
-        <v>1677.809623723833</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I206" t="n">
-        <v>1544.088196713044</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J206" t="n">
-        <v>1750.069562154564</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K206" t="n">
-        <v>1412.131129702517</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D207" t="n">
         <v>1000</v>
       </c>
       <c r="E207" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F207" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G207" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H207" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I207" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J207" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K207" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -24004,36 +24066,36 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D208" t="n">
         <v>1000</v>
       </c>
       <c r="E208" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F208" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G208" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H208" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I208" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J208" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K208" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -24041,36 +24103,36 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D209" t="n">
         <v>1000</v>
       </c>
       <c r="E209" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F209" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G209" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H209" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I209" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J209" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K209" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -24078,147 +24140,147 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D210" t="n">
         <v>1000</v>
       </c>
       <c r="E210" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F210" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G210" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H210" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I210" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J210" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K210" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D211" t="n">
         <v>1000</v>
       </c>
       <c r="E211" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F211" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G211" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H211" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I211" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J211" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K211" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="D212" t="n">
         <v>1000</v>
       </c>
       <c r="E212" t="n">
-        <v>1127.9</v>
+        <v>1141.5</v>
       </c>
       <c r="F212" t="n">
-        <v>1108.7257</v>
+        <v>884.8908</v>
       </c>
       <c r="G212" t="n">
-        <v>1251.64044273</v>
+        <v>789.49957176</v>
       </c>
       <c r="H212" t="n">
-        <v>1235.619445063056</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I212" t="n">
-        <v>1202.010596157341</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J212" t="n">
-        <v>1559.849150633381</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K212" t="n">
-        <v>2161.015013287486</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="D213" t="n">
         <v>1000</v>
       </c>
       <c r="E213" t="n">
-        <v>1342</v>
+        <v>1127.9</v>
       </c>
       <c r="F213" t="n">
-        <v>1365.6192</v>
+        <v>1108.7257</v>
       </c>
       <c r="G213" t="n">
-        <v>1401.67154688</v>
+        <v>1251.64044273</v>
       </c>
       <c r="H213" t="n">
-        <v>1356.1172216064</v>
+        <v>1235.619445063056</v>
       </c>
       <c r="I213" t="n">
-        <v>1614.321940600259</v>
+        <v>1202.010596157341</v>
       </c>
       <c r="J213" t="n">
-        <v>1682.93062307577</v>
+        <v>1559.849150633381</v>
       </c>
       <c r="K213" t="n">
-        <v>1547.623000980478</v>
+        <v>2161.015013287486</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -24255,266 +24317,266 @@
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>220</v>
+        <v>39</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>-1.6978</v>
+        <v>-1.5423</v>
       </c>
       <c r="D215" t="n">
         <v>1000</v>
       </c>
       <c r="E215" t="n">
-        <v>901.6999999999999</v>
+        <v>1342</v>
       </c>
       <c r="F215" t="n">
-        <v>774.1094499999999</v>
+        <v>1365.6192</v>
       </c>
       <c r="G215" t="n">
-        <v>749.570180435</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H215" t="n">
-        <v>634.3612437021405</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I215" t="n">
-        <v>618.502212609587</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J215" t="n">
-        <v>338.3207102974441</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K215" t="n">
-        <v>264.9389482339285</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>14</v>
+        <v>220</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>-1.7077</v>
+        <v>-1.6978</v>
       </c>
       <c r="D216" t="n">
         <v>1000</v>
       </c>
       <c r="E216" t="n">
-        <v>1067.7</v>
+        <v>901.6999999999999</v>
       </c>
       <c r="F216" t="n">
-        <v>1380.10902</v>
+        <v>774.1094499999999</v>
       </c>
       <c r="G216" t="n">
-        <v>1542.409840752</v>
+        <v>749.570180435</v>
       </c>
       <c r="H216" t="n">
-        <v>1525.751814471878</v>
+        <v>634.3612437021405</v>
       </c>
       <c r="I216" t="n">
-        <v>1571.066643361693</v>
+        <v>618.502212609587</v>
       </c>
       <c r="J216" t="n">
-        <v>1715.918987879641</v>
+        <v>338.3207102974441</v>
       </c>
       <c r="K216" t="n">
-        <v>1440.513990324959</v>
+        <v>264.9389482339285</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D217" t="n">
         <v>1000</v>
       </c>
       <c r="E217" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F217" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G217" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H217" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I217" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J217" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K217" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D218" t="n">
         <v>1000</v>
       </c>
       <c r="E218" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F218" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G218" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H218" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I218" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J218" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K218" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="D219" t="n">
         <v>1000</v>
       </c>
       <c r="E219" t="n">
-        <v>1222.6</v>
+        <v>942</v>
       </c>
       <c r="F219" t="n">
-        <v>1122.46906</v>
+        <v>730.2384</v>
       </c>
       <c r="G219" t="n">
-        <v>1222.481053246</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H219" t="n">
-        <v>1198.520424602378</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I219" t="n">
-        <v>1133.440765546469</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J219" t="n">
-        <v>1142.73497982395</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K219" t="n">
-        <v>813.6273056346525</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D220" t="n">
         <v>1000</v>
       </c>
       <c r="E220" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F220" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G220" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H220" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I220" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J220" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K220" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D221" t="n">
         <v>1000</v>
       </c>
       <c r="E221" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F221" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G221" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H221" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I221" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J221" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K221" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B222" t="inlineStr">
         <is>
@@ -24522,30 +24584,67 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D222" t="n">
         <v>1000</v>
       </c>
       <c r="E222" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F222" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G222" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H222" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I222" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J222" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K222" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>41</v>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D223" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E223" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F222" t="n">
+      <c r="F223" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G222" t="n">
+      <c r="G223" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H222" t="n">
+      <c r="H223" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I222" t="n">
+      <c r="I223" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J222" t="n">
+      <c r="J223" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K222" t="n">
+      <c r="K223" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 247 xLSTM seed=13 -1.42 catastrophic (6-seed median -0.30); exp 248 seed=11 #7/10
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$247</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$248</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>249</row>
+      <row>250</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T247"/>
+  <dimension ref="A1:T248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -16475,16 +16475,16 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>110</v>
+        <v>247</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>xLSTM seq=60 seed=13 #6/10</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -16493,60 +16493,60 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>-1.4189</v>
+        <v>-1.4181</v>
       </c>
       <c r="F226" t="n">
-        <v>-0.8189</v>
+        <v>-0.9181</v>
       </c>
       <c r="G226" t="n">
-        <v>1.1456</v>
+        <v>-0.0286</v>
       </c>
       <c r="I226" t="n">
-        <v>-58.71</v>
+        <v>-62.4</v>
       </c>
       <c r="J226" t="n">
-        <v>412.9</v>
+        <v>376</v>
       </c>
       <c r="K226" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L226" t="n">
         <v>3</v>
       </c>
       <c r="N226" t="n">
-        <v>0.0089</v>
+        <v>-0.01</v>
       </c>
       <c r="O226" t="n">
-        <v>41.44</v>
+        <v>42.1</v>
       </c>
       <c r="P226" t="n">
-        <v>0.68</v>
+        <v>0.5412</v>
       </c>
       <c r="Q226" t="n">
-        <v>0.0271</v>
+        <v>0.1672</v>
       </c>
       <c r="R226" t="n">
-        <v>0.0521</v>
+        <v>0.2555</v>
       </c>
       <c r="S226" t="n">
-        <v>0.0277</v>
+        <v>-0.0493</v>
       </c>
       <c r="T226" t="n">
-        <v>8786.5</v>
+        <v>1037.1</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -16555,60 +16555,60 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="F227" t="n">
-        <v>0.2144</v>
+        <v>-0.8189</v>
       </c>
       <c r="G227" t="n">
-        <v>-1.2304</v>
+        <v>1.1456</v>
       </c>
       <c r="I227" t="n">
-        <v>10.12</v>
+        <v>-58.71</v>
       </c>
       <c r="J227" t="n">
-        <v>1101.2</v>
+        <v>412.9</v>
       </c>
       <c r="K227" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L227" t="n">
         <v>3</v>
       </c>
       <c r="N227" t="n">
-        <v>0.0027</v>
+        <v>0.0089</v>
       </c>
       <c r="O227" t="n">
-        <v>53.55</v>
+        <v>41.44</v>
       </c>
       <c r="P227" t="n">
-        <v>0.5858</v>
+        <v>0.68</v>
       </c>
       <c r="Q227" t="n">
-        <v>0.7341</v>
+        <v>0.0271</v>
       </c>
       <c r="R227" t="n">
-        <v>0.6516</v>
+        <v>0.0521</v>
       </c>
       <c r="S227" t="n">
-        <v>-0.0231</v>
+        <v>0.0277</v>
       </c>
       <c r="T227" t="n">
-        <v>69.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -16617,51 +16617,51 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="F228" t="n">
-        <v>-0.6042</v>
+        <v>0.2144</v>
       </c>
       <c r="G228" t="n">
-        <v>-0.8305</v>
+        <v>-1.2304</v>
       </c>
       <c r="I228" t="n">
-        <v>-67.48999999999999</v>
+        <v>10.12</v>
       </c>
       <c r="J228" t="n">
-        <v>325.1000000000001</v>
+        <v>1101.2</v>
       </c>
       <c r="K228" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L228" t="n">
         <v>3</v>
       </c>
       <c r="N228" t="n">
-        <v>0.0111</v>
+        <v>0.0027</v>
       </c>
       <c r="O228" t="n">
-        <v>42.64</v>
+        <v>53.55</v>
       </c>
       <c r="P228" t="n">
-        <v>0</v>
+        <v>0.5858</v>
       </c>
       <c r="Q228" t="n">
-        <v>0</v>
+        <v>0.7341</v>
       </c>
       <c r="R228" t="n">
-        <v>0</v>
+        <v>0.6516</v>
       </c>
       <c r="S228" t="n">
-        <v>0</v>
+        <v>-0.0231</v>
       </c>
       <c r="T228" t="n">
-        <v>82.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -16670,7 +16670,7 @@
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -16700,7 +16700,7 @@
         <v>3</v>
       </c>
       <c r="N229" t="n">
-        <v>0.032</v>
+        <v>0.0111</v>
       </c>
       <c r="O229" t="n">
         <v>42.64</v>
@@ -16718,21 +16718,21 @@
         <v>0</v>
       </c>
       <c r="T229" t="n">
-        <v>62.3</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -16741,60 +16741,60 @@
         </is>
       </c>
       <c r="E230" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F230" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G230" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I230" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J230" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K230" t="n">
         <v>1</v>
       </c>
       <c r="L230" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N230" t="n">
-        <v>0.0284</v>
+        <v>0.032</v>
       </c>
       <c r="O230" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P230" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q230" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R230" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S230" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T230" t="n">
-        <v>79.8</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -16803,60 +16803,60 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="F231" t="n">
-        <v>0.4732</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G231" t="n">
-        <v>-1.1536</v>
+        <v>-0.8347</v>
       </c>
       <c r="I231" t="n">
-        <v>41.21</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J231" t="n">
-        <v>1412.1</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K231" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L231" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N231" t="n">
-        <v>0.0231</v>
+        <v>0.0284</v>
       </c>
       <c r="O231" t="n">
-        <v>48.31</v>
+        <v>44.07</v>
       </c>
       <c r="P231" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.5588</v>
       </c>
       <c r="Q231" t="n">
-        <v>0.3418</v>
+        <v>0.1177</v>
       </c>
       <c r="R231" t="n">
-        <v>0.4395</v>
+        <v>0.1945</v>
       </c>
       <c r="S231" t="n">
-        <v>0.0329</v>
+        <v>-0.0101</v>
       </c>
       <c r="T231" t="n">
-        <v>1311.2</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -16865,39 +16865,51 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F232" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G232" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I232" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J232" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K232" t="n">
         <v>4</v>
       </c>
       <c r="L232" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N232" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O232" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P232" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R232" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S232" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T232" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -16906,7 +16918,7 @@
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -16915,51 +16927,39 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F233" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G233" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I233" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J233" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K233" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L233" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N233" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O233" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P233" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q233" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R233" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S233" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T233" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -16968,7 +16968,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -16977,51 +16977,51 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F234" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G234" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I234" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J234" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K234" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L234" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N234" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O234" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P234" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q234" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R234" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S234" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T234" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -17030,7 +17030,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -17039,60 +17039,60 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F235" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G235" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I235" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J235" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K235" t="n">
         <v>1</v>
       </c>
       <c r="L235" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N235" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O235" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P235" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q235" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R235" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S235" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T235" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -17101,60 +17101,60 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F236" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G236" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I236" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J236" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K236" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L236" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N236" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O236" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P236" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q236" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R236" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S236" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T236" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -17163,113 +17163,113 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="F237" t="n">
-        <v>0.9243</v>
+        <v>-1.0225</v>
       </c>
       <c r="G237" t="n">
-        <v>-1.2246</v>
+        <v>-0.2617</v>
       </c>
       <c r="I237" t="n">
-        <v>116.09</v>
+        <v>-65.97</v>
       </c>
       <c r="J237" t="n">
-        <v>2160.9</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K237" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L237" t="n">
         <v>3</v>
       </c>
       <c r="N237" t="n">
-        <v>0.0283</v>
+        <v>-0.0076</v>
       </c>
       <c r="O237" t="n">
-        <v>53.93</v>
+        <v>40.96</v>
       </c>
       <c r="P237" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5526</v>
       </c>
       <c r="Q237" t="n">
-        <v>0.7548</v>
+        <v>0.0334</v>
       </c>
       <c r="R237" t="n">
-        <v>0.6592</v>
+        <v>0.0631</v>
       </c>
       <c r="S237" t="n">
-        <v>-0.0266</v>
+        <v>-0.0156</v>
       </c>
       <c r="T237" t="n">
-        <v>97.5</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="F238" t="n">
-        <v>0.5694</v>
+        <v>0.9243</v>
       </c>
       <c r="G238" t="n">
-        <v>-1.3423</v>
+        <v>-1.2246</v>
       </c>
       <c r="I238" t="n">
-        <v>54.77</v>
+        <v>116.09</v>
       </c>
       <c r="J238" t="n">
-        <v>1547.7</v>
+        <v>2160.9</v>
       </c>
       <c r="K238" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L238" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N238" t="n">
-        <v>0.0103</v>
+        <v>0.0283</v>
       </c>
       <c r="O238" t="n">
-        <v>51.13</v>
+        <v>53.93</v>
       </c>
       <c r="P238" t="n">
-        <v>0.5968</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="Q238" t="n">
-        <v>0.5364</v>
+        <v>0.7548</v>
       </c>
       <c r="R238" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="S238" t="n">
-        <v>0.0098</v>
+        <v>-0.0266</v>
       </c>
       <c r="T238" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
@@ -17278,12 +17278,12 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E239" t="n">
@@ -17326,21 +17326,21 @@
         <v>0.0098</v>
       </c>
       <c r="T239" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>220</v>
+        <v>39</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>MLP seq=35 seed=13 (#6/10 user directive) - Picard 2021</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
@@ -17349,60 +17349,60 @@
         </is>
       </c>
       <c r="E240" t="n">
-        <v>-1.6978</v>
+        <v>-1.5423</v>
       </c>
       <c r="F240" t="n">
-        <v>-0.9978</v>
+        <v>0.5694</v>
       </c>
       <c r="G240" t="n">
-        <v>-0.2639</v>
+        <v>-1.3423</v>
       </c>
       <c r="I240" t="n">
-        <v>-73.51000000000001</v>
+        <v>54.77</v>
       </c>
       <c r="J240" t="n">
-        <v>264.8999999999999</v>
+        <v>1547.7</v>
       </c>
       <c r="K240" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L240" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N240" t="n">
-        <v>-0.0151</v>
+        <v>0.0103</v>
       </c>
       <c r="O240" t="n">
-        <v>44.4</v>
+        <v>51.13</v>
       </c>
       <c r="P240" t="n">
-        <v>0.5636</v>
+        <v>0.5968</v>
       </c>
       <c r="Q240" t="n">
-        <v>0.1858</v>
+        <v>0.5364</v>
       </c>
       <c r="R240" t="n">
-        <v>0.2794</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S240" t="n">
-        <v>-0.0159</v>
+        <v>0.0098</v>
       </c>
       <c r="T240" t="n">
-        <v>30.8</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>14</v>
+        <v>220</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>MLP seq=35 seed=13 (#6/10 user directive) - Picard 2021</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -17411,60 +17411,60 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>-1.7077</v>
+        <v>-1.6978</v>
       </c>
       <c r="F241" t="n">
-        <v>0.4944</v>
+        <v>-0.9978</v>
       </c>
       <c r="G241" t="n">
-        <v>-1.5077</v>
+        <v>-0.2639</v>
       </c>
       <c r="I241" t="n">
-        <v>44.06</v>
+        <v>-73.51000000000001</v>
       </c>
       <c r="J241" t="n">
-        <v>1440.6</v>
+        <v>264.8999999999999</v>
       </c>
       <c r="K241" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L241" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N241" t="n">
-        <v>0.0102</v>
+        <v>-0.0151</v>
       </c>
       <c r="O241" t="n">
-        <v>52.26</v>
+        <v>44.4</v>
       </c>
       <c r="P241" t="n">
-        <v>0.5959</v>
+        <v>0.5636</v>
       </c>
       <c r="Q241" t="n">
-        <v>0.6044</v>
+        <v>0.1858</v>
       </c>
       <c r="R241" t="n">
-        <v>0.6002</v>
+        <v>0.2794</v>
       </c>
       <c r="S241" t="n">
-        <v>0.0091</v>
+        <v>-0.0159</v>
       </c>
       <c r="T241" t="n">
-        <v>1076.7</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -17473,60 +17473,60 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F242" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G242" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I242" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J242" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K242" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L242" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N242" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O242" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P242" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q242" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R242" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S242" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T242" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -17535,60 +17535,60 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F243" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G243" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I243" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J243" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K243" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L243" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N243" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O243" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P243" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q243" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R243" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S243" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T243" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -17597,60 +17597,60 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="F244" t="n">
-        <v>-0.1044</v>
+        <v>-1.2201</v>
       </c>
       <c r="G244" t="n">
-        <v>-1.6173</v>
+        <v>-0.255</v>
       </c>
       <c r="I244" t="n">
-        <v>-18.65</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J244" t="n">
-        <v>813.5</v>
+        <v>282.4</v>
       </c>
       <c r="K244" t="n">
+        <v>1</v>
+      </c>
+      <c r="L244" t="n">
         <v>3</v>
       </c>
-      <c r="L244" t="n">
-        <v>2</v>
-      </c>
       <c r="N244" t="n">
-        <v>-0.0416</v>
+        <v>-0.0322</v>
       </c>
       <c r="O244" t="n">
-        <v>48.72</v>
+        <v>40.59</v>
       </c>
       <c r="P244" t="n">
-        <v>0.5679999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q244" t="n">
-        <v>0.5653</v>
+        <v>0</v>
       </c>
       <c r="R244" t="n">
-        <v>0.5666</v>
+        <v>0</v>
       </c>
       <c r="S244" t="n">
-        <v>-0.0596</v>
+        <v>0</v>
       </c>
       <c r="T244" t="n">
-        <v>73</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -17659,60 +17659,60 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F245" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G245" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I245" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J245" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K245" t="n">
         <v>3</v>
       </c>
       <c r="L245" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N245" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O245" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P245" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q245" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R245" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S245" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T245" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -17721,51 +17721,51 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F246" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G246" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I246" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J246" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K246" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L246" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N246" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O246" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P246" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q246" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R246" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S246" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T246" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
@@ -17774,7 +17774,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -17783,51 +17783,113 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F247" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G247" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I247" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J247" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K247" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L247" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N247" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O247" t="n">
         <v>47.65</v>
       </c>
       <c r="P247" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q247" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R247" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S247" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T247" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>41</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E248" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F248" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G248" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I248" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J248" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K248" t="n">
+        <v>4</v>
+      </c>
+      <c r="L248" t="n">
+        <v>2</v>
+      </c>
+      <c r="N248" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O248" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P248" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q247" t="n">
+      <c r="Q248" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R247" t="n">
+      <c r="R248" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S247" t="n">
+      <c r="S248" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T247" t="n">
+      <c r="T248" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T247"/>
-  <conditionalFormatting sqref="E2:E247">
+  <autoFilter ref="A1:T248"/>
+  <conditionalFormatting sqref="E2:E248">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -17849,7 +17911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K247"/>
+  <dimension ref="A1:K248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -26212,118 +26274,118 @@
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>110</v>
+        <v>247</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>-1.4189</v>
+        <v>-1.4181</v>
       </c>
       <c r="D226" t="n">
         <v>1000</v>
       </c>
       <c r="E226" t="n">
-        <v>942</v>
+        <v>1092.5</v>
       </c>
       <c r="F226" t="n">
-        <v>730.2384</v>
+        <v>846.9059999999999</v>
       </c>
       <c r="G226" t="n">
-        <v>637.6441708799999</v>
+        <v>824.3783003999999</v>
       </c>
       <c r="H226" t="n">
-        <v>706.8923278375679</v>
+        <v>849.0272115819599</v>
       </c>
       <c r="I226" t="n">
-        <v>605.0291433961744</v>
+        <v>607.8185807715251</v>
       </c>
       <c r="J226" t="n">
-        <v>435.9234978169437</v>
+        <v>416.7812008350348</v>
       </c>
       <c r="K226" t="n">
-        <v>412.9503294819908</v>
+        <v>375.9783212732849</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="D227" t="n">
         <v>1000</v>
       </c>
       <c r="E227" t="n">
-        <v>999.6</v>
+        <v>942</v>
       </c>
       <c r="F227" t="n">
-        <v>1076.66916</v>
+        <v>730.2384</v>
       </c>
       <c r="G227" t="n">
-        <v>1127.918612016</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H227" t="n">
-        <v>1009.261574031917</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I227" t="n">
-        <v>837.9898849187007</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J227" t="n">
-        <v>1032.403538219839</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K227" t="n">
-        <v>1101.161613865281</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="D228" t="n">
         <v>1000</v>
       </c>
       <c r="E228" t="n">
-        <v>1045.3</v>
+        <v>999.6</v>
       </c>
       <c r="F228" t="n">
-        <v>853.06933</v>
+        <v>1076.66916</v>
       </c>
       <c r="G228" t="n">
-        <v>749.933248003</v>
+        <v>1127.918612016</v>
       </c>
       <c r="H228" t="n">
-        <v>740.3341024285616</v>
+        <v>1009.261574031917</v>
       </c>
       <c r="I228" t="n">
-        <v>691.1759180273051</v>
+        <v>837.9898849187007</v>
       </c>
       <c r="J228" t="n">
-        <v>482.7172611502699</v>
+        <v>1032.403538219839</v>
       </c>
       <c r="K228" t="n">
-        <v>325.0618036585918</v>
+        <v>1101.161613865281</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
@@ -26360,118 +26422,118 @@
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D230" t="n">
         <v>1000</v>
       </c>
       <c r="E230" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F230" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G230" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H230" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I230" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J230" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K230" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="D231" t="n">
         <v>1000</v>
       </c>
       <c r="E231" t="n">
-        <v>1236.4</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F231" t="n">
-        <v>1500.74232</v>
+        <v>692.62656</v>
       </c>
       <c r="G231" t="n">
-        <v>1734.708047688</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H231" t="n">
-        <v>1677.809623723833</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I231" t="n">
-        <v>1544.088196713044</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J231" t="n">
-        <v>1750.069562154564</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K231" t="n">
-        <v>1412.131129702517</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D232" t="n">
         <v>1000</v>
       </c>
       <c r="E232" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F232" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G232" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H232" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I232" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J232" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K232" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
@@ -26479,36 +26541,36 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D233" t="n">
         <v>1000</v>
       </c>
       <c r="E233" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F233" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G233" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H233" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I233" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J233" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K233" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -26516,36 +26578,36 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D234" t="n">
         <v>1000</v>
       </c>
       <c r="E234" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F234" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G234" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H234" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I234" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J234" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K234" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -26553,147 +26615,147 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D235" t="n">
         <v>1000</v>
       </c>
       <c r="E235" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F235" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G235" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H235" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I235" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J235" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K235" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D236" t="n">
         <v>1000</v>
       </c>
       <c r="E236" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F236" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G236" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H236" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I236" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J236" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K236" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="D237" t="n">
         <v>1000</v>
       </c>
       <c r="E237" t="n">
-        <v>1127.9</v>
+        <v>1141.5</v>
       </c>
       <c r="F237" t="n">
-        <v>1108.7257</v>
+        <v>884.8908</v>
       </c>
       <c r="G237" t="n">
-        <v>1251.64044273</v>
+        <v>789.49957176</v>
       </c>
       <c r="H237" t="n">
-        <v>1235.619445063056</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I237" t="n">
-        <v>1202.010596157341</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J237" t="n">
-        <v>1559.849150633381</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K237" t="n">
-        <v>2161.015013287486</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="D238" t="n">
         <v>1000</v>
       </c>
       <c r="E238" t="n">
-        <v>1342</v>
+        <v>1127.9</v>
       </c>
       <c r="F238" t="n">
-        <v>1365.6192</v>
+        <v>1108.7257</v>
       </c>
       <c r="G238" t="n">
-        <v>1401.67154688</v>
+        <v>1251.64044273</v>
       </c>
       <c r="H238" t="n">
-        <v>1356.1172216064</v>
+        <v>1235.619445063056</v>
       </c>
       <c r="I238" t="n">
-        <v>1614.321940600259</v>
+        <v>1202.010596157341</v>
       </c>
       <c r="J238" t="n">
-        <v>1682.93062307577</v>
+        <v>1559.849150633381</v>
       </c>
       <c r="K238" t="n">
-        <v>1547.623000980478</v>
+        <v>2161.015013287486</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
@@ -26730,266 +26792,266 @@
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>220</v>
+        <v>39</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>-1.6978</v>
+        <v>-1.5423</v>
       </c>
       <c r="D240" t="n">
         <v>1000</v>
       </c>
       <c r="E240" t="n">
-        <v>901.6999999999999</v>
+        <v>1342</v>
       </c>
       <c r="F240" t="n">
-        <v>774.1094499999999</v>
+        <v>1365.6192</v>
       </c>
       <c r="G240" t="n">
-        <v>749.570180435</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H240" t="n">
-        <v>634.3612437021405</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I240" t="n">
-        <v>618.502212609587</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J240" t="n">
-        <v>338.3207102974441</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K240" t="n">
-        <v>264.9389482339285</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>14</v>
+        <v>220</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>-1.7077</v>
+        <v>-1.6978</v>
       </c>
       <c r="D241" t="n">
         <v>1000</v>
       </c>
       <c r="E241" t="n">
-        <v>1067.7</v>
+        <v>901.6999999999999</v>
       </c>
       <c r="F241" t="n">
-        <v>1380.10902</v>
+        <v>774.1094499999999</v>
       </c>
       <c r="G241" t="n">
-        <v>1542.409840752</v>
+        <v>749.570180435</v>
       </c>
       <c r="H241" t="n">
-        <v>1525.751814471878</v>
+        <v>634.3612437021405</v>
       </c>
       <c r="I241" t="n">
-        <v>1571.066643361693</v>
+        <v>618.502212609587</v>
       </c>
       <c r="J241" t="n">
-        <v>1715.918987879641</v>
+        <v>338.3207102974441</v>
       </c>
       <c r="K241" t="n">
-        <v>1440.513990324959</v>
+        <v>264.9389482339285</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D242" t="n">
         <v>1000</v>
       </c>
       <c r="E242" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F242" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G242" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H242" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I242" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J242" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K242" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D243" t="n">
         <v>1000</v>
       </c>
       <c r="E243" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F243" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G243" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H243" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I243" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J243" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K243" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="D244" t="n">
         <v>1000</v>
       </c>
       <c r="E244" t="n">
-        <v>1222.6</v>
+        <v>942</v>
       </c>
       <c r="F244" t="n">
-        <v>1122.46906</v>
+        <v>730.2384</v>
       </c>
       <c r="G244" t="n">
-        <v>1222.481053246</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H244" t="n">
-        <v>1198.520424602378</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I244" t="n">
-        <v>1133.440765546469</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J244" t="n">
-        <v>1142.73497982395</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K244" t="n">
-        <v>813.6273056346525</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D245" t="n">
         <v>1000</v>
       </c>
       <c r="E245" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F245" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G245" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H245" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I245" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J245" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K245" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D246" t="n">
         <v>1000</v>
       </c>
       <c r="E246" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F246" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G246" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H246" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I246" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J246" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K246" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
@@ -26997,30 +27059,67 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D247" t="n">
         <v>1000</v>
       </c>
       <c r="E247" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F247" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G247" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H247" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I247" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J247" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K247" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>41</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D248" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E248" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F247" t="n">
+      <c r="F248" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G247" t="n">
+      <c r="G248" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H247" t="n">
+      <c r="H248" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I247" t="n">
+      <c r="I248" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J247" t="n">
+      <c r="J248" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K247" t="n">
+      <c r="K248" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>

<commit_message>
QQQ exp 248 xLSTM seed=11 -1.34; exp 249 seed=3 #8/10
</commit_message>
<xml_diff>
--- a/docs/index_stock_dashboard/autoresearch_equity.xlsx
+++ b/docs/index_stock_dashboard/autoresearch_equity.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Champion Detail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$248</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$T$249</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2133,7 +2133,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>250</row>
+      <row>251</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="4320000"/>
@@ -2470,7 +2470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T248"/>
+  <dimension ref="A1:T249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -16351,16 +16351,16 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>27</v>
+        <v>248</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
+          <t>xLSTM seq=60 seed=11 #7/10</t>
         </is>
       </c>
       <c r="D224" t="inlineStr">
@@ -16369,60 +16369,60 @@
         </is>
       </c>
       <c r="E224" t="n">
-        <v>-1.3564</v>
+        <v>-1.3385</v>
       </c>
       <c r="F224" t="n">
-        <v>0.011</v>
+        <v>-0.7385</v>
       </c>
       <c r="G224" t="n">
-        <v>-0.9564</v>
+        <v>-0.1564</v>
       </c>
       <c r="I224" t="n">
-        <v>-17.26</v>
+        <v>-55.45</v>
       </c>
       <c r="J224" t="n">
-        <v>827.4</v>
+        <v>445.5</v>
       </c>
       <c r="K224" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L224" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N224" t="n">
-        <v>-0.0003</v>
+        <v>0.0009</v>
       </c>
       <c r="O224" t="n">
-        <v>48.19</v>
+        <v>47.21</v>
       </c>
       <c r="P224" t="n">
-        <v>0.5666</v>
+        <v>0.5839</v>
       </c>
       <c r="Q224" t="n">
-        <v>0.4114</v>
+        <v>0.3822</v>
       </c>
       <c r="R224" t="n">
-        <v>0.4767</v>
+        <v>0.462</v>
       </c>
       <c r="S224" t="n">
-        <v>-0.009900000000000001</v>
+        <v>-0.0138</v>
       </c>
       <c r="T224" t="n">
-        <v>37.9</v>
+        <v>1335.6</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
+          <t>MLP @ FX-Exp32 lr=1e-4 (down from 3e-4) - flat-minima hill-climb on lucky-seed champ; Kesk</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
@@ -16431,60 +16431,60 @@
         </is>
       </c>
       <c r="E225" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="F225" t="n">
-        <v>-0.6131</v>
+        <v>0.011</v>
       </c>
       <c r="G225" t="n">
-        <v>-0.9054</v>
+        <v>-0.9564</v>
       </c>
       <c r="I225" t="n">
-        <v>-49.86</v>
+        <v>-17.26</v>
       </c>
       <c r="J225" t="n">
-        <v>501.4000000000001</v>
+        <v>827.4</v>
       </c>
       <c r="K225" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L225" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N225" t="n">
-        <v>0.0074</v>
+        <v>-0.0003</v>
       </c>
       <c r="O225" t="n">
-        <v>44.37</v>
+        <v>48.19</v>
       </c>
       <c r="P225" t="n">
-        <v>0.6127</v>
+        <v>0.5666</v>
       </c>
       <c r="Q225" t="n">
-        <v>0.1688</v>
+        <v>0.4114</v>
       </c>
       <c r="R225" t="n">
-        <v>0.2647</v>
+        <v>0.4767</v>
       </c>
       <c r="S225" t="n">
-        <v>0.0182</v>
+        <v>-0.009900000000000001</v>
       </c>
       <c r="T225" t="n">
-        <v>54.7</v>
+        <v>37.9</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>247</v>
+        <v>108</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>xlstm</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>xLSTM seq=60 seed=13 #6/10</t>
+          <t>iTransformer Liu 2024 ICLR baseline on QQQ - paper recipe lr=1e-4 bs=32 ep=100 pat=20 seq=</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
@@ -16493,19 +16493,19 @@
         </is>
       </c>
       <c r="E226" t="n">
-        <v>-1.4181</v>
+        <v>-1.4054</v>
       </c>
       <c r="F226" t="n">
-        <v>-0.9181</v>
+        <v>-0.6131</v>
       </c>
       <c r="G226" t="n">
-        <v>-0.0286</v>
+        <v>-0.9054</v>
       </c>
       <c r="I226" t="n">
-        <v>-62.4</v>
+        <v>-49.86</v>
       </c>
       <c r="J226" t="n">
-        <v>376</v>
+        <v>501.4000000000001</v>
       </c>
       <c r="K226" t="n">
         <v>2</v>
@@ -16514,39 +16514,39 @@
         <v>3</v>
       </c>
       <c r="N226" t="n">
-        <v>-0.01</v>
+        <v>0.0074</v>
       </c>
       <c r="O226" t="n">
-        <v>42.1</v>
+        <v>44.37</v>
       </c>
       <c r="P226" t="n">
-        <v>0.5412</v>
+        <v>0.6127</v>
       </c>
       <c r="Q226" t="n">
-        <v>0.1672</v>
+        <v>0.1688</v>
       </c>
       <c r="R226" t="n">
-        <v>0.2555</v>
+        <v>0.2647</v>
       </c>
       <c r="S226" t="n">
-        <v>-0.0493</v>
+        <v>0.0182</v>
       </c>
       <c r="T226" t="n">
-        <v>1037.1</v>
+        <v>54.7</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>110</v>
+        <v>247</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
+          <t>xLSTM seq=60 seed=13 #6/10</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
@@ -16555,60 +16555,60 @@
         </is>
       </c>
       <c r="E227" t="n">
-        <v>-1.4189</v>
+        <v>-1.4181</v>
       </c>
       <c r="F227" t="n">
-        <v>-0.8189</v>
+        <v>-0.9181</v>
       </c>
       <c r="G227" t="n">
-        <v>1.1456</v>
+        <v>-0.0286</v>
       </c>
       <c r="I227" t="n">
-        <v>-58.71</v>
+        <v>-62.4</v>
       </c>
       <c r="J227" t="n">
-        <v>412.9</v>
+        <v>376</v>
       </c>
       <c r="K227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L227" t="n">
         <v>3</v>
       </c>
       <c r="N227" t="n">
-        <v>0.0089</v>
+        <v>-0.01</v>
       </c>
       <c r="O227" t="n">
-        <v>41.44</v>
+        <v>42.1</v>
       </c>
       <c r="P227" t="n">
-        <v>0.68</v>
+        <v>0.5412</v>
       </c>
       <c r="Q227" t="n">
-        <v>0.0271</v>
+        <v>0.1672</v>
       </c>
       <c r="R227" t="n">
-        <v>0.0521</v>
+        <v>0.2555</v>
       </c>
       <c r="S227" t="n">
-        <v>0.0277</v>
+        <v>-0.0493</v>
       </c>
       <c r="T227" t="n">
-        <v>8786.5</v>
+        <v>1037.1</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
+          <t>PatchTST Nie 2023 ICLR baseline on QQQ at paper-required seq=60 (FX violated with seq=10)</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -16617,60 +16617,60 @@
         </is>
       </c>
       <c r="E228" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="F228" t="n">
-        <v>0.2144</v>
+        <v>-0.8189</v>
       </c>
       <c r="G228" t="n">
-        <v>-1.2304</v>
+        <v>1.1456</v>
       </c>
       <c r="I228" t="n">
-        <v>10.12</v>
+        <v>-58.71</v>
       </c>
       <c r="J228" t="n">
-        <v>1101.2</v>
+        <v>412.9</v>
       </c>
       <c r="K228" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L228" t="n">
         <v>3</v>
       </c>
       <c r="N228" t="n">
-        <v>0.0027</v>
+        <v>0.0089</v>
       </c>
       <c r="O228" t="n">
-        <v>53.55</v>
+        <v>41.44</v>
       </c>
       <c r="P228" t="n">
-        <v>0.5858</v>
+        <v>0.68</v>
       </c>
       <c r="Q228" t="n">
-        <v>0.7341</v>
+        <v>0.0271</v>
       </c>
       <c r="R228" t="n">
-        <v>0.6516</v>
+        <v>0.0521</v>
       </c>
       <c r="S228" t="n">
-        <v>-0.0231</v>
+        <v>0.0277</v>
       </c>
       <c r="T228" t="n">
-        <v>69.40000000000001</v>
+        <v>8786.5</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
+          <t>iTransformer paper-recipe seed=99 (3-seed median lock) - Picard 2021</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
@@ -16679,51 +16679,51 @@
         </is>
       </c>
       <c r="E229" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="F229" t="n">
-        <v>-0.6042</v>
+        <v>0.2144</v>
       </c>
       <c r="G229" t="n">
-        <v>-0.8305</v>
+        <v>-1.2304</v>
       </c>
       <c r="I229" t="n">
-        <v>-67.48999999999999</v>
+        <v>10.12</v>
       </c>
       <c r="J229" t="n">
-        <v>325.1000000000001</v>
+        <v>1101.2</v>
       </c>
       <c r="K229" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L229" t="n">
         <v>3</v>
       </c>
       <c r="N229" t="n">
-        <v>0.0111</v>
+        <v>0.0027</v>
       </c>
       <c r="O229" t="n">
-        <v>42.64</v>
+        <v>53.55</v>
       </c>
       <c r="P229" t="n">
-        <v>0</v>
+        <v>0.5858</v>
       </c>
       <c r="Q229" t="n">
-        <v>0</v>
+        <v>0.7341</v>
       </c>
       <c r="R229" t="n">
-        <v>0</v>
+        <v>0.6516</v>
       </c>
       <c r="S229" t="n">
-        <v>0</v>
+        <v>-0.0231</v>
       </c>
       <c r="T229" t="n">
-        <v>82.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -16732,7 +16732,7 @@
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
+          <t>N-BEATS Oreshkin 2020 ICLR baseline on QQQ - paper recipe (FX paper section 4.7 all 8 conf</t>
         </is>
       </c>
       <c r="D230" t="inlineStr">
@@ -16762,7 +16762,7 @@
         <v>3</v>
       </c>
       <c r="N230" t="n">
-        <v>0.032</v>
+        <v>0.0111</v>
       </c>
       <c r="O230" t="n">
         <v>42.64</v>
@@ -16780,21 +16780,21 @@
         <v>0</v>
       </c>
       <c r="T230" t="n">
-        <v>62.3</v>
+        <v>82.40000000000001</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
+          <t>N-BEATS seed=0 (variance baseline) - Oreshkin 2020 ICLR Section 4.2 bootstrap; Picard 2021</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
@@ -16803,60 +16803,60 @@
         </is>
       </c>
       <c r="E231" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="F231" t="n">
-        <v>-0.6758999999999999</v>
+        <v>-0.6042</v>
       </c>
       <c r="G231" t="n">
-        <v>-0.8347</v>
+        <v>-0.8305</v>
       </c>
       <c r="I231" t="n">
-        <v>-70.84999999999999</v>
+        <v>-67.48999999999999</v>
       </c>
       <c r="J231" t="n">
-        <v>291.5000000000001</v>
+        <v>325.1000000000001</v>
       </c>
       <c r="K231" t="n">
         <v>1</v>
       </c>
       <c r="L231" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N231" t="n">
-        <v>0.0284</v>
+        <v>0.032</v>
       </c>
       <c r="O231" t="n">
-        <v>44.07</v>
+        <v>42.64</v>
       </c>
       <c r="P231" t="n">
-        <v>0.5588</v>
+        <v>0</v>
       </c>
       <c r="Q231" t="n">
-        <v>0.1177</v>
+        <v>0</v>
       </c>
       <c r="R231" t="n">
-        <v>0.1945</v>
+        <v>0</v>
       </c>
       <c r="S231" t="n">
-        <v>-0.0101</v>
+        <v>0</v>
       </c>
       <c r="T231" t="n">
-        <v>79.8</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
+          <t>LSTM @ exp 8 baseline ep=200 pat=30 (up from 100/15) - Goyal 2017 longer training; Fischer</t>
         </is>
       </c>
       <c r="D232" t="inlineStr">
@@ -16865,60 +16865,60 @@
         </is>
       </c>
       <c r="E232" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="F232" t="n">
-        <v>0.4732</v>
+        <v>-0.6758999999999999</v>
       </c>
       <c r="G232" t="n">
-        <v>-1.1536</v>
+        <v>-0.8347</v>
       </c>
       <c r="I232" t="n">
-        <v>41.21</v>
+        <v>-70.84999999999999</v>
       </c>
       <c r="J232" t="n">
-        <v>1412.1</v>
+        <v>291.5000000000001</v>
       </c>
       <c r="K232" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L232" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N232" t="n">
-        <v>0.0231</v>
+        <v>0.0284</v>
       </c>
       <c r="O232" t="n">
-        <v>48.31</v>
+        <v>44.07</v>
       </c>
       <c r="P232" t="n">
-        <v>0.6153999999999999</v>
+        <v>0.5588</v>
       </c>
       <c r="Q232" t="n">
-        <v>0.3418</v>
+        <v>0.1177</v>
       </c>
       <c r="R232" t="n">
-        <v>0.4395</v>
+        <v>0.1945</v>
       </c>
       <c r="S232" t="n">
-        <v>0.0329</v>
+        <v>-0.0101</v>
       </c>
       <c r="T232" t="n">
-        <v>1311.2</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
+          <t>CatBoost lr=0.05 n_est=1000 seed=99 (3-seed median lock) - per CLAUDE.md 3-seed median rul</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
@@ -16927,39 +16927,51 @@
         </is>
       </c>
       <c r="E233" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="F233" t="n">
-        <v>-0.0343</v>
+        <v>0.4732</v>
       </c>
       <c r="G233" t="n">
-        <v>-1.2001</v>
+        <v>-1.1536</v>
       </c>
       <c r="I233" t="n">
-        <v>-22.74</v>
+        <v>41.21</v>
       </c>
       <c r="J233" t="n">
-        <v>772.5999999999999</v>
+        <v>1412.1</v>
       </c>
       <c r="K233" t="n">
         <v>4</v>
       </c>
       <c r="L233" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N233" t="n">
-        <v>-0.008200000000000001</v>
+        <v>0.0231</v>
       </c>
       <c r="O233" t="n">
-        <v>47.05</v>
+        <v>48.31</v>
+      </c>
+      <c r="P233" t="n">
+        <v>0.6153999999999999</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>0.3418</v>
+      </c>
+      <c r="R233" t="n">
+        <v>0.4395</v>
+      </c>
+      <c r="S233" t="n">
+        <v>0.0329</v>
       </c>
       <c r="T233" t="n">
-        <v>38.6</v>
+        <v>1311.2</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -16968,7 +16980,7 @@
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
+          <t>MLP @ FX-Exp32 HPs seed=7 — multi-seed variance check on champion</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
@@ -16977,51 +16989,39 @@
         </is>
       </c>
       <c r="E234" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="F234" t="n">
-        <v>-0.4997</v>
+        <v>-0.0343</v>
       </c>
       <c r="G234" t="n">
-        <v>-1.0008</v>
+        <v>-1.2001</v>
       </c>
       <c r="I234" t="n">
-        <v>-61.92</v>
+        <v>-22.74</v>
       </c>
       <c r="J234" t="n">
-        <v>380.8</v>
+        <v>772.5999999999999</v>
       </c>
       <c r="K234" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L234" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N234" t="n">
-        <v>-0.0369</v>
+        <v>-0.008200000000000001</v>
       </c>
       <c r="O234" t="n">
-        <v>46.98</v>
-      </c>
-      <c r="P234" t="n">
-        <v>0.5685</v>
-      </c>
-      <c r="Q234" t="n">
-        <v>0.3086</v>
-      </c>
-      <c r="R234" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="S234" t="n">
-        <v>-0.0052</v>
+        <v>47.05</v>
       </c>
       <c r="T234" t="n">
-        <v>36</v>
+        <v>38.6</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -17030,7 +17030,7 @@
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
+          <t>MLP @ FX-Exp32 HPs seed=42 — fills the missing seed (we have 0,7,99). 4-seed multi-seed ta</t>
         </is>
       </c>
       <c r="D235" t="inlineStr">
@@ -17039,51 +17039,51 @@
         </is>
       </c>
       <c r="E235" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="F235" t="n">
-        <v>-0.5149</v>
+        <v>-0.4997</v>
       </c>
       <c r="G235" t="n">
-        <v>-0.9094</v>
+        <v>-1.0008</v>
       </c>
       <c r="I235" t="n">
-        <v>-62.76</v>
+        <v>-61.92</v>
       </c>
       <c r="J235" t="n">
-        <v>372.4000000000001</v>
+        <v>380.8</v>
       </c>
       <c r="K235" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L235" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N235" t="n">
-        <v>-0.0196</v>
+        <v>-0.0369</v>
       </c>
       <c r="O235" t="n">
-        <v>43.43</v>
+        <v>46.98</v>
       </c>
       <c r="P235" t="n">
-        <v>0.524</v>
+        <v>0.5685</v>
       </c>
       <c r="Q235" t="n">
-        <v>0.1487</v>
+        <v>0.3086</v>
       </c>
       <c r="R235" t="n">
-        <v>0.2317</v>
+        <v>0.4</v>
       </c>
       <c r="S235" t="n">
-        <v>-0.043</v>
+        <v>-0.0052</v>
       </c>
       <c r="T235" t="n">
-        <v>45.9</v>
+        <v>36</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
@@ -17092,7 +17092,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
+          <t>MLP @ FX-Exp32 bs=16 (down from 32) - small-batch flat-minima per Keskar 2017 ICLR; last M</t>
         </is>
       </c>
       <c r="D236" t="inlineStr">
@@ -17101,60 +17101,60 @@
         </is>
       </c>
       <c r="E236" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="F236" t="n">
-        <v>-0.5178</v>
+        <v>-0.5149</v>
       </c>
       <c r="G236" t="n">
-        <v>-0.9134</v>
+        <v>-0.9094</v>
       </c>
       <c r="I236" t="n">
-        <v>-62.95</v>
+        <v>-62.76</v>
       </c>
       <c r="J236" t="n">
-        <v>370.4999999999999</v>
+        <v>372.4000000000001</v>
       </c>
       <c r="K236" t="n">
         <v>1</v>
       </c>
       <c r="L236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N236" t="n">
-        <v>-0.0025</v>
+        <v>-0.0196</v>
       </c>
       <c r="O236" t="n">
-        <v>44.99</v>
+        <v>43.43</v>
       </c>
       <c r="P236" t="n">
-        <v>0.5558999999999999</v>
+        <v>0.524</v>
       </c>
       <c r="Q236" t="n">
-        <v>0.2032</v>
+        <v>0.1487</v>
       </c>
       <c r="R236" t="n">
-        <v>0.2976</v>
+        <v>0.2317</v>
       </c>
       <c r="S236" t="n">
-        <v>-0.0171</v>
+        <v>-0.043</v>
       </c>
       <c r="T236" t="n">
-        <v>18.8</v>
+        <v>45.9</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
+          <t>MLP @ exp 6 bs=64 (up from 32) - Keskar 2017 reverse direction; larger batch stability tes</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
@@ -17163,60 +17163,60 @@
         </is>
       </c>
       <c r="E237" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="F237" t="n">
-        <v>-1.0225</v>
+        <v>-0.5178</v>
       </c>
       <c r="G237" t="n">
-        <v>-0.2617</v>
+        <v>-0.9134</v>
       </c>
       <c r="I237" t="n">
-        <v>-65.97</v>
+        <v>-62.95</v>
       </c>
       <c r="J237" t="n">
-        <v>340.3000000000001</v>
+        <v>370.4999999999999</v>
       </c>
       <c r="K237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L237" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N237" t="n">
-        <v>-0.0076</v>
+        <v>-0.0025</v>
       </c>
       <c r="O237" t="n">
-        <v>40.96</v>
+        <v>44.99</v>
       </c>
       <c r="P237" t="n">
-        <v>0.5526</v>
+        <v>0.5558999999999999</v>
       </c>
       <c r="Q237" t="n">
-        <v>0.0334</v>
+        <v>0.2032</v>
       </c>
       <c r="R237" t="n">
-        <v>0.0631</v>
+        <v>0.2976</v>
       </c>
       <c r="S237" t="n">
-        <v>-0.0156</v>
+        <v>-0.0171</v>
       </c>
       <c r="T237" t="n">
-        <v>938.7</v>
+        <v>18.8</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
+          <t>dMamba num_layers=3 (up from 2) - depth axis untested</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
@@ -17225,113 +17225,113 @@
         </is>
       </c>
       <c r="E238" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="F238" t="n">
-        <v>0.9243</v>
+        <v>-1.0225</v>
       </c>
       <c r="G238" t="n">
-        <v>-1.2246</v>
+        <v>-0.2617</v>
       </c>
       <c r="I238" t="n">
-        <v>116.09</v>
+        <v>-65.97</v>
       </c>
       <c r="J238" t="n">
-        <v>2160.9</v>
+        <v>340.3000000000001</v>
       </c>
       <c r="K238" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L238" t="n">
         <v>3</v>
       </c>
       <c r="N238" t="n">
-        <v>0.0283</v>
+        <v>-0.0076</v>
       </c>
       <c r="O238" t="n">
-        <v>53.93</v>
+        <v>40.96</v>
       </c>
       <c r="P238" t="n">
-        <v>0.5852000000000001</v>
+        <v>0.5526</v>
       </c>
       <c r="Q238" t="n">
-        <v>0.7548</v>
+        <v>0.0334</v>
       </c>
       <c r="R238" t="n">
-        <v>0.6592</v>
+        <v>0.0631</v>
       </c>
       <c r="S238" t="n">
-        <v>-0.0266</v>
+        <v>-0.0156</v>
       </c>
       <c r="T238" t="n">
-        <v>97.5</v>
+        <v>938.7</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>iTransformer paper-recipe lr=5e-5 warmup=10 (Liu 2024 ICLR Section 4.1) - one knob from ex</t>
         </is>
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>KEEP</t>
+          <t>DISCARD</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="F239" t="n">
-        <v>0.5694</v>
+        <v>0.9243</v>
       </c>
       <c r="G239" t="n">
-        <v>-1.3423</v>
+        <v>-1.2246</v>
       </c>
       <c r="I239" t="n">
-        <v>54.77</v>
+        <v>116.09</v>
       </c>
       <c r="J239" t="n">
-        <v>1547.7</v>
+        <v>2160.9</v>
       </c>
       <c r="K239" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L239" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N239" t="n">
-        <v>0.0103</v>
+        <v>0.0283</v>
       </c>
       <c r="O239" t="n">
-        <v>51.13</v>
+        <v>53.93</v>
       </c>
       <c r="P239" t="n">
-        <v>0.5968</v>
+        <v>0.5852000000000001</v>
       </c>
       <c r="Q239" t="n">
-        <v>0.5364</v>
+        <v>0.7548</v>
       </c>
       <c r="R239" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.6592</v>
       </c>
       <c r="S239" t="n">
-        <v>0.0098</v>
+        <v>-0.0266</v>
       </c>
       <c r="T239" t="n">
-        <v>97.8</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
@@ -17340,12 +17340,12 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
+          <t>smoke</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>DISCARD</t>
+          <t>KEEP</t>
         </is>
       </c>
       <c r="E240" t="n">
@@ -17388,21 +17388,21 @@
         <v>0.0098</v>
       </c>
       <c r="T240" t="n">
-        <v>49.8</v>
+        <v>97.8</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>220</v>
+        <v>39</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>MLP seq=35 seed=13 (#6/10 user directive) - Picard 2021</t>
+          <t>XGBoost @ exp 1 max_depth=4 (down from 6) - Chen-Guestrin 2016 regularised tabular default</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
@@ -17411,60 +17411,60 @@
         </is>
       </c>
       <c r="E241" t="n">
-        <v>-1.6978</v>
+        <v>-1.5423</v>
       </c>
       <c r="F241" t="n">
-        <v>-0.9978</v>
+        <v>0.5694</v>
       </c>
       <c r="G241" t="n">
-        <v>-0.2639</v>
+        <v>-1.3423</v>
       </c>
       <c r="I241" t="n">
-        <v>-73.51000000000001</v>
+        <v>54.77</v>
       </c>
       <c r="J241" t="n">
-        <v>264.8999999999999</v>
+        <v>1547.7</v>
       </c>
       <c r="K241" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L241" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N241" t="n">
-        <v>-0.0151</v>
+        <v>0.0103</v>
       </c>
       <c r="O241" t="n">
-        <v>44.4</v>
+        <v>51.13</v>
       </c>
       <c r="P241" t="n">
-        <v>0.5636</v>
+        <v>0.5968</v>
       </c>
       <c r="Q241" t="n">
-        <v>0.1858</v>
+        <v>0.5364</v>
       </c>
       <c r="R241" t="n">
-        <v>0.2794</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="S241" t="n">
-        <v>-0.0159</v>
+        <v>0.0098</v>
       </c>
       <c r="T241" t="n">
-        <v>30.8</v>
+        <v>49.8</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>14</v>
+        <v>220</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
+          <t>MLP seq=35 seed=13 (#6/10 user directive) - Picard 2021</t>
         </is>
       </c>
       <c r="D242" t="inlineStr">
@@ -17473,60 +17473,60 @@
         </is>
       </c>
       <c r="E242" t="n">
-        <v>-1.7077</v>
+        <v>-1.6978</v>
       </c>
       <c r="F242" t="n">
-        <v>0.4944</v>
+        <v>-0.9978</v>
       </c>
       <c r="G242" t="n">
-        <v>-1.5077</v>
+        <v>-0.2639</v>
       </c>
       <c r="I242" t="n">
-        <v>44.06</v>
+        <v>-73.51000000000001</v>
       </c>
       <c r="J242" t="n">
-        <v>1440.6</v>
+        <v>264.8999999999999</v>
       </c>
       <c r="K242" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L242" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N242" t="n">
-        <v>0.0102</v>
+        <v>-0.0151</v>
       </c>
       <c r="O242" t="n">
-        <v>52.26</v>
+        <v>44.4</v>
       </c>
       <c r="P242" t="n">
-        <v>0.5959</v>
+        <v>0.5636</v>
       </c>
       <c r="Q242" t="n">
-        <v>0.6044</v>
+        <v>0.1858</v>
       </c>
       <c r="R242" t="n">
-        <v>0.6002</v>
+        <v>0.2794</v>
       </c>
       <c r="S242" t="n">
-        <v>0.0091</v>
+        <v>-0.0159</v>
       </c>
       <c r="T242" t="n">
-        <v>1076.7</v>
+        <v>30.8</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
+          <t>CatBoost @ FX-Exp236-lite n_est=500 (Prokhorenkova 2018 NeurIPS); QQQ — 3rd ensemble compo</t>
         </is>
       </c>
       <c r="D243" t="inlineStr">
@@ -17535,60 +17535,60 @@
         </is>
       </c>
       <c r="E243" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="F243" t="n">
-        <v>0.2915</v>
+        <v>0.4944</v>
       </c>
       <c r="G243" t="n">
-        <v>-1.4766</v>
+        <v>-1.5077</v>
       </c>
       <c r="I243" t="n">
-        <v>18.69</v>
+        <v>44.06</v>
       </c>
       <c r="J243" t="n">
-        <v>1186.9</v>
+        <v>1440.6</v>
       </c>
       <c r="K243" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L243" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N243" t="n">
-        <v>0.0052</v>
+        <v>0.0102</v>
       </c>
       <c r="O243" t="n">
-        <v>47.84</v>
+        <v>52.26</v>
       </c>
       <c r="P243" t="n">
-        <v>0.5918</v>
+        <v>0.5959</v>
       </c>
       <c r="Q243" t="n">
-        <v>0.3877</v>
+        <v>0.6044</v>
       </c>
       <c r="R243" t="n">
-        <v>0.4685</v>
+        <v>0.6002</v>
       </c>
       <c r="S243" t="n">
-        <v>-0.0009</v>
+        <v>0.0091</v>
       </c>
       <c r="T243" t="n">
-        <v>2340.4</v>
+        <v>1076.7</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
+          <t>XGBoost @ FX-Exp203 FULL n_est=1500 (Chen-Guestrin 2016 KDD); QQQ — final FX-winner baseli</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
@@ -17597,60 +17597,60 @@
         </is>
       </c>
       <c r="E244" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="F244" t="n">
-        <v>-1.2201</v>
+        <v>0.2915</v>
       </c>
       <c r="G244" t="n">
-        <v>-0.255</v>
+        <v>-1.4766</v>
       </c>
       <c r="I244" t="n">
-        <v>-71.76000000000001</v>
+        <v>18.69</v>
       </c>
       <c r="J244" t="n">
-        <v>282.4</v>
+        <v>1186.9</v>
       </c>
       <c r="K244" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L244" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N244" t="n">
-        <v>-0.0322</v>
+        <v>0.0052</v>
       </c>
       <c r="O244" t="n">
-        <v>40.59</v>
+        <v>47.84</v>
       </c>
       <c r="P244" t="n">
-        <v>0</v>
+        <v>0.5918</v>
       </c>
       <c r="Q244" t="n">
-        <v>0</v>
+        <v>0.3877</v>
       </c>
       <c r="R244" t="n">
-        <v>0</v>
+        <v>0.4685</v>
       </c>
       <c r="S244" t="n">
-        <v>0</v>
+        <v>-0.0009</v>
       </c>
       <c r="T244" t="n">
-        <v>464.4</v>
+        <v>2340.4</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
+          <t>PatchTSMixer seed=0 - multi-seed verify exp 145 +0.06</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
@@ -17659,60 +17659,60 @@
         </is>
       </c>
       <c r="E245" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="F245" t="n">
-        <v>-0.1044</v>
+        <v>-1.2201</v>
       </c>
       <c r="G245" t="n">
-        <v>-1.6173</v>
+        <v>-0.255</v>
       </c>
       <c r="I245" t="n">
-        <v>-18.65</v>
+        <v>-71.76000000000001</v>
       </c>
       <c r="J245" t="n">
-        <v>813.5</v>
+        <v>282.4</v>
       </c>
       <c r="K245" t="n">
+        <v>1</v>
+      </c>
+      <c r="L245" t="n">
         <v>3</v>
       </c>
-      <c r="L245" t="n">
-        <v>2</v>
-      </c>
       <c r="N245" t="n">
-        <v>-0.0416</v>
+        <v>-0.0322</v>
       </c>
       <c r="O245" t="n">
-        <v>48.72</v>
+        <v>40.59</v>
       </c>
       <c r="P245" t="n">
-        <v>0.5679999999999999</v>
+        <v>0</v>
       </c>
       <c r="Q245" t="n">
-        <v>0.5653</v>
+        <v>0</v>
       </c>
       <c r="R245" t="n">
-        <v>0.5666</v>
+        <v>0</v>
       </c>
       <c r="S245" t="n">
-        <v>-0.0596</v>
+        <v>0</v>
       </c>
       <c r="T245" t="n">
-        <v>73</v>
+        <v>464.4</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
+          <t>iTransformer paper-recipe seed=0 (variance check on exp 193 A_sh+0.92) - Picard 2021</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -17721,60 +17721,60 @@
         </is>
       </c>
       <c r="E246" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="F246" t="n">
-        <v>-0.3397</v>
+        <v>-0.1044</v>
       </c>
       <c r="G246" t="n">
-        <v>-1.8082</v>
+        <v>-1.6173</v>
       </c>
       <c r="I246" t="n">
-        <v>-51.44</v>
+        <v>-18.65</v>
       </c>
       <c r="J246" t="n">
-        <v>485.6</v>
+        <v>813.5</v>
       </c>
       <c r="K246" t="n">
         <v>3</v>
       </c>
       <c r="L246" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N246" t="n">
-        <v>-0.0003</v>
+        <v>-0.0416</v>
       </c>
       <c r="O246" t="n">
-        <v>45.06</v>
+        <v>48.72</v>
       </c>
       <c r="P246" t="n">
-        <v>0.5895</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="Q246" t="n">
-        <v>0.1388</v>
+        <v>0.5653</v>
       </c>
       <c r="R246" t="n">
-        <v>0.2247</v>
+        <v>0.5666</v>
       </c>
       <c r="S246" t="n">
-        <v>0.0137</v>
+        <v>-0.0596</v>
       </c>
       <c r="T246" t="n">
-        <v>40.3</v>
+        <v>73</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
+          <t>MLP hidden=96 + bs=16 - cross-axis combo of two known-good axes</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -17783,51 +17783,51 @@
         </is>
       </c>
       <c r="E247" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="F247" t="n">
-        <v>-0.0045</v>
+        <v>-0.3397</v>
       </c>
       <c r="G247" t="n">
-        <v>-2.1923</v>
+        <v>-1.8082</v>
       </c>
       <c r="I247" t="n">
-        <v>-10.56</v>
+        <v>-51.44</v>
       </c>
       <c r="J247" t="n">
-        <v>894.4</v>
+        <v>485.6</v>
       </c>
       <c r="K247" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="L247" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N247" t="n">
-        <v>-0.0018</v>
+        <v>-0.0003</v>
       </c>
       <c r="O247" t="n">
-        <v>47.65</v>
+        <v>45.06</v>
       </c>
       <c r="P247" t="n">
-        <v>0.583</v>
+        <v>0.5895</v>
       </c>
       <c r="Q247" t="n">
-        <v>0.4114</v>
+        <v>0.1388</v>
       </c>
       <c r="R247" t="n">
-        <v>0.4824</v>
+        <v>0.2247</v>
       </c>
       <c r="S247" t="n">
-        <v>-0.0161</v>
+        <v>0.0137</v>
       </c>
       <c r="T247" t="n">
-        <v>335.3</v>
+        <v>40.3</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
@@ -17836,7 +17836,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+          <t>xgboost SOTA-lite n_est=300 (Chen-Guestrin 2016 KDD); regime-aware folds + extended featur</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
@@ -17845,51 +17845,113 @@
         </is>
       </c>
       <c r="E248" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="F248" t="n">
-        <v>-0.0887</v>
+        <v>-0.0045</v>
       </c>
       <c r="G248" t="n">
-        <v>-2.3905</v>
+        <v>-2.1923</v>
       </c>
       <c r="I248" t="n">
-        <v>-17.48</v>
+        <v>-10.56</v>
       </c>
       <c r="J248" t="n">
-        <v>825.1999999999999</v>
+        <v>894.4</v>
       </c>
       <c r="K248" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L248" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N248" t="n">
-        <v>-0.0067</v>
+        <v>-0.0018</v>
       </c>
       <c r="O248" t="n">
         <v>47.65</v>
       </c>
       <c r="P248" t="n">
+        <v>0.583</v>
+      </c>
+      <c r="Q248" t="n">
+        <v>0.4114</v>
+      </c>
+      <c r="R248" t="n">
+        <v>0.4824</v>
+      </c>
+      <c r="S248" t="n">
+        <v>-0.0161</v>
+      </c>
+      <c r="T248" t="n">
+        <v>335.3</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>41</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>XGBoost depth=4 n_est=200 - upper capacity boundary test (sweet spot between 100 and 300)</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>DISCARD</t>
+        </is>
+      </c>
+      <c r="E249" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="F249" t="n">
+        <v>-0.0887</v>
+      </c>
+      <c r="G249" t="n">
+        <v>-2.3905</v>
+      </c>
+      <c r="I249" t="n">
+        <v>-17.48</v>
+      </c>
+      <c r="J249" t="n">
+        <v>825.1999999999999</v>
+      </c>
+      <c r="K249" t="n">
+        <v>4</v>
+      </c>
+      <c r="L249" t="n">
+        <v>2</v>
+      </c>
+      <c r="N249" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="O249" t="n">
+        <v>47.65</v>
+      </c>
+      <c r="P249" t="n">
         <v>0.5790999999999999</v>
       </c>
-      <c r="Q248" t="n">
+      <c r="Q249" t="n">
         <v>0.4288</v>
       </c>
-      <c r="R248" t="n">
+      <c r="R249" t="n">
         <v>0.4927</v>
       </c>
-      <c r="S248" t="n">
+      <c r="S249" t="n">
         <v>-0.0238</v>
       </c>
-      <c r="T248" t="n">
+      <c r="T249" t="n">
         <v>138.3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T248"/>
-  <conditionalFormatting sqref="E2:E248">
+  <autoFilter ref="A1:T249"/>
+  <conditionalFormatting sqref="E2:E249">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -17911,7 +17973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K248"/>
+  <dimension ref="A1:K249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -26200,229 +26262,229 @@
     </row>
     <row r="224">
       <c r="A224" t="n">
-        <v>27</v>
+        <v>248</v>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>-1.3564</v>
+        <v>-1.3385</v>
       </c>
       <c r="D224" t="n">
         <v>1000</v>
       </c>
       <c r="E224" t="n">
-        <v>799.9</v>
+        <v>911.3</v>
       </c>
       <c r="F224" t="n">
-        <v>677.35532</v>
+        <v>840.58312</v>
       </c>
       <c r="G224" t="n">
-        <v>658.660313168</v>
+        <v>827.806256576</v>
       </c>
       <c r="H224" t="n">
-        <v>699.1679224278321</v>
+        <v>733.9330270802817</v>
       </c>
       <c r="I224" t="n">
-        <v>703.2230963779135</v>
+        <v>734.5201735019459</v>
       </c>
       <c r="J224" t="n">
-        <v>1025.22895220936</v>
+        <v>615.0137412731793</v>
       </c>
       <c r="K224" t="n">
-        <v>827.3597644329536</v>
+        <v>445.4544528041637</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
-        <v>108</v>
+        <v>27</v>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>-1.4054</v>
+        <v>-1.3564</v>
       </c>
       <c r="D225" t="n">
         <v>1000</v>
       </c>
       <c r="E225" t="n">
-        <v>951.8</v>
+        <v>799.9</v>
       </c>
       <c r="F225" t="n">
-        <v>762.2014399999999</v>
+        <v>677.35532</v>
       </c>
       <c r="G225" t="n">
-        <v>716.4693535999999</v>
+        <v>658.660313168</v>
       </c>
       <c r="H225" t="n">
-        <v>909.7727852012798</v>
+        <v>699.1679224278321</v>
       </c>
       <c r="I225" t="n">
-        <v>665.9536787673368</v>
+        <v>703.2230963779135</v>
       </c>
       <c r="J225" t="n">
-        <v>657.0298994718545</v>
+        <v>1025.22895220936</v>
       </c>
       <c r="K225" t="n">
-        <v>501.3795162869721</v>
+        <v>827.3597644329536</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
-        <v>247</v>
+        <v>108</v>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>xlstm</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>-1.4181</v>
+        <v>-1.4054</v>
       </c>
       <c r="D226" t="n">
         <v>1000</v>
       </c>
       <c r="E226" t="n">
-        <v>1092.5</v>
+        <v>951.8</v>
       </c>
       <c r="F226" t="n">
-        <v>846.9059999999999</v>
+        <v>762.2014399999999</v>
       </c>
       <c r="G226" t="n">
-        <v>824.3783003999999</v>
+        <v>716.4693535999999</v>
       </c>
       <c r="H226" t="n">
-        <v>849.0272115819599</v>
+        <v>909.7727852012798</v>
       </c>
       <c r="I226" t="n">
-        <v>607.8185807715251</v>
+        <v>665.9536787673368</v>
       </c>
       <c r="J226" t="n">
-        <v>416.7812008350348</v>
+        <v>657.0298994718545</v>
       </c>
       <c r="K226" t="n">
-        <v>375.9783212732849</v>
+        <v>501.3795162869721</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>110</v>
+        <v>247</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>patchtst</t>
+          <t>xlstm</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>-1.4189</v>
+        <v>-1.4181</v>
       </c>
       <c r="D227" t="n">
         <v>1000</v>
       </c>
       <c r="E227" t="n">
-        <v>942</v>
+        <v>1092.5</v>
       </c>
       <c r="F227" t="n">
-        <v>730.2384</v>
+        <v>846.9059999999999</v>
       </c>
       <c r="G227" t="n">
-        <v>637.6441708799999</v>
+        <v>824.3783003999999</v>
       </c>
       <c r="H227" t="n">
-        <v>706.8923278375679</v>
+        <v>849.0272115819599</v>
       </c>
       <c r="I227" t="n">
-        <v>605.0291433961744</v>
+        <v>607.8185807715251</v>
       </c>
       <c r="J227" t="n">
-        <v>435.9234978169437</v>
+        <v>416.7812008350348</v>
       </c>
       <c r="K227" t="n">
-        <v>412.9503294819908</v>
+        <v>375.9783212732849</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>195</v>
+        <v>110</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtst</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>-1.4304</v>
+        <v>-1.4189</v>
       </c>
       <c r="D228" t="n">
         <v>1000</v>
       </c>
       <c r="E228" t="n">
-        <v>999.6</v>
+        <v>942</v>
       </c>
       <c r="F228" t="n">
-        <v>1076.66916</v>
+        <v>730.2384</v>
       </c>
       <c r="G228" t="n">
-        <v>1127.918612016</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H228" t="n">
-        <v>1009.261574031917</v>
+        <v>706.8923278375679</v>
       </c>
       <c r="I228" t="n">
-        <v>837.9898849187007</v>
+        <v>605.0291433961744</v>
       </c>
       <c r="J228" t="n">
-        <v>1032.403538219839</v>
+        <v>435.9234978169437</v>
       </c>
       <c r="K228" t="n">
-        <v>1101.161613865281</v>
+        <v>412.9503294819908</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>144</v>
+        <v>195</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>nbeats</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>-1.4305</v>
+        <v>-1.4304</v>
       </c>
       <c r="D229" t="n">
         <v>1000</v>
       </c>
       <c r="E229" t="n">
-        <v>1045.3</v>
+        <v>999.6</v>
       </c>
       <c r="F229" t="n">
-        <v>853.06933</v>
+        <v>1076.66916</v>
       </c>
       <c r="G229" t="n">
-        <v>749.933248003</v>
+        <v>1127.918612016</v>
       </c>
       <c r="H229" t="n">
-        <v>740.3341024285616</v>
+        <v>1009.261574031917</v>
       </c>
       <c r="I229" t="n">
-        <v>691.1759180273051</v>
+        <v>837.9898849187007</v>
       </c>
       <c r="J229" t="n">
-        <v>482.7172611502699</v>
+        <v>1032.403538219839</v>
       </c>
       <c r="K229" t="n">
-        <v>325.0618036585918</v>
+        <v>1101.161613865281</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>196</v>
+        <v>144</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
@@ -26459,118 +26521,118 @@
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>35</v>
+        <v>196</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>lstm</t>
+          <t>nbeats</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>-1.4347</v>
+        <v>-1.4305</v>
       </c>
       <c r="D231" t="n">
         <v>1000</v>
       </c>
       <c r="E231" t="n">
-        <v>743.8000000000001</v>
+        <v>1045.3</v>
       </c>
       <c r="F231" t="n">
-        <v>692.62656</v>
+        <v>853.06933</v>
       </c>
       <c r="G231" t="n">
-        <v>666.7223266560001</v>
+        <v>749.933248003</v>
       </c>
       <c r="H231" t="n">
-        <v>724.7938413077377</v>
+        <v>740.3341024285616</v>
       </c>
       <c r="I231" t="n">
-        <v>681.3786902134042</v>
+        <v>691.1759180273051</v>
       </c>
       <c r="J231" t="n">
-        <v>441.2608397822005</v>
+        <v>482.7172611502699</v>
       </c>
       <c r="K231" t="n">
-        <v>291.4527846761434</v>
+        <v>325.0618036585918</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>170</v>
+        <v>35</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>lstm</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>-1.4536</v>
+        <v>-1.4347</v>
       </c>
       <c r="D232" t="n">
         <v>1000</v>
       </c>
       <c r="E232" t="n">
-        <v>1236.4</v>
+        <v>743.8000000000001</v>
       </c>
       <c r="F232" t="n">
-        <v>1500.74232</v>
+        <v>692.62656</v>
       </c>
       <c r="G232" t="n">
-        <v>1734.708047688</v>
+        <v>666.7223266560001</v>
       </c>
       <c r="H232" t="n">
-        <v>1677.809623723833</v>
+        <v>724.7938413077377</v>
       </c>
       <c r="I232" t="n">
-        <v>1544.088196713044</v>
+        <v>681.3786902134042</v>
       </c>
       <c r="J232" t="n">
-        <v>1750.069562154564</v>
+        <v>441.2608397822005</v>
       </c>
       <c r="K232" t="n">
-        <v>1412.131129702517</v>
+        <v>291.4527846761434</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>7</v>
+        <v>170</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>-1.5001</v>
+        <v>-1.4536</v>
       </c>
       <c r="D233" t="n">
         <v>1000</v>
       </c>
       <c r="E233" t="n">
-        <v>969.0999999999999</v>
+        <v>1236.4</v>
       </c>
       <c r="F233" t="n">
-        <v>872.5776399999999</v>
+        <v>1500.74232</v>
       </c>
       <c r="G233" t="n">
-        <v>1116.724863672</v>
+        <v>1734.708047688</v>
       </c>
       <c r="H233" t="n">
-        <v>1199.809193529197</v>
+        <v>1677.809623723833</v>
       </c>
       <c r="I233" t="n">
-        <v>1246.001847480071</v>
+        <v>1544.088196713044</v>
       </c>
       <c r="J233" t="n">
-        <v>1151.804107810577</v>
+        <v>1750.069562154564</v>
       </c>
       <c r="K233" t="n">
-        <v>772.5150151085543</v>
+        <v>1412.131129702517</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
@@ -26578,36 +26640,36 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>-1.5008</v>
+        <v>-1.5001</v>
       </c>
       <c r="D234" t="n">
         <v>1000</v>
       </c>
       <c r="E234" t="n">
-        <v>875.8000000000001</v>
+        <v>969.0999999999999</v>
       </c>
       <c r="F234" t="n">
-        <v>762.9093800000001</v>
+        <v>872.5776399999999</v>
       </c>
       <c r="G234" t="n">
-        <v>793.883500828</v>
+        <v>1116.724863672</v>
       </c>
       <c r="H234" t="n">
-        <v>753.6336073360204</v>
+        <v>1199.809193529197</v>
       </c>
       <c r="I234" t="n">
-        <v>764.9381114460607</v>
+        <v>1246.001847480071</v>
       </c>
       <c r="J234" t="n">
-        <v>525.3594949411546</v>
+        <v>1151.804107810577</v>
       </c>
       <c r="K234" t="n">
-        <v>380.9381697818312</v>
+        <v>772.5150151085543</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
@@ -26615,36 +26677,36 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>-1.5094</v>
+        <v>-1.5008</v>
       </c>
       <c r="D235" t="n">
         <v>1000</v>
       </c>
       <c r="E235" t="n">
-        <v>929.4</v>
+        <v>875.8000000000001</v>
       </c>
       <c r="F235" t="n">
-        <v>792.49938</v>
+        <v>762.9093800000001</v>
       </c>
       <c r="G235" t="n">
-        <v>743.681418192</v>
+        <v>793.883500828</v>
       </c>
       <c r="H235" t="n">
-        <v>625.8079134085681</v>
+        <v>753.6336073360204</v>
       </c>
       <c r="I235" t="n">
-        <v>559.0967898392147</v>
+        <v>764.9381114460607</v>
       </c>
       <c r="J235" t="n">
-        <v>584.8711518508026</v>
+        <v>525.3594949411546</v>
       </c>
       <c r="K235" t="n">
-        <v>372.4459494985911</v>
+        <v>380.9381697818312</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
@@ -26652,147 +26714,147 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>-1.5134</v>
+        <v>-1.5094</v>
       </c>
       <c r="D236" t="n">
         <v>1000</v>
       </c>
       <c r="E236" t="n">
-        <v>892.7</v>
+        <v>929.4</v>
       </c>
       <c r="F236" t="n">
-        <v>712.64241</v>
+        <v>792.49938</v>
       </c>
       <c r="G236" t="n">
-        <v>685.8470553840001</v>
+        <v>743.681418192</v>
       </c>
       <c r="H236" t="n">
-        <v>634.4771109357386</v>
+        <v>625.8079134085681</v>
       </c>
       <c r="I236" t="n">
-        <v>652.43281317522</v>
+        <v>559.0967898392147</v>
       </c>
       <c r="J236" t="n">
-        <v>434.5202535746965</v>
+        <v>584.8711518508026</v>
       </c>
       <c r="K236" t="n">
-        <v>370.5154202231437</v>
+        <v>372.4459494985911</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>157</v>
+        <v>59</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>mamba</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>-1.5225</v>
+        <v>-1.5134</v>
       </c>
       <c r="D237" t="n">
         <v>1000</v>
       </c>
       <c r="E237" t="n">
-        <v>1141.5</v>
+        <v>892.7</v>
       </c>
       <c r="F237" t="n">
-        <v>884.8908</v>
+        <v>712.64241</v>
       </c>
       <c r="G237" t="n">
-        <v>789.49957176</v>
+        <v>685.8470553840001</v>
       </c>
       <c r="H237" t="n">
-        <v>805.7632629382559</v>
+        <v>634.4771109357386</v>
       </c>
       <c r="I237" t="n">
-        <v>674.1015457741449</v>
+        <v>652.43281317522</v>
       </c>
       <c r="J237" t="n">
-        <v>457.9171800443767</v>
+        <v>434.5202535746965</v>
       </c>
       <c r="K237" t="n">
-        <v>340.3698399269852</v>
+        <v>370.5154202231437</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>mamba</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>-1.5246</v>
+        <v>-1.5225</v>
       </c>
       <c r="D238" t="n">
         <v>1000</v>
       </c>
       <c r="E238" t="n">
-        <v>1127.9</v>
+        <v>1141.5</v>
       </c>
       <c r="F238" t="n">
-        <v>1108.7257</v>
+        <v>884.8908</v>
       </c>
       <c r="G238" t="n">
-        <v>1251.64044273</v>
+        <v>789.49957176</v>
       </c>
       <c r="H238" t="n">
-        <v>1235.619445063056</v>
+        <v>805.7632629382559</v>
       </c>
       <c r="I238" t="n">
-        <v>1202.010596157341</v>
+        <v>674.1015457741449</v>
       </c>
       <c r="J238" t="n">
-        <v>1559.849150633381</v>
+        <v>457.9171800443767</v>
       </c>
       <c r="K238" t="n">
-        <v>2161.015013287486</v>
+        <v>340.3698399269852</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>1</v>
+        <v>193</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>-1.5423</v>
+        <v>-1.5246</v>
       </c>
       <c r="D239" t="n">
         <v>1000</v>
       </c>
       <c r="E239" t="n">
-        <v>1342</v>
+        <v>1127.9</v>
       </c>
       <c r="F239" t="n">
-        <v>1365.6192</v>
+        <v>1108.7257</v>
       </c>
       <c r="G239" t="n">
-        <v>1401.67154688</v>
+        <v>1251.64044273</v>
       </c>
       <c r="H239" t="n">
-        <v>1356.1172216064</v>
+        <v>1235.619445063056</v>
       </c>
       <c r="I239" t="n">
-        <v>1614.321940600259</v>
+        <v>1202.010596157341</v>
       </c>
       <c r="J239" t="n">
-        <v>1682.93062307577</v>
+        <v>1559.849150633381</v>
       </c>
       <c r="K239" t="n">
-        <v>1547.623000980478</v>
+        <v>2161.015013287486</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
@@ -26829,266 +26891,266 @@
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>220</v>
+        <v>39</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>-1.6978</v>
+        <v>-1.5423</v>
       </c>
       <c r="D241" t="n">
         <v>1000</v>
       </c>
       <c r="E241" t="n">
-        <v>901.6999999999999</v>
+        <v>1342</v>
       </c>
       <c r="F241" t="n">
-        <v>774.1094499999999</v>
+        <v>1365.6192</v>
       </c>
       <c r="G241" t="n">
-        <v>749.570180435</v>
+        <v>1401.67154688</v>
       </c>
       <c r="H241" t="n">
-        <v>634.3612437021405</v>
+        <v>1356.1172216064</v>
       </c>
       <c r="I241" t="n">
-        <v>618.502212609587</v>
+        <v>1614.321940600259</v>
       </c>
       <c r="J241" t="n">
-        <v>338.3207102974441</v>
+        <v>1682.93062307577</v>
       </c>
       <c r="K241" t="n">
-        <v>264.9389482339285</v>
+        <v>1547.623000980478</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>14</v>
+        <v>220</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>catboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>-1.7077</v>
+        <v>-1.6978</v>
       </c>
       <c r="D242" t="n">
         <v>1000</v>
       </c>
       <c r="E242" t="n">
-        <v>1067.7</v>
+        <v>901.6999999999999</v>
       </c>
       <c r="F242" t="n">
-        <v>1380.10902</v>
+        <v>774.1094499999999</v>
       </c>
       <c r="G242" t="n">
-        <v>1542.409840752</v>
+        <v>749.570180435</v>
       </c>
       <c r="H242" t="n">
-        <v>1525.751814471878</v>
+        <v>634.3612437021405</v>
       </c>
       <c r="I242" t="n">
-        <v>1571.066643361693</v>
+        <v>618.502212609587</v>
       </c>
       <c r="J242" t="n">
-        <v>1715.918987879641</v>
+        <v>338.3207102974441</v>
       </c>
       <c r="K242" t="n">
-        <v>1440.513990324959</v>
+        <v>264.9389482339285</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>catboost</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>-1.7766</v>
+        <v>-1.7077</v>
       </c>
       <c r="D243" t="n">
         <v>1000</v>
       </c>
       <c r="E243" t="n">
-        <v>1165.9</v>
+        <v>1067.7</v>
       </c>
       <c r="F243" t="n">
-        <v>1389.63621</v>
+        <v>1380.10902</v>
       </c>
       <c r="G243" t="n">
-        <v>1502.613633873</v>
+        <v>1542.409840752</v>
       </c>
       <c r="H243" t="n">
-        <v>1405.244270398029</v>
+        <v>1525.751814471878</v>
       </c>
       <c r="I243" t="n">
-        <v>1637.531148294824</v>
+        <v>1571.066643361693</v>
       </c>
       <c r="J243" t="n">
-        <v>1327.382748807784</v>
+        <v>1715.918987879641</v>
       </c>
       <c r="K243" t="n">
-        <v>1186.94565398392</v>
+        <v>1440.513990324959</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>146</v>
+        <v>22</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>patchtsmixer</t>
+          <t>xgboost</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>-1.8201</v>
+        <v>-1.7766</v>
       </c>
       <c r="D244" t="n">
         <v>1000</v>
       </c>
       <c r="E244" t="n">
-        <v>942</v>
+        <v>1165.9</v>
       </c>
       <c r="F244" t="n">
-        <v>730.2384</v>
+        <v>1389.63621</v>
       </c>
       <c r="G244" t="n">
-        <v>637.6441708799999</v>
+        <v>1502.613633873</v>
       </c>
       <c r="H244" t="n">
-        <v>677.6882248112639</v>
+        <v>1405.244270398029</v>
       </c>
       <c r="I244" t="n">
-        <v>580.0333516159608</v>
+        <v>1637.531148294824</v>
       </c>
       <c r="J244" t="n">
-        <v>381.8939587039486</v>
+        <v>1327.382748807784</v>
       </c>
       <c r="K244" t="n">
-        <v>282.3723930656996</v>
+        <v>1186.94565398392</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>194</v>
+        <v>146</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>itransformer</t>
+          <t>patchtsmixer</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>-2.0173</v>
+        <v>-1.8201</v>
       </c>
       <c r="D245" t="n">
         <v>1000</v>
       </c>
       <c r="E245" t="n">
-        <v>1222.6</v>
+        <v>942</v>
       </c>
       <c r="F245" t="n">
-        <v>1122.46906</v>
+        <v>730.2384</v>
       </c>
       <c r="G245" t="n">
-        <v>1222.481053246</v>
+        <v>637.6441708799999</v>
       </c>
       <c r="H245" t="n">
-        <v>1198.520424602378</v>
+        <v>677.6882248112639</v>
       </c>
       <c r="I245" t="n">
-        <v>1133.440765546469</v>
+        <v>580.0333516159608</v>
       </c>
       <c r="J245" t="n">
-        <v>1142.73497982395</v>
+        <v>381.8939587039486</v>
       </c>
       <c r="K245" t="n">
-        <v>813.6273056346525</v>
+        <v>282.3723930656996</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>158</v>
+        <v>194</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>mlp</t>
+          <t>itransformer</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>-2.2082</v>
+        <v>-2.0173</v>
       </c>
       <c r="D246" t="n">
         <v>1000</v>
       </c>
       <c r="E246" t="n">
-        <v>1000.2</v>
+        <v>1222.6</v>
       </c>
       <c r="F246" t="n">
-        <v>765.0529799999999</v>
+        <v>1122.46906</v>
       </c>
       <c r="G246" t="n">
-        <v>773.1625415879998</v>
+        <v>1222.481053246</v>
       </c>
       <c r="H246" t="n">
-        <v>742.158723670321</v>
+        <v>1198.520424602378</v>
       </c>
       <c r="I246" t="n">
-        <v>765.9078028277713</v>
+        <v>1133.440765546469</v>
       </c>
       <c r="J246" t="n">
-        <v>571.2906301292346</v>
+        <v>1142.73497982395</v>
       </c>
       <c r="K246" t="n">
-        <v>485.5970356098494</v>
+        <v>813.6273056346525</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>2</v>
+        <v>158</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>xgboost</t>
+          <t>mlp</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>-2.3923</v>
+        <v>-2.2082</v>
       </c>
       <c r="D247" t="n">
         <v>1000</v>
       </c>
       <c r="E247" t="n">
-        <v>982.1</v>
+        <v>1000.2</v>
       </c>
       <c r="F247" t="n">
-        <v>1102.11262</v>
+        <v>765.0529799999999</v>
       </c>
       <c r="G247" t="n">
-        <v>1215.07916355</v>
+        <v>773.1625415879998</v>
       </c>
       <c r="H247" t="n">
-        <v>1137.07108125009</v>
+        <v>742.158723670321</v>
       </c>
       <c r="I247" t="n">
-        <v>1227.127110885097</v>
+        <v>765.9078028277713</v>
       </c>
       <c r="J247" t="n">
-        <v>1233.5081718617</v>
+        <v>571.2906301292346</v>
       </c>
       <c r="K247" t="n">
-        <v>894.5401262341047</v>
+        <v>485.5970356098494</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
@@ -27096,30 +27158,67 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>-2.6905</v>
+        <v>-2.3923</v>
       </c>
       <c r="D248" t="n">
         <v>1000</v>
       </c>
       <c r="E248" t="n">
+        <v>982.1</v>
+      </c>
+      <c r="F248" t="n">
+        <v>1102.11262</v>
+      </c>
+      <c r="G248" t="n">
+        <v>1215.07916355</v>
+      </c>
+      <c r="H248" t="n">
+        <v>1137.07108125009</v>
+      </c>
+      <c r="I248" t="n">
+        <v>1227.127110885097</v>
+      </c>
+      <c r="J248" t="n">
+        <v>1233.5081718617</v>
+      </c>
+      <c r="K248" t="n">
+        <v>894.5401262341047</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>41</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>xgboost</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>-2.6905</v>
+      </c>
+      <c r="D249" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E249" t="n">
         <v>1067.8</v>
       </c>
-      <c r="F248" t="n">
+      <c r="F249" t="n">
         <v>1221.5632</v>
       </c>
-      <c r="G248" t="n">
+      <c r="G249" t="n">
         <v>1298.76599424</v>
       </c>
-      <c r="H248" t="n">
+      <c r="H249" t="n">
         <v>1152.784696487424</v>
       </c>
-      <c r="I248" t="n">
+      <c r="I249" t="n">
         <v>1298.381403653786</v>
       </c>
-      <c r="J248" t="n">
+      <c r="J249" t="n">
         <v>1191.264937852349</v>
       </c>
-      <c r="K248" t="n">
+      <c r="K249" t="n">
         <v>825.3083489441071</v>
       </c>
     </row>

</xml_diff>